<commit_message>
Named, specialised upgrade paths (UPGRADES.md)
UPGRADES.md is the approved vision: every tower's three paths specialise
(attack speed, anti-armour, support, control, economy) and all 75 tiers have
their own names, with ability tiers and the phase that builds each mechanic.

- Spreadsheet: Scout paths renamed Lookout / Trigger Happy / Hardliner,
  Sniper Pierce -> Deadeye; new Name column on Tower Upgrades.
- Exporter reads names and refuses a tier without one.
- Tower panel shows the tier name, path and real stat change.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Storm-Split-Balance.xlsx
+++ b/Storm-Split-Balance.xlsx
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="376">
   <si>
     <t>STORM SPLIT — Balance Model</t>
   </si>
@@ -454,7 +454,7 @@
     <t>TOWER UPGRADES — 5 towers x 3 paths x 5 tiers</t>
   </si>
   <si>
-    <t>Multipliers are blue because they define each path's character. Costs are formulas off Tuning. Range x multiplies the tower's base range (range-focus paths only).</t>
+    <t>Multipliers are blue because they define each path's character. Costs are formulas off Tuning. Range x multiplies the tower's base range (range-focus paths only). Name is the tier's in-game name (full design: UPGRADES.md).</t>
   </si>
   <si>
     <t>Path</t>
@@ -490,51 +490,234 @@
     <t>Range x</t>
   </si>
   <si>
-    <t>Range</t>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Lookout</t>
   </si>
   <si>
     <t>range</t>
   </si>
   <si>
-    <t>Rate</t>
+    <t>Keen Eyes</t>
+  </si>
+  <si>
+    <t>Long Barrel</t>
+  </si>
+  <si>
+    <t>Flare Gun</t>
+  </si>
+  <si>
+    <t>Watch Post</t>
+  </si>
+  <si>
+    <t>Signal Tower</t>
+  </si>
+  <si>
+    <t>Trigger Happy</t>
   </si>
   <si>
     <t>rate</t>
   </si>
   <si>
+    <t>Quick Hands</t>
+  </si>
+  <si>
+    <t>Extended Mag</t>
+  </si>
+  <si>
+    <t>Double Tap</t>
+  </si>
+  <si>
+    <t>Bullet Hose</t>
+  </si>
+  <si>
+    <t>Stormgunner</t>
+  </si>
+  <si>
+    <t>Hardliner</t>
+  </si>
+  <si>
     <t>damage</t>
   </si>
   <si>
-    <t>Pierce</t>
+    <t>Heavy Slugs</t>
+  </si>
+  <si>
+    <t>Armor Breaker</t>
+  </si>
+  <si>
+    <t>Hollow Points</t>
+  </si>
+  <si>
+    <t>Railshot</t>
+  </si>
+  <si>
+    <t>Tank Buster</t>
+  </si>
+  <si>
+    <t>Deadeye</t>
   </si>
   <si>
     <t>targets</t>
   </si>
   <si>
+    <t>Full Metal Jacket</t>
+  </si>
+  <si>
+    <t>Through-and-Through</t>
+  </si>
+  <si>
+    <t>Ricochet</t>
+  </si>
+  <si>
+    <t>Tungsten Core</t>
+  </si>
+  <si>
+    <t>Linebreaker</t>
+  </si>
+  <si>
     <t>Spotter</t>
   </si>
   <si>
+    <t>Steady Breath</t>
+  </si>
+  <si>
+    <t>Bolt Racking</t>
+  </si>
+  <si>
+    <t>Marked Target</t>
+  </si>
+  <si>
+    <t>Tactical Spotter</t>
+  </si>
+  <si>
+    <t>Eye in the Sky</t>
+  </si>
+  <si>
     <t>Siege</t>
   </si>
   <si>
+    <t>Large Calibre</t>
+  </si>
+  <si>
+    <t>Anti-Materiel</t>
+  </si>
+  <si>
+    <t>Concussion Round</t>
+  </si>
+  <si>
+    <t>Siege Gun</t>
+  </si>
+  <si>
+    <t>Skybreaker</t>
+  </si>
+  <si>
     <t>Blast</t>
   </si>
   <si>
+    <t>Bigger Bang</t>
+  </si>
+  <si>
+    <t>Shrapnel</t>
+  </si>
+  <si>
+    <t>Napalm</t>
+  </si>
+  <si>
+    <t>Firestorm</t>
+  </si>
+  <si>
+    <t>Scorched Earth</t>
+  </si>
+  <si>
     <t>Cluster</t>
   </si>
   <si>
+    <t>Cluster Shell</t>
+  </si>
+  <si>
+    <t>Rapid Loader</t>
+  </si>
+  <si>
+    <t>Chain Reaction</t>
+  </si>
+  <si>
+    <t>Carpet Shelling</t>
+  </si>
+  <si>
+    <t>Storm of Steel</t>
+  </si>
+  <si>
     <t>Concussive</t>
   </si>
   <si>
+    <t>Shockwave</t>
+  </si>
+  <si>
+    <t>Armor Crack</t>
+  </si>
+  <si>
+    <t>Stun Grenade</t>
+  </si>
+  <si>
+    <t>Earthshaker</t>
+  </si>
+  <si>
+    <t>Tectonic Slam</t>
+  </si>
+  <si>
     <t>Field</t>
   </si>
   <si>
+    <t>Cold Snap</t>
+  </si>
+  <si>
+    <t>Frostbite</t>
+  </si>
+  <si>
+    <t>Permafrost</t>
+  </si>
+  <si>
+    <t>Glacier Zone</t>
+  </si>
+  <si>
+    <t>Absolute Zero</t>
+  </si>
+  <si>
     <t>Freeze</t>
   </si>
   <si>
+    <t>Flash Freeze</t>
+  </si>
+  <si>
+    <t>Deep Freeze</t>
+  </si>
+  <si>
+    <t>Ice Shards</t>
+  </si>
+  <si>
+    <t>Cryo Pulse</t>
+  </si>
+  <si>
+    <t>Stasis</t>
+  </si>
+  <si>
     <t>Brittle</t>
   </si>
   <si>
+    <t>Shatter</t>
+  </si>
+  <si>
+    <t>Cold Front</t>
+  </si>
+  <si>
+    <t>Frozen Core</t>
+  </si>
+  <si>
+    <t>Winter's Edge</t>
+  </si>
+  <si>
     <t>Yield</t>
   </si>
   <si>
@@ -544,10 +727,55 @@
     <t>n/a</t>
   </si>
   <si>
+    <t>Supply Crate</t>
+  </si>
+  <si>
+    <t>Bigger Budget</t>
+  </si>
+  <si>
+    <t>Trade Route</t>
+  </si>
+  <si>
+    <t>War Chest</t>
+  </si>
+  <si>
+    <t>Storm Bank</t>
+  </si>
+  <si>
     <t>Airdrop</t>
   </si>
   <si>
+    <t>Air Drop</t>
+  </si>
+  <si>
+    <t>Double Drop</t>
+  </si>
+  <si>
+    <t>Care Package</t>
+  </si>
+  <si>
+    <t>Supply Chain</t>
+  </si>
+  <si>
+    <t>Treasure Barge</t>
+  </si>
+  <si>
     <t>Logistics</t>
+  </si>
+  <si>
+    <t>Bulk Order</t>
+  </si>
+  <si>
+    <t>Field Engineer</t>
+  </si>
+  <si>
+    <t>Recycler</t>
+  </si>
+  <si>
+    <t>Forward Base</t>
+  </si>
+  <si>
+    <t>Command Center</t>
   </si>
   <si>
     <t>PLAYER WEAPONS — in-round track</t>
@@ -3745,7 +3973,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:L79"/>
+  <dimension ref="A1:M79"/>
   <sheetFormatPr defaultColWidth="8.66667" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="15" style="49" customWidth="1"/>
@@ -3760,7 +3988,8 @@
     <col min="10" max="10" width="13" style="49" customWidth="1"/>
     <col min="11" max="11" width="12" style="49" customWidth="1"/>
     <col min="12" max="12" width="10" style="49" customWidth="1"/>
-    <col min="13" max="16384" width="8.67188" style="49" customWidth="1"/>
+    <col min="13" max="13" width="22" style="49" customWidth="1"/>
+    <col min="14" max="16384" width="8.67188" style="49" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.5" customHeight="1">
@@ -3778,6 +4007,7 @@
       <c r="J1" s="3"/>
       <c r="K1" s="4"/>
       <c r="L1" s="50"/>
+      <c r="M1" s="50"/>
     </row>
     <row r="2" ht="13.65" customHeight="1">
       <c r="A2" t="s" s="5">
@@ -3794,6 +4024,7 @@
       <c r="J2" s="6"/>
       <c r="K2" s="7"/>
       <c r="L2" s="51"/>
+      <c r="M2" s="51"/>
     </row>
     <row r="3" ht="13.55" customHeight="1">
       <c r="A3" s="19"/>
@@ -3808,6 +4039,7 @@
       <c r="J3" s="20"/>
       <c r="K3" s="37"/>
       <c r="L3" s="52"/>
+      <c r="M3" s="52"/>
     </row>
     <row r="4" ht="27.75" customHeight="1">
       <c r="A4" t="s" s="21">
@@ -3846,16 +4078,19 @@
       <c r="L4" t="s" s="21">
         <v>148</v>
       </c>
+      <c r="M4" t="s" s="21">
+        <v>149</v>
+      </c>
     </row>
     <row r="5" ht="13.65" customHeight="1">
       <c r="A5" t="s" s="38">
         <v>117</v>
       </c>
       <c r="B5" t="s" s="38">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C5" t="s" s="38">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D5" s="53">
         <v>1</v>
@@ -3888,16 +4123,19 @@
       <c r="L5" s="54">
         <v>1.15</v>
       </c>
+      <c r="M5" t="s" s="38">
+        <v>152</v>
+      </c>
     </row>
     <row r="6" ht="13.65" customHeight="1">
       <c r="A6" t="s" s="38">
         <v>117</v>
       </c>
       <c r="B6" t="s" s="38">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C6" t="s" s="38">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D6" s="53">
         <v>2</v>
@@ -3930,16 +4168,19 @@
       <c r="L6" s="54">
         <v>1.3</v>
       </c>
+      <c r="M6" t="s" s="38">
+        <v>153</v>
+      </c>
     </row>
     <row r="7" ht="13.65" customHeight="1">
       <c r="A7" t="s" s="38">
         <v>117</v>
       </c>
       <c r="B7" t="s" s="38">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C7" t="s" s="38">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D7" s="53">
         <v>3</v>
@@ -3972,16 +4213,19 @@
       <c r="L7" s="54">
         <v>1.5</v>
       </c>
+      <c r="M7" t="s" s="38">
+        <v>154</v>
+      </c>
     </row>
     <row r="8" ht="13.65" customHeight="1">
       <c r="A8" t="s" s="38">
         <v>117</v>
       </c>
       <c r="B8" t="s" s="38">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C8" t="s" s="38">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D8" s="53">
         <v>4</v>
@@ -4014,16 +4258,19 @@
       <c r="L8" s="54">
         <v>1.75</v>
       </c>
+      <c r="M8" t="s" s="38">
+        <v>155</v>
+      </c>
     </row>
     <row r="9" ht="13.65" customHeight="1">
       <c r="A9" t="s" s="38">
         <v>117</v>
       </c>
       <c r="B9" t="s" s="38">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C9" t="s" s="38">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D9" s="53">
         <v>5</v>
@@ -4056,16 +4303,19 @@
       <c r="L9" s="54">
         <v>2</v>
       </c>
+      <c r="M9" t="s" s="38">
+        <v>156</v>
+      </c>
     </row>
     <row r="10" ht="13.65" customHeight="1">
       <c r="A10" t="s" s="38">
         <v>117</v>
       </c>
       <c r="B10" t="s" s="38">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="C10" t="s" s="38">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="D10" s="53">
         <v>1</v>
@@ -4098,16 +4348,19 @@
       <c r="L10" s="54">
         <v>1</v>
       </c>
+      <c r="M10" t="s" s="38">
+        <v>159</v>
+      </c>
     </row>
     <row r="11" ht="13.65" customHeight="1">
       <c r="A11" t="s" s="38">
         <v>117</v>
       </c>
       <c r="B11" t="s" s="38">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="C11" t="s" s="38">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="D11" s="53">
         <v>2</v>
@@ -4140,16 +4393,19 @@
       <c r="L11" s="54">
         <v>1</v>
       </c>
+      <c r="M11" t="s" s="38">
+        <v>160</v>
+      </c>
     </row>
     <row r="12" ht="13.65" customHeight="1">
       <c r="A12" t="s" s="38">
         <v>117</v>
       </c>
       <c r="B12" t="s" s="38">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="C12" t="s" s="38">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="D12" s="53">
         <v>3</v>
@@ -4182,16 +4438,19 @@
       <c r="L12" s="54">
         <v>1</v>
       </c>
+      <c r="M12" t="s" s="38">
+        <v>161</v>
+      </c>
     </row>
     <row r="13" ht="13.65" customHeight="1">
       <c r="A13" t="s" s="38">
         <v>117</v>
       </c>
       <c r="B13" t="s" s="38">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="C13" t="s" s="38">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="D13" s="53">
         <v>4</v>
@@ -4224,16 +4483,19 @@
       <c r="L13" s="54">
         <v>1</v>
       </c>
+      <c r="M13" t="s" s="38">
+        <v>162</v>
+      </c>
     </row>
     <row r="14" ht="13.65" customHeight="1">
       <c r="A14" t="s" s="38">
         <v>117</v>
       </c>
       <c r="B14" t="s" s="38">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="C14" t="s" s="38">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="D14" s="53">
         <v>5</v>
@@ -4266,16 +4528,19 @@
       <c r="L14" s="54">
         <v>1</v>
       </c>
+      <c r="M14" t="s" s="38">
+        <v>163</v>
+      </c>
     </row>
     <row r="15" ht="13.65" customHeight="1">
       <c r="A15" t="s" s="38">
         <v>117</v>
       </c>
       <c r="B15" t="s" s="38">
-        <v>109</v>
+        <v>164</v>
       </c>
       <c r="C15" t="s" s="38">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="D15" s="53">
         <v>1</v>
@@ -4308,16 +4573,19 @@
       <c r="L15" s="54">
         <v>1</v>
       </c>
+      <c r="M15" t="s" s="38">
+        <v>166</v>
+      </c>
     </row>
     <row r="16" ht="13.65" customHeight="1">
       <c r="A16" t="s" s="38">
         <v>117</v>
       </c>
       <c r="B16" t="s" s="38">
-        <v>109</v>
+        <v>164</v>
       </c>
       <c r="C16" t="s" s="38">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="D16" s="53">
         <v>2</v>
@@ -4350,16 +4618,19 @@
       <c r="L16" s="54">
         <v>1</v>
       </c>
+      <c r="M16" t="s" s="38">
+        <v>167</v>
+      </c>
     </row>
     <row r="17" ht="13.65" customHeight="1">
       <c r="A17" t="s" s="38">
         <v>117</v>
       </c>
       <c r="B17" t="s" s="38">
-        <v>109</v>
+        <v>164</v>
       </c>
       <c r="C17" t="s" s="38">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="D17" s="53">
         <v>3</v>
@@ -4392,16 +4663,19 @@
       <c r="L17" s="54">
         <v>1</v>
       </c>
+      <c r="M17" t="s" s="38">
+        <v>168</v>
+      </c>
     </row>
     <row r="18" ht="13.65" customHeight="1">
       <c r="A18" t="s" s="38">
         <v>117</v>
       </c>
       <c r="B18" t="s" s="38">
-        <v>109</v>
+        <v>164</v>
       </c>
       <c r="C18" t="s" s="38">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="D18" s="53">
         <v>4</v>
@@ -4434,16 +4708,19 @@
       <c r="L18" s="54">
         <v>1</v>
       </c>
+      <c r="M18" t="s" s="38">
+        <v>169</v>
+      </c>
     </row>
     <row r="19" ht="13.65" customHeight="1">
       <c r="A19" t="s" s="38">
         <v>117</v>
       </c>
       <c r="B19" t="s" s="38">
-        <v>109</v>
+        <v>164</v>
       </c>
       <c r="C19" t="s" s="38">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="D19" s="53">
         <v>5</v>
@@ -4476,16 +4753,19 @@
       <c r="L19" s="54">
         <v>1</v>
       </c>
+      <c r="M19" t="s" s="38">
+        <v>170</v>
+      </c>
     </row>
     <row r="20" ht="13.65" customHeight="1">
       <c r="A20" t="s" s="38">
         <v>121</v>
       </c>
       <c r="B20" t="s" s="38">
-        <v>154</v>
+        <v>171</v>
       </c>
       <c r="C20" t="s" s="38">
-        <v>155</v>
+        <v>172</v>
       </c>
       <c r="D20" s="53">
         <v>1</v>
@@ -4518,16 +4798,19 @@
       <c r="L20" s="54">
         <v>1</v>
       </c>
+      <c r="M20" t="s" s="38">
+        <v>173</v>
+      </c>
     </row>
     <row r="21" ht="13.65" customHeight="1">
       <c r="A21" t="s" s="38">
         <v>121</v>
       </c>
       <c r="B21" t="s" s="38">
-        <v>154</v>
+        <v>171</v>
       </c>
       <c r="C21" t="s" s="38">
-        <v>155</v>
+        <v>172</v>
       </c>
       <c r="D21" s="53">
         <v>2</v>
@@ -4560,16 +4843,19 @@
       <c r="L21" s="54">
         <v>1</v>
       </c>
+      <c r="M21" t="s" s="38">
+        <v>174</v>
+      </c>
     </row>
     <row r="22" ht="13.65" customHeight="1">
       <c r="A22" t="s" s="38">
         <v>121</v>
       </c>
       <c r="B22" t="s" s="38">
-        <v>154</v>
+        <v>171</v>
       </c>
       <c r="C22" t="s" s="38">
-        <v>155</v>
+        <v>172</v>
       </c>
       <c r="D22" s="53">
         <v>3</v>
@@ -4602,16 +4888,19 @@
       <c r="L22" s="54">
         <v>1</v>
       </c>
+      <c r="M22" t="s" s="38">
+        <v>175</v>
+      </c>
     </row>
     <row r="23" ht="13.65" customHeight="1">
       <c r="A23" t="s" s="38">
         <v>121</v>
       </c>
       <c r="B23" t="s" s="38">
-        <v>154</v>
+        <v>171</v>
       </c>
       <c r="C23" t="s" s="38">
-        <v>155</v>
+        <v>172</v>
       </c>
       <c r="D23" s="53">
         <v>4</v>
@@ -4644,16 +4933,19 @@
       <c r="L23" s="54">
         <v>1</v>
       </c>
+      <c r="M23" t="s" s="38">
+        <v>176</v>
+      </c>
     </row>
     <row r="24" ht="13.65" customHeight="1">
       <c r="A24" t="s" s="38">
         <v>121</v>
       </c>
       <c r="B24" t="s" s="38">
-        <v>154</v>
+        <v>171</v>
       </c>
       <c r="C24" t="s" s="38">
-        <v>155</v>
+        <v>172</v>
       </c>
       <c r="D24" s="53">
         <v>5</v>
@@ -4686,16 +4978,19 @@
       <c r="L24" s="54">
         <v>1</v>
       </c>
+      <c r="M24" t="s" s="38">
+        <v>177</v>
+      </c>
     </row>
     <row r="25" ht="13.65" customHeight="1">
       <c r="A25" t="s" s="38">
         <v>121</v>
       </c>
       <c r="B25" t="s" s="38">
-        <v>156</v>
+        <v>178</v>
       </c>
       <c r="C25" t="s" s="38">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="D25" s="53">
         <v>1</v>
@@ -4728,16 +5023,19 @@
       <c r="L25" s="54">
         <v>1</v>
       </c>
+      <c r="M25" t="s" s="38">
+        <v>179</v>
+      </c>
     </row>
     <row r="26" ht="13.65" customHeight="1">
       <c r="A26" t="s" s="38">
         <v>121</v>
       </c>
       <c r="B26" t="s" s="38">
-        <v>156</v>
+        <v>178</v>
       </c>
       <c r="C26" t="s" s="38">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="D26" s="53">
         <v>2</v>
@@ -4770,16 +5068,19 @@
       <c r="L26" s="54">
         <v>1</v>
       </c>
+      <c r="M26" t="s" s="38">
+        <v>180</v>
+      </c>
     </row>
     <row r="27" ht="13.65" customHeight="1">
       <c r="A27" t="s" s="38">
         <v>121</v>
       </c>
       <c r="B27" t="s" s="38">
-        <v>156</v>
+        <v>178</v>
       </c>
       <c r="C27" t="s" s="38">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="D27" s="53">
         <v>3</v>
@@ -4812,16 +5113,19 @@
       <c r="L27" s="54">
         <v>1</v>
       </c>
+      <c r="M27" t="s" s="38">
+        <v>181</v>
+      </c>
     </row>
     <row r="28" ht="13.65" customHeight="1">
       <c r="A28" t="s" s="38">
         <v>121</v>
       </c>
       <c r="B28" t="s" s="38">
-        <v>156</v>
+        <v>178</v>
       </c>
       <c r="C28" t="s" s="38">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="D28" s="53">
         <v>4</v>
@@ -4854,16 +5158,19 @@
       <c r="L28" s="54">
         <v>1</v>
       </c>
+      <c r="M28" t="s" s="38">
+        <v>182</v>
+      </c>
     </row>
     <row r="29" ht="13.65" customHeight="1">
       <c r="A29" t="s" s="38">
         <v>121</v>
       </c>
       <c r="B29" t="s" s="38">
-        <v>156</v>
+        <v>178</v>
       </c>
       <c r="C29" t="s" s="38">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="D29" s="53">
         <v>5</v>
@@ -4896,16 +5203,19 @@
       <c r="L29" s="54">
         <v>1</v>
       </c>
+      <c r="M29" t="s" s="38">
+        <v>183</v>
+      </c>
     </row>
     <row r="30" ht="13.65" customHeight="1">
       <c r="A30" t="s" s="38">
         <v>121</v>
       </c>
       <c r="B30" t="s" s="38">
-        <v>157</v>
+        <v>184</v>
       </c>
       <c r="C30" t="s" s="38">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="D30" s="53">
         <v>1</v>
@@ -4938,16 +5248,19 @@
       <c r="L30" s="54">
         <v>1</v>
       </c>
+      <c r="M30" t="s" s="38">
+        <v>185</v>
+      </c>
     </row>
     <row r="31" ht="13.65" customHeight="1">
       <c r="A31" t="s" s="38">
         <v>121</v>
       </c>
       <c r="B31" t="s" s="38">
-        <v>157</v>
+        <v>184</v>
       </c>
       <c r="C31" t="s" s="38">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="D31" s="53">
         <v>2</v>
@@ -4980,16 +5293,19 @@
       <c r="L31" s="54">
         <v>1</v>
       </c>
+      <c r="M31" t="s" s="38">
+        <v>186</v>
+      </c>
     </row>
     <row r="32" ht="13.65" customHeight="1">
       <c r="A32" t="s" s="38">
         <v>121</v>
       </c>
       <c r="B32" t="s" s="38">
-        <v>157</v>
+        <v>184</v>
       </c>
       <c r="C32" t="s" s="38">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="D32" s="53">
         <v>3</v>
@@ -5022,16 +5338,19 @@
       <c r="L32" s="54">
         <v>1</v>
       </c>
+      <c r="M32" t="s" s="38">
+        <v>187</v>
+      </c>
     </row>
     <row r="33" ht="13.65" customHeight="1">
       <c r="A33" t="s" s="38">
         <v>121</v>
       </c>
       <c r="B33" t="s" s="38">
-        <v>157</v>
+        <v>184</v>
       </c>
       <c r="C33" t="s" s="38">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="D33" s="53">
         <v>4</v>
@@ -5064,16 +5383,19 @@
       <c r="L33" s="54">
         <v>1</v>
       </c>
+      <c r="M33" t="s" s="38">
+        <v>188</v>
+      </c>
     </row>
     <row r="34" ht="13.65" customHeight="1">
       <c r="A34" t="s" s="38">
         <v>121</v>
       </c>
       <c r="B34" t="s" s="38">
-        <v>157</v>
+        <v>184</v>
       </c>
       <c r="C34" t="s" s="38">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="D34" s="53">
         <v>5</v>
@@ -5106,16 +5428,19 @@
       <c r="L34" s="54">
         <v>1</v>
       </c>
+      <c r="M34" t="s" s="38">
+        <v>189</v>
+      </c>
     </row>
     <row r="35" ht="13.65" customHeight="1">
       <c r="A35" t="s" s="38">
         <v>124</v>
       </c>
       <c r="B35" t="s" s="38">
-        <v>158</v>
+        <v>190</v>
       </c>
       <c r="C35" t="s" s="38">
-        <v>155</v>
+        <v>172</v>
       </c>
       <c r="D35" s="53">
         <v>1</v>
@@ -5148,16 +5473,19 @@
       <c r="L35" s="54">
         <v>1</v>
       </c>
+      <c r="M35" t="s" s="38">
+        <v>191</v>
+      </c>
     </row>
     <row r="36" ht="13.65" customHeight="1">
       <c r="A36" t="s" s="38">
         <v>124</v>
       </c>
       <c r="B36" t="s" s="38">
-        <v>158</v>
+        <v>190</v>
       </c>
       <c r="C36" t="s" s="38">
-        <v>155</v>
+        <v>172</v>
       </c>
       <c r="D36" s="53">
         <v>2</v>
@@ -5190,16 +5518,19 @@
       <c r="L36" s="54">
         <v>1</v>
       </c>
+      <c r="M36" t="s" s="38">
+        <v>192</v>
+      </c>
     </row>
     <row r="37" ht="13.65" customHeight="1">
       <c r="A37" t="s" s="38">
         <v>124</v>
       </c>
       <c r="B37" t="s" s="38">
-        <v>158</v>
+        <v>190</v>
       </c>
       <c r="C37" t="s" s="38">
-        <v>155</v>
+        <v>172</v>
       </c>
       <c r="D37" s="53">
         <v>3</v>
@@ -5232,16 +5563,19 @@
       <c r="L37" s="54">
         <v>1</v>
       </c>
+      <c r="M37" t="s" s="38">
+        <v>193</v>
+      </c>
     </row>
     <row r="38" ht="13.65" customHeight="1">
       <c r="A38" t="s" s="38">
         <v>124</v>
       </c>
       <c r="B38" t="s" s="38">
-        <v>158</v>
+        <v>190</v>
       </c>
       <c r="C38" t="s" s="38">
-        <v>155</v>
+        <v>172</v>
       </c>
       <c r="D38" s="53">
         <v>4</v>
@@ -5274,16 +5608,19 @@
       <c r="L38" s="54">
         <v>1</v>
       </c>
+      <c r="M38" t="s" s="38">
+        <v>194</v>
+      </c>
     </row>
     <row r="39" ht="13.65" customHeight="1">
       <c r="A39" t="s" s="38">
         <v>124</v>
       </c>
       <c r="B39" t="s" s="38">
-        <v>158</v>
+        <v>190</v>
       </c>
       <c r="C39" t="s" s="38">
-        <v>155</v>
+        <v>172</v>
       </c>
       <c r="D39" s="53">
         <v>5</v>
@@ -5316,16 +5653,19 @@
       <c r="L39" s="54">
         <v>1</v>
       </c>
+      <c r="M39" t="s" s="38">
+        <v>195</v>
+      </c>
     </row>
     <row r="40" ht="13.65" customHeight="1">
       <c r="A40" t="s" s="38">
         <v>124</v>
       </c>
       <c r="B40" t="s" s="38">
-        <v>159</v>
+        <v>196</v>
       </c>
       <c r="C40" t="s" s="38">
-        <v>155</v>
+        <v>172</v>
       </c>
       <c r="D40" s="53">
         <v>1</v>
@@ -5358,16 +5698,19 @@
       <c r="L40" s="54">
         <v>1</v>
       </c>
+      <c r="M40" t="s" s="38">
+        <v>197</v>
+      </c>
     </row>
     <row r="41" ht="13.65" customHeight="1">
       <c r="A41" t="s" s="38">
         <v>124</v>
       </c>
       <c r="B41" t="s" s="38">
-        <v>159</v>
+        <v>196</v>
       </c>
       <c r="C41" t="s" s="38">
-        <v>155</v>
+        <v>172</v>
       </c>
       <c r="D41" s="53">
         <v>2</v>
@@ -5400,16 +5743,19 @@
       <c r="L41" s="54">
         <v>1</v>
       </c>
+      <c r="M41" t="s" s="38">
+        <v>198</v>
+      </c>
     </row>
     <row r="42" ht="13.65" customHeight="1">
       <c r="A42" t="s" s="38">
         <v>124</v>
       </c>
       <c r="B42" t="s" s="38">
-        <v>159</v>
+        <v>196</v>
       </c>
       <c r="C42" t="s" s="38">
-        <v>155</v>
+        <v>172</v>
       </c>
       <c r="D42" s="53">
         <v>3</v>
@@ -5442,16 +5788,19 @@
       <c r="L42" s="54">
         <v>1</v>
       </c>
+      <c r="M42" t="s" s="38">
+        <v>199</v>
+      </c>
     </row>
     <row r="43" ht="13.65" customHeight="1">
       <c r="A43" t="s" s="38">
         <v>124</v>
       </c>
       <c r="B43" t="s" s="38">
-        <v>159</v>
+        <v>196</v>
       </c>
       <c r="C43" t="s" s="38">
-        <v>155</v>
+        <v>172</v>
       </c>
       <c r="D43" s="53">
         <v>4</v>
@@ -5484,16 +5833,19 @@
       <c r="L43" s="54">
         <v>1</v>
       </c>
+      <c r="M43" t="s" s="38">
+        <v>200</v>
+      </c>
     </row>
     <row r="44" ht="13.65" customHeight="1">
       <c r="A44" t="s" s="38">
         <v>124</v>
       </c>
       <c r="B44" t="s" s="38">
-        <v>159</v>
+        <v>196</v>
       </c>
       <c r="C44" t="s" s="38">
-        <v>155</v>
+        <v>172</v>
       </c>
       <c r="D44" s="53">
         <v>5</v>
@@ -5526,16 +5878,19 @@
       <c r="L44" s="54">
         <v>1</v>
       </c>
+      <c r="M44" t="s" s="38">
+        <v>201</v>
+      </c>
     </row>
     <row r="45" ht="13.65" customHeight="1">
       <c r="A45" t="s" s="38">
         <v>124</v>
       </c>
       <c r="B45" t="s" s="38">
-        <v>160</v>
+        <v>202</v>
       </c>
       <c r="C45" t="s" s="38">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="D45" s="53">
         <v>1</v>
@@ -5568,16 +5923,19 @@
       <c r="L45" s="54">
         <v>1</v>
       </c>
+      <c r="M45" t="s" s="38">
+        <v>203</v>
+      </c>
     </row>
     <row r="46" ht="13.65" customHeight="1">
       <c r="A46" t="s" s="38">
         <v>124</v>
       </c>
       <c r="B46" t="s" s="38">
-        <v>160</v>
+        <v>202</v>
       </c>
       <c r="C46" t="s" s="38">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="D46" s="53">
         <v>2</v>
@@ -5610,16 +5968,19 @@
       <c r="L46" s="54">
         <v>1</v>
       </c>
+      <c r="M46" t="s" s="38">
+        <v>204</v>
+      </c>
     </row>
     <row r="47" ht="13.65" customHeight="1">
       <c r="A47" t="s" s="38">
         <v>124</v>
       </c>
       <c r="B47" t="s" s="38">
-        <v>160</v>
+        <v>202</v>
       </c>
       <c r="C47" t="s" s="38">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="D47" s="53">
         <v>3</v>
@@ -5652,16 +6013,19 @@
       <c r="L47" s="54">
         <v>1</v>
       </c>
+      <c r="M47" t="s" s="38">
+        <v>205</v>
+      </c>
     </row>
     <row r="48" ht="13.65" customHeight="1">
       <c r="A48" t="s" s="38">
         <v>124</v>
       </c>
       <c r="B48" t="s" s="38">
-        <v>160</v>
+        <v>202</v>
       </c>
       <c r="C48" t="s" s="38">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="D48" s="53">
         <v>4</v>
@@ -5694,16 +6058,19 @@
       <c r="L48" s="54">
         <v>1</v>
       </c>
+      <c r="M48" t="s" s="38">
+        <v>206</v>
+      </c>
     </row>
     <row r="49" ht="13.65" customHeight="1">
       <c r="A49" t="s" s="38">
         <v>124</v>
       </c>
       <c r="B49" t="s" s="38">
-        <v>160</v>
+        <v>202</v>
       </c>
       <c r="C49" t="s" s="38">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="D49" s="53">
         <v>5</v>
@@ -5736,16 +6103,19 @@
       <c r="L49" s="54">
         <v>1</v>
       </c>
+      <c r="M49" t="s" s="38">
+        <v>207</v>
+      </c>
     </row>
     <row r="50" ht="13.65" customHeight="1">
       <c r="A50" t="s" s="38">
         <v>128</v>
       </c>
       <c r="B50" t="s" s="38">
-        <v>161</v>
+        <v>208</v>
       </c>
       <c r="C50" t="s" s="38">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D50" s="53">
         <v>1</v>
@@ -5778,16 +6148,19 @@
       <c r="L50" s="54">
         <v>1.15</v>
       </c>
+      <c r="M50" t="s" s="38">
+        <v>209</v>
+      </c>
     </row>
     <row r="51" ht="13.65" customHeight="1">
       <c r="A51" t="s" s="38">
         <v>128</v>
       </c>
       <c r="B51" t="s" s="38">
-        <v>161</v>
+        <v>208</v>
       </c>
       <c r="C51" t="s" s="38">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D51" s="53">
         <v>2</v>
@@ -5820,16 +6193,19 @@
       <c r="L51" s="54">
         <v>1.3</v>
       </c>
+      <c r="M51" t="s" s="38">
+        <v>210</v>
+      </c>
     </row>
     <row r="52" ht="13.65" customHeight="1">
       <c r="A52" t="s" s="38">
         <v>128</v>
       </c>
       <c r="B52" t="s" s="38">
-        <v>161</v>
+        <v>208</v>
       </c>
       <c r="C52" t="s" s="38">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D52" s="53">
         <v>3</v>
@@ -5862,16 +6238,19 @@
       <c r="L52" s="54">
         <v>1.5</v>
       </c>
+      <c r="M52" t="s" s="38">
+        <v>211</v>
+      </c>
     </row>
     <row r="53" ht="13.65" customHeight="1">
       <c r="A53" t="s" s="38">
         <v>128</v>
       </c>
       <c r="B53" t="s" s="38">
-        <v>161</v>
+        <v>208</v>
       </c>
       <c r="C53" t="s" s="38">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D53" s="53">
         <v>4</v>
@@ -5904,16 +6283,19 @@
       <c r="L53" s="54">
         <v>1.75</v>
       </c>
+      <c r="M53" t="s" s="38">
+        <v>212</v>
+      </c>
     </row>
     <row r="54" ht="13.65" customHeight="1">
       <c r="A54" t="s" s="38">
         <v>128</v>
       </c>
       <c r="B54" t="s" s="38">
-        <v>161</v>
+        <v>208</v>
       </c>
       <c r="C54" t="s" s="38">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D54" s="53">
         <v>5</v>
@@ -5946,16 +6328,19 @@
       <c r="L54" s="54">
         <v>2</v>
       </c>
+      <c r="M54" t="s" s="38">
+        <v>213</v>
+      </c>
     </row>
     <row r="55" ht="13.65" customHeight="1">
       <c r="A55" t="s" s="38">
         <v>128</v>
       </c>
       <c r="B55" t="s" s="38">
-        <v>162</v>
+        <v>214</v>
       </c>
       <c r="C55" t="s" s="38">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="D55" s="53">
         <v>1</v>
@@ -5988,16 +6373,19 @@
       <c r="L55" s="54">
         <v>1</v>
       </c>
+      <c r="M55" t="s" s="38">
+        <v>215</v>
+      </c>
     </row>
     <row r="56" ht="13.65" customHeight="1">
       <c r="A56" t="s" s="38">
         <v>128</v>
       </c>
       <c r="B56" t="s" s="38">
-        <v>162</v>
+        <v>214</v>
       </c>
       <c r="C56" t="s" s="38">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="D56" s="53">
         <v>2</v>
@@ -6030,16 +6418,19 @@
       <c r="L56" s="54">
         <v>1</v>
       </c>
+      <c r="M56" t="s" s="38">
+        <v>216</v>
+      </c>
     </row>
     <row r="57" ht="13.65" customHeight="1">
       <c r="A57" t="s" s="38">
         <v>128</v>
       </c>
       <c r="B57" t="s" s="38">
-        <v>162</v>
+        <v>214</v>
       </c>
       <c r="C57" t="s" s="38">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="D57" s="53">
         <v>3</v>
@@ -6072,16 +6463,19 @@
       <c r="L57" s="54">
         <v>1</v>
       </c>
+      <c r="M57" t="s" s="38">
+        <v>217</v>
+      </c>
     </row>
     <row r="58" ht="13.65" customHeight="1">
       <c r="A58" t="s" s="38">
         <v>128</v>
       </c>
       <c r="B58" t="s" s="38">
-        <v>162</v>
+        <v>214</v>
       </c>
       <c r="C58" t="s" s="38">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="D58" s="53">
         <v>4</v>
@@ -6114,16 +6508,19 @@
       <c r="L58" s="54">
         <v>1</v>
       </c>
+      <c r="M58" t="s" s="38">
+        <v>218</v>
+      </c>
     </row>
     <row r="59" ht="13.65" customHeight="1">
       <c r="A59" t="s" s="38">
         <v>128</v>
       </c>
       <c r="B59" t="s" s="38">
-        <v>162</v>
+        <v>214</v>
       </c>
       <c r="C59" t="s" s="38">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="D59" s="53">
         <v>5</v>
@@ -6156,16 +6553,19 @@
       <c r="L59" s="54">
         <v>1</v>
       </c>
+      <c r="M59" t="s" s="38">
+        <v>219</v>
+      </c>
     </row>
     <row r="60" ht="13.65" customHeight="1">
       <c r="A60" t="s" s="38">
         <v>128</v>
       </c>
       <c r="B60" t="s" s="38">
-        <v>163</v>
+        <v>220</v>
       </c>
       <c r="C60" t="s" s="38">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="D60" s="53">
         <v>1</v>
@@ -6198,16 +6598,19 @@
       <c r="L60" s="54">
         <v>1</v>
       </c>
+      <c r="M60" t="s" s="38">
+        <v>220</v>
+      </c>
     </row>
     <row r="61" ht="13.65" customHeight="1">
       <c r="A61" t="s" s="38">
         <v>128</v>
       </c>
       <c r="B61" t="s" s="38">
-        <v>163</v>
+        <v>220</v>
       </c>
       <c r="C61" t="s" s="38">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="D61" s="53">
         <v>2</v>
@@ -6240,16 +6643,19 @@
       <c r="L61" s="54">
         <v>1</v>
       </c>
+      <c r="M61" t="s" s="38">
+        <v>221</v>
+      </c>
     </row>
     <row r="62" ht="13.65" customHeight="1">
       <c r="A62" t="s" s="38">
         <v>128</v>
       </c>
       <c r="B62" t="s" s="38">
-        <v>163</v>
+        <v>220</v>
       </c>
       <c r="C62" t="s" s="38">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="D62" s="53">
         <v>3</v>
@@ -6282,16 +6688,19 @@
       <c r="L62" s="54">
         <v>1</v>
       </c>
+      <c r="M62" t="s" s="38">
+        <v>222</v>
+      </c>
     </row>
     <row r="63" ht="13.65" customHeight="1">
       <c r="A63" t="s" s="38">
         <v>128</v>
       </c>
       <c r="B63" t="s" s="38">
-        <v>163</v>
+        <v>220</v>
       </c>
       <c r="C63" t="s" s="38">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="D63" s="53">
         <v>4</v>
@@ -6324,16 +6733,19 @@
       <c r="L63" s="54">
         <v>1</v>
       </c>
+      <c r="M63" t="s" s="38">
+        <v>223</v>
+      </c>
     </row>
     <row r="64" ht="13.65" customHeight="1">
       <c r="A64" t="s" s="38">
         <v>128</v>
       </c>
       <c r="B64" t="s" s="38">
-        <v>163</v>
+        <v>220</v>
       </c>
       <c r="C64" t="s" s="38">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="D64" s="53">
         <v>5</v>
@@ -6366,16 +6778,19 @@
       <c r="L64" s="54">
         <v>1</v>
       </c>
+      <c r="M64" t="s" s="38">
+        <v>224</v>
+      </c>
     </row>
     <row r="65" ht="13.65" customHeight="1">
       <c r="A65" t="s" s="38">
         <v>131</v>
       </c>
       <c r="B65" t="s" s="38">
-        <v>164</v>
+        <v>225</v>
       </c>
       <c r="C65" t="s" s="38">
-        <v>165</v>
+        <v>226</v>
       </c>
       <c r="D65" s="53">
         <v>1</v>
@@ -6401,10 +6816,13 @@
         <v>0</v>
       </c>
       <c r="K65" t="s" s="38">
-        <v>166</v>
+        <v>227</v>
       </c>
       <c r="L65" s="54">
         <v>1</v>
+      </c>
+      <c r="M65" t="s" s="38">
+        <v>228</v>
       </c>
     </row>
     <row r="66" ht="13.65" customHeight="1">
@@ -6412,10 +6830,10 @@
         <v>131</v>
       </c>
       <c r="B66" t="s" s="38">
-        <v>164</v>
+        <v>225</v>
       </c>
       <c r="C66" t="s" s="38">
-        <v>165</v>
+        <v>226</v>
       </c>
       <c r="D66" s="53">
         <v>2</v>
@@ -6441,10 +6859,13 @@
         <v>0</v>
       </c>
       <c r="K66" t="s" s="38">
-        <v>166</v>
+        <v>227</v>
       </c>
       <c r="L66" s="54">
         <v>1</v>
+      </c>
+      <c r="M66" t="s" s="38">
+        <v>229</v>
       </c>
     </row>
     <row r="67" ht="13.65" customHeight="1">
@@ -6452,10 +6873,10 @@
         <v>131</v>
       </c>
       <c r="B67" t="s" s="38">
-        <v>164</v>
+        <v>225</v>
       </c>
       <c r="C67" t="s" s="38">
-        <v>165</v>
+        <v>226</v>
       </c>
       <c r="D67" s="53">
         <v>3</v>
@@ -6481,10 +6902,13 @@
         <v>0</v>
       </c>
       <c r="K67" t="s" s="38">
-        <v>166</v>
+        <v>227</v>
       </c>
       <c r="L67" s="54">
         <v>1</v>
+      </c>
+      <c r="M67" t="s" s="38">
+        <v>230</v>
       </c>
     </row>
     <row r="68" ht="13.65" customHeight="1">
@@ -6492,10 +6916,10 @@
         <v>131</v>
       </c>
       <c r="B68" t="s" s="38">
-        <v>164</v>
+        <v>225</v>
       </c>
       <c r="C68" t="s" s="38">
-        <v>165</v>
+        <v>226</v>
       </c>
       <c r="D68" s="53">
         <v>4</v>
@@ -6521,10 +6945,13 @@
         <v>0</v>
       </c>
       <c r="K68" t="s" s="38">
-        <v>166</v>
+        <v>227</v>
       </c>
       <c r="L68" s="54">
         <v>1</v>
+      </c>
+      <c r="M68" t="s" s="38">
+        <v>231</v>
       </c>
     </row>
     <row r="69" ht="13.65" customHeight="1">
@@ -6532,10 +6959,10 @@
         <v>131</v>
       </c>
       <c r="B69" t="s" s="38">
-        <v>164</v>
+        <v>225</v>
       </c>
       <c r="C69" t="s" s="38">
-        <v>165</v>
+        <v>226</v>
       </c>
       <c r="D69" s="53">
         <v>5</v>
@@ -6561,10 +6988,13 @@
         <v>0</v>
       </c>
       <c r="K69" t="s" s="38">
-        <v>166</v>
+        <v>227</v>
       </c>
       <c r="L69" s="54">
         <v>1</v>
+      </c>
+      <c r="M69" t="s" s="38">
+        <v>232</v>
       </c>
     </row>
     <row r="70" ht="13.65" customHeight="1">
@@ -6572,10 +7002,10 @@
         <v>131</v>
       </c>
       <c r="B70" t="s" s="38">
-        <v>167</v>
+        <v>233</v>
       </c>
       <c r="C70" t="s" s="38">
-        <v>165</v>
+        <v>226</v>
       </c>
       <c r="D70" s="53">
         <v>1</v>
@@ -6601,10 +7031,13 @@
         <v>0</v>
       </c>
       <c r="K70" t="s" s="38">
-        <v>166</v>
+        <v>227</v>
       </c>
       <c r="L70" s="54">
         <v>1</v>
+      </c>
+      <c r="M70" t="s" s="38">
+        <v>234</v>
       </c>
     </row>
     <row r="71" ht="13.65" customHeight="1">
@@ -6612,10 +7045,10 @@
         <v>131</v>
       </c>
       <c r="B71" t="s" s="38">
-        <v>167</v>
+        <v>233</v>
       </c>
       <c r="C71" t="s" s="38">
-        <v>165</v>
+        <v>226</v>
       </c>
       <c r="D71" s="53">
         <v>2</v>
@@ -6641,10 +7074,13 @@
         <v>0</v>
       </c>
       <c r="K71" t="s" s="38">
-        <v>166</v>
+        <v>227</v>
       </c>
       <c r="L71" s="54">
         <v>1</v>
+      </c>
+      <c r="M71" t="s" s="38">
+        <v>235</v>
       </c>
     </row>
     <row r="72" ht="13.65" customHeight="1">
@@ -6652,10 +7088,10 @@
         <v>131</v>
       </c>
       <c r="B72" t="s" s="38">
-        <v>167</v>
+        <v>233</v>
       </c>
       <c r="C72" t="s" s="38">
-        <v>165</v>
+        <v>226</v>
       </c>
       <c r="D72" s="53">
         <v>3</v>
@@ -6681,10 +7117,13 @@
         <v>0</v>
       </c>
       <c r="K72" t="s" s="38">
-        <v>166</v>
+        <v>227</v>
       </c>
       <c r="L72" s="54">
         <v>1</v>
+      </c>
+      <c r="M72" t="s" s="38">
+        <v>236</v>
       </c>
     </row>
     <row r="73" ht="13.65" customHeight="1">
@@ -6692,10 +7131,10 @@
         <v>131</v>
       </c>
       <c r="B73" t="s" s="38">
-        <v>167</v>
+        <v>233</v>
       </c>
       <c r="C73" t="s" s="38">
-        <v>165</v>
+        <v>226</v>
       </c>
       <c r="D73" s="53">
         <v>4</v>
@@ -6721,10 +7160,13 @@
         <v>0</v>
       </c>
       <c r="K73" t="s" s="38">
-        <v>166</v>
+        <v>227</v>
       </c>
       <c r="L73" s="54">
         <v>1</v>
+      </c>
+      <c r="M73" t="s" s="38">
+        <v>237</v>
       </c>
     </row>
     <row r="74" ht="13.65" customHeight="1">
@@ -6732,10 +7174,10 @@
         <v>131</v>
       </c>
       <c r="B74" t="s" s="38">
-        <v>167</v>
+        <v>233</v>
       </c>
       <c r="C74" t="s" s="38">
-        <v>165</v>
+        <v>226</v>
       </c>
       <c r="D74" s="53">
         <v>5</v>
@@ -6761,10 +7203,13 @@
         <v>0</v>
       </c>
       <c r="K74" t="s" s="38">
-        <v>166</v>
+        <v>227</v>
       </c>
       <c r="L74" s="54">
         <v>1</v>
+      </c>
+      <c r="M74" t="s" s="38">
+        <v>238</v>
       </c>
     </row>
     <row r="75" ht="13.65" customHeight="1">
@@ -6772,10 +7217,10 @@
         <v>131</v>
       </c>
       <c r="B75" t="s" s="38">
-        <v>168</v>
+        <v>239</v>
       </c>
       <c r="C75" t="s" s="38">
-        <v>165</v>
+        <v>226</v>
       </c>
       <c r="D75" s="53">
         <v>1</v>
@@ -6801,10 +7246,13 @@
         <v>0</v>
       </c>
       <c r="K75" t="s" s="38">
-        <v>166</v>
+        <v>227</v>
       </c>
       <c r="L75" s="54">
         <v>1</v>
+      </c>
+      <c r="M75" t="s" s="38">
+        <v>240</v>
       </c>
     </row>
     <row r="76" ht="13.65" customHeight="1">
@@ -6812,10 +7260,10 @@
         <v>131</v>
       </c>
       <c r="B76" t="s" s="38">
-        <v>168</v>
+        <v>239</v>
       </c>
       <c r="C76" t="s" s="38">
-        <v>165</v>
+        <v>226</v>
       </c>
       <c r="D76" s="53">
         <v>2</v>
@@ -6841,10 +7289,13 @@
         <v>0</v>
       </c>
       <c r="K76" t="s" s="38">
-        <v>166</v>
+        <v>227</v>
       </c>
       <c r="L76" s="54">
         <v>1</v>
+      </c>
+      <c r="M76" t="s" s="38">
+        <v>241</v>
       </c>
     </row>
     <row r="77" ht="13.65" customHeight="1">
@@ -6852,10 +7303,10 @@
         <v>131</v>
       </c>
       <c r="B77" t="s" s="38">
-        <v>168</v>
+        <v>239</v>
       </c>
       <c r="C77" t="s" s="38">
-        <v>165</v>
+        <v>226</v>
       </c>
       <c r="D77" s="53">
         <v>3</v>
@@ -6881,10 +7332,13 @@
         <v>0</v>
       </c>
       <c r="K77" t="s" s="38">
-        <v>166</v>
+        <v>227</v>
       </c>
       <c r="L77" s="54">
         <v>1</v>
+      </c>
+      <c r="M77" t="s" s="38">
+        <v>242</v>
       </c>
     </row>
     <row r="78" ht="13.65" customHeight="1">
@@ -6892,10 +7346,10 @@
         <v>131</v>
       </c>
       <c r="B78" t="s" s="38">
-        <v>168</v>
+        <v>239</v>
       </c>
       <c r="C78" t="s" s="38">
-        <v>165</v>
+        <v>226</v>
       </c>
       <c r="D78" s="53">
         <v>4</v>
@@ -6921,10 +7375,13 @@
         <v>0</v>
       </c>
       <c r="K78" t="s" s="38">
-        <v>166</v>
+        <v>227</v>
       </c>
       <c r="L78" s="54">
         <v>1</v>
+      </c>
+      <c r="M78" t="s" s="38">
+        <v>243</v>
       </c>
     </row>
     <row r="79" ht="13.65" customHeight="1">
@@ -6932,10 +7389,10 @@
         <v>131</v>
       </c>
       <c r="B79" t="s" s="38">
-        <v>168</v>
+        <v>239</v>
       </c>
       <c r="C79" t="s" s="38">
-        <v>165</v>
+        <v>226</v>
       </c>
       <c r="D79" s="53">
         <v>5</v>
@@ -6961,10 +7418,13 @@
         <v>0</v>
       </c>
       <c r="K79" t="s" s="38">
-        <v>166</v>
+        <v>227</v>
       </c>
       <c r="L79" s="54">
         <v>1</v>
+      </c>
+      <c r="M79" t="s" s="38">
+        <v>244</v>
       </c>
     </row>
   </sheetData>
@@ -6998,7 +7458,7 @@
   <sheetData>
     <row r="1" ht="18.5" customHeight="1">
       <c r="A1" t="s" s="2">
-        <v>169</v>
+        <v>245</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -7014,7 +7474,7 @@
     </row>
     <row r="2" ht="13.65" customHeight="1">
       <c r="A2" t="s" s="5">
-        <v>170</v>
+        <v>246</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -7044,22 +7504,22 @@
     </row>
     <row r="4" ht="27.75" customHeight="1">
       <c r="A4" t="s" s="21">
-        <v>171</v>
+        <v>247</v>
       </c>
       <c r="B4" t="s" s="21">
-        <v>172</v>
+        <v>248</v>
       </c>
       <c r="C4" t="s" s="21">
         <v>140</v>
       </c>
       <c r="D4" t="s" s="21">
-        <v>173</v>
+        <v>249</v>
       </c>
       <c r="E4" t="s" s="21">
         <v>108</v>
       </c>
       <c r="F4" t="s" s="21">
-        <v>174</v>
+        <v>250</v>
       </c>
       <c r="G4" t="s" s="21">
         <v>109</v>
@@ -7068,30 +7528,30 @@
         <v>110</v>
       </c>
       <c r="I4" t="s" s="21">
-        <v>175</v>
+        <v>251</v>
       </c>
       <c r="J4" t="s" s="21">
-        <v>176</v>
+        <v>252</v>
       </c>
       <c r="K4" t="s" s="21">
-        <v>177</v>
+        <v>253</v>
       </c>
       <c r="L4" t="s" s="21">
-        <v>178</v>
+        <v>254</v>
       </c>
     </row>
     <row r="5" ht="13.65" customHeight="1">
       <c r="A5" t="s" s="38">
-        <v>179</v>
+        <v>255</v>
       </c>
       <c r="B5" t="s" s="56">
-        <v>180</v>
+        <v>256</v>
       </c>
       <c r="C5" s="53">
         <v>1</v>
       </c>
       <c r="D5" t="s" s="38">
-        <v>181</v>
+        <v>257</v>
       </c>
       <c r="E5" s="53" cm="1">
         <f t="array" ref="E5">ROUND('Tuning'!$B$21*POWER('Tuning'!$B$22,C5-1),0)</f>
@@ -7117,21 +7577,21 @@
       </c>
       <c r="K5" s="53"/>
       <c r="L5" t="s" s="42">
-        <v>182</v>
+        <v>258</v>
       </c>
     </row>
     <row r="6" ht="13.65" customHeight="1">
       <c r="A6" t="s" s="38">
-        <v>179</v>
+        <v>255</v>
       </c>
       <c r="B6" t="s" s="38">
-        <v>183</v>
+        <v>259</v>
       </c>
       <c r="C6" s="53">
         <v>2</v>
       </c>
       <c r="D6" t="s" s="38">
-        <v>184</v>
+        <v>260</v>
       </c>
       <c r="E6" s="53" cm="1">
         <f t="array" ref="E6">ROUND('Tuning'!$B$21*POWER('Tuning'!$B$22,C6-1),0)</f>
@@ -7162,16 +7622,16 @@
     </row>
     <row r="7" ht="13.65" customHeight="1">
       <c r="A7" t="s" s="38">
-        <v>179</v>
+        <v>255</v>
       </c>
       <c r="B7" t="s" s="38">
-        <v>183</v>
+        <v>259</v>
       </c>
       <c r="C7" s="53">
         <v>3</v>
       </c>
       <c r="D7" t="s" s="38">
-        <v>185</v>
+        <v>261</v>
       </c>
       <c r="E7" s="53" cm="1">
         <f t="array" ref="E7">ROUND('Tuning'!$B$21*POWER('Tuning'!$B$22,C7-1),0)</f>
@@ -7202,16 +7662,16 @@
     </row>
     <row r="8" ht="13.65" customHeight="1">
       <c r="A8" t="s" s="38">
-        <v>179</v>
+        <v>255</v>
       </c>
       <c r="B8" t="s" s="38">
-        <v>183</v>
+        <v>259</v>
       </c>
       <c r="C8" s="53">
         <v>4</v>
       </c>
       <c r="D8" t="s" s="38">
-        <v>186</v>
+        <v>262</v>
       </c>
       <c r="E8" s="53" cm="1">
         <f t="array" ref="E8">ROUND('Tuning'!$B$21*POWER('Tuning'!$B$22,C8-1),0)</f>
@@ -7242,16 +7702,16 @@
     </row>
     <row r="9" ht="13.65" customHeight="1">
       <c r="A9" t="s" s="38">
-        <v>179</v>
+        <v>255</v>
       </c>
       <c r="B9" t="s" s="38">
-        <v>183</v>
+        <v>259</v>
       </c>
       <c r="C9" s="53">
         <v>5</v>
       </c>
       <c r="D9" t="s" s="38">
-        <v>187</v>
+        <v>263</v>
       </c>
       <c r="E9" s="53" cm="1">
         <f t="array" ref="E9">ROUND('Tuning'!$B$21*POWER('Tuning'!$B$22,C9-1),0)</f>
@@ -7282,16 +7742,16 @@
     </row>
     <row r="10" ht="13.65" customHeight="1">
       <c r="A10" t="s" s="38">
-        <v>188</v>
+        <v>264</v>
       </c>
       <c r="B10" t="s" s="56">
-        <v>180</v>
+        <v>256</v>
       </c>
       <c r="C10" s="53">
         <v>1</v>
       </c>
       <c r="D10" t="s" s="38">
-        <v>189</v>
+        <v>265</v>
       </c>
       <c r="E10" s="53" cm="1">
         <f t="array" ref="E10">ROUND('Tuning'!$B$21*POWER('Tuning'!$B$22,C10-1),0)</f>
@@ -7317,21 +7777,21 @@
       </c>
       <c r="K10" s="53"/>
       <c r="L10" t="s" s="42">
-        <v>190</v>
+        <v>266</v>
       </c>
     </row>
     <row r="11" ht="13.65" customHeight="1">
       <c r="A11" t="s" s="38">
-        <v>188</v>
+        <v>264</v>
       </c>
       <c r="B11" t="s" s="38">
-        <v>191</v>
+        <v>267</v>
       </c>
       <c r="C11" s="53">
         <v>2</v>
       </c>
       <c r="D11" t="s" s="38">
-        <v>192</v>
+        <v>268</v>
       </c>
       <c r="E11" s="53" cm="1">
         <f t="array" ref="E11">ROUND('Tuning'!$B$21*POWER('Tuning'!$B$22,C11-1),0)</f>
@@ -7362,16 +7822,16 @@
     </row>
     <row r="12" ht="13.65" customHeight="1">
       <c r="A12" t="s" s="38">
-        <v>188</v>
+        <v>264</v>
       </c>
       <c r="B12" t="s" s="38">
-        <v>191</v>
+        <v>267</v>
       </c>
       <c r="C12" s="53">
         <v>3</v>
       </c>
       <c r="D12" t="s" s="38">
-        <v>193</v>
+        <v>269</v>
       </c>
       <c r="E12" s="53" cm="1">
         <f t="array" ref="E12">ROUND('Tuning'!$B$21*POWER('Tuning'!$B$22,C12-1),0)</f>
@@ -7402,16 +7862,16 @@
     </row>
     <row r="13" ht="13.65" customHeight="1">
       <c r="A13" t="s" s="38">
-        <v>188</v>
+        <v>264</v>
       </c>
       <c r="B13" t="s" s="38">
-        <v>191</v>
+        <v>267</v>
       </c>
       <c r="C13" s="53">
         <v>4</v>
       </c>
       <c r="D13" t="s" s="38">
-        <v>194</v>
+        <v>270</v>
       </c>
       <c r="E13" s="53" cm="1">
         <f t="array" ref="E13">ROUND('Tuning'!$B$21*POWER('Tuning'!$B$22,C13-1),0)</f>
@@ -7442,16 +7902,16 @@
     </row>
     <row r="14" ht="13.65" customHeight="1">
       <c r="A14" t="s" s="38">
-        <v>188</v>
+        <v>264</v>
       </c>
       <c r="B14" t="s" s="38">
-        <v>191</v>
+        <v>267</v>
       </c>
       <c r="C14" s="53">
         <v>5</v>
       </c>
       <c r="D14" t="s" s="38">
-        <v>195</v>
+        <v>271</v>
       </c>
       <c r="E14" s="53" cm="1">
         <f t="array" ref="E14">ROUND('Tuning'!$B$21*POWER('Tuning'!$B$22,C14-1),0)</f>
@@ -7482,16 +7942,16 @@
     </row>
     <row r="15" ht="13.65" customHeight="1">
       <c r="A15" t="s" s="38">
-        <v>196</v>
+        <v>272</v>
       </c>
       <c r="B15" t="s" s="56">
-        <v>180</v>
+        <v>256</v>
       </c>
       <c r="C15" s="53">
         <v>1</v>
       </c>
       <c r="D15" t="s" s="38">
-        <v>197</v>
+        <v>273</v>
       </c>
       <c r="E15" s="53" cm="1">
         <f t="array" ref="E15">ROUND('Tuning'!$B$21*POWER('Tuning'!$B$22,C15-1),0)</f>
@@ -7517,21 +7977,21 @@
       </c>
       <c r="K15" s="53"/>
       <c r="L15" t="s" s="42">
-        <v>198</v>
+        <v>274</v>
       </c>
     </row>
     <row r="16" ht="13.65" customHeight="1">
       <c r="A16" t="s" s="38">
-        <v>196</v>
+        <v>272</v>
       </c>
       <c r="B16" t="s" s="38">
-        <v>199</v>
+        <v>275</v>
       </c>
       <c r="C16" s="53">
         <v>2</v>
       </c>
       <c r="D16" t="s" s="38">
-        <v>200</v>
+        <v>276</v>
       </c>
       <c r="E16" s="53" cm="1">
         <f t="array" ref="E16">ROUND('Tuning'!$B$21*POWER('Tuning'!$B$22,C16-1),0)</f>
@@ -7562,16 +8022,16 @@
     </row>
     <row r="17" ht="13.65" customHeight="1">
       <c r="A17" t="s" s="38">
-        <v>196</v>
+        <v>272</v>
       </c>
       <c r="B17" t="s" s="38">
-        <v>199</v>
+        <v>275</v>
       </c>
       <c r="C17" s="53">
         <v>3</v>
       </c>
       <c r="D17" t="s" s="38">
-        <v>201</v>
+        <v>277</v>
       </c>
       <c r="E17" s="53" cm="1">
         <f t="array" ref="E17">ROUND('Tuning'!$B$21*POWER('Tuning'!$B$22,C17-1),0)</f>
@@ -7602,16 +8062,16 @@
     </row>
     <row r="18" ht="13.65" customHeight="1">
       <c r="A18" t="s" s="38">
-        <v>196</v>
+        <v>272</v>
       </c>
       <c r="B18" t="s" s="38">
-        <v>199</v>
+        <v>275</v>
       </c>
       <c r="C18" s="53">
         <v>4</v>
       </c>
       <c r="D18" t="s" s="38">
-        <v>202</v>
+        <v>278</v>
       </c>
       <c r="E18" s="53" cm="1">
         <f t="array" ref="E18">ROUND('Tuning'!$B$21*POWER('Tuning'!$B$22,C18-1),0)</f>
@@ -7642,16 +8102,16 @@
     </row>
     <row r="19" ht="13.65" customHeight="1">
       <c r="A19" t="s" s="38">
-        <v>196</v>
+        <v>272</v>
       </c>
       <c r="B19" t="s" s="38">
-        <v>199</v>
+        <v>275</v>
       </c>
       <c r="C19" s="53">
         <v>5</v>
       </c>
       <c r="D19" t="s" s="38">
-        <v>203</v>
+        <v>279</v>
       </c>
       <c r="E19" s="53" cm="1">
         <f t="array" ref="E19">ROUND('Tuning'!$B$21*POWER('Tuning'!$B$22,C19-1),0)</f>
@@ -7696,7 +8156,7 @@
     </row>
     <row r="21" ht="14.6" customHeight="1">
       <c r="A21" t="s" s="11">
-        <v>204</v>
+        <v>280</v>
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="6"/>
@@ -7712,7 +8172,7 @@
     </row>
     <row r="22" ht="13.55" customHeight="1">
       <c r="A22" t="s" s="60">
-        <v>205</v>
+        <v>281</v>
       </c>
       <c r="B22" s="16"/>
       <c r="C22" s="16"/>
@@ -7750,7 +8210,7 @@
   <sheetData>
     <row r="1" ht="18.5" customHeight="1">
       <c r="A1" t="s" s="2">
-        <v>206</v>
+        <v>282</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -7759,7 +8219,7 @@
     </row>
     <row r="2" ht="13.65" customHeight="1">
       <c r="A2" t="s" s="5">
-        <v>207</v>
+        <v>283</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -7775,19 +8235,19 @@
     </row>
     <row r="4" ht="27.75" customHeight="1">
       <c r="A4" t="s" s="21">
-        <v>208</v>
+        <v>284</v>
       </c>
       <c r="B4" t="s" s="21">
-        <v>209</v>
+        <v>285</v>
       </c>
       <c r="C4" t="s" s="21">
-        <v>210</v>
+        <v>286</v>
       </c>
       <c r="D4" t="s" s="21">
-        <v>211</v>
+        <v>287</v>
       </c>
       <c r="E4" t="s" s="21">
-        <v>212</v>
+        <v>288</v>
       </c>
     </row>
     <row r="5" ht="13.65" customHeight="1">
@@ -7807,7 +8267,7 @@
         <v>0.6</v>
       </c>
       <c r="E5" t="s" s="62">
-        <v>213</v>
+        <v>289</v>
       </c>
     </row>
     <row r="6" ht="13.65" customHeight="1">
@@ -7827,7 +8287,7 @@
         <v>1.3</v>
       </c>
       <c r="E6" t="s" s="62">
-        <v>214</v>
+        <v>290</v>
       </c>
     </row>
     <row r="7" ht="13.65" customHeight="1">
@@ -7847,7 +8307,7 @@
         <v>2.1</v>
       </c>
       <c r="E7" t="s" s="62">
-        <v>215</v>
+        <v>291</v>
       </c>
     </row>
     <row r="8" ht="13.65" customHeight="1">
@@ -7867,7 +8327,7 @@
         <v>3.1</v>
       </c>
       <c r="E8" t="s" s="62">
-        <v>216</v>
+        <v>292</v>
       </c>
     </row>
     <row r="9" ht="13.65" customHeight="1">
@@ -7887,7 +8347,7 @@
         <v>4.2</v>
       </c>
       <c r="E9" t="s" s="65">
-        <v>217</v>
+        <v>293</v>
       </c>
     </row>
     <row r="10" ht="13.65" customHeight="1">
@@ -7979,7 +8439,7 @@
         <v>13.8</v>
       </c>
       <c r="E14" t="s" s="65">
-        <v>218</v>
+        <v>294</v>
       </c>
     </row>
     <row r="15" ht="13.65" customHeight="1">
@@ -8071,7 +8531,7 @@
         <v>35.9</v>
       </c>
       <c r="E19" t="s" s="65">
-        <v>219</v>
+        <v>295</v>
       </c>
     </row>
     <row r="20" ht="13.65" customHeight="1">
@@ -8163,7 +8623,7 @@
         <v>86.2</v>
       </c>
       <c r="E24" t="s" s="65">
-        <v>220</v>
+        <v>296</v>
       </c>
     </row>
     <row r="25" ht="13.55" customHeight="1">
@@ -8175,7 +8635,7 @@
     </row>
     <row r="26" ht="13.55" customHeight="1">
       <c r="A26" t="s" s="67">
-        <v>221</v>
+        <v>297</v>
       </c>
       <c r="B26" s="16"/>
       <c r="C26" s="16"/>
@@ -8212,7 +8672,7 @@
   <sheetData>
     <row r="1" ht="18.5" customHeight="1">
       <c r="A1" t="s" s="2">
-        <v>222</v>
+        <v>298</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -8227,7 +8687,7 @@
     </row>
     <row r="2" ht="13.65" customHeight="1">
       <c r="A2" t="s" s="5">
-        <v>223</v>
+        <v>299</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -8255,45 +8715,45 @@
     </row>
     <row r="4" ht="27.75" customHeight="1">
       <c r="A4" t="s" s="21">
-        <v>224</v>
+        <v>300</v>
       </c>
       <c r="B4" t="s" s="21">
-        <v>225</v>
+        <v>301</v>
       </c>
       <c r="C4" t="s" s="21">
-        <v>226</v>
+        <v>302</v>
       </c>
       <c r="D4" t="s" s="21">
-        <v>227</v>
+        <v>303</v>
       </c>
       <c r="E4" t="s" s="21">
-        <v>228</v>
+        <v>304</v>
       </c>
       <c r="F4" t="s" s="21">
-        <v>229</v>
+        <v>305</v>
       </c>
       <c r="G4" t="s" s="21">
-        <v>230</v>
+        <v>306</v>
       </c>
       <c r="H4" t="s" s="21">
-        <v>231</v>
+        <v>307</v>
       </c>
       <c r="I4" t="s" s="21">
-        <v>232</v>
+        <v>308</v>
       </c>
       <c r="J4" t="s" s="21">
-        <v>233</v>
+        <v>309</v>
       </c>
       <c r="K4" t="s" s="21">
-        <v>234</v>
+        <v>310</v>
       </c>
     </row>
     <row r="5" ht="13.65" customHeight="1">
       <c r="A5" t="s" s="62">
-        <v>235</v>
+        <v>311</v>
       </c>
       <c r="B5" t="s" s="38">
-        <v>236</v>
+        <v>312</v>
       </c>
       <c r="C5" s="27">
         <v>1</v>
@@ -8306,7 +8766,7 @@
         <v>1</v>
       </c>
       <c r="F5" t="s" s="38">
-        <v>237</v>
+        <v>313</v>
       </c>
       <c r="G5" s="57">
         <v>0</v>
@@ -8323,15 +8783,15 @@
         <v>126</v>
       </c>
       <c r="K5" t="s" s="42">
-        <v>238</v>
+        <v>314</v>
       </c>
     </row>
     <row r="6" ht="13.65" customHeight="1">
       <c r="A6" t="s" s="62">
-        <v>239</v>
+        <v>315</v>
       </c>
       <c r="B6" t="s" s="38">
-        <v>240</v>
+        <v>316</v>
       </c>
       <c r="C6" s="27">
         <v>1</v>
@@ -8344,7 +8804,7 @@
         <v>1.2</v>
       </c>
       <c r="F6" t="s" s="38">
-        <v>235</v>
+        <v>311</v>
       </c>
       <c r="G6" s="57">
         <v>2</v>
@@ -8364,10 +8824,10 @@
     </row>
     <row r="7" ht="13.65" customHeight="1">
       <c r="A7" t="s" s="62">
-        <v>241</v>
+        <v>317</v>
       </c>
       <c r="B7" t="s" s="38">
-        <v>242</v>
+        <v>318</v>
       </c>
       <c r="C7" s="27">
         <v>2</v>
@@ -8380,7 +8840,7 @@
         <v>1</v>
       </c>
       <c r="F7" t="s" s="38">
-        <v>239</v>
+        <v>315</v>
       </c>
       <c r="G7" s="57">
         <v>2</v>
@@ -8400,10 +8860,10 @@
     </row>
     <row r="8" ht="13.65" customHeight="1">
       <c r="A8" t="s" s="62">
-        <v>243</v>
+        <v>319</v>
       </c>
       <c r="B8" t="s" s="38">
-        <v>244</v>
+        <v>320</v>
       </c>
       <c r="C8" s="27">
         <v>3</v>
@@ -8416,7 +8876,7 @@
         <v>0.8</v>
       </c>
       <c r="F8" t="s" s="38">
-        <v>241</v>
+        <v>317</v>
       </c>
       <c r="G8" s="57">
         <v>2</v>
@@ -8433,15 +8893,15 @@
         <v>126</v>
       </c>
       <c r="K8" t="s" s="42">
-        <v>245</v>
+        <v>321</v>
       </c>
     </row>
     <row r="9" ht="13.65" customHeight="1">
       <c r="A9" t="s" s="62">
-        <v>246</v>
+        <v>322</v>
       </c>
       <c r="B9" t="s" s="38">
-        <v>247</v>
+        <v>323</v>
       </c>
       <c r="C9" s="27">
         <v>4</v>
@@ -8454,7 +8914,7 @@
         <v>1.4</v>
       </c>
       <c r="F9" t="s" s="38">
-        <v>243</v>
+        <v>319</v>
       </c>
       <c r="G9" s="57">
         <v>3</v>
@@ -8471,15 +8931,15 @@
         <v>126</v>
       </c>
       <c r="K9" t="s" s="42">
-        <v>248</v>
+        <v>324</v>
       </c>
     </row>
     <row r="10" ht="13.65" customHeight="1">
       <c r="A10" t="s" s="62">
-        <v>249</v>
+        <v>325</v>
       </c>
       <c r="B10" t="s" s="38">
-        <v>250</v>
+        <v>326</v>
       </c>
       <c r="C10" s="27">
         <v>4</v>
@@ -8492,7 +8952,7 @@
         <v>0.9</v>
       </c>
       <c r="F10" t="s" s="38">
-        <v>241</v>
+        <v>317</v>
       </c>
       <c r="G10" s="57">
         <v>2</v>
@@ -8509,15 +8969,15 @@
         <v>119</v>
       </c>
       <c r="K10" t="s" s="42">
-        <v>251</v>
+        <v>327</v>
       </c>
     </row>
     <row r="11" ht="13.65" customHeight="1">
       <c r="A11" t="s" s="62">
-        <v>252</v>
+        <v>328</v>
       </c>
       <c r="B11" t="s" s="38">
-        <v>253</v>
+        <v>329</v>
       </c>
       <c r="C11" s="27">
         <v>200</v>
@@ -8530,7 +8990,7 @@
         <v>0.5</v>
       </c>
       <c r="F11" t="s" s="38">
-        <v>249</v>
+        <v>325</v>
       </c>
       <c r="G11" s="57">
         <v>4</v>
@@ -8547,15 +9007,15 @@
         <v>119</v>
       </c>
       <c r="K11" t="s" s="42">
-        <v>254</v>
+        <v>330</v>
       </c>
     </row>
     <row r="12" ht="13.65" customHeight="1">
       <c r="A12" t="s" s="62">
-        <v>255</v>
+        <v>331</v>
       </c>
       <c r="B12" t="s" s="38">
-        <v>256</v>
+        <v>332</v>
       </c>
       <c r="C12" s="27">
         <v>700</v>
@@ -8568,7 +9028,7 @@
         <v>0.4</v>
       </c>
       <c r="F12" t="s" s="38">
-        <v>252</v>
+        <v>328</v>
       </c>
       <c r="G12" s="57">
         <v>4</v>
@@ -8585,7 +9045,7 @@
         <v>119</v>
       </c>
       <c r="K12" t="s" s="42">
-        <v>257</v>
+        <v>333</v>
       </c>
     </row>
     <row r="13" ht="13.55" customHeight="1">
@@ -8603,7 +9063,7 @@
     </row>
     <row r="14" ht="14.6" customHeight="1">
       <c r="A14" t="s" s="11">
-        <v>258</v>
+        <v>334</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
@@ -8618,7 +9078,7 @@
     </row>
     <row r="15" ht="13.55" customHeight="1">
       <c r="A15" t="s" s="60">
-        <v>259</v>
+        <v>335</v>
       </c>
       <c r="B15" s="16"/>
       <c r="C15" s="16"/>
@@ -8661,7 +9121,7 @@
   <sheetData>
     <row r="1" ht="18.5" customHeight="1">
       <c r="A1" t="s" s="2">
-        <v>260</v>
+        <v>336</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -8684,7 +9144,7 @@
     </row>
     <row r="2" ht="13.65" customHeight="1">
       <c r="A2" t="s" s="5">
-        <v>261</v>
+        <v>337</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -8728,61 +9188,61 @@
     </row>
     <row r="4" ht="27.75" customHeight="1">
       <c r="A4" t="s" s="21">
-        <v>262</v>
+        <v>338</v>
       </c>
       <c r="B4" t="s" s="21">
-        <v>236</v>
+        <v>312</v>
       </c>
       <c r="C4" t="s" s="21">
-        <v>263</v>
+        <v>339</v>
       </c>
       <c r="D4" t="s" s="21">
-        <v>264</v>
+        <v>340</v>
       </c>
       <c r="E4" t="s" s="21">
-        <v>265</v>
+        <v>341</v>
       </c>
       <c r="F4" t="s" s="21">
-        <v>266</v>
+        <v>342</v>
       </c>
       <c r="G4" t="s" s="21">
-        <v>267</v>
+        <v>343</v>
       </c>
       <c r="H4" t="s" s="21">
-        <v>268</v>
+        <v>344</v>
       </c>
       <c r="I4" t="s" s="21">
-        <v>269</v>
+        <v>345</v>
       </c>
       <c r="J4" t="s" s="21">
         <v>22</v>
       </c>
       <c r="K4" t="s" s="21">
-        <v>270</v>
+        <v>346</v>
       </c>
       <c r="L4" t="s" s="21">
-        <v>271</v>
+        <v>347</v>
       </c>
       <c r="M4" t="s" s="21">
-        <v>272</v>
+        <v>348</v>
       </c>
       <c r="N4" t="s" s="21">
-        <v>273</v>
+        <v>349</v>
       </c>
       <c r="O4" t="s" s="21">
-        <v>274</v>
+        <v>350</v>
       </c>
       <c r="P4" t="s" s="21">
-        <v>275</v>
+        <v>351</v>
       </c>
       <c r="Q4" t="s" s="21">
-        <v>276</v>
+        <v>352</v>
       </c>
       <c r="R4" t="s" s="21">
-        <v>277</v>
+        <v>353</v>
       </c>
       <c r="S4" t="s" s="21">
-        <v>278</v>
+        <v>354</v>
       </c>
     </row>
     <row r="5" ht="13.65" customHeight="1">
@@ -11528,7 +11988,7 @@
     </row>
     <row r="46" ht="13.55" customHeight="1">
       <c r="A46" t="s" s="76">
-        <v>279</v>
+        <v>355</v>
       </c>
       <c r="B46" s="6"/>
       <c r="C46" s="6"/>
@@ -11551,7 +12011,7 @@
     </row>
     <row r="47" ht="13.55" customHeight="1">
       <c r="A47" t="s" s="76">
-        <v>280</v>
+        <v>356</v>
       </c>
       <c r="B47" s="6"/>
       <c r="C47" s="6"/>
@@ -11574,7 +12034,7 @@
     </row>
     <row r="48" ht="13.55" customHeight="1">
       <c r="A48" t="s" s="67">
-        <v>281</v>
+        <v>357</v>
       </c>
       <c r="B48" s="16"/>
       <c r="C48" s="16"/>
@@ -11621,7 +12081,7 @@
   <sheetData>
     <row r="1" ht="18.5" customHeight="1">
       <c r="A1" t="s" s="2">
-        <v>282</v>
+        <v>358</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -11634,7 +12094,7 @@
     </row>
     <row r="2" ht="13.65" customHeight="1">
       <c r="A2" t="s" s="5">
-        <v>283</v>
+        <v>359</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -11658,31 +12118,31 @@
     </row>
     <row r="4" ht="27.75" customHeight="1">
       <c r="A4" t="s" s="21">
-        <v>262</v>
+        <v>338</v>
       </c>
       <c r="B4" t="s" s="21">
-        <v>274</v>
+        <v>350</v>
       </c>
       <c r="C4" t="s" s="21">
-        <v>284</v>
+        <v>360</v>
       </c>
       <c r="D4" t="s" s="21">
         <v>147</v>
       </c>
       <c r="E4" t="s" s="21">
-        <v>285</v>
+        <v>361</v>
       </c>
       <c r="F4" t="s" s="21">
-        <v>278</v>
+        <v>354</v>
       </c>
       <c r="G4" t="s" s="21">
-        <v>286</v>
+        <v>362</v>
       </c>
       <c r="H4" t="s" s="21">
-        <v>287</v>
+        <v>363</v>
       </c>
       <c r="I4" t="s" s="21">
-        <v>288</v>
+        <v>364</v>
       </c>
     </row>
     <row r="5" ht="13.65" customHeight="1">
@@ -13178,7 +13638,7 @@
     </row>
     <row r="46" ht="14.6" customHeight="1">
       <c r="A46" t="s" s="11">
-        <v>292</v>
+        <v>368</v>
       </c>
       <c r="B46" s="6"/>
       <c r="C46" s="6"/>
@@ -13191,7 +13651,7 @@
     </row>
     <row r="47" ht="13.55" customHeight="1">
       <c r="A47" t="s" s="84">
-        <v>293</v>
+        <v>369</v>
       </c>
       <c r="B47" s="6"/>
       <c r="C47" s="6"/>
@@ -13215,7 +13675,7 @@
     </row>
     <row r="49" ht="13.55" customHeight="1">
       <c r="A49" t="s" s="84">
-        <v>294</v>
+        <v>370</v>
       </c>
       <c r="B49" s="6"/>
       <c r="C49" s="6"/>
@@ -13228,7 +13688,7 @@
     </row>
     <row r="50" ht="13.55" customHeight="1">
       <c r="A50" t="s" s="84">
-        <v>295</v>
+        <v>371</v>
       </c>
       <c r="B50" s="6"/>
       <c r="C50" s="6"/>
@@ -13241,7 +13701,7 @@
     </row>
     <row r="51" ht="13.55" customHeight="1">
       <c r="A51" t="s" s="84">
-        <v>296</v>
+        <v>372</v>
       </c>
       <c r="B51" s="6"/>
       <c r="C51" s="6"/>
@@ -13265,7 +13725,7 @@
     </row>
     <row r="53" ht="14.6" customHeight="1">
       <c r="A53" t="s" s="11">
-        <v>297</v>
+        <v>373</v>
       </c>
       <c r="B53" s="6"/>
       <c r="C53" s="6"/>
@@ -13278,7 +13738,7 @@
     </row>
     <row r="54" ht="13.55" customHeight="1">
       <c r="A54" t="s" s="84">
-        <v>298</v>
+        <v>374</v>
       </c>
       <c r="B54" s="6"/>
       <c r="C54" s="6"/>
@@ -13291,7 +13751,7 @@
     </row>
     <row r="55" ht="13.55" customHeight="1">
       <c r="A55" t="s" s="60">
-        <v>299</v>
+        <v>375</v>
       </c>
       <c r="B55" s="16"/>
       <c r="C55" s="16"/>

</xml_diff>

<commit_message>
Phase 5: Chiller and Quartermaster; fix burns dealing no damage
Chiller (UPGRADES.md): every frame it chills enemies in range - slow (Field
grows it, Permafrost makes it linger, Absolute Zero slows bosses), brittle
damage amp and armour strip (Brittle / Shatter), and Freeze pulses hard
stops that later deal damage and hold bosses. Chilled enemies turn icy.

Quartermaster: round income scaled by Yield plus Storm Bank interest on
banked cash; Airdrop chests land around it each round for players to run
over; Logistics discounts upgrades and raises sell refunds for towers in
its range (shown in the tower panel). Both towers are now for sale.

Fix: burning patches (Napalm, Incendiary, Dragon's Breath) have dealt no
damage since the hero redesign moved them into Server/Hazards - its step
and init were never wired into Main.

Statically checked; not yet playtested.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Storm-Split-Balance.xlsx
+++ b/Storm-Split-Balance.xlsx
@@ -4182,7 +4182,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66667" defaultRowHeight="15" customHeight="1" outlineLevelRow="0"/>
   <cols>
     <col width="34" customWidth="1" style="81" min="1" max="1"/>
@@ -5077,6 +5077,56 @@
       <c r="D52" s="29" t="inlineStr">
         <is>
           <t>Time between calling an Airburst and the strike landing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="31" t="inlineStr">
+        <is>
+          <t>QUARTERMASTER / CHILLER</t>
+        </is>
+      </c>
+      <c r="B54" s="24" t="n"/>
+      <c r="C54" s="32" t="n"/>
+      <c r="D54" s="32" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="26" t="inlineStr">
+        <is>
+          <t>Chest lifetime</t>
+        </is>
+      </c>
+      <c r="B55" s="30" t="n">
+        <v>20</v>
+      </c>
+      <c r="C55" s="28" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="D55" s="29" t="inlineStr">
+        <is>
+          <t>Airdrop chests vanish if nobody collects them in time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="26" t="inlineStr">
+        <is>
+          <t>Chest spread</t>
+        </is>
+      </c>
+      <c r="B56" s="30" t="n">
+        <v>25</v>
+      </c>
+      <c r="C56" s="28" t="inlineStr">
+        <is>
+          <t>studs</t>
+        </is>
+      </c>
+      <c r="D56" s="29" t="inlineStr">
+        <is>
+          <t>Chests land this far around their Quartermaster at most.</t>
         </is>
       </c>
     </row>
@@ -5100,7 +5150,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66667" defaultRowHeight="15" customHeight="1" outlineLevelRow="0"/>
   <cols>
     <col width="15" customWidth="1" style="81" min="1" max="1"/>
@@ -5229,6 +5279,11 @@
           <t>Splash radius (m)</t>
         </is>
       </c>
+      <c r="M4" s="21" t="inlineStr">
+        <is>
+          <t>Slow %</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="13.65" customHeight="1" s="90">
       <c r="A5" s="43" t="inlineStr">
@@ -5276,6 +5331,9 @@
       <c r="L5" s="27" t="n">
         <v>0</v>
       </c>
+      <c r="M5" s="27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" ht="13.65" customHeight="1" s="90">
       <c r="A6" s="43" t="inlineStr">
@@ -5323,6 +5381,9 @@
       <c r="L6" s="27" t="n">
         <v>0</v>
       </c>
+      <c r="M6" s="27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7" ht="13.65" customHeight="1" s="90">
       <c r="A7" s="43" t="inlineStr">
@@ -5370,6 +5431,9 @@
       <c r="L7" s="27" t="n">
         <v>6</v>
       </c>
+      <c r="M7" s="27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" ht="13.65" customHeight="1" s="90">
       <c r="A8" s="43" t="inlineStr">
@@ -5417,6 +5481,9 @@
       <c r="L8" s="27" t="n">
         <v>6</v>
       </c>
+      <c r="M8" s="27" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="9" ht="13.65" customHeight="1" s="90">
       <c r="A9" s="43" t="inlineStr">
@@ -5446,7 +5513,7 @@
         <v/>
       </c>
       <c r="H9" s="27" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I9" s="46" t="inlineStr">
         <is>
@@ -5462,6 +5529,9 @@
         </is>
       </c>
       <c r="L9" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="27" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5524,7 +5594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD79"/>
+  <dimension ref="A1:AT79"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66667" defaultRowHeight="15" customHeight="1" outlineLevelRow="0"/>
   <cols>
     <col width="15" customWidth="1" style="81" min="1" max="1"/>
@@ -5541,7 +5611,22 @@
     <col width="10" customWidth="1" style="81" min="12" max="12"/>
     <col width="22" customWidth="1" style="81" min="13" max="13"/>
     <col width="12" customWidth="1" style="81" min="14" max="30"/>
-    <col width="8.67188" customWidth="1" style="81" min="31" max="16384"/>
+    <col width="12" customWidth="1" style="81" min="31" max="16384"/>
+    <col width="12" customWidth="1" style="90" min="32" max="32"/>
+    <col width="12" customWidth="1" style="90" min="33" max="33"/>
+    <col width="12" customWidth="1" style="90" min="34" max="34"/>
+    <col width="12" customWidth="1" style="90" min="35" max="35"/>
+    <col width="12" customWidth="1" style="90" min="36" max="36"/>
+    <col width="12" customWidth="1" style="90" min="37" max="37"/>
+    <col width="12" customWidth="1" style="90" min="38" max="38"/>
+    <col width="12" customWidth="1" style="90" min="39" max="39"/>
+    <col width="12" customWidth="1" style="90" min="40" max="40"/>
+    <col width="12" customWidth="1" style="90" min="41" max="41"/>
+    <col width="12" customWidth="1" style="90" min="42" max="42"/>
+    <col width="12" customWidth="1" style="90" min="43" max="43"/>
+    <col width="12" customWidth="1" style="90" min="44" max="44"/>
+    <col width="12" customWidth="1" style="90" min="45" max="45"/>
+    <col width="12" customWidth="1" style="90" min="46" max="46"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.5" customHeight="1" s="90">
@@ -5799,6 +5884,86 @@
           <t>Aura pierces armour</t>
         </is>
       </c>
+      <c r="AE4" s="21" t="inlineStr">
+        <is>
+          <t>Slow %</t>
+        </is>
+      </c>
+      <c r="AF4" s="21" t="inlineStr">
+        <is>
+          <t>Slow linger (s)</t>
+        </is>
+      </c>
+      <c r="AG4" s="21" t="inlineStr">
+        <is>
+          <t>Slows bosses</t>
+        </is>
+      </c>
+      <c r="AH4" s="21" t="inlineStr">
+        <is>
+          <t>Freeze every (s)</t>
+        </is>
+      </c>
+      <c r="AI4" s="21" t="inlineStr">
+        <is>
+          <t>Freeze (s)</t>
+        </is>
+      </c>
+      <c r="AJ4" s="21" t="inlineStr">
+        <is>
+          <t>Freeze damage</t>
+        </is>
+      </c>
+      <c r="AK4" s="21" t="inlineStr">
+        <is>
+          <t>Freeze holds bosses</t>
+        </is>
+      </c>
+      <c r="AL4" s="21" t="inlineStr">
+        <is>
+          <t>Brittle %</t>
+        </is>
+      </c>
+      <c r="AM4" s="21" t="inlineStr">
+        <is>
+          <t>Strips armour</t>
+        </is>
+      </c>
+      <c r="AN4" s="21" t="inlineStr">
+        <is>
+          <t>Income x</t>
+        </is>
+      </c>
+      <c r="AO4" s="21" t="inlineStr">
+        <is>
+          <t>Interest %</t>
+        </is>
+      </c>
+      <c r="AP4" s="21" t="inlineStr">
+        <is>
+          <t>Interest cap</t>
+        </is>
+      </c>
+      <c r="AQ4" s="21" t="inlineStr">
+        <is>
+          <t>Chests</t>
+        </is>
+      </c>
+      <c r="AR4" s="21" t="inlineStr">
+        <is>
+          <t>Chest cash</t>
+        </is>
+      </c>
+      <c r="AS4" s="21" t="inlineStr">
+        <is>
+          <t>Upgrade discount %</t>
+        </is>
+      </c>
+      <c r="AT4" s="21" t="inlineStr">
+        <is>
+          <t>Sell refund</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="13.65" customHeight="1" s="90">
       <c r="A5" s="43" t="inlineStr">
@@ -5869,6 +6034,22 @@
       <c r="AB5" s="57" t="n"/>
       <c r="AC5" s="57" t="n"/>
       <c r="AD5" s="57" t="n"/>
+      <c r="AE5" s="57" t="n"/>
+      <c r="AF5" s="57" t="n"/>
+      <c r="AG5" s="57" t="n"/>
+      <c r="AH5" s="57" t="n"/>
+      <c r="AI5" s="57" t="n"/>
+      <c r="AJ5" s="57" t="n"/>
+      <c r="AK5" s="57" t="n"/>
+      <c r="AL5" s="57" t="n"/>
+      <c r="AM5" s="57" t="n"/>
+      <c r="AN5" s="57" t="n"/>
+      <c r="AO5" s="57" t="n"/>
+      <c r="AP5" s="57" t="n"/>
+      <c r="AQ5" s="57" t="n"/>
+      <c r="AR5" s="57" t="n"/>
+      <c r="AS5" s="57" t="n"/>
+      <c r="AT5" s="57" t="n"/>
     </row>
     <row r="6" ht="13.65" customHeight="1" s="90">
       <c r="A6" s="43" t="inlineStr">
@@ -5939,6 +6120,22 @@
       <c r="AB6" s="57" t="n"/>
       <c r="AC6" s="57" t="n"/>
       <c r="AD6" s="57" t="n"/>
+      <c r="AE6" s="57" t="n"/>
+      <c r="AF6" s="57" t="n"/>
+      <c r="AG6" s="57" t="n"/>
+      <c r="AH6" s="57" t="n"/>
+      <c r="AI6" s="57" t="n"/>
+      <c r="AJ6" s="57" t="n"/>
+      <c r="AK6" s="57" t="n"/>
+      <c r="AL6" s="57" t="n"/>
+      <c r="AM6" s="57" t="n"/>
+      <c r="AN6" s="57" t="n"/>
+      <c r="AO6" s="57" t="n"/>
+      <c r="AP6" s="57" t="n"/>
+      <c r="AQ6" s="57" t="n"/>
+      <c r="AR6" s="57" t="n"/>
+      <c r="AS6" s="57" t="n"/>
+      <c r="AT6" s="57" t="n"/>
     </row>
     <row r="7" ht="13.65" customHeight="1" s="90">
       <c r="A7" s="43" t="inlineStr">
@@ -6011,6 +6208,22 @@
       </c>
       <c r="AC7" s="57" t="n"/>
       <c r="AD7" s="57" t="n"/>
+      <c r="AE7" s="57" t="n"/>
+      <c r="AF7" s="57" t="n"/>
+      <c r="AG7" s="57" t="n"/>
+      <c r="AH7" s="57" t="n"/>
+      <c r="AI7" s="57" t="n"/>
+      <c r="AJ7" s="57" t="n"/>
+      <c r="AK7" s="57" t="n"/>
+      <c r="AL7" s="57" t="n"/>
+      <c r="AM7" s="57" t="n"/>
+      <c r="AN7" s="57" t="n"/>
+      <c r="AO7" s="57" t="n"/>
+      <c r="AP7" s="57" t="n"/>
+      <c r="AQ7" s="57" t="n"/>
+      <c r="AR7" s="57" t="n"/>
+      <c r="AS7" s="57" t="n"/>
+      <c r="AT7" s="57" t="n"/>
     </row>
     <row r="8" ht="13.65" customHeight="1" s="90">
       <c r="A8" s="43" t="inlineStr">
@@ -6083,6 +6296,22 @@
       </c>
       <c r="AC8" s="57" t="n"/>
       <c r="AD8" s="57" t="n"/>
+      <c r="AE8" s="57" t="n"/>
+      <c r="AF8" s="57" t="n"/>
+      <c r="AG8" s="57" t="n"/>
+      <c r="AH8" s="57" t="n"/>
+      <c r="AI8" s="57" t="n"/>
+      <c r="AJ8" s="57" t="n"/>
+      <c r="AK8" s="57" t="n"/>
+      <c r="AL8" s="57" t="n"/>
+      <c r="AM8" s="57" t="n"/>
+      <c r="AN8" s="57" t="n"/>
+      <c r="AO8" s="57" t="n"/>
+      <c r="AP8" s="57" t="n"/>
+      <c r="AQ8" s="57" t="n"/>
+      <c r="AR8" s="57" t="n"/>
+      <c r="AS8" s="57" t="n"/>
+      <c r="AT8" s="57" t="n"/>
     </row>
     <row r="9" ht="13.65" customHeight="1" s="90">
       <c r="A9" s="43" t="inlineStr">
@@ -6161,6 +6390,22 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="AE9" s="57" t="n"/>
+      <c r="AF9" s="57" t="n"/>
+      <c r="AG9" s="57" t="n"/>
+      <c r="AH9" s="57" t="n"/>
+      <c r="AI9" s="57" t="n"/>
+      <c r="AJ9" s="57" t="n"/>
+      <c r="AK9" s="57" t="n"/>
+      <c r="AL9" s="57" t="n"/>
+      <c r="AM9" s="57" t="n"/>
+      <c r="AN9" s="57" t="n"/>
+      <c r="AO9" s="57" t="n"/>
+      <c r="AP9" s="57" t="n"/>
+      <c r="AQ9" s="57" t="n"/>
+      <c r="AR9" s="57" t="n"/>
+      <c r="AS9" s="57" t="n"/>
+      <c r="AT9" s="57" t="n"/>
     </row>
     <row r="10" ht="13.65" customHeight="1" s="90">
       <c r="A10" s="43" t="inlineStr">
@@ -6231,6 +6476,22 @@
       <c r="AB10" s="57" t="n"/>
       <c r="AC10" s="57" t="n"/>
       <c r="AD10" s="57" t="n"/>
+      <c r="AE10" s="57" t="n"/>
+      <c r="AF10" s="57" t="n"/>
+      <c r="AG10" s="57" t="n"/>
+      <c r="AH10" s="57" t="n"/>
+      <c r="AI10" s="57" t="n"/>
+      <c r="AJ10" s="57" t="n"/>
+      <c r="AK10" s="57" t="n"/>
+      <c r="AL10" s="57" t="n"/>
+      <c r="AM10" s="57" t="n"/>
+      <c r="AN10" s="57" t="n"/>
+      <c r="AO10" s="57" t="n"/>
+      <c r="AP10" s="57" t="n"/>
+      <c r="AQ10" s="57" t="n"/>
+      <c r="AR10" s="57" t="n"/>
+      <c r="AS10" s="57" t="n"/>
+      <c r="AT10" s="57" t="n"/>
     </row>
     <row r="11" ht="13.65" customHeight="1" s="90">
       <c r="A11" s="43" t="inlineStr">
@@ -6301,6 +6562,22 @@
       <c r="AB11" s="57" t="n"/>
       <c r="AC11" s="57" t="n"/>
       <c r="AD11" s="57" t="n"/>
+      <c r="AE11" s="57" t="n"/>
+      <c r="AF11" s="57" t="n"/>
+      <c r="AG11" s="57" t="n"/>
+      <c r="AH11" s="57" t="n"/>
+      <c r="AI11" s="57" t="n"/>
+      <c r="AJ11" s="57" t="n"/>
+      <c r="AK11" s="57" t="n"/>
+      <c r="AL11" s="57" t="n"/>
+      <c r="AM11" s="57" t="n"/>
+      <c r="AN11" s="57" t="n"/>
+      <c r="AO11" s="57" t="n"/>
+      <c r="AP11" s="57" t="n"/>
+      <c r="AQ11" s="57" t="n"/>
+      <c r="AR11" s="57" t="n"/>
+      <c r="AS11" s="57" t="n"/>
+      <c r="AT11" s="57" t="n"/>
     </row>
     <row r="12" ht="13.65" customHeight="1" s="90">
       <c r="A12" s="43" t="inlineStr">
@@ -6373,6 +6650,22 @@
       <c r="AB12" s="57" t="n"/>
       <c r="AC12" s="57" t="n"/>
       <c r="AD12" s="57" t="n"/>
+      <c r="AE12" s="57" t="n"/>
+      <c r="AF12" s="57" t="n"/>
+      <c r="AG12" s="57" t="n"/>
+      <c r="AH12" s="57" t="n"/>
+      <c r="AI12" s="57" t="n"/>
+      <c r="AJ12" s="57" t="n"/>
+      <c r="AK12" s="57" t="n"/>
+      <c r="AL12" s="57" t="n"/>
+      <c r="AM12" s="57" t="n"/>
+      <c r="AN12" s="57" t="n"/>
+      <c r="AO12" s="57" t="n"/>
+      <c r="AP12" s="57" t="n"/>
+      <c r="AQ12" s="57" t="n"/>
+      <c r="AR12" s="57" t="n"/>
+      <c r="AS12" s="57" t="n"/>
+      <c r="AT12" s="57" t="n"/>
     </row>
     <row r="13" ht="13.65" customHeight="1" s="90">
       <c r="A13" s="43" t="inlineStr">
@@ -6445,6 +6738,22 @@
       <c r="AB13" s="57" t="n"/>
       <c r="AC13" s="57" t="n"/>
       <c r="AD13" s="57" t="n"/>
+      <c r="AE13" s="57" t="n"/>
+      <c r="AF13" s="57" t="n"/>
+      <c r="AG13" s="57" t="n"/>
+      <c r="AH13" s="57" t="n"/>
+      <c r="AI13" s="57" t="n"/>
+      <c r="AJ13" s="57" t="n"/>
+      <c r="AK13" s="57" t="n"/>
+      <c r="AL13" s="57" t="n"/>
+      <c r="AM13" s="57" t="n"/>
+      <c r="AN13" s="57" t="n"/>
+      <c r="AO13" s="57" t="n"/>
+      <c r="AP13" s="57" t="n"/>
+      <c r="AQ13" s="57" t="n"/>
+      <c r="AR13" s="57" t="n"/>
+      <c r="AS13" s="57" t="n"/>
+      <c r="AT13" s="57" t="n"/>
     </row>
     <row r="14" ht="13.65" customHeight="1" s="90">
       <c r="A14" s="43" t="inlineStr">
@@ -6517,6 +6826,22 @@
       <c r="AB14" s="57" t="n"/>
       <c r="AC14" s="57" t="n"/>
       <c r="AD14" s="57" t="n"/>
+      <c r="AE14" s="57" t="n"/>
+      <c r="AF14" s="57" t="n"/>
+      <c r="AG14" s="57" t="n"/>
+      <c r="AH14" s="57" t="n"/>
+      <c r="AI14" s="57" t="n"/>
+      <c r="AJ14" s="57" t="n"/>
+      <c r="AK14" s="57" t="n"/>
+      <c r="AL14" s="57" t="n"/>
+      <c r="AM14" s="57" t="n"/>
+      <c r="AN14" s="57" t="n"/>
+      <c r="AO14" s="57" t="n"/>
+      <c r="AP14" s="57" t="n"/>
+      <c r="AQ14" s="57" t="n"/>
+      <c r="AR14" s="57" t="n"/>
+      <c r="AS14" s="57" t="n"/>
+      <c r="AT14" s="57" t="n"/>
     </row>
     <row r="15" ht="13.65" customHeight="1" s="90">
       <c r="A15" s="43" t="inlineStr">
@@ -6587,6 +6912,22 @@
       <c r="AB15" s="57" t="n"/>
       <c r="AC15" s="57" t="n"/>
       <c r="AD15" s="57" t="n"/>
+      <c r="AE15" s="57" t="n"/>
+      <c r="AF15" s="57" t="n"/>
+      <c r="AG15" s="57" t="n"/>
+      <c r="AH15" s="57" t="n"/>
+      <c r="AI15" s="57" t="n"/>
+      <c r="AJ15" s="57" t="n"/>
+      <c r="AK15" s="57" t="n"/>
+      <c r="AL15" s="57" t="n"/>
+      <c r="AM15" s="57" t="n"/>
+      <c r="AN15" s="57" t="n"/>
+      <c r="AO15" s="57" t="n"/>
+      <c r="AP15" s="57" t="n"/>
+      <c r="AQ15" s="57" t="n"/>
+      <c r="AR15" s="57" t="n"/>
+      <c r="AS15" s="57" t="n"/>
+      <c r="AT15" s="57" t="n"/>
     </row>
     <row r="16" ht="13.65" customHeight="1" s="90">
       <c r="A16" s="43" t="inlineStr">
@@ -6661,6 +7002,22 @@
       <c r="AB16" s="57" t="n"/>
       <c r="AC16" s="57" t="n"/>
       <c r="AD16" s="57" t="n"/>
+      <c r="AE16" s="57" t="n"/>
+      <c r="AF16" s="57" t="n"/>
+      <c r="AG16" s="57" t="n"/>
+      <c r="AH16" s="57" t="n"/>
+      <c r="AI16" s="57" t="n"/>
+      <c r="AJ16" s="57" t="n"/>
+      <c r="AK16" s="57" t="n"/>
+      <c r="AL16" s="57" t="n"/>
+      <c r="AM16" s="57" t="n"/>
+      <c r="AN16" s="57" t="n"/>
+      <c r="AO16" s="57" t="n"/>
+      <c r="AP16" s="57" t="n"/>
+      <c r="AQ16" s="57" t="n"/>
+      <c r="AR16" s="57" t="n"/>
+      <c r="AS16" s="57" t="n"/>
+      <c r="AT16" s="57" t="n"/>
     </row>
     <row r="17" ht="13.65" customHeight="1" s="90">
       <c r="A17" s="43" t="inlineStr">
@@ -6737,6 +7094,22 @@
       <c r="AB17" s="57" t="n"/>
       <c r="AC17" s="57" t="n"/>
       <c r="AD17" s="57" t="n"/>
+      <c r="AE17" s="57" t="n"/>
+      <c r="AF17" s="57" t="n"/>
+      <c r="AG17" s="57" t="n"/>
+      <c r="AH17" s="57" t="n"/>
+      <c r="AI17" s="57" t="n"/>
+      <c r="AJ17" s="57" t="n"/>
+      <c r="AK17" s="57" t="n"/>
+      <c r="AL17" s="57" t="n"/>
+      <c r="AM17" s="57" t="n"/>
+      <c r="AN17" s="57" t="n"/>
+      <c r="AO17" s="57" t="n"/>
+      <c r="AP17" s="57" t="n"/>
+      <c r="AQ17" s="57" t="n"/>
+      <c r="AR17" s="57" t="n"/>
+      <c r="AS17" s="57" t="n"/>
+      <c r="AT17" s="57" t="n"/>
     </row>
     <row r="18" ht="13.65" customHeight="1" s="90">
       <c r="A18" s="43" t="inlineStr">
@@ -6815,6 +7188,22 @@
       <c r="AB18" s="57" t="n"/>
       <c r="AC18" s="57" t="n"/>
       <c r="AD18" s="57" t="n"/>
+      <c r="AE18" s="57" t="n"/>
+      <c r="AF18" s="57" t="n"/>
+      <c r="AG18" s="57" t="n"/>
+      <c r="AH18" s="57" t="n"/>
+      <c r="AI18" s="57" t="n"/>
+      <c r="AJ18" s="57" t="n"/>
+      <c r="AK18" s="57" t="n"/>
+      <c r="AL18" s="57" t="n"/>
+      <c r="AM18" s="57" t="n"/>
+      <c r="AN18" s="57" t="n"/>
+      <c r="AO18" s="57" t="n"/>
+      <c r="AP18" s="57" t="n"/>
+      <c r="AQ18" s="57" t="n"/>
+      <c r="AR18" s="57" t="n"/>
+      <c r="AS18" s="57" t="n"/>
+      <c r="AT18" s="57" t="n"/>
     </row>
     <row r="19" ht="13.65" customHeight="1" s="90">
       <c r="A19" s="43" t="inlineStr">
@@ -6895,6 +7284,22 @@
       <c r="AB19" s="57" t="n"/>
       <c r="AC19" s="57" t="n"/>
       <c r="AD19" s="57" t="n"/>
+      <c r="AE19" s="57" t="n"/>
+      <c r="AF19" s="57" t="n"/>
+      <c r="AG19" s="57" t="n"/>
+      <c r="AH19" s="57" t="n"/>
+      <c r="AI19" s="57" t="n"/>
+      <c r="AJ19" s="57" t="n"/>
+      <c r="AK19" s="57" t="n"/>
+      <c r="AL19" s="57" t="n"/>
+      <c r="AM19" s="57" t="n"/>
+      <c r="AN19" s="57" t="n"/>
+      <c r="AO19" s="57" t="n"/>
+      <c r="AP19" s="57" t="n"/>
+      <c r="AQ19" s="57" t="n"/>
+      <c r="AR19" s="57" t="n"/>
+      <c r="AS19" s="57" t="n"/>
+      <c r="AT19" s="57" t="n"/>
     </row>
     <row r="20" ht="13.65" customHeight="1" s="90">
       <c r="A20" s="43" t="inlineStr">
@@ -6967,6 +7372,22 @@
       <c r="AB20" s="57" t="n"/>
       <c r="AC20" s="57" t="n"/>
       <c r="AD20" s="57" t="n"/>
+      <c r="AE20" s="57" t="n"/>
+      <c r="AF20" s="57" t="n"/>
+      <c r="AG20" s="57" t="n"/>
+      <c r="AH20" s="57" t="n"/>
+      <c r="AI20" s="57" t="n"/>
+      <c r="AJ20" s="57" t="n"/>
+      <c r="AK20" s="57" t="n"/>
+      <c r="AL20" s="57" t="n"/>
+      <c r="AM20" s="57" t="n"/>
+      <c r="AN20" s="57" t="n"/>
+      <c r="AO20" s="57" t="n"/>
+      <c r="AP20" s="57" t="n"/>
+      <c r="AQ20" s="57" t="n"/>
+      <c r="AR20" s="57" t="n"/>
+      <c r="AS20" s="57" t="n"/>
+      <c r="AT20" s="57" t="n"/>
     </row>
     <row r="21" ht="13.65" customHeight="1" s="90">
       <c r="A21" s="43" t="inlineStr">
@@ -7043,6 +7464,22 @@
       <c r="AB21" s="57" t="n"/>
       <c r="AC21" s="57" t="n"/>
       <c r="AD21" s="57" t="n"/>
+      <c r="AE21" s="57" t="n"/>
+      <c r="AF21" s="57" t="n"/>
+      <c r="AG21" s="57" t="n"/>
+      <c r="AH21" s="57" t="n"/>
+      <c r="AI21" s="57" t="n"/>
+      <c r="AJ21" s="57" t="n"/>
+      <c r="AK21" s="57" t="n"/>
+      <c r="AL21" s="57" t="n"/>
+      <c r="AM21" s="57" t="n"/>
+      <c r="AN21" s="57" t="n"/>
+      <c r="AO21" s="57" t="n"/>
+      <c r="AP21" s="57" t="n"/>
+      <c r="AQ21" s="57" t="n"/>
+      <c r="AR21" s="57" t="n"/>
+      <c r="AS21" s="57" t="n"/>
+      <c r="AT21" s="57" t="n"/>
     </row>
     <row r="22" ht="13.65" customHeight="1" s="90">
       <c r="A22" s="43" t="inlineStr">
@@ -7119,6 +7556,22 @@
       <c r="AB22" s="57" t="n"/>
       <c r="AC22" s="57" t="n"/>
       <c r="AD22" s="57" t="n"/>
+      <c r="AE22" s="57" t="n"/>
+      <c r="AF22" s="57" t="n"/>
+      <c r="AG22" s="57" t="n"/>
+      <c r="AH22" s="57" t="n"/>
+      <c r="AI22" s="57" t="n"/>
+      <c r="AJ22" s="57" t="n"/>
+      <c r="AK22" s="57" t="n"/>
+      <c r="AL22" s="57" t="n"/>
+      <c r="AM22" s="57" t="n"/>
+      <c r="AN22" s="57" t="n"/>
+      <c r="AO22" s="57" t="n"/>
+      <c r="AP22" s="57" t="n"/>
+      <c r="AQ22" s="57" t="n"/>
+      <c r="AR22" s="57" t="n"/>
+      <c r="AS22" s="57" t="n"/>
+      <c r="AT22" s="57" t="n"/>
     </row>
     <row r="23" ht="13.65" customHeight="1" s="90">
       <c r="A23" s="43" t="inlineStr">
@@ -7195,6 +7648,22 @@
       <c r="AB23" s="57" t="n"/>
       <c r="AC23" s="57" t="n"/>
       <c r="AD23" s="57" t="n"/>
+      <c r="AE23" s="57" t="n"/>
+      <c r="AF23" s="57" t="n"/>
+      <c r="AG23" s="57" t="n"/>
+      <c r="AH23" s="57" t="n"/>
+      <c r="AI23" s="57" t="n"/>
+      <c r="AJ23" s="57" t="n"/>
+      <c r="AK23" s="57" t="n"/>
+      <c r="AL23" s="57" t="n"/>
+      <c r="AM23" s="57" t="n"/>
+      <c r="AN23" s="57" t="n"/>
+      <c r="AO23" s="57" t="n"/>
+      <c r="AP23" s="57" t="n"/>
+      <c r="AQ23" s="57" t="n"/>
+      <c r="AR23" s="57" t="n"/>
+      <c r="AS23" s="57" t="n"/>
+      <c r="AT23" s="57" t="n"/>
     </row>
     <row r="24" ht="13.65" customHeight="1" s="90">
       <c r="A24" s="43" t="inlineStr">
@@ -7271,6 +7740,22 @@
       <c r="AB24" s="57" t="n"/>
       <c r="AC24" s="57" t="n"/>
       <c r="AD24" s="57" t="n"/>
+      <c r="AE24" s="57" t="n"/>
+      <c r="AF24" s="57" t="n"/>
+      <c r="AG24" s="57" t="n"/>
+      <c r="AH24" s="57" t="n"/>
+      <c r="AI24" s="57" t="n"/>
+      <c r="AJ24" s="57" t="n"/>
+      <c r="AK24" s="57" t="n"/>
+      <c r="AL24" s="57" t="n"/>
+      <c r="AM24" s="57" t="n"/>
+      <c r="AN24" s="57" t="n"/>
+      <c r="AO24" s="57" t="n"/>
+      <c r="AP24" s="57" t="n"/>
+      <c r="AQ24" s="57" t="n"/>
+      <c r="AR24" s="57" t="n"/>
+      <c r="AS24" s="57" t="n"/>
+      <c r="AT24" s="57" t="n"/>
     </row>
     <row r="25" ht="13.65" customHeight="1" s="90">
       <c r="A25" s="43" t="inlineStr">
@@ -7341,6 +7826,22 @@
       <c r="AB25" s="57" t="n"/>
       <c r="AC25" s="57" t="n"/>
       <c r="AD25" s="57" t="n"/>
+      <c r="AE25" s="57" t="n"/>
+      <c r="AF25" s="57" t="n"/>
+      <c r="AG25" s="57" t="n"/>
+      <c r="AH25" s="57" t="n"/>
+      <c r="AI25" s="57" t="n"/>
+      <c r="AJ25" s="57" t="n"/>
+      <c r="AK25" s="57" t="n"/>
+      <c r="AL25" s="57" t="n"/>
+      <c r="AM25" s="57" t="n"/>
+      <c r="AN25" s="57" t="n"/>
+      <c r="AO25" s="57" t="n"/>
+      <c r="AP25" s="57" t="n"/>
+      <c r="AQ25" s="57" t="n"/>
+      <c r="AR25" s="57" t="n"/>
+      <c r="AS25" s="57" t="n"/>
+      <c r="AT25" s="57" t="n"/>
     </row>
     <row r="26" ht="13.65" customHeight="1" s="90">
       <c r="A26" s="43" t="inlineStr">
@@ -7411,6 +7912,22 @@
       <c r="AB26" s="57" t="n"/>
       <c r="AC26" s="57" t="n"/>
       <c r="AD26" s="57" t="n"/>
+      <c r="AE26" s="57" t="n"/>
+      <c r="AF26" s="57" t="n"/>
+      <c r="AG26" s="57" t="n"/>
+      <c r="AH26" s="57" t="n"/>
+      <c r="AI26" s="57" t="n"/>
+      <c r="AJ26" s="57" t="n"/>
+      <c r="AK26" s="57" t="n"/>
+      <c r="AL26" s="57" t="n"/>
+      <c r="AM26" s="57" t="n"/>
+      <c r="AN26" s="57" t="n"/>
+      <c r="AO26" s="57" t="n"/>
+      <c r="AP26" s="57" t="n"/>
+      <c r="AQ26" s="57" t="n"/>
+      <c r="AR26" s="57" t="n"/>
+      <c r="AS26" s="57" t="n"/>
+      <c r="AT26" s="57" t="n"/>
     </row>
     <row r="27" ht="13.65" customHeight="1" s="90">
       <c r="A27" s="43" t="inlineStr">
@@ -7483,6 +8000,22 @@
       <c r="AB27" s="57" t="n"/>
       <c r="AC27" s="57" t="n"/>
       <c r="AD27" s="57" t="n"/>
+      <c r="AE27" s="57" t="n"/>
+      <c r="AF27" s="57" t="n"/>
+      <c r="AG27" s="57" t="n"/>
+      <c r="AH27" s="57" t="n"/>
+      <c r="AI27" s="57" t="n"/>
+      <c r="AJ27" s="57" t="n"/>
+      <c r="AK27" s="57" t="n"/>
+      <c r="AL27" s="57" t="n"/>
+      <c r="AM27" s="57" t="n"/>
+      <c r="AN27" s="57" t="n"/>
+      <c r="AO27" s="57" t="n"/>
+      <c r="AP27" s="57" t="n"/>
+      <c r="AQ27" s="57" t="n"/>
+      <c r="AR27" s="57" t="n"/>
+      <c r="AS27" s="57" t="n"/>
+      <c r="AT27" s="57" t="n"/>
     </row>
     <row r="28" ht="13.65" customHeight="1" s="90">
       <c r="A28" s="43" t="inlineStr">
@@ -7555,6 +8088,22 @@
       <c r="AB28" s="57" t="n"/>
       <c r="AC28" s="57" t="n"/>
       <c r="AD28" s="57" t="n"/>
+      <c r="AE28" s="57" t="n"/>
+      <c r="AF28" s="57" t="n"/>
+      <c r="AG28" s="57" t="n"/>
+      <c r="AH28" s="57" t="n"/>
+      <c r="AI28" s="57" t="n"/>
+      <c r="AJ28" s="57" t="n"/>
+      <c r="AK28" s="57" t="n"/>
+      <c r="AL28" s="57" t="n"/>
+      <c r="AM28" s="57" t="n"/>
+      <c r="AN28" s="57" t="n"/>
+      <c r="AO28" s="57" t="n"/>
+      <c r="AP28" s="57" t="n"/>
+      <c r="AQ28" s="57" t="n"/>
+      <c r="AR28" s="57" t="n"/>
+      <c r="AS28" s="57" t="n"/>
+      <c r="AT28" s="57" t="n"/>
     </row>
     <row r="29" ht="13.65" customHeight="1" s="90">
       <c r="A29" s="43" t="inlineStr">
@@ -7629,6 +8178,22 @@
       </c>
       <c r="AC29" s="57" t="n"/>
       <c r="AD29" s="57" t="n"/>
+      <c r="AE29" s="57" t="n"/>
+      <c r="AF29" s="57" t="n"/>
+      <c r="AG29" s="57" t="n"/>
+      <c r="AH29" s="57" t="n"/>
+      <c r="AI29" s="57" t="n"/>
+      <c r="AJ29" s="57" t="n"/>
+      <c r="AK29" s="57" t="n"/>
+      <c r="AL29" s="57" t="n"/>
+      <c r="AM29" s="57" t="n"/>
+      <c r="AN29" s="57" t="n"/>
+      <c r="AO29" s="57" t="n"/>
+      <c r="AP29" s="57" t="n"/>
+      <c r="AQ29" s="57" t="n"/>
+      <c r="AR29" s="57" t="n"/>
+      <c r="AS29" s="57" t="n"/>
+      <c r="AT29" s="57" t="n"/>
     </row>
     <row r="30" ht="13.65" customHeight="1" s="90">
       <c r="A30" s="43" t="inlineStr">
@@ -7699,6 +8264,22 @@
       <c r="AB30" s="57" t="n"/>
       <c r="AC30" s="57" t="n"/>
       <c r="AD30" s="57" t="n"/>
+      <c r="AE30" s="57" t="n"/>
+      <c r="AF30" s="57" t="n"/>
+      <c r="AG30" s="57" t="n"/>
+      <c r="AH30" s="57" t="n"/>
+      <c r="AI30" s="57" t="n"/>
+      <c r="AJ30" s="57" t="n"/>
+      <c r="AK30" s="57" t="n"/>
+      <c r="AL30" s="57" t="n"/>
+      <c r="AM30" s="57" t="n"/>
+      <c r="AN30" s="57" t="n"/>
+      <c r="AO30" s="57" t="n"/>
+      <c r="AP30" s="57" t="n"/>
+      <c r="AQ30" s="57" t="n"/>
+      <c r="AR30" s="57" t="n"/>
+      <c r="AS30" s="57" t="n"/>
+      <c r="AT30" s="57" t="n"/>
     </row>
     <row r="31" ht="13.65" customHeight="1" s="90">
       <c r="A31" s="43" t="inlineStr">
@@ -7771,6 +8352,22 @@
       <c r="AB31" s="57" t="n"/>
       <c r="AC31" s="57" t="n"/>
       <c r="AD31" s="57" t="n"/>
+      <c r="AE31" s="57" t="n"/>
+      <c r="AF31" s="57" t="n"/>
+      <c r="AG31" s="57" t="n"/>
+      <c r="AH31" s="57" t="n"/>
+      <c r="AI31" s="57" t="n"/>
+      <c r="AJ31" s="57" t="n"/>
+      <c r="AK31" s="57" t="n"/>
+      <c r="AL31" s="57" t="n"/>
+      <c r="AM31" s="57" t="n"/>
+      <c r="AN31" s="57" t="n"/>
+      <c r="AO31" s="57" t="n"/>
+      <c r="AP31" s="57" t="n"/>
+      <c r="AQ31" s="57" t="n"/>
+      <c r="AR31" s="57" t="n"/>
+      <c r="AS31" s="57" t="n"/>
+      <c r="AT31" s="57" t="n"/>
     </row>
     <row r="32" ht="13.65" customHeight="1" s="90">
       <c r="A32" s="43" t="inlineStr">
@@ -7845,6 +8442,22 @@
       <c r="AB32" s="57" t="n"/>
       <c r="AC32" s="57" t="n"/>
       <c r="AD32" s="57" t="n"/>
+      <c r="AE32" s="57" t="n"/>
+      <c r="AF32" s="57" t="n"/>
+      <c r="AG32" s="57" t="n"/>
+      <c r="AH32" s="57" t="n"/>
+      <c r="AI32" s="57" t="n"/>
+      <c r="AJ32" s="57" t="n"/>
+      <c r="AK32" s="57" t="n"/>
+      <c r="AL32" s="57" t="n"/>
+      <c r="AM32" s="57" t="n"/>
+      <c r="AN32" s="57" t="n"/>
+      <c r="AO32" s="57" t="n"/>
+      <c r="AP32" s="57" t="n"/>
+      <c r="AQ32" s="57" t="n"/>
+      <c r="AR32" s="57" t="n"/>
+      <c r="AS32" s="57" t="n"/>
+      <c r="AT32" s="57" t="n"/>
     </row>
     <row r="33" ht="13.65" customHeight="1" s="90">
       <c r="A33" s="43" t="inlineStr">
@@ -7919,6 +8532,22 @@
       <c r="AB33" s="57" t="n"/>
       <c r="AC33" s="57" t="n"/>
       <c r="AD33" s="57" t="n"/>
+      <c r="AE33" s="57" t="n"/>
+      <c r="AF33" s="57" t="n"/>
+      <c r="AG33" s="57" t="n"/>
+      <c r="AH33" s="57" t="n"/>
+      <c r="AI33" s="57" t="n"/>
+      <c r="AJ33" s="57" t="n"/>
+      <c r="AK33" s="57" t="n"/>
+      <c r="AL33" s="57" t="n"/>
+      <c r="AM33" s="57" t="n"/>
+      <c r="AN33" s="57" t="n"/>
+      <c r="AO33" s="57" t="n"/>
+      <c r="AP33" s="57" t="n"/>
+      <c r="AQ33" s="57" t="n"/>
+      <c r="AR33" s="57" t="n"/>
+      <c r="AS33" s="57" t="n"/>
+      <c r="AT33" s="57" t="n"/>
     </row>
     <row r="34" ht="13.65" customHeight="1" s="90">
       <c r="A34" s="43" t="inlineStr">
@@ -7997,6 +8626,22 @@
       <c r="AB34" s="57" t="n"/>
       <c r="AC34" s="57" t="n"/>
       <c r="AD34" s="57" t="n"/>
+      <c r="AE34" s="57" t="n"/>
+      <c r="AF34" s="57" t="n"/>
+      <c r="AG34" s="57" t="n"/>
+      <c r="AH34" s="57" t="n"/>
+      <c r="AI34" s="57" t="n"/>
+      <c r="AJ34" s="57" t="n"/>
+      <c r="AK34" s="57" t="n"/>
+      <c r="AL34" s="57" t="n"/>
+      <c r="AM34" s="57" t="n"/>
+      <c r="AN34" s="57" t="n"/>
+      <c r="AO34" s="57" t="n"/>
+      <c r="AP34" s="57" t="n"/>
+      <c r="AQ34" s="57" t="n"/>
+      <c r="AR34" s="57" t="n"/>
+      <c r="AS34" s="57" t="n"/>
+      <c r="AT34" s="57" t="n"/>
     </row>
     <row r="35" ht="13.65" customHeight="1" s="90">
       <c r="A35" s="43" t="inlineStr">
@@ -8069,6 +8714,22 @@
       <c r="AB35" s="57" t="n"/>
       <c r="AC35" s="57" t="n"/>
       <c r="AD35" s="57" t="n"/>
+      <c r="AE35" s="57" t="n"/>
+      <c r="AF35" s="57" t="n"/>
+      <c r="AG35" s="57" t="n"/>
+      <c r="AH35" s="57" t="n"/>
+      <c r="AI35" s="57" t="n"/>
+      <c r="AJ35" s="57" t="n"/>
+      <c r="AK35" s="57" t="n"/>
+      <c r="AL35" s="57" t="n"/>
+      <c r="AM35" s="57" t="n"/>
+      <c r="AN35" s="57" t="n"/>
+      <c r="AO35" s="57" t="n"/>
+      <c r="AP35" s="57" t="n"/>
+      <c r="AQ35" s="57" t="n"/>
+      <c r="AR35" s="57" t="n"/>
+      <c r="AS35" s="57" t="n"/>
+      <c r="AT35" s="57" t="n"/>
     </row>
     <row r="36" ht="13.65" customHeight="1" s="90">
       <c r="A36" s="43" t="inlineStr">
@@ -8141,6 +8802,22 @@
       <c r="AB36" s="57" t="n"/>
       <c r="AC36" s="57" t="n"/>
       <c r="AD36" s="57" t="n"/>
+      <c r="AE36" s="57" t="n"/>
+      <c r="AF36" s="57" t="n"/>
+      <c r="AG36" s="57" t="n"/>
+      <c r="AH36" s="57" t="n"/>
+      <c r="AI36" s="57" t="n"/>
+      <c r="AJ36" s="57" t="n"/>
+      <c r="AK36" s="57" t="n"/>
+      <c r="AL36" s="57" t="n"/>
+      <c r="AM36" s="57" t="n"/>
+      <c r="AN36" s="57" t="n"/>
+      <c r="AO36" s="57" t="n"/>
+      <c r="AP36" s="57" t="n"/>
+      <c r="AQ36" s="57" t="n"/>
+      <c r="AR36" s="57" t="n"/>
+      <c r="AS36" s="57" t="n"/>
+      <c r="AT36" s="57" t="n"/>
     </row>
     <row r="37" ht="13.65" customHeight="1" s="90">
       <c r="A37" s="43" t="inlineStr">
@@ -8217,6 +8894,22 @@
       <c r="AB37" s="57" t="n"/>
       <c r="AC37" s="57" t="n"/>
       <c r="AD37" s="57" t="n"/>
+      <c r="AE37" s="57" t="n"/>
+      <c r="AF37" s="57" t="n"/>
+      <c r="AG37" s="57" t="n"/>
+      <c r="AH37" s="57" t="n"/>
+      <c r="AI37" s="57" t="n"/>
+      <c r="AJ37" s="57" t="n"/>
+      <c r="AK37" s="57" t="n"/>
+      <c r="AL37" s="57" t="n"/>
+      <c r="AM37" s="57" t="n"/>
+      <c r="AN37" s="57" t="n"/>
+      <c r="AO37" s="57" t="n"/>
+      <c r="AP37" s="57" t="n"/>
+      <c r="AQ37" s="57" t="n"/>
+      <c r="AR37" s="57" t="n"/>
+      <c r="AS37" s="57" t="n"/>
+      <c r="AT37" s="57" t="n"/>
     </row>
     <row r="38" ht="13.65" customHeight="1" s="90">
       <c r="A38" s="43" t="inlineStr">
@@ -8293,6 +8986,22 @@
       <c r="AB38" s="57" t="n"/>
       <c r="AC38" s="57" t="n"/>
       <c r="AD38" s="57" t="n"/>
+      <c r="AE38" s="57" t="n"/>
+      <c r="AF38" s="57" t="n"/>
+      <c r="AG38" s="57" t="n"/>
+      <c r="AH38" s="57" t="n"/>
+      <c r="AI38" s="57" t="n"/>
+      <c r="AJ38" s="57" t="n"/>
+      <c r="AK38" s="57" t="n"/>
+      <c r="AL38" s="57" t="n"/>
+      <c r="AM38" s="57" t="n"/>
+      <c r="AN38" s="57" t="n"/>
+      <c r="AO38" s="57" t="n"/>
+      <c r="AP38" s="57" t="n"/>
+      <c r="AQ38" s="57" t="n"/>
+      <c r="AR38" s="57" t="n"/>
+      <c r="AS38" s="57" t="n"/>
+      <c r="AT38" s="57" t="n"/>
     </row>
     <row r="39" ht="13.65" customHeight="1" s="90">
       <c r="A39" s="43" t="inlineStr">
@@ -8369,6 +9078,22 @@
       <c r="AB39" s="57" t="n"/>
       <c r="AC39" s="57" t="n"/>
       <c r="AD39" s="57" t="n"/>
+      <c r="AE39" s="57" t="n"/>
+      <c r="AF39" s="57" t="n"/>
+      <c r="AG39" s="57" t="n"/>
+      <c r="AH39" s="57" t="n"/>
+      <c r="AI39" s="57" t="n"/>
+      <c r="AJ39" s="57" t="n"/>
+      <c r="AK39" s="57" t="n"/>
+      <c r="AL39" s="57" t="n"/>
+      <c r="AM39" s="57" t="n"/>
+      <c r="AN39" s="57" t="n"/>
+      <c r="AO39" s="57" t="n"/>
+      <c r="AP39" s="57" t="n"/>
+      <c r="AQ39" s="57" t="n"/>
+      <c r="AR39" s="57" t="n"/>
+      <c r="AS39" s="57" t="n"/>
+      <c r="AT39" s="57" t="n"/>
     </row>
     <row r="40" ht="13.65" customHeight="1" s="90">
       <c r="A40" s="43" t="inlineStr">
@@ -8443,6 +9168,22 @@
       <c r="AB40" s="57" t="n"/>
       <c r="AC40" s="57" t="n"/>
       <c r="AD40" s="57" t="n"/>
+      <c r="AE40" s="57" t="n"/>
+      <c r="AF40" s="57" t="n"/>
+      <c r="AG40" s="57" t="n"/>
+      <c r="AH40" s="57" t="n"/>
+      <c r="AI40" s="57" t="n"/>
+      <c r="AJ40" s="57" t="n"/>
+      <c r="AK40" s="57" t="n"/>
+      <c r="AL40" s="57" t="n"/>
+      <c r="AM40" s="57" t="n"/>
+      <c r="AN40" s="57" t="n"/>
+      <c r="AO40" s="57" t="n"/>
+      <c r="AP40" s="57" t="n"/>
+      <c r="AQ40" s="57" t="n"/>
+      <c r="AR40" s="57" t="n"/>
+      <c r="AS40" s="57" t="n"/>
+      <c r="AT40" s="57" t="n"/>
     </row>
     <row r="41" ht="13.65" customHeight="1" s="90">
       <c r="A41" s="43" t="inlineStr">
@@ -8517,6 +9258,22 @@
       <c r="AB41" s="57" t="n"/>
       <c r="AC41" s="57" t="n"/>
       <c r="AD41" s="57" t="n"/>
+      <c r="AE41" s="57" t="n"/>
+      <c r="AF41" s="57" t="n"/>
+      <c r="AG41" s="57" t="n"/>
+      <c r="AH41" s="57" t="n"/>
+      <c r="AI41" s="57" t="n"/>
+      <c r="AJ41" s="57" t="n"/>
+      <c r="AK41" s="57" t="n"/>
+      <c r="AL41" s="57" t="n"/>
+      <c r="AM41" s="57" t="n"/>
+      <c r="AN41" s="57" t="n"/>
+      <c r="AO41" s="57" t="n"/>
+      <c r="AP41" s="57" t="n"/>
+      <c r="AQ41" s="57" t="n"/>
+      <c r="AR41" s="57" t="n"/>
+      <c r="AS41" s="57" t="n"/>
+      <c r="AT41" s="57" t="n"/>
     </row>
     <row r="42" ht="13.65" customHeight="1" s="90">
       <c r="A42" s="43" t="inlineStr">
@@ -8591,6 +9348,22 @@
       <c r="AB42" s="57" t="n"/>
       <c r="AC42" s="57" t="n"/>
       <c r="AD42" s="57" t="n"/>
+      <c r="AE42" s="57" t="n"/>
+      <c r="AF42" s="57" t="n"/>
+      <c r="AG42" s="57" t="n"/>
+      <c r="AH42" s="57" t="n"/>
+      <c r="AI42" s="57" t="n"/>
+      <c r="AJ42" s="57" t="n"/>
+      <c r="AK42" s="57" t="n"/>
+      <c r="AL42" s="57" t="n"/>
+      <c r="AM42" s="57" t="n"/>
+      <c r="AN42" s="57" t="n"/>
+      <c r="AO42" s="57" t="n"/>
+      <c r="AP42" s="57" t="n"/>
+      <c r="AQ42" s="57" t="n"/>
+      <c r="AR42" s="57" t="n"/>
+      <c r="AS42" s="57" t="n"/>
+      <c r="AT42" s="57" t="n"/>
     </row>
     <row r="43" ht="13.65" customHeight="1" s="90">
       <c r="A43" s="43" t="inlineStr">
@@ -8665,6 +9438,22 @@
       <c r="AB43" s="57" t="n"/>
       <c r="AC43" s="57" t="n"/>
       <c r="AD43" s="57" t="n"/>
+      <c r="AE43" s="57" t="n"/>
+      <c r="AF43" s="57" t="n"/>
+      <c r="AG43" s="57" t="n"/>
+      <c r="AH43" s="57" t="n"/>
+      <c r="AI43" s="57" t="n"/>
+      <c r="AJ43" s="57" t="n"/>
+      <c r="AK43" s="57" t="n"/>
+      <c r="AL43" s="57" t="n"/>
+      <c r="AM43" s="57" t="n"/>
+      <c r="AN43" s="57" t="n"/>
+      <c r="AO43" s="57" t="n"/>
+      <c r="AP43" s="57" t="n"/>
+      <c r="AQ43" s="57" t="n"/>
+      <c r="AR43" s="57" t="n"/>
+      <c r="AS43" s="57" t="n"/>
+      <c r="AT43" s="57" t="n"/>
     </row>
     <row r="44" ht="13.65" customHeight="1" s="90">
       <c r="A44" s="43" t="inlineStr">
@@ -8739,6 +9528,22 @@
       <c r="AB44" s="57" t="n"/>
       <c r="AC44" s="57" t="n"/>
       <c r="AD44" s="57" t="n"/>
+      <c r="AE44" s="57" t="n"/>
+      <c r="AF44" s="57" t="n"/>
+      <c r="AG44" s="57" t="n"/>
+      <c r="AH44" s="57" t="n"/>
+      <c r="AI44" s="57" t="n"/>
+      <c r="AJ44" s="57" t="n"/>
+      <c r="AK44" s="57" t="n"/>
+      <c r="AL44" s="57" t="n"/>
+      <c r="AM44" s="57" t="n"/>
+      <c r="AN44" s="57" t="n"/>
+      <c r="AO44" s="57" t="n"/>
+      <c r="AP44" s="57" t="n"/>
+      <c r="AQ44" s="57" t="n"/>
+      <c r="AR44" s="57" t="n"/>
+      <c r="AS44" s="57" t="n"/>
+      <c r="AT44" s="57" t="n"/>
     </row>
     <row r="45" ht="13.65" customHeight="1" s="90">
       <c r="A45" s="43" t="inlineStr">
@@ -8811,6 +9616,22 @@
       <c r="AB45" s="57" t="n"/>
       <c r="AC45" s="57" t="n"/>
       <c r="AD45" s="57" t="n"/>
+      <c r="AE45" s="57" t="n"/>
+      <c r="AF45" s="57" t="n"/>
+      <c r="AG45" s="57" t="n"/>
+      <c r="AH45" s="57" t="n"/>
+      <c r="AI45" s="57" t="n"/>
+      <c r="AJ45" s="57" t="n"/>
+      <c r="AK45" s="57" t="n"/>
+      <c r="AL45" s="57" t="n"/>
+      <c r="AM45" s="57" t="n"/>
+      <c r="AN45" s="57" t="n"/>
+      <c r="AO45" s="57" t="n"/>
+      <c r="AP45" s="57" t="n"/>
+      <c r="AQ45" s="57" t="n"/>
+      <c r="AR45" s="57" t="n"/>
+      <c r="AS45" s="57" t="n"/>
+      <c r="AT45" s="57" t="n"/>
     </row>
     <row r="46" ht="13.65" customHeight="1" s="90">
       <c r="A46" s="43" t="inlineStr">
@@ -8889,6 +9710,22 @@
       <c r="AB46" s="57" t="n"/>
       <c r="AC46" s="57" t="n"/>
       <c r="AD46" s="57" t="n"/>
+      <c r="AE46" s="57" t="n"/>
+      <c r="AF46" s="57" t="n"/>
+      <c r="AG46" s="57" t="n"/>
+      <c r="AH46" s="57" t="n"/>
+      <c r="AI46" s="57" t="n"/>
+      <c r="AJ46" s="57" t="n"/>
+      <c r="AK46" s="57" t="n"/>
+      <c r="AL46" s="57" t="n"/>
+      <c r="AM46" s="57" t="n"/>
+      <c r="AN46" s="57" t="n"/>
+      <c r="AO46" s="57" t="n"/>
+      <c r="AP46" s="57" t="n"/>
+      <c r="AQ46" s="57" t="n"/>
+      <c r="AR46" s="57" t="n"/>
+      <c r="AS46" s="57" t="n"/>
+      <c r="AT46" s="57" t="n"/>
     </row>
     <row r="47" ht="13.65" customHeight="1" s="90">
       <c r="A47" s="43" t="inlineStr">
@@ -8969,6 +9806,22 @@
       <c r="AB47" s="57" t="n"/>
       <c r="AC47" s="57" t="n"/>
       <c r="AD47" s="57" t="n"/>
+      <c r="AE47" s="57" t="n"/>
+      <c r="AF47" s="57" t="n"/>
+      <c r="AG47" s="57" t="n"/>
+      <c r="AH47" s="57" t="n"/>
+      <c r="AI47" s="57" t="n"/>
+      <c r="AJ47" s="57" t="n"/>
+      <c r="AK47" s="57" t="n"/>
+      <c r="AL47" s="57" t="n"/>
+      <c r="AM47" s="57" t="n"/>
+      <c r="AN47" s="57" t="n"/>
+      <c r="AO47" s="57" t="n"/>
+      <c r="AP47" s="57" t="n"/>
+      <c r="AQ47" s="57" t="n"/>
+      <c r="AR47" s="57" t="n"/>
+      <c r="AS47" s="57" t="n"/>
+      <c r="AT47" s="57" t="n"/>
     </row>
     <row r="48" ht="13.65" customHeight="1" s="90">
       <c r="A48" s="43" t="inlineStr">
@@ -9049,6 +9902,22 @@
       <c r="AB48" s="57" t="n"/>
       <c r="AC48" s="57" t="n"/>
       <c r="AD48" s="57" t="n"/>
+      <c r="AE48" s="57" t="n"/>
+      <c r="AF48" s="57" t="n"/>
+      <c r="AG48" s="57" t="n"/>
+      <c r="AH48" s="57" t="n"/>
+      <c r="AI48" s="57" t="n"/>
+      <c r="AJ48" s="57" t="n"/>
+      <c r="AK48" s="57" t="n"/>
+      <c r="AL48" s="57" t="n"/>
+      <c r="AM48" s="57" t="n"/>
+      <c r="AN48" s="57" t="n"/>
+      <c r="AO48" s="57" t="n"/>
+      <c r="AP48" s="57" t="n"/>
+      <c r="AQ48" s="57" t="n"/>
+      <c r="AR48" s="57" t="n"/>
+      <c r="AS48" s="57" t="n"/>
+      <c r="AT48" s="57" t="n"/>
     </row>
     <row r="49" ht="13.65" customHeight="1" s="90">
       <c r="A49" s="43" t="inlineStr">
@@ -9129,6 +9998,22 @@
       <c r="AB49" s="57" t="n"/>
       <c r="AC49" s="57" t="n"/>
       <c r="AD49" s="57" t="n"/>
+      <c r="AE49" s="57" t="n"/>
+      <c r="AF49" s="57" t="n"/>
+      <c r="AG49" s="57" t="n"/>
+      <c r="AH49" s="57" t="n"/>
+      <c r="AI49" s="57" t="n"/>
+      <c r="AJ49" s="57" t="n"/>
+      <c r="AK49" s="57" t="n"/>
+      <c r="AL49" s="57" t="n"/>
+      <c r="AM49" s="57" t="n"/>
+      <c r="AN49" s="57" t="n"/>
+      <c r="AO49" s="57" t="n"/>
+      <c r="AP49" s="57" t="n"/>
+      <c r="AQ49" s="57" t="n"/>
+      <c r="AR49" s="57" t="n"/>
+      <c r="AS49" s="57" t="n"/>
+      <c r="AT49" s="57" t="n"/>
     </row>
     <row r="50" ht="13.65" customHeight="1" s="90">
       <c r="A50" s="43" t="inlineStr">
@@ -9199,6 +10084,24 @@
       <c r="AB50" s="57" t="n"/>
       <c r="AC50" s="57" t="n"/>
       <c r="AD50" s="57" t="n"/>
+      <c r="AE50" s="57" t="n">
+        <v>35</v>
+      </c>
+      <c r="AF50" s="57" t="n"/>
+      <c r="AG50" s="57" t="n"/>
+      <c r="AH50" s="57" t="n"/>
+      <c r="AI50" s="57" t="n"/>
+      <c r="AJ50" s="57" t="n"/>
+      <c r="AK50" s="57" t="n"/>
+      <c r="AL50" s="57" t="n"/>
+      <c r="AM50" s="57" t="n"/>
+      <c r="AN50" s="57" t="n"/>
+      <c r="AO50" s="57" t="n"/>
+      <c r="AP50" s="57" t="n"/>
+      <c r="AQ50" s="57" t="n"/>
+      <c r="AR50" s="57" t="n"/>
+      <c r="AS50" s="57" t="n"/>
+      <c r="AT50" s="57" t="n"/>
     </row>
     <row r="51" ht="13.65" customHeight="1" s="90">
       <c r="A51" s="43" t="inlineStr">
@@ -9269,6 +10172,24 @@
       <c r="AB51" s="57" t="n"/>
       <c r="AC51" s="57" t="n"/>
       <c r="AD51" s="57" t="n"/>
+      <c r="AE51" s="57" t="n">
+        <v>45</v>
+      </c>
+      <c r="AF51" s="57" t="n"/>
+      <c r="AG51" s="57" t="n"/>
+      <c r="AH51" s="57" t="n"/>
+      <c r="AI51" s="57" t="n"/>
+      <c r="AJ51" s="57" t="n"/>
+      <c r="AK51" s="57" t="n"/>
+      <c r="AL51" s="57" t="n"/>
+      <c r="AM51" s="57" t="n"/>
+      <c r="AN51" s="57" t="n"/>
+      <c r="AO51" s="57" t="n"/>
+      <c r="AP51" s="57" t="n"/>
+      <c r="AQ51" s="57" t="n"/>
+      <c r="AR51" s="57" t="n"/>
+      <c r="AS51" s="57" t="n"/>
+      <c r="AT51" s="57" t="n"/>
     </row>
     <row r="52" ht="13.65" customHeight="1" s="90">
       <c r="A52" s="43" t="inlineStr">
@@ -9339,6 +10260,26 @@
       <c r="AB52" s="57" t="n"/>
       <c r="AC52" s="57" t="n"/>
       <c r="AD52" s="57" t="n"/>
+      <c r="AE52" s="57" t="n">
+        <v>45</v>
+      </c>
+      <c r="AF52" s="57" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG52" s="57" t="n"/>
+      <c r="AH52" s="57" t="n"/>
+      <c r="AI52" s="57" t="n"/>
+      <c r="AJ52" s="57" t="n"/>
+      <c r="AK52" s="57" t="n"/>
+      <c r="AL52" s="57" t="n"/>
+      <c r="AM52" s="57" t="n"/>
+      <c r="AN52" s="57" t="n"/>
+      <c r="AO52" s="57" t="n"/>
+      <c r="AP52" s="57" t="n"/>
+      <c r="AQ52" s="57" t="n"/>
+      <c r="AR52" s="57" t="n"/>
+      <c r="AS52" s="57" t="n"/>
+      <c r="AT52" s="57" t="n"/>
     </row>
     <row r="53" ht="13.65" customHeight="1" s="90">
       <c r="A53" s="43" t="inlineStr">
@@ -9409,6 +10350,26 @@
       <c r="AB53" s="57" t="n"/>
       <c r="AC53" s="57" t="n"/>
       <c r="AD53" s="57" t="n"/>
+      <c r="AE53" s="57" t="n">
+        <v>50</v>
+      </c>
+      <c r="AF53" s="57" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG53" s="57" t="n"/>
+      <c r="AH53" s="57" t="n"/>
+      <c r="AI53" s="57" t="n"/>
+      <c r="AJ53" s="57" t="n"/>
+      <c r="AK53" s="57" t="n"/>
+      <c r="AL53" s="57" t="n"/>
+      <c r="AM53" s="57" t="n"/>
+      <c r="AN53" s="57" t="n"/>
+      <c r="AO53" s="57" t="n"/>
+      <c r="AP53" s="57" t="n"/>
+      <c r="AQ53" s="57" t="n"/>
+      <c r="AR53" s="57" t="n"/>
+      <c r="AS53" s="57" t="n"/>
+      <c r="AT53" s="57" t="n"/>
     </row>
     <row r="54" ht="13.65" customHeight="1" s="90">
       <c r="A54" s="43" t="inlineStr">
@@ -9479,6 +10440,30 @@
       <c r="AB54" s="57" t="n"/>
       <c r="AC54" s="57" t="n"/>
       <c r="AD54" s="57" t="n"/>
+      <c r="AE54" s="57" t="n">
+        <v>60</v>
+      </c>
+      <c r="AF54" s="57" t="n">
+        <v>3</v>
+      </c>
+      <c r="AG54" s="57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AH54" s="57" t="n"/>
+      <c r="AI54" s="57" t="n"/>
+      <c r="AJ54" s="57" t="n"/>
+      <c r="AK54" s="57" t="n"/>
+      <c r="AL54" s="57" t="n"/>
+      <c r="AM54" s="57" t="n"/>
+      <c r="AN54" s="57" t="n"/>
+      <c r="AO54" s="57" t="n"/>
+      <c r="AP54" s="57" t="n"/>
+      <c r="AQ54" s="57" t="n"/>
+      <c r="AR54" s="57" t="n"/>
+      <c r="AS54" s="57" t="n"/>
+      <c r="AT54" s="57" t="n"/>
     </row>
     <row r="55" ht="13.65" customHeight="1" s="90">
       <c r="A55" s="43" t="inlineStr">
@@ -9549,6 +10534,26 @@
       <c r="AB55" s="57" t="n"/>
       <c r="AC55" s="57" t="n"/>
       <c r="AD55" s="57" t="n"/>
+      <c r="AE55" s="57" t="n"/>
+      <c r="AF55" s="57" t="n"/>
+      <c r="AG55" s="57" t="n"/>
+      <c r="AH55" s="57" t="n">
+        <v>8</v>
+      </c>
+      <c r="AI55" s="57" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="AJ55" s="57" t="n"/>
+      <c r="AK55" s="57" t="n"/>
+      <c r="AL55" s="57" t="n"/>
+      <c r="AM55" s="57" t="n"/>
+      <c r="AN55" s="57" t="n"/>
+      <c r="AO55" s="57" t="n"/>
+      <c r="AP55" s="57" t="n"/>
+      <c r="AQ55" s="57" t="n"/>
+      <c r="AR55" s="57" t="n"/>
+      <c r="AS55" s="57" t="n"/>
+      <c r="AT55" s="57" t="n"/>
     </row>
     <row r="56" ht="13.65" customHeight="1" s="90">
       <c r="A56" s="43" t="inlineStr">
@@ -9619,6 +10624,26 @@
       <c r="AB56" s="57" t="n"/>
       <c r="AC56" s="57" t="n"/>
       <c r="AD56" s="57" t="n"/>
+      <c r="AE56" s="57" t="n"/>
+      <c r="AF56" s="57" t="n"/>
+      <c r="AG56" s="57" t="n"/>
+      <c r="AH56" s="57" t="n">
+        <v>8</v>
+      </c>
+      <c r="AI56" s="57" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ56" s="57" t="n"/>
+      <c r="AK56" s="57" t="n"/>
+      <c r="AL56" s="57" t="n"/>
+      <c r="AM56" s="57" t="n"/>
+      <c r="AN56" s="57" t="n"/>
+      <c r="AO56" s="57" t="n"/>
+      <c r="AP56" s="57" t="n"/>
+      <c r="AQ56" s="57" t="n"/>
+      <c r="AR56" s="57" t="n"/>
+      <c r="AS56" s="57" t="n"/>
+      <c r="AT56" s="57" t="n"/>
     </row>
     <row r="57" ht="13.65" customHeight="1" s="90">
       <c r="A57" s="43" t="inlineStr">
@@ -9689,6 +10714,28 @@
       <c r="AB57" s="57" t="n"/>
       <c r="AC57" s="57" t="n"/>
       <c r="AD57" s="57" t="n"/>
+      <c r="AE57" s="57" t="n"/>
+      <c r="AF57" s="57" t="n"/>
+      <c r="AG57" s="57" t="n"/>
+      <c r="AH57" s="57" t="n">
+        <v>7</v>
+      </c>
+      <c r="AI57" s="57" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ57" s="57" t="n">
+        <v>2</v>
+      </c>
+      <c r="AK57" s="57" t="n"/>
+      <c r="AL57" s="57" t="n"/>
+      <c r="AM57" s="57" t="n"/>
+      <c r="AN57" s="57" t="n"/>
+      <c r="AO57" s="57" t="n"/>
+      <c r="AP57" s="57" t="n"/>
+      <c r="AQ57" s="57" t="n"/>
+      <c r="AR57" s="57" t="n"/>
+      <c r="AS57" s="57" t="n"/>
+      <c r="AT57" s="57" t="n"/>
     </row>
     <row r="58" ht="13.65" customHeight="1" s="90">
       <c r="A58" s="43" t="inlineStr">
@@ -9759,6 +10806,28 @@
       <c r="AB58" s="57" t="n"/>
       <c r="AC58" s="57" t="n"/>
       <c r="AD58" s="57" t="n"/>
+      <c r="AE58" s="57" t="n"/>
+      <c r="AF58" s="57" t="n"/>
+      <c r="AG58" s="57" t="n"/>
+      <c r="AH58" s="57" t="n">
+        <v>5</v>
+      </c>
+      <c r="AI58" s="57" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ58" s="57" t="n">
+        <v>3</v>
+      </c>
+      <c r="AK58" s="57" t="n"/>
+      <c r="AL58" s="57" t="n"/>
+      <c r="AM58" s="57" t="n"/>
+      <c r="AN58" s="57" t="n"/>
+      <c r="AO58" s="57" t="n"/>
+      <c r="AP58" s="57" t="n"/>
+      <c r="AQ58" s="57" t="n"/>
+      <c r="AR58" s="57" t="n"/>
+      <c r="AS58" s="57" t="n"/>
+      <c r="AT58" s="57" t="n"/>
     </row>
     <row r="59" ht="13.65" customHeight="1" s="90">
       <c r="A59" s="43" t="inlineStr">
@@ -9829,6 +10898,32 @@
       <c r="AB59" s="57" t="n"/>
       <c r="AC59" s="57" t="n"/>
       <c r="AD59" s="57" t="n"/>
+      <c r="AE59" s="57" t="n"/>
+      <c r="AF59" s="57" t="n"/>
+      <c r="AG59" s="57" t="n"/>
+      <c r="AH59" s="57" t="n">
+        <v>5</v>
+      </c>
+      <c r="AI59" s="57" t="n">
+        <v>2</v>
+      </c>
+      <c r="AJ59" s="57" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK59" s="57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AL59" s="57" t="n"/>
+      <c r="AM59" s="57" t="n"/>
+      <c r="AN59" s="57" t="n"/>
+      <c r="AO59" s="57" t="n"/>
+      <c r="AP59" s="57" t="n"/>
+      <c r="AQ59" s="57" t="n"/>
+      <c r="AR59" s="57" t="n"/>
+      <c r="AS59" s="57" t="n"/>
+      <c r="AT59" s="57" t="n"/>
     </row>
     <row r="60" ht="13.65" customHeight="1" s="90">
       <c r="A60" s="43" t="inlineStr">
@@ -9899,6 +10994,24 @@
       <c r="AB60" s="57" t="n"/>
       <c r="AC60" s="57" t="n"/>
       <c r="AD60" s="57" t="n"/>
+      <c r="AE60" s="57" t="n"/>
+      <c r="AF60" s="57" t="n"/>
+      <c r="AG60" s="57" t="n"/>
+      <c r="AH60" s="57" t="n"/>
+      <c r="AI60" s="57" t="n"/>
+      <c r="AJ60" s="57" t="n"/>
+      <c r="AK60" s="57" t="n"/>
+      <c r="AL60" s="57" t="n">
+        <v>25</v>
+      </c>
+      <c r="AM60" s="57" t="n"/>
+      <c r="AN60" s="57" t="n"/>
+      <c r="AO60" s="57" t="n"/>
+      <c r="AP60" s="57" t="n"/>
+      <c r="AQ60" s="57" t="n"/>
+      <c r="AR60" s="57" t="n"/>
+      <c r="AS60" s="57" t="n"/>
+      <c r="AT60" s="57" t="n"/>
     </row>
     <row r="61" ht="13.65" customHeight="1" s="90">
       <c r="A61" s="43" t="inlineStr">
@@ -9969,6 +11082,28 @@
       <c r="AB61" s="57" t="n"/>
       <c r="AC61" s="57" t="n"/>
       <c r="AD61" s="57" t="n"/>
+      <c r="AE61" s="57" t="n"/>
+      <c r="AF61" s="57" t="n"/>
+      <c r="AG61" s="57" t="n"/>
+      <c r="AH61" s="57" t="n"/>
+      <c r="AI61" s="57" t="n"/>
+      <c r="AJ61" s="57" t="n"/>
+      <c r="AK61" s="57" t="n"/>
+      <c r="AL61" s="57" t="n">
+        <v>35</v>
+      </c>
+      <c r="AM61" s="57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AN61" s="57" t="n"/>
+      <c r="AO61" s="57" t="n"/>
+      <c r="AP61" s="57" t="n"/>
+      <c r="AQ61" s="57" t="n"/>
+      <c r="AR61" s="57" t="n"/>
+      <c r="AS61" s="57" t="n"/>
+      <c r="AT61" s="57" t="n"/>
     </row>
     <row r="62" ht="13.65" customHeight="1" s="90">
       <c r="A62" s="43" t="inlineStr">
@@ -10036,9 +11171,33 @@
       <c r="Y62" s="57" t="n"/>
       <c r="Z62" s="57" t="n"/>
       <c r="AA62" s="57" t="n"/>
-      <c r="AB62" s="57" t="n"/>
+      <c r="AB62" s="57" t="n">
+        <v>10</v>
+      </c>
       <c r="AC62" s="57" t="n"/>
       <c r="AD62" s="57" t="n"/>
+      <c r="AE62" s="57" t="n"/>
+      <c r="AF62" s="57" t="n"/>
+      <c r="AG62" s="57" t="n"/>
+      <c r="AH62" s="57" t="n"/>
+      <c r="AI62" s="57" t="n"/>
+      <c r="AJ62" s="57" t="n"/>
+      <c r="AK62" s="57" t="n"/>
+      <c r="AL62" s="57" t="n">
+        <v>35</v>
+      </c>
+      <c r="AM62" s="57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AN62" s="57" t="n"/>
+      <c r="AO62" s="57" t="n"/>
+      <c r="AP62" s="57" t="n"/>
+      <c r="AQ62" s="57" t="n"/>
+      <c r="AR62" s="57" t="n"/>
+      <c r="AS62" s="57" t="n"/>
+      <c r="AT62" s="57" t="n"/>
     </row>
     <row r="63" ht="13.65" customHeight="1" s="90">
       <c r="A63" s="43" t="inlineStr">
@@ -10106,9 +11265,33 @@
       <c r="Y63" s="57" t="n"/>
       <c r="Z63" s="57" t="n"/>
       <c r="AA63" s="57" t="n"/>
-      <c r="AB63" s="57" t="n"/>
+      <c r="AB63" s="57" t="n">
+        <v>10</v>
+      </c>
       <c r="AC63" s="57" t="n"/>
       <c r="AD63" s="57" t="n"/>
+      <c r="AE63" s="57" t="n"/>
+      <c r="AF63" s="57" t="n"/>
+      <c r="AG63" s="57" t="n"/>
+      <c r="AH63" s="57" t="n"/>
+      <c r="AI63" s="57" t="n"/>
+      <c r="AJ63" s="57" t="n"/>
+      <c r="AK63" s="57" t="n"/>
+      <c r="AL63" s="57" t="n">
+        <v>50</v>
+      </c>
+      <c r="AM63" s="57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AN63" s="57" t="n"/>
+      <c r="AO63" s="57" t="n"/>
+      <c r="AP63" s="57" t="n"/>
+      <c r="AQ63" s="57" t="n"/>
+      <c r="AR63" s="57" t="n"/>
+      <c r="AS63" s="57" t="n"/>
+      <c r="AT63" s="57" t="n"/>
     </row>
     <row r="64" ht="13.65" customHeight="1" s="90">
       <c r="A64" s="43" t="inlineStr">
@@ -10176,9 +11359,35 @@
       <c r="Y64" s="57" t="n"/>
       <c r="Z64" s="57" t="n"/>
       <c r="AA64" s="57" t="n"/>
-      <c r="AB64" s="57" t="n"/>
-      <c r="AC64" s="57" t="n"/>
+      <c r="AB64" s="57" t="n">
+        <v>10</v>
+      </c>
+      <c r="AC64" s="57" t="n">
+        <v>20</v>
+      </c>
       <c r="AD64" s="57" t="n"/>
+      <c r="AE64" s="57" t="n"/>
+      <c r="AF64" s="57" t="n"/>
+      <c r="AG64" s="57" t="n"/>
+      <c r="AH64" s="57" t="n"/>
+      <c r="AI64" s="57" t="n"/>
+      <c r="AJ64" s="57" t="n"/>
+      <c r="AK64" s="57" t="n"/>
+      <c r="AL64" s="57" t="n">
+        <v>75</v>
+      </c>
+      <c r="AM64" s="57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AN64" s="57" t="n"/>
+      <c r="AO64" s="57" t="n"/>
+      <c r="AP64" s="57" t="n"/>
+      <c r="AQ64" s="57" t="n"/>
+      <c r="AR64" s="57" t="n"/>
+      <c r="AS64" s="57" t="n"/>
+      <c r="AT64" s="57" t="n"/>
     </row>
     <row r="65" ht="13.65" customHeight="1" s="90">
       <c r="A65" s="43" t="inlineStr">
@@ -10249,6 +11458,24 @@
       <c r="AB65" s="57" t="n"/>
       <c r="AC65" s="57" t="n"/>
       <c r="AD65" s="57" t="n"/>
+      <c r="AE65" s="57" t="n"/>
+      <c r="AF65" s="57" t="n"/>
+      <c r="AG65" s="57" t="n"/>
+      <c r="AH65" s="57" t="n"/>
+      <c r="AI65" s="57" t="n"/>
+      <c r="AJ65" s="57" t="n"/>
+      <c r="AK65" s="57" t="n"/>
+      <c r="AL65" s="57" t="n"/>
+      <c r="AM65" s="57" t="n"/>
+      <c r="AN65" s="57" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="AO65" s="57" t="n"/>
+      <c r="AP65" s="57" t="n"/>
+      <c r="AQ65" s="57" t="n"/>
+      <c r="AR65" s="57" t="n"/>
+      <c r="AS65" s="57" t="n"/>
+      <c r="AT65" s="57" t="n"/>
     </row>
     <row r="66" ht="13.65" customHeight="1" s="90">
       <c r="A66" s="43" t="inlineStr">
@@ -10319,6 +11546,24 @@
       <c r="AB66" s="57" t="n"/>
       <c r="AC66" s="57" t="n"/>
       <c r="AD66" s="57" t="n"/>
+      <c r="AE66" s="57" t="n"/>
+      <c r="AF66" s="57" t="n"/>
+      <c r="AG66" s="57" t="n"/>
+      <c r="AH66" s="57" t="n"/>
+      <c r="AI66" s="57" t="n"/>
+      <c r="AJ66" s="57" t="n"/>
+      <c r="AK66" s="57" t="n"/>
+      <c r="AL66" s="57" t="n"/>
+      <c r="AM66" s="57" t="n"/>
+      <c r="AN66" s="57" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="AO66" s="57" t="n"/>
+      <c r="AP66" s="57" t="n"/>
+      <c r="AQ66" s="57" t="n"/>
+      <c r="AR66" s="57" t="n"/>
+      <c r="AS66" s="57" t="n"/>
+      <c r="AT66" s="57" t="n"/>
     </row>
     <row r="67" ht="13.65" customHeight="1" s="90">
       <c r="A67" s="43" t="inlineStr">
@@ -10389,6 +11634,24 @@
       <c r="AB67" s="57" t="n"/>
       <c r="AC67" s="57" t="n"/>
       <c r="AD67" s="57" t="n"/>
+      <c r="AE67" s="57" t="n"/>
+      <c r="AF67" s="57" t="n"/>
+      <c r="AG67" s="57" t="n"/>
+      <c r="AH67" s="57" t="n"/>
+      <c r="AI67" s="57" t="n"/>
+      <c r="AJ67" s="57" t="n"/>
+      <c r="AK67" s="57" t="n"/>
+      <c r="AL67" s="57" t="n"/>
+      <c r="AM67" s="57" t="n"/>
+      <c r="AN67" s="57" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="AO67" s="57" t="n"/>
+      <c r="AP67" s="57" t="n"/>
+      <c r="AQ67" s="57" t="n"/>
+      <c r="AR67" s="57" t="n"/>
+      <c r="AS67" s="57" t="n"/>
+      <c r="AT67" s="57" t="n"/>
     </row>
     <row r="68" ht="13.65" customHeight="1" s="90">
       <c r="A68" s="43" t="inlineStr">
@@ -10459,6 +11722,24 @@
       <c r="AB68" s="57" t="n"/>
       <c r="AC68" s="57" t="n"/>
       <c r="AD68" s="57" t="n"/>
+      <c r="AE68" s="57" t="n"/>
+      <c r="AF68" s="57" t="n"/>
+      <c r="AG68" s="57" t="n"/>
+      <c r="AH68" s="57" t="n"/>
+      <c r="AI68" s="57" t="n"/>
+      <c r="AJ68" s="57" t="n"/>
+      <c r="AK68" s="57" t="n"/>
+      <c r="AL68" s="57" t="n"/>
+      <c r="AM68" s="57" t="n"/>
+      <c r="AN68" s="57" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO68" s="57" t="n"/>
+      <c r="AP68" s="57" t="n"/>
+      <c r="AQ68" s="57" t="n"/>
+      <c r="AR68" s="57" t="n"/>
+      <c r="AS68" s="57" t="n"/>
+      <c r="AT68" s="57" t="n"/>
     </row>
     <row r="69" ht="13.65" customHeight="1" s="90">
       <c r="A69" s="43" t="inlineStr">
@@ -10529,6 +11810,28 @@
       <c r="AB69" s="57" t="n"/>
       <c r="AC69" s="57" t="n"/>
       <c r="AD69" s="57" t="n"/>
+      <c r="AE69" s="57" t="n"/>
+      <c r="AF69" s="57" t="n"/>
+      <c r="AG69" s="57" t="n"/>
+      <c r="AH69" s="57" t="n"/>
+      <c r="AI69" s="57" t="n"/>
+      <c r="AJ69" s="57" t="n"/>
+      <c r="AK69" s="57" t="n"/>
+      <c r="AL69" s="57" t="n"/>
+      <c r="AM69" s="57" t="n"/>
+      <c r="AN69" s="57" t="n">
+        <v>4</v>
+      </c>
+      <c r="AO69" s="57" t="n">
+        <v>5</v>
+      </c>
+      <c r="AP69" s="57" t="n">
+        <v>500</v>
+      </c>
+      <c r="AQ69" s="57" t="n"/>
+      <c r="AR69" s="57" t="n"/>
+      <c r="AS69" s="57" t="n"/>
+      <c r="AT69" s="57" t="n"/>
     </row>
     <row r="70" ht="13.65" customHeight="1" s="90">
       <c r="A70" s="43" t="inlineStr">
@@ -10599,6 +11902,26 @@
       <c r="AB70" s="57" t="n"/>
       <c r="AC70" s="57" t="n"/>
       <c r="AD70" s="57" t="n"/>
+      <c r="AE70" s="57" t="n"/>
+      <c r="AF70" s="57" t="n"/>
+      <c r="AG70" s="57" t="n"/>
+      <c r="AH70" s="57" t="n"/>
+      <c r="AI70" s="57" t="n"/>
+      <c r="AJ70" s="57" t="n"/>
+      <c r="AK70" s="57" t="n"/>
+      <c r="AL70" s="57" t="n"/>
+      <c r="AM70" s="57" t="n"/>
+      <c r="AN70" s="57" t="n"/>
+      <c r="AO70" s="57" t="n"/>
+      <c r="AP70" s="57" t="n"/>
+      <c r="AQ70" s="57" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR70" s="57" t="n">
+        <v>60</v>
+      </c>
+      <c r="AS70" s="57" t="n"/>
+      <c r="AT70" s="57" t="n"/>
     </row>
     <row r="71" ht="13.65" customHeight="1" s="90">
       <c r="A71" s="43" t="inlineStr">
@@ -10669,6 +11992,26 @@
       <c r="AB71" s="57" t="n"/>
       <c r="AC71" s="57" t="n"/>
       <c r="AD71" s="57" t="n"/>
+      <c r="AE71" s="57" t="n"/>
+      <c r="AF71" s="57" t="n"/>
+      <c r="AG71" s="57" t="n"/>
+      <c r="AH71" s="57" t="n"/>
+      <c r="AI71" s="57" t="n"/>
+      <c r="AJ71" s="57" t="n"/>
+      <c r="AK71" s="57" t="n"/>
+      <c r="AL71" s="57" t="n"/>
+      <c r="AM71" s="57" t="n"/>
+      <c r="AN71" s="57" t="n"/>
+      <c r="AO71" s="57" t="n"/>
+      <c r="AP71" s="57" t="n"/>
+      <c r="AQ71" s="57" t="n">
+        <v>2</v>
+      </c>
+      <c r="AR71" s="57" t="n">
+        <v>60</v>
+      </c>
+      <c r="AS71" s="57" t="n"/>
+      <c r="AT71" s="57" t="n"/>
     </row>
     <row r="72" ht="13.65" customHeight="1" s="90">
       <c r="A72" s="43" t="inlineStr">
@@ -10739,6 +12082,26 @@
       <c r="AB72" s="57" t="n"/>
       <c r="AC72" s="57" t="n"/>
       <c r="AD72" s="57" t="n"/>
+      <c r="AE72" s="57" t="n"/>
+      <c r="AF72" s="57" t="n"/>
+      <c r="AG72" s="57" t="n"/>
+      <c r="AH72" s="57" t="n"/>
+      <c r="AI72" s="57" t="n"/>
+      <c r="AJ72" s="57" t="n"/>
+      <c r="AK72" s="57" t="n"/>
+      <c r="AL72" s="57" t="n"/>
+      <c r="AM72" s="57" t="n"/>
+      <c r="AN72" s="57" t="n"/>
+      <c r="AO72" s="57" t="n"/>
+      <c r="AP72" s="57" t="n"/>
+      <c r="AQ72" s="57" t="n">
+        <v>2</v>
+      </c>
+      <c r="AR72" s="57" t="n">
+        <v>120</v>
+      </c>
+      <c r="AS72" s="57" t="n"/>
+      <c r="AT72" s="57" t="n"/>
     </row>
     <row r="73" ht="13.65" customHeight="1" s="90">
       <c r="A73" s="43" t="inlineStr">
@@ -10809,6 +12172,26 @@
       <c r="AB73" s="57" t="n"/>
       <c r="AC73" s="57" t="n"/>
       <c r="AD73" s="57" t="n"/>
+      <c r="AE73" s="57" t="n"/>
+      <c r="AF73" s="57" t="n"/>
+      <c r="AG73" s="57" t="n"/>
+      <c r="AH73" s="57" t="n"/>
+      <c r="AI73" s="57" t="n"/>
+      <c r="AJ73" s="57" t="n"/>
+      <c r="AK73" s="57" t="n"/>
+      <c r="AL73" s="57" t="n"/>
+      <c r="AM73" s="57" t="n"/>
+      <c r="AN73" s="57" t="n"/>
+      <c r="AO73" s="57" t="n"/>
+      <c r="AP73" s="57" t="n"/>
+      <c r="AQ73" s="57" t="n">
+        <v>3</v>
+      </c>
+      <c r="AR73" s="57" t="n">
+        <v>120</v>
+      </c>
+      <c r="AS73" s="57" t="n"/>
+      <c r="AT73" s="57" t="n"/>
     </row>
     <row r="74" ht="13.65" customHeight="1" s="90">
       <c r="A74" s="43" t="inlineStr">
@@ -10879,6 +12262,26 @@
       <c r="AB74" s="57" t="n"/>
       <c r="AC74" s="57" t="n"/>
       <c r="AD74" s="57" t="n"/>
+      <c r="AE74" s="57" t="n"/>
+      <c r="AF74" s="57" t="n"/>
+      <c r="AG74" s="57" t="n"/>
+      <c r="AH74" s="57" t="n"/>
+      <c r="AI74" s="57" t="n"/>
+      <c r="AJ74" s="57" t="n"/>
+      <c r="AK74" s="57" t="n"/>
+      <c r="AL74" s="57" t="n"/>
+      <c r="AM74" s="57" t="n"/>
+      <c r="AN74" s="57" t="n"/>
+      <c r="AO74" s="57" t="n"/>
+      <c r="AP74" s="57" t="n"/>
+      <c r="AQ74" s="57" t="n">
+        <v>4</v>
+      </c>
+      <c r="AR74" s="57" t="n">
+        <v>250</v>
+      </c>
+      <c r="AS74" s="57" t="n"/>
+      <c r="AT74" s="57" t="n"/>
     </row>
     <row r="75" ht="13.65" customHeight="1" s="90">
       <c r="A75" s="43" t="inlineStr">
@@ -10949,6 +12352,24 @@
       <c r="AB75" s="57" t="n"/>
       <c r="AC75" s="57" t="n"/>
       <c r="AD75" s="57" t="n"/>
+      <c r="AE75" s="57" t="n"/>
+      <c r="AF75" s="57" t="n"/>
+      <c r="AG75" s="57" t="n"/>
+      <c r="AH75" s="57" t="n"/>
+      <c r="AI75" s="57" t="n"/>
+      <c r="AJ75" s="57" t="n"/>
+      <c r="AK75" s="57" t="n"/>
+      <c r="AL75" s="57" t="n"/>
+      <c r="AM75" s="57" t="n"/>
+      <c r="AN75" s="57" t="n"/>
+      <c r="AO75" s="57" t="n"/>
+      <c r="AP75" s="57" t="n"/>
+      <c r="AQ75" s="57" t="n"/>
+      <c r="AR75" s="57" t="n"/>
+      <c r="AS75" s="57" t="n">
+        <v>5</v>
+      </c>
+      <c r="AT75" s="57" t="n"/>
     </row>
     <row r="76" ht="13.65" customHeight="1" s="90">
       <c r="A76" s="43" t="inlineStr">
@@ -11019,6 +12440,24 @@
       <c r="AB76" s="57" t="n"/>
       <c r="AC76" s="57" t="n"/>
       <c r="AD76" s="57" t="n"/>
+      <c r="AE76" s="57" t="n"/>
+      <c r="AF76" s="57" t="n"/>
+      <c r="AG76" s="57" t="n"/>
+      <c r="AH76" s="57" t="n"/>
+      <c r="AI76" s="57" t="n"/>
+      <c r="AJ76" s="57" t="n"/>
+      <c r="AK76" s="57" t="n"/>
+      <c r="AL76" s="57" t="n"/>
+      <c r="AM76" s="57" t="n"/>
+      <c r="AN76" s="57" t="n"/>
+      <c r="AO76" s="57" t="n"/>
+      <c r="AP76" s="57" t="n"/>
+      <c r="AQ76" s="57" t="n"/>
+      <c r="AR76" s="57" t="n"/>
+      <c r="AS76" s="57" t="n">
+        <v>10</v>
+      </c>
+      <c r="AT76" s="57" t="n"/>
     </row>
     <row r="77" ht="13.65" customHeight="1" s="90">
       <c r="A77" s="43" t="inlineStr">
@@ -11089,6 +12528,26 @@
       <c r="AB77" s="57" t="n"/>
       <c r="AC77" s="57" t="n"/>
       <c r="AD77" s="57" t="n"/>
+      <c r="AE77" s="57" t="n"/>
+      <c r="AF77" s="57" t="n"/>
+      <c r="AG77" s="57" t="n"/>
+      <c r="AH77" s="57" t="n"/>
+      <c r="AI77" s="57" t="n"/>
+      <c r="AJ77" s="57" t="n"/>
+      <c r="AK77" s="57" t="n"/>
+      <c r="AL77" s="57" t="n"/>
+      <c r="AM77" s="57" t="n"/>
+      <c r="AN77" s="57" t="n"/>
+      <c r="AO77" s="57" t="n"/>
+      <c r="AP77" s="57" t="n"/>
+      <c r="AQ77" s="57" t="n"/>
+      <c r="AR77" s="57" t="n"/>
+      <c r="AS77" s="57" t="n">
+        <v>10</v>
+      </c>
+      <c r="AT77" s="57" t="n">
+        <v>0.9</v>
+      </c>
     </row>
     <row r="78" ht="13.65" customHeight="1" s="90">
       <c r="A78" s="43" t="inlineStr">
@@ -11156,9 +12615,31 @@
       <c r="Y78" s="57" t="n"/>
       <c r="Z78" s="57" t="n"/>
       <c r="AA78" s="57" t="n"/>
-      <c r="AB78" s="57" t="n"/>
+      <c r="AB78" s="57" t="n">
+        <v>10</v>
+      </c>
       <c r="AC78" s="57" t="n"/>
       <c r="AD78" s="57" t="n"/>
+      <c r="AE78" s="57" t="n"/>
+      <c r="AF78" s="57" t="n"/>
+      <c r="AG78" s="57" t="n"/>
+      <c r="AH78" s="57" t="n"/>
+      <c r="AI78" s="57" t="n"/>
+      <c r="AJ78" s="57" t="n"/>
+      <c r="AK78" s="57" t="n"/>
+      <c r="AL78" s="57" t="n"/>
+      <c r="AM78" s="57" t="n"/>
+      <c r="AN78" s="57" t="n"/>
+      <c r="AO78" s="57" t="n"/>
+      <c r="AP78" s="57" t="n"/>
+      <c r="AQ78" s="57" t="n"/>
+      <c r="AR78" s="57" t="n"/>
+      <c r="AS78" s="57" t="n">
+        <v>10</v>
+      </c>
+      <c r="AT78" s="57" t="n">
+        <v>0.9</v>
+      </c>
     </row>
     <row r="79" ht="13.65" customHeight="1" s="90">
       <c r="A79" s="43" t="inlineStr">
@@ -11226,9 +12707,31 @@
       <c r="Y79" s="57" t="n"/>
       <c r="Z79" s="57" t="n"/>
       <c r="AA79" s="57" t="n"/>
-      <c r="AB79" s="57" t="n"/>
+      <c r="AB79" s="57" t="n">
+        <v>10</v>
+      </c>
       <c r="AC79" s="57" t="n"/>
       <c r="AD79" s="57" t="n"/>
+      <c r="AE79" s="57" t="n"/>
+      <c r="AF79" s="57" t="n"/>
+      <c r="AG79" s="57" t="n"/>
+      <c r="AH79" s="57" t="n"/>
+      <c r="AI79" s="57" t="n"/>
+      <c r="AJ79" s="57" t="n"/>
+      <c r="AK79" s="57" t="n"/>
+      <c r="AL79" s="57" t="n"/>
+      <c r="AM79" s="57" t="n"/>
+      <c r="AN79" s="57" t="n"/>
+      <c r="AO79" s="57" t="n"/>
+      <c r="AP79" s="57" t="n"/>
+      <c r="AQ79" s="57" t="n"/>
+      <c r="AR79" s="57" t="n"/>
+      <c r="AS79" s="57" t="n">
+        <v>20</v>
+      </c>
+      <c r="AT79" s="57" t="n">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811" footer="0.511811"/>

</xml_diff>

<commit_message>
Buff the Chiller's slow
Base slow 30% -> 40%; Field path 35/45/45/50/60% -> 50/60/60/70/80%.
Linger and boss slow unchanged. (User: the slow needed a buff.)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Storm-Split-Balance.xlsx
+++ b/Storm-Split-Balance.xlsx
@@ -5482,7 +5482,7 @@
         <v>6</v>
       </c>
       <c r="M8" s="27" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" ht="13.65" customHeight="1" s="90">
@@ -10085,7 +10085,7 @@
       <c r="AC50" s="57" t="n"/>
       <c r="AD50" s="57" t="n"/>
       <c r="AE50" s="57" t="n">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="AF50" s="57" t="n"/>
       <c r="AG50" s="57" t="n"/>
@@ -10173,7 +10173,7 @@
       <c r="AC51" s="57" t="n"/>
       <c r="AD51" s="57" t="n"/>
       <c r="AE51" s="57" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="AF51" s="57" t="n"/>
       <c r="AG51" s="57" t="n"/>
@@ -10261,7 +10261,7 @@
       <c r="AC52" s="57" t="n"/>
       <c r="AD52" s="57" t="n"/>
       <c r="AE52" s="57" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="AF52" s="57" t="n">
         <v>2</v>
@@ -10351,7 +10351,7 @@
       <c r="AC53" s="57" t="n"/>
       <c r="AD53" s="57" t="n"/>
       <c r="AE53" s="57" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="AF53" s="57" t="n">
         <v>2</v>
@@ -10441,7 +10441,7 @@
       <c r="AC54" s="57" t="n"/>
       <c r="AD54" s="57" t="n"/>
       <c r="AE54" s="57" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="AF54" s="57" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Dragon's Breath ignites what it hits
Dragon's Breath (and the Buckshot tiers after it) now set the enemy they hit
on fire as well as leaving burning ground: it takes the burn damage for
Ignite (s) = 1.5s, then loses its current layer if it's still alive, so it
burns down one level. Split children aren't on fire; the patch on the ground
catches them. Bosses take the burn damage but never lose a whole layer.

- Hero Upgrades: new Ignite (s) column; exporter, HeroStats and the upgrade
  panel read it.
- Server/Hazards tracks ignited enemies next to burning patches (one fire
  per enemy, refreshed not stacked; kills credited to whoever lit it).
- Enemies.showBurning: flames on burning enemies (visual only).

Statically checked; not yet playtested.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Storm-Split-Balance.xlsx
+++ b/Storm-Split-Balance.xlsx
@@ -13184,7 +13184,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG49"/>
+  <dimension ref="A1:AH49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" style="90" min="1" max="1"/>
@@ -13232,7 +13232,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Effect columns are cumulative per tier (like Tower Upgrades); blank = no change. x columns multiply the hero's base; Fire mode / Guns / Pellets / Pierce / Bounces override it. Crossover rule as towers: two paths, one past tier 2. Damage is per shot: pellets share the hero's base damage x its base pellet count, so more pellets spread the same damage wider and a slug concentrates it.</t>
+          <t>Effect columns are cumulative per tier (like Tower Upgrades); blank = no change. x columns multiply the hero's base; Fire mode / Guns / Pellets / Pierce / Bounces override it. Crossover rule as towers: two paths, one past tier 2. Damage is per shot: pellets share the hero's base damage x its base pellet count, so more pellets spread the same damage wider and a slug concentrates it. Ignite (s): an enemy hit burns (Burn DPS) for this long, then loses its current layer if it's still alive (not bosses).</t>
         </is>
       </c>
     </row>
@@ -13400,6 +13400,11 @@
       <c r="AG4" s="21" t="inlineStr">
         <is>
           <t>Scope</t>
+        </is>
+      </c>
+      <c r="AH4" s="21" t="inlineStr">
+        <is>
+          <t>Ignite (s)</t>
         </is>
       </c>
     </row>
@@ -13462,6 +13467,7 @@
       <c r="AE5" s="57" t="n"/>
       <c r="AF5" s="57" t="n"/>
       <c r="AG5" s="57" t="n"/>
+      <c r="AH5" s="57" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="43" t="inlineStr">
@@ -13522,6 +13528,7 @@
       <c r="AE6" s="57" t="n"/>
       <c r="AF6" s="57" t="n"/>
       <c r="AG6" s="57" t="n"/>
+      <c r="AH6" s="57" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="43" t="inlineStr">
@@ -13584,6 +13591,7 @@
       <c r="AE7" s="57" t="n"/>
       <c r="AF7" s="57" t="n"/>
       <c r="AG7" s="57" t="n"/>
+      <c r="AH7" s="57" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="43" t="inlineStr">
@@ -13646,6 +13654,7 @@
       <c r="AE8" s="57" t="n"/>
       <c r="AF8" s="57" t="n"/>
       <c r="AG8" s="57" t="n"/>
+      <c r="AH8" s="57" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="43" t="inlineStr">
@@ -13714,6 +13723,7 @@
       <c r="AE9" s="57" t="n"/>
       <c r="AF9" s="57" t="n"/>
       <c r="AG9" s="57" t="n"/>
+      <c r="AH9" s="57" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="43" t="inlineStr">
@@ -13772,6 +13782,7 @@
       <c r="AE10" s="57" t="n"/>
       <c r="AF10" s="57" t="n"/>
       <c r="AG10" s="57" t="n"/>
+      <c r="AH10" s="57" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="43" t="inlineStr">
@@ -13832,6 +13843,7 @@
       <c r="AE11" s="57" t="n"/>
       <c r="AF11" s="57" t="n"/>
       <c r="AG11" s="57" t="n"/>
+      <c r="AH11" s="57" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="43" t="inlineStr">
@@ -13898,6 +13910,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="AH12" s="57" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="43" t="inlineStr">
@@ -13968,6 +13981,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="AH13" s="57" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="43" t="inlineStr">
@@ -14040,6 +14054,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="AH14" s="57" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="43" t="inlineStr">
@@ -14098,6 +14113,7 @@
       <c r="AE15" s="57" t="n"/>
       <c r="AF15" s="57" t="n"/>
       <c r="AG15" s="57" t="n"/>
+      <c r="AH15" s="57" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="43" t="inlineStr">
@@ -14158,6 +14174,7 @@
       <c r="AE16" s="57" t="n"/>
       <c r="AF16" s="57" t="n"/>
       <c r="AG16" s="57" t="n"/>
+      <c r="AH16" s="57" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="43" t="inlineStr">
@@ -14220,6 +14237,7 @@
       <c r="AE17" s="57" t="n"/>
       <c r="AF17" s="57" t="n"/>
       <c r="AG17" s="57" t="n"/>
+      <c r="AH17" s="57" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="43" t="inlineStr">
@@ -14284,6 +14302,7 @@
       <c r="AE18" s="57" t="n"/>
       <c r="AF18" s="57" t="n"/>
       <c r="AG18" s="57" t="n"/>
+      <c r="AH18" s="57" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="43" t="inlineStr">
@@ -14348,6 +14367,7 @@
       <c r="AE19" s="57" t="n"/>
       <c r="AF19" s="57" t="n"/>
       <c r="AG19" s="57" t="n"/>
+      <c r="AH19" s="57" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="43" t="inlineStr">
@@ -14406,6 +14426,7 @@
       <c r="AE20" s="57" t="n"/>
       <c r="AF20" s="57" t="n"/>
       <c r="AG20" s="57" t="n"/>
+      <c r="AH20" s="57" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="43" t="inlineStr">
@@ -14466,6 +14487,7 @@
       <c r="AE21" s="57" t="n"/>
       <c r="AF21" s="57" t="n"/>
       <c r="AG21" s="57" t="n"/>
+      <c r="AH21" s="57" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="43" t="inlineStr">
@@ -14534,6 +14556,7 @@
       <c r="AE22" s="57" t="n"/>
       <c r="AF22" s="57" t="n"/>
       <c r="AG22" s="57" t="n"/>
+      <c r="AH22" s="57" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="43" t="inlineStr">
@@ -14604,6 +14627,7 @@
       <c r="AE23" s="57" t="n"/>
       <c r="AF23" s="57" t="n"/>
       <c r="AG23" s="57" t="n"/>
+      <c r="AH23" s="57" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="43" t="inlineStr">
@@ -14676,6 +14700,7 @@
       <c r="AE24" s="57" t="n"/>
       <c r="AF24" s="57" t="n"/>
       <c r="AG24" s="57" t="n"/>
+      <c r="AH24" s="57" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="43" t="inlineStr">
@@ -14734,6 +14759,7 @@
       <c r="AE25" s="57" t="n"/>
       <c r="AF25" s="57" t="n"/>
       <c r="AG25" s="57" t="n"/>
+      <c r="AH25" s="57" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="43" t="inlineStr">
@@ -14794,6 +14820,7 @@
       <c r="AE26" s="57" t="n"/>
       <c r="AF26" s="57" t="n"/>
       <c r="AG26" s="57" t="n"/>
+      <c r="AH26" s="57" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="43" t="inlineStr">
@@ -14858,6 +14885,7 @@
       <c r="AE27" s="57" t="n"/>
       <c r="AF27" s="57" t="n"/>
       <c r="AG27" s="57" t="n"/>
+      <c r="AH27" s="57" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="43" t="inlineStr">
@@ -14924,6 +14952,7 @@
       </c>
       <c r="AF28" s="57" t="n"/>
       <c r="AG28" s="57" t="n"/>
+      <c r="AH28" s="57" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="43" t="inlineStr">
@@ -14992,6 +15021,7 @@
         <v>2.5</v>
       </c>
       <c r="AG29" s="57" t="n"/>
+      <c r="AH29" s="57" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="43" t="inlineStr">
@@ -15050,6 +15080,7 @@
       <c r="AE30" s="57" t="n"/>
       <c r="AF30" s="57" t="n"/>
       <c r="AG30" s="57" t="n"/>
+      <c r="AH30" s="57" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="43" t="inlineStr">
@@ -15112,6 +15143,7 @@
       <c r="AE31" s="57" t="n"/>
       <c r="AF31" s="57" t="n"/>
       <c r="AG31" s="57" t="n"/>
+      <c r="AH31" s="57" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="43" t="inlineStr">
@@ -15178,6 +15210,7 @@
       <c r="AE32" s="57" t="n"/>
       <c r="AF32" s="57" t="n"/>
       <c r="AG32" s="57" t="n"/>
+      <c r="AH32" s="57" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="43" t="inlineStr">
@@ -15248,6 +15281,7 @@
       <c r="AE33" s="57" t="n"/>
       <c r="AF33" s="57" t="n"/>
       <c r="AG33" s="57" t="n"/>
+      <c r="AH33" s="57" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="43" t="inlineStr">
@@ -15320,6 +15354,7 @@
       <c r="AE34" s="57" t="n"/>
       <c r="AF34" s="57" t="n"/>
       <c r="AG34" s="57" t="n"/>
+      <c r="AH34" s="57" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="43" t="inlineStr">
@@ -15386,6 +15421,7 @@
       <c r="AE35" s="57" t="n"/>
       <c r="AF35" s="57" t="n"/>
       <c r="AG35" s="57" t="n"/>
+      <c r="AH35" s="57" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="43" t="inlineStr">
@@ -15456,6 +15492,7 @@
       <c r="AE36" s="57" t="n"/>
       <c r="AF36" s="57" t="n"/>
       <c r="AG36" s="57" t="n"/>
+      <c r="AH36" s="57" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="43" t="inlineStr">
@@ -15530,6 +15567,7 @@
       <c r="AE37" s="57" t="n"/>
       <c r="AF37" s="57" t="n"/>
       <c r="AG37" s="57" t="n"/>
+      <c r="AH37" s="57" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="43" t="inlineStr">
@@ -15604,6 +15642,7 @@
       <c r="AE38" s="57" t="n"/>
       <c r="AF38" s="57" t="n"/>
       <c r="AG38" s="57" t="n"/>
+      <c r="AH38" s="57" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="43" t="inlineStr">
@@ -15678,6 +15717,7 @@
       <c r="AE39" s="57" t="n"/>
       <c r="AF39" s="57" t="n"/>
       <c r="AG39" s="57" t="n"/>
+      <c r="AH39" s="57" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="43" t="inlineStr">
@@ -15736,6 +15776,7 @@
       <c r="AE40" s="57" t="n"/>
       <c r="AF40" s="57" t="n"/>
       <c r="AG40" s="57" t="n"/>
+      <c r="AH40" s="57" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="43" t="inlineStr">
@@ -15796,6 +15837,7 @@
       <c r="AE41" s="57" t="n"/>
       <c r="AF41" s="57" t="n"/>
       <c r="AG41" s="57" t="n"/>
+      <c r="AH41" s="57" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="43" t="inlineStr">
@@ -15860,6 +15902,9 @@
       <c r="AE42" s="57" t="n"/>
       <c r="AF42" s="57" t="n"/>
       <c r="AG42" s="57" t="n"/>
+      <c r="AH42" s="57" t="n">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="43" t="inlineStr">
@@ -15928,6 +15973,9 @@
       <c r="AE43" s="57" t="n"/>
       <c r="AF43" s="57" t="n"/>
       <c r="AG43" s="57" t="n"/>
+      <c r="AH43" s="57" t="n">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="43" t="inlineStr">
@@ -16002,6 +16050,9 @@
       <c r="AE44" s="57" t="n"/>
       <c r="AF44" s="57" t="n"/>
       <c r="AG44" s="57" t="n"/>
+      <c r="AH44" s="57" t="n">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="43" t="inlineStr">
@@ -16060,6 +16111,7 @@
       <c r="AE45" s="57" t="n"/>
       <c r="AF45" s="57" t="n"/>
       <c r="AG45" s="57" t="n"/>
+      <c r="AH45" s="57" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="43" t="inlineStr">
@@ -16120,6 +16172,7 @@
       <c r="AE46" s="57" t="n"/>
       <c r="AF46" s="57" t="n"/>
       <c r="AG46" s="57" t="n"/>
+      <c r="AH46" s="57" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="43" t="inlineStr">
@@ -16182,6 +16235,7 @@
       <c r="AE47" s="57" t="n"/>
       <c r="AF47" s="57" t="n"/>
       <c r="AG47" s="57" t="n"/>
+      <c r="AH47" s="57" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="43" t="inlineStr">
@@ -16246,6 +16300,7 @@
       <c r="AE48" s="57" t="n"/>
       <c r="AF48" s="57" t="n"/>
       <c r="AG48" s="57" t="n"/>
+      <c r="AH48" s="57" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="43" t="inlineStr">
@@ -16312,6 +16367,7 @@
       <c r="AE49" s="57" t="n"/>
       <c r="AF49" s="57" t="n"/>
       <c r="AG49" s="57" t="n"/>
+      <c r="AH49" s="57" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Ignite: one burn tick instead of an automatic layer pop
User clarification: Dragon's Breath should be able to take an enemy down a
level early on, not remove a layer automatically. An ignited enemy now shows
flames for Ignite (s) = 1.5s, then takes one tick of damage equal to
Ignite tick (x shot) = 0.25 of the whole shot's damage (all pellets):
about 1.2 on the base shotgun, enough to pop an early 1-2 HP layer, a small
extra against later ones. Bosses get the same tick. The burning ground patch
is unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Storm-Split-Balance.xlsx
+++ b/Storm-Split-Balance.xlsx
@@ -13184,7 +13184,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH49"/>
+  <dimension ref="A1:AI49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" style="90" min="1" max="1"/>
@@ -13232,7 +13232,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Effect columns are cumulative per tier (like Tower Upgrades); blank = no change. x columns multiply the hero's base; Fire mode / Guns / Pellets / Pierce / Bounces override it. Crossover rule as towers: two paths, one past tier 2. Damage is per shot: pellets share the hero's base damage x its base pellet count, so more pellets spread the same damage wider and a slug concentrates it. Ignite (s): an enemy hit burns (Burn DPS) for this long, then loses its current layer if it's still alive (not bosses).</t>
+          <t>Effect columns are cumulative per tier (like Tower Upgrades); blank = no change. x columns multiply the hero's base; Fire mode / Guns / Pellets / Pierce / Bounces override it. Crossover rule as towers: two paths, one past tier 2. Damage is per shot: pellets share the hero's base damage x its base pellet count, so more pellets spread the same damage wider and a slug concentrates it. Ignite: an enemy hit burns for Ignite (s), then takes one tick of Ignite tick x the whole shot's damage.</t>
         </is>
       </c>
     </row>
@@ -13405,6 +13405,11 @@
       <c r="AH4" s="21" t="inlineStr">
         <is>
           <t>Ignite (s)</t>
+        </is>
+      </c>
+      <c r="AI4" s="21" t="inlineStr">
+        <is>
+          <t>Ignite tick (x shot)</t>
         </is>
       </c>
     </row>
@@ -13468,6 +13473,7 @@
       <c r="AF5" s="57" t="n"/>
       <c r="AG5" s="57" t="n"/>
       <c r="AH5" s="57" t="n"/>
+      <c r="AI5" s="57" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="43" t="inlineStr">
@@ -13529,6 +13535,7 @@
       <c r="AF6" s="57" t="n"/>
       <c r="AG6" s="57" t="n"/>
       <c r="AH6" s="57" t="n"/>
+      <c r="AI6" s="57" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="43" t="inlineStr">
@@ -13592,6 +13599,7 @@
       <c r="AF7" s="57" t="n"/>
       <c r="AG7" s="57" t="n"/>
       <c r="AH7" s="57" t="n"/>
+      <c r="AI7" s="57" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="43" t="inlineStr">
@@ -13655,6 +13663,7 @@
       <c r="AF8" s="57" t="n"/>
       <c r="AG8" s="57" t="n"/>
       <c r="AH8" s="57" t="n"/>
+      <c r="AI8" s="57" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="43" t="inlineStr">
@@ -13724,6 +13733,7 @@
       <c r="AF9" s="57" t="n"/>
       <c r="AG9" s="57" t="n"/>
       <c r="AH9" s="57" t="n"/>
+      <c r="AI9" s="57" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="43" t="inlineStr">
@@ -13783,6 +13793,7 @@
       <c r="AF10" s="57" t="n"/>
       <c r="AG10" s="57" t="n"/>
       <c r="AH10" s="57" t="n"/>
+      <c r="AI10" s="57" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="43" t="inlineStr">
@@ -13844,6 +13855,7 @@
       <c r="AF11" s="57" t="n"/>
       <c r="AG11" s="57" t="n"/>
       <c r="AH11" s="57" t="n"/>
+      <c r="AI11" s="57" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="43" t="inlineStr">
@@ -13911,6 +13923,7 @@
         </is>
       </c>
       <c r="AH12" s="57" t="n"/>
+      <c r="AI12" s="57" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="43" t="inlineStr">
@@ -13982,6 +13995,7 @@
         </is>
       </c>
       <c r="AH13" s="57" t="n"/>
+      <c r="AI13" s="57" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="43" t="inlineStr">
@@ -14055,6 +14069,7 @@
         </is>
       </c>
       <c r="AH14" s="57" t="n"/>
+      <c r="AI14" s="57" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="43" t="inlineStr">
@@ -14114,6 +14129,7 @@
       <c r="AF15" s="57" t="n"/>
       <c r="AG15" s="57" t="n"/>
       <c r="AH15" s="57" t="n"/>
+      <c r="AI15" s="57" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="43" t="inlineStr">
@@ -14175,6 +14191,7 @@
       <c r="AF16" s="57" t="n"/>
       <c r="AG16" s="57" t="n"/>
       <c r="AH16" s="57" t="n"/>
+      <c r="AI16" s="57" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="43" t="inlineStr">
@@ -14238,6 +14255,7 @@
       <c r="AF17" s="57" t="n"/>
       <c r="AG17" s="57" t="n"/>
       <c r="AH17" s="57" t="n"/>
+      <c r="AI17" s="57" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="43" t="inlineStr">
@@ -14303,6 +14321,7 @@
       <c r="AF18" s="57" t="n"/>
       <c r="AG18" s="57" t="n"/>
       <c r="AH18" s="57" t="n"/>
+      <c r="AI18" s="57" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="43" t="inlineStr">
@@ -14368,6 +14387,7 @@
       <c r="AF19" s="57" t="n"/>
       <c r="AG19" s="57" t="n"/>
       <c r="AH19" s="57" t="n"/>
+      <c r="AI19" s="57" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="43" t="inlineStr">
@@ -14427,6 +14447,7 @@
       <c r="AF20" s="57" t="n"/>
       <c r="AG20" s="57" t="n"/>
       <c r="AH20" s="57" t="n"/>
+      <c r="AI20" s="57" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="43" t="inlineStr">
@@ -14488,6 +14509,7 @@
       <c r="AF21" s="57" t="n"/>
       <c r="AG21" s="57" t="n"/>
       <c r="AH21" s="57" t="n"/>
+      <c r="AI21" s="57" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="43" t="inlineStr">
@@ -14557,6 +14579,7 @@
       <c r="AF22" s="57" t="n"/>
       <c r="AG22" s="57" t="n"/>
       <c r="AH22" s="57" t="n"/>
+      <c r="AI22" s="57" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="43" t="inlineStr">
@@ -14628,6 +14651,7 @@
       <c r="AF23" s="57" t="n"/>
       <c r="AG23" s="57" t="n"/>
       <c r="AH23" s="57" t="n"/>
+      <c r="AI23" s="57" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="43" t="inlineStr">
@@ -14701,6 +14725,7 @@
       <c r="AF24" s="57" t="n"/>
       <c r="AG24" s="57" t="n"/>
       <c r="AH24" s="57" t="n"/>
+      <c r="AI24" s="57" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="43" t="inlineStr">
@@ -14760,6 +14785,7 @@
       <c r="AF25" s="57" t="n"/>
       <c r="AG25" s="57" t="n"/>
       <c r="AH25" s="57" t="n"/>
+      <c r="AI25" s="57" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="43" t="inlineStr">
@@ -14821,6 +14847,7 @@
       <c r="AF26" s="57" t="n"/>
       <c r="AG26" s="57" t="n"/>
       <c r="AH26" s="57" t="n"/>
+      <c r="AI26" s="57" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="43" t="inlineStr">
@@ -14886,6 +14913,7 @@
       <c r="AF27" s="57" t="n"/>
       <c r="AG27" s="57" t="n"/>
       <c r="AH27" s="57" t="n"/>
+      <c r="AI27" s="57" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="43" t="inlineStr">
@@ -14953,6 +14981,7 @@
       <c r="AF28" s="57" t="n"/>
       <c r="AG28" s="57" t="n"/>
       <c r="AH28" s="57" t="n"/>
+      <c r="AI28" s="57" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="43" t="inlineStr">
@@ -15022,6 +15051,7 @@
       </c>
       <c r="AG29" s="57" t="n"/>
       <c r="AH29" s="57" t="n"/>
+      <c r="AI29" s="57" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="43" t="inlineStr">
@@ -15081,6 +15111,7 @@
       <c r="AF30" s="57" t="n"/>
       <c r="AG30" s="57" t="n"/>
       <c r="AH30" s="57" t="n"/>
+      <c r="AI30" s="57" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="43" t="inlineStr">
@@ -15144,6 +15175,7 @@
       <c r="AF31" s="57" t="n"/>
       <c r="AG31" s="57" t="n"/>
       <c r="AH31" s="57" t="n"/>
+      <c r="AI31" s="57" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="43" t="inlineStr">
@@ -15211,6 +15243,7 @@
       <c r="AF32" s="57" t="n"/>
       <c r="AG32" s="57" t="n"/>
       <c r="AH32" s="57" t="n"/>
+      <c r="AI32" s="57" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="43" t="inlineStr">
@@ -15282,6 +15315,7 @@
       <c r="AF33" s="57" t="n"/>
       <c r="AG33" s="57" t="n"/>
       <c r="AH33" s="57" t="n"/>
+      <c r="AI33" s="57" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="43" t="inlineStr">
@@ -15355,6 +15389,7 @@
       <c r="AF34" s="57" t="n"/>
       <c r="AG34" s="57" t="n"/>
       <c r="AH34" s="57" t="n"/>
+      <c r="AI34" s="57" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="43" t="inlineStr">
@@ -15422,6 +15457,7 @@
       <c r="AF35" s="57" t="n"/>
       <c r="AG35" s="57" t="n"/>
       <c r="AH35" s="57" t="n"/>
+      <c r="AI35" s="57" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="43" t="inlineStr">
@@ -15493,6 +15529,7 @@
       <c r="AF36" s="57" t="n"/>
       <c r="AG36" s="57" t="n"/>
       <c r="AH36" s="57" t="n"/>
+      <c r="AI36" s="57" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="43" t="inlineStr">
@@ -15568,6 +15605,7 @@
       <c r="AF37" s="57" t="n"/>
       <c r="AG37" s="57" t="n"/>
       <c r="AH37" s="57" t="n"/>
+      <c r="AI37" s="57" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="43" t="inlineStr">
@@ -15643,6 +15681,7 @@
       <c r="AF38" s="57" t="n"/>
       <c r="AG38" s="57" t="n"/>
       <c r="AH38" s="57" t="n"/>
+      <c r="AI38" s="57" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="43" t="inlineStr">
@@ -15718,6 +15757,7 @@
       <c r="AF39" s="57" t="n"/>
       <c r="AG39" s="57" t="n"/>
       <c r="AH39" s="57" t="n"/>
+      <c r="AI39" s="57" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="43" t="inlineStr">
@@ -15777,6 +15817,7 @@
       <c r="AF40" s="57" t="n"/>
       <c r="AG40" s="57" t="n"/>
       <c r="AH40" s="57" t="n"/>
+      <c r="AI40" s="57" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="43" t="inlineStr">
@@ -15838,6 +15879,7 @@
       <c r="AF41" s="57" t="n"/>
       <c r="AG41" s="57" t="n"/>
       <c r="AH41" s="57" t="n"/>
+      <c r="AI41" s="57" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="43" t="inlineStr">
@@ -15905,6 +15947,9 @@
       <c r="AH42" s="57" t="n">
         <v>1.5</v>
       </c>
+      <c r="AI42" s="57" t="n">
+        <v>0.25</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="43" t="inlineStr">
@@ -15976,6 +16021,9 @@
       <c r="AH43" s="57" t="n">
         <v>1.5</v>
       </c>
+      <c r="AI43" s="57" t="n">
+        <v>0.25</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="43" t="inlineStr">
@@ -16052,6 +16100,9 @@
       <c r="AG44" s="57" t="n"/>
       <c r="AH44" s="57" t="n">
         <v>1.5</v>
+      </c>
+      <c r="AI44" s="57" t="n">
+        <v>0.25</v>
       </c>
     </row>
     <row r="45">
@@ -16112,6 +16163,7 @@
       <c r="AF45" s="57" t="n"/>
       <c r="AG45" s="57" t="n"/>
       <c r="AH45" s="57" t="n"/>
+      <c r="AI45" s="57" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="43" t="inlineStr">
@@ -16173,6 +16225,7 @@
       <c r="AF46" s="57" t="n"/>
       <c r="AG46" s="57" t="n"/>
       <c r="AH46" s="57" t="n"/>
+      <c r="AI46" s="57" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="43" t="inlineStr">
@@ -16236,6 +16289,7 @@
       <c r="AF47" s="57" t="n"/>
       <c r="AG47" s="57" t="n"/>
       <c r="AH47" s="57" t="n"/>
+      <c r="AI47" s="57" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="43" t="inlineStr">
@@ -16301,6 +16355,7 @@
       <c r="AF48" s="57" t="n"/>
       <c r="AG48" s="57" t="n"/>
       <c r="AH48" s="57" t="n"/>
+      <c r="AI48" s="57" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="43" t="inlineStr">
@@ -16368,6 +16423,7 @@
       <c r="AF49" s="57" t="n"/>
       <c r="AG49" s="57" t="n"/>
       <c r="AH49" s="57" t="n"/>
+      <c r="AI49" s="57" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Ignite passes to split children; tick 35% of the shot
User: a Dragon's Breath shot should take a Brute (blue) down to Husks
(green), and the Husks should die on the fire tick.

- The fire now lives on the enemy (Enemies.ignite / extinguish) and passes
  to split children like a Mark, on the same timer, so a Brute popped by
  the blast leaves Husks that burn out together when the tick lands.
- Hero rounds ignite before dealing damage, so a pellet that pops the enemy
  still lights its children.
- Tick 0.25 -> 0.35 of the shot (~1.7 on the base shotgun): kills Husks to
  about round 11 on Easy, round 6 on Normal, round 1 on Hard. 0.25 (1.2)
  missed round-1 Husks on Normal (x1.25 HP).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Storm-Split-Balance.xlsx
+++ b/Storm-Split-Balance.xlsx
@@ -13232,7 +13232,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Effect columns are cumulative per tier (like Tower Upgrades); blank = no change. x columns multiply the hero's base; Fire mode / Guns / Pellets / Pierce / Bounces override it. Crossover rule as towers: two paths, one past tier 2. Damage is per shot: pellets share the hero's base damage x its base pellet count, so more pellets spread the same damage wider and a slug concentrates it. Ignite: an enemy hit burns for Ignite (s), then takes one tick of Ignite tick x the whole shot's damage.</t>
+          <t>Effect columns are cumulative per tier (like Tower Upgrades); blank = no change. x columns multiply the hero's base; Fire mode / Guns / Pellets / Pierce / Bounces override it. Crossover rule as towers: two paths, one past tier 2. Damage is per shot: pellets share the hero's base damage x its base pellet count, so more pellets spread the same damage wider and a slug concentrates it. Ignite: an enemy hit burns for Ignite (s), then takes one tick of Ignite tick x the whole shot's damage. The fire passes to the enemy's split children, so a Brute shot down to Husks sees them burn out together.</t>
         </is>
       </c>
     </row>
@@ -15948,7 +15948,7 @@
         <v>1.5</v>
       </c>
       <c r="AI42" s="57" t="n">
-        <v>0.25</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="43">
@@ -16022,7 +16022,7 @@
         <v>1.5</v>
       </c>
       <c r="AI43" s="57" t="n">
-        <v>0.25</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="44">
@@ -16102,7 +16102,7 @@
         <v>1.5</v>
       </c>
       <c r="AI44" s="57" t="n">
-        <v>0.25</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="45">

</xml_diff>

<commit_message>
Levels: heroes and towers keep pace with enemy HP
Enemy HP compounds ~5% a round (x7 by round 40) and hero upgrades are about
handling, so the hero fell behind. Every 5 rounds cleared, everyone levels
up: all hero damage (rounds, splash, fire, Airburst) x1.25 and all tower
damage (shots, bomblets, freeze, burns) x1.1, compounding. A banner
announces it and the status bar shows the level.

Levels are stored per player (HeroLevel) so the planned next step - hero XP
from your own pops - only changes the trigger (HEROES.md).

Tuning: Rounds per level, Hero / Tower damage per level. The exporter's
hero-vs-tower guard now compares at the last round's level (206 vs 826 DPS
at level 9).

Statically checked; not yet playtested.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Storm-Split-Balance.xlsx
+++ b/Storm-Split-Balance.xlsx
@@ -4182,7 +4182,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66667" defaultRowHeight="15" customHeight="1" outlineLevelRow="0"/>
   <cols>
     <col width="34" customWidth="1" style="81" min="1" max="1"/>
@@ -5127,6 +5127,76 @@
       <c r="D56" s="29" t="inlineStr">
         <is>
           <t>Chests land this far around their Quartermaster at most.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="31" t="inlineStr">
+        <is>
+          <t>HERO LEVELS</t>
+        </is>
+      </c>
+      <c r="B58" s="24" t="n"/>
+      <c r="C58" s="32" t="n"/>
+      <c r="D58" s="32" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="26" t="inlineStr">
+        <is>
+          <t>Rounds per level</t>
+        </is>
+      </c>
+      <c r="B59" s="30" t="n">
+        <v>5</v>
+      </c>
+      <c r="C59" s="28" t="inlineStr">
+        <is>
+          <t>rounds</t>
+        </is>
+      </c>
+      <c r="D59" s="29" t="inlineStr">
+        <is>
+          <t>Every this many rounds cleared, heroes level up and towers get stronger. (Later: hero XP from pops.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="26" t="inlineStr">
+        <is>
+          <t>Hero damage per level</t>
+        </is>
+      </c>
+      <c r="B60" s="30" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C60" s="28" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="D60" s="29" t="inlineStr">
+        <is>
+          <t>Each hero level multiplies all hero damage by 1 + this (compounding).</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="26" t="inlineStr">
+        <is>
+          <t>Tower damage per level</t>
+        </is>
+      </c>
+      <c r="B61" s="30" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C61" s="28" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="D61" s="29" t="inlineStr">
+        <is>
+          <t>Each level multiplies all tower damage by 1 + this (compounding).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Readable hero burn patch: Burn patch min reach lever
T10b of the gauntlet plan (DECISIONS #32).

Spreadsheet: Tuning row 75 (A75:E75 asserted empty, style copied from the
row above): "Burn patch min reach" = 3 studs, with a note. Exporter: added
to `needed`. Config diff, the one line: Tuning BurnPatchMinReach = 3.

Hazards.burn: reach = math.max(reach, Config.Tuning.BurnPatchMinReach)
instead of the literal 1 (Hazards now requires Shared/Config). No other
change: tower burns (Napalm and up) have splash radii >= 9, so only a
hero patch with no splash (Big Game Hunter Incendiary / AP / Hot Load)
changes, from 1 stud to 3.

Spec: heroes +1, Incendiary's patch reach >= 3 (and the lever is 3); it can
fail (expecting 4 failed it, then reverted). tools/check.sh clean;
tools/test.sh 89 passed; audit: only Tuning.MaxProjectiles (T12).
Statically checked and headless-tested, not playtested.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Storm-Split-Balance.xlsx
+++ b/Storm-Split-Balance.xlsx
@@ -4199,7 +4199,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E74"/>
+  <dimension ref="A1:E75"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66667" defaultRowHeight="15" customHeight="1" outlineLevelRow="0"/>
   <cols>
     <col width="34" customWidth="1" style="81" min="1" max="1"/>
@@ -5414,6 +5414,26 @@
       <c r="D74" s="29" t="inlineStr">
         <is>
           <t>Repairing a tower from 0 HP costs this share of the cash put into it (less for partial damage).</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="26" t="inlineStr">
+        <is>
+          <t>Burn patch min reach</t>
+        </is>
+      </c>
+      <c r="B75" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="C75" s="28" t="inlineStr">
+        <is>
+          <t>studs</t>
+        </is>
+      </c>
+      <c r="D75" s="29" t="inlineStr">
+        <is>
+          <t>Burning ground is at least this wide either side, so a hero patch with no splash (Incendiary) is visible.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rename four tiers Jovan approved (DECISIONS #52)
Skybreaker -> Extinction Round (Longshot Perch Siege T5), Storm of Steel
-> Meteor Shower (Mortar Pit Cluster T5), Crack Armor -> Find the Gap
(Tranq Station Weak Spot T2), Quick Mark -> Quick Dart (Tracker Trick
Shot T4). Cells found by (tower/hero, path, tier) and asserted before
writing; Config changed by exactly those four name lines. Design docs and
specs updated; audit compares 165 tier names with 0 findings; tests pass.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Storm-Split-Balance.xlsx
+++ b/Storm-Split-Balance.xlsx
@@ -9243,7 +9243,7 @@
       </c>
       <c r="M34" s="43" t="inlineStr">
         <is>
-          <t>Skybreaker</t>
+          <t>Extinction Round</t>
         </is>
       </c>
       <c r="N34" s="57" t="n"/>
@@ -10149,7 +10149,7 @@
       </c>
       <c r="M44" s="43" t="inlineStr">
         <is>
-          <t>Storm of Steel</t>
+          <t>Meteor Shower</t>
         </is>
       </c>
       <c r="N44" s="57" t="n"/>
@@ -11707,7 +11707,7 @@
       </c>
       <c r="M61" s="43" t="inlineStr">
         <is>
-          <t>Crack Armor</t>
+          <t>Find the Gap</t>
         </is>
       </c>
       <c r="N61" s="57" t="n"/>
@@ -18162,7 +18162,7 @@
       </c>
       <c r="E18" s="43" t="inlineStr">
         <is>
-          <t>Quick Mark</t>
+          <t>Quick Dart</t>
         </is>
       </c>
       <c r="F18" s="56">

</xml_diff>

<commit_message>
T24b: round 39 below the finale; round-11 step named in value.py
Rounds!H43 (round 39 Triceratops) 12 -> 10 (DECISIONS #78). Config: round 39
ZEP 12 -> 10 and its derived effectiveHp 44314 -> 40470; nothing else.
threat.py: round 39 defended mid-gap 241.6 -> 212.1 (round 40: 215.8).
Finale EHP 285,725 = -11.6% of the pre-T21 323,127 (bar +/-12%). Normal solo
minimum over rounds 11-39 0.77 (r39) -> 0.78 (r37); round 40 slips 0.01
(less cash from round 39).

value.py: the step check runs from round 2 at 1.6x; round 11 is a named
exception ("first armour and air wave", x2.02) with its own 2.1x bar, printed
in the pacing report (#77). Comment citing #79 on the damage medians. No new
finding.

Statically checked and headless-tested, not playtested.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Storm-Split-Balance.xlsx
+++ b/Storm-Split-Balance.xlsx
@@ -5405,7 +5405,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E89"/>
+  <dimension ref="A1:E85"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66667" defaultRowHeight="15" customHeight="1" outlineLevelRow="0"/>
   <cols>
     <col width="34" customWidth="1" style="81" min="1" max="1"/>
@@ -6663,7 +6663,6 @@
         </is>
       </c>
     </row>
-    <row r="77"/>
     <row r="78">
       <c r="A78" s="31" t="inlineStr">
         <is>
@@ -6811,10 +6810,6 @@
         </is>
       </c>
     </row>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811" footer="0.511811"/>
   <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" firstPageNumber="1" useFirstPageNumber="0" pageOrder="downThenOver"/>
@@ -27303,7 +27298,7 @@
         <v>18</v>
       </c>
       <c r="H43" s="60" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="I43" s="60" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
T44: softer boss throws vs towers, lever 0.3 (DECISIONS #138, #154)
Tuning gains block BOSS THROWS (rows 97-98), `Boss ranged vs towers x`
= 0.3; Config diff is the one Tuning line BossRangedVsTowersX = 0.3.
Combat.throwDamage applies it when a Boss species' throw lands on a
tower; hunters and other dinos' throws are unchanged (spec added).

threat.py splits rounds 31-40 mid-gap defended damage into boss / other
/ total and judges the boss share in 31-39 (< 50% of every non-Perch
tower's T0 HP; Hunting Blind 100 binds). Max boss share in 31-39:
0.5 -> 73.6 (7 misses), 0.4 -> 58.9 (3 misses), 0.3 -> 44.1 (0), so
0.3. Totals stay report-only (31-39: 51.6-109.1; other dinos 47-65).

Not playtested.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Storm-Split-Balance.xlsx
+++ b/Storm-Split-Balance.xlsx
@@ -5720,7 +5720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E95"/>
+  <dimension ref="A1:E98"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66667" defaultRowHeight="15" customHeight="1" outlineLevelRow="0"/>
   <cols>
     <col width="34" customWidth="1" style="81" min="1" max="1"/>
@@ -7232,14 +7232,14 @@
         </is>
       </c>
     </row>
-    <row r="94">
+    <row r="94" s="90">
       <c r="A94" s="31" t="inlineStr">
         <is>
           <t>MASTERY PERKS</t>
         </is>
       </c>
     </row>
-    <row r="95">
+    <row r="95" s="90">
       <c r="A95" s="26" t="inlineStr">
         <is>
           <t>Mastery perk worth cap</t>
@@ -7256,6 +7256,33 @@
       <c r="D95" s="29" t="inlineStr">
         <is>
           <t>The most a mastery perk may be worth, in % of one cast (Mastery Perks sheet, DECISIONS #99). Read by the exporter only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="31" t="inlineStr">
+        <is>
+          <t>BOSS THROWS</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="26" t="inlineStr">
+        <is>
+          <t>Boss ranged vs towers x</t>
+        </is>
+      </c>
+      <c r="B98" s="27" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C98" s="28" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="D98" s="29" t="inlineStr">
+        <is>
+          <t>A Boss species' projectile damage to a tower is multiplied by this; hunters take full damage (they can dodge). DECISIONS #138, #154. 1 = off.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
T52: hero tier 6 on all twelve paths (#133-#134)
Hero Upgrades gains twelve tier-6 rows (cost 6,400 from the ladder formula)
and eight columns: Burn patch reach, Staggered reload, Ricochet reload,
Burst recoil reset, Spun-up belt, Still spread x, Scoped spread x, Ability
charges. Heart Shot and Thunder Slug carry Size breaks 2 (hero path, no
level term). The exporter requires six tiers per path and in-order rows.

New pure Shared/GunRules holds the mechanics (spread cone, Hot Swap
staggered reload, Trick Reload, Five-Round Burst recoil reset, Endless
Belt, ability charges); server Hero and the client crosshair both use it.
Wildfire Drum's 4-stud patch goes through Combat.burnPatchReach.
tiersix.spec covers each tier 6; sizebreaks.spec covers the two 2s.
Config diff is additive only: 12 tiers + 8 default fields per tier.
Not playtested.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Storm-Split-Balance.xlsx
+++ b/Storm-Split-Balance.xlsx
@@ -18975,7 +18975,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS64"/>
+  <dimension ref="A1:BA79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" style="90" min="1" max="1"/>
@@ -19016,7 +19016,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>HERO UPGRADES — 4 heroes x 3 paths x 5 tiers (HEROES.md)</t>
+          <t>HERO UPGRADES — 4 heroes x 3 paths x 6 tiers (HEROES.md)</t>
         </is>
       </c>
     </row>
@@ -19251,6 +19251,46 @@
       <c r="AS4" s="104" t="inlineStr">
         <is>
           <t>Size breaks</t>
+        </is>
+      </c>
+      <c r="AT4" s="104" t="inlineStr">
+        <is>
+          <t>Burn patch reach (studs)</t>
+        </is>
+      </c>
+      <c r="AU4" s="104" t="inlineStr">
+        <is>
+          <t>Staggered reload</t>
+        </is>
+      </c>
+      <c r="AV4" s="104" t="inlineStr">
+        <is>
+          <t>Ricochet reload (rounds)</t>
+        </is>
+      </c>
+      <c r="AW4" s="104" t="inlineStr">
+        <is>
+          <t>Burst recoil reset</t>
+        </is>
+      </c>
+      <c r="AX4" s="104" t="inlineStr">
+        <is>
+          <t>Spun-up belt</t>
+        </is>
+      </c>
+      <c r="AY4" s="104" t="inlineStr">
+        <is>
+          <t>Still spread x</t>
+        </is>
+      </c>
+      <c r="AZ4" s="104" t="inlineStr">
+        <is>
+          <t>Scoped spread x</t>
+        </is>
+      </c>
+      <c r="BA4" s="104" t="inlineStr">
+        <is>
+          <t>Ability charges</t>
         </is>
       </c>
     </row>
@@ -23274,6 +23314,914 @@
         <v>6</v>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" s="43" t="inlineStr">
+        <is>
+          <t>Tracker</t>
+        </is>
+      </c>
+      <c r="B65" s="43" t="inlineStr">
+        <is>
+          <t>Gunslinger</t>
+        </is>
+      </c>
+      <c r="C65" s="43" t="inlineStr">
+        <is>
+          <t>handling</t>
+        </is>
+      </c>
+      <c r="D65" s="43" t="n">
+        <v>6</v>
+      </c>
+      <c r="E65" s="43" t="inlineStr">
+        <is>
+          <t>Hot Swap</t>
+        </is>
+      </c>
+      <c r="F65" s="56">
+        <f>ROUND(Tuning!$B$21*POWER(Tuning!$B$22,D65-1),0)</f>
+        <v/>
+      </c>
+      <c r="G65" s="57" t="n">
+        <v>2</v>
+      </c>
+      <c r="H65" s="57" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I65" s="57" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="J65" s="57" t="n"/>
+      <c r="K65" s="57" t="n"/>
+      <c r="L65" s="57" t="n"/>
+      <c r="M65" s="57" t="n"/>
+      <c r="N65" s="57" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="O65" s="57" t="n"/>
+      <c r="P65" s="57" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q65" s="57" t="n"/>
+      <c r="R65" s="57" t="n"/>
+      <c r="S65" s="57" t="n"/>
+      <c r="T65" s="57" t="n"/>
+      <c r="U65" s="57" t="n"/>
+      <c r="V65" s="57" t="n"/>
+      <c r="W65" s="57" t="n"/>
+      <c r="X65" s="57" t="n"/>
+      <c r="Y65" s="57" t="n"/>
+      <c r="Z65" s="57" t="n"/>
+      <c r="AA65" s="57" t="n"/>
+      <c r="AB65" s="57" t="n"/>
+      <c r="AC65" s="57" t="n"/>
+      <c r="AD65" s="57" t="n"/>
+      <c r="AE65" s="57" t="n"/>
+      <c r="AF65" s="57" t="n"/>
+      <c r="AG65" s="57" t="n"/>
+      <c r="AH65" s="57" t="n"/>
+      <c r="AI65" s="57" t="n"/>
+      <c r="AU65" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="43" t="inlineStr">
+        <is>
+          <t>Tracker</t>
+        </is>
+      </c>
+      <c r="B66" s="43" t="inlineStr">
+        <is>
+          <t>Marksman</t>
+        </is>
+      </c>
+      <c r="C66" s="43" t="inlineStr">
+        <is>
+          <t>accuracy</t>
+        </is>
+      </c>
+      <c r="D66" s="43" t="n">
+        <v>6</v>
+      </c>
+      <c r="E66" s="43" t="inlineStr">
+        <is>
+          <t>Heart Shot</t>
+        </is>
+      </c>
+      <c r="F66" s="56">
+        <f>ROUND(Tuning!$B$21*POWER(Tuning!$B$22,D66-1),0)</f>
+        <v/>
+      </c>
+      <c r="G66" s="57" t="n"/>
+      <c r="H66" s="57" t="n"/>
+      <c r="I66" s="57" t="n"/>
+      <c r="J66" s="57" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="K66" s="57" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L66" s="57" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="M66" s="57" t="n"/>
+      <c r="N66" s="57" t="n"/>
+      <c r="O66" s="57" t="n"/>
+      <c r="P66" s="57" t="n"/>
+      <c r="Q66" s="57" t="n"/>
+      <c r="R66" s="57" t="n"/>
+      <c r="S66" s="57" t="n"/>
+      <c r="T66" s="57" t="n"/>
+      <c r="U66" s="57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V66" s="57" t="n"/>
+      <c r="W66" s="57" t="n"/>
+      <c r="X66" s="57" t="n"/>
+      <c r="Y66" s="57" t="n"/>
+      <c r="Z66" s="57" t="n"/>
+      <c r="AA66" s="57" t="n"/>
+      <c r="AB66" s="57" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC66" s="57" t="n"/>
+      <c r="AD66" s="57" t="n"/>
+      <c r="AE66" s="57" t="n"/>
+      <c r="AF66" s="57" t="n"/>
+      <c r="AG66" s="57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AH66" s="57" t="n"/>
+      <c r="AI66" s="57" t="n"/>
+      <c r="AS66" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ66" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="43" t="inlineStr">
+        <is>
+          <t>Tracker</t>
+        </is>
+      </c>
+      <c r="B67" s="43" t="inlineStr">
+        <is>
+          <t>Trick Shot</t>
+        </is>
+      </c>
+      <c r="C67" s="43" t="inlineStr">
+        <is>
+          <t>utility</t>
+        </is>
+      </c>
+      <c r="D67" s="43" t="n">
+        <v>6</v>
+      </c>
+      <c r="E67" s="43" t="inlineStr">
+        <is>
+          <t>Trick Reload</t>
+        </is>
+      </c>
+      <c r="F67" s="56">
+        <f>ROUND(Tuning!$B$21*POWER(Tuning!$B$22,D67-1),0)</f>
+        <v/>
+      </c>
+      <c r="G67" s="57" t="n"/>
+      <c r="H67" s="57" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="I67" s="57" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J67" s="57" t="n"/>
+      <c r="K67" s="57" t="n"/>
+      <c r="L67" s="57" t="n"/>
+      <c r="M67" s="57" t="n"/>
+      <c r="N67" s="57" t="n"/>
+      <c r="O67" s="57" t="n"/>
+      <c r="P67" s="57" t="n"/>
+      <c r="Q67" s="57" t="n"/>
+      <c r="R67" s="57" t="n"/>
+      <c r="S67" s="57" t="n"/>
+      <c r="T67" s="57" t="n">
+        <v>4</v>
+      </c>
+      <c r="U67" s="57" t="n"/>
+      <c r="V67" s="57" t="n"/>
+      <c r="W67" s="57" t="n"/>
+      <c r="X67" s="57" t="n"/>
+      <c r="Y67" s="57" t="n"/>
+      <c r="Z67" s="57" t="n"/>
+      <c r="AA67" s="57" t="n"/>
+      <c r="AB67" s="57" t="n"/>
+      <c r="AC67" s="57" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="AD67" s="57" t="n"/>
+      <c r="AE67" s="57" t="n"/>
+      <c r="AF67" s="57" t="n"/>
+      <c r="AG67" s="57" t="n"/>
+      <c r="AH67" s="57" t="n"/>
+      <c r="AI67" s="57" t="n"/>
+      <c r="AV67" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="43" t="inlineStr">
+        <is>
+          <t>Big Game Hunter</t>
+        </is>
+      </c>
+      <c r="B68" s="43" t="inlineStr">
+        <is>
+          <t>Stalker</t>
+        </is>
+      </c>
+      <c r="C68" s="43" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D68" s="43" t="n">
+        <v>6</v>
+      </c>
+      <c r="E68" s="43" t="inlineStr">
+        <is>
+          <t>Five-Round Burst</t>
+        </is>
+      </c>
+      <c r="F68" s="56">
+        <f>ROUND(Tuning!$B$21*POWER(Tuning!$B$22,D68-1),0)</f>
+        <v/>
+      </c>
+      <c r="G68" s="57" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H68" s="57" t="n"/>
+      <c r="I68" s="57" t="n"/>
+      <c r="J68" s="57" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="K68" s="57" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="L68" s="57" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="M68" s="57" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="N68" s="57" t="inlineStr">
+        <is>
+          <t>burst</t>
+        </is>
+      </c>
+      <c r="O68" s="57" t="n">
+        <v>5</v>
+      </c>
+      <c r="P68" s="57" t="n"/>
+      <c r="Q68" s="57" t="n"/>
+      <c r="R68" s="57" t="n"/>
+      <c r="S68" s="57" t="n"/>
+      <c r="T68" s="57" t="n"/>
+      <c r="U68" s="57" t="n"/>
+      <c r="V68" s="57" t="n"/>
+      <c r="W68" s="57" t="n"/>
+      <c r="X68" s="57" t="n"/>
+      <c r="Y68" s="57" t="n"/>
+      <c r="Z68" s="57" t="n"/>
+      <c r="AA68" s="57" t="n"/>
+      <c r="AB68" s="57" t="n"/>
+      <c r="AC68" s="57" t="n"/>
+      <c r="AD68" s="57" t="n"/>
+      <c r="AE68" s="57" t="n"/>
+      <c r="AF68" s="57" t="n"/>
+      <c r="AG68" s="57" t="n"/>
+      <c r="AH68" s="57" t="n"/>
+      <c r="AI68" s="57" t="n"/>
+      <c r="AW68" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="43" t="inlineStr">
+        <is>
+          <t>Big Game Hunter</t>
+        </is>
+      </c>
+      <c r="B69" s="43" t="inlineStr">
+        <is>
+          <t>Heavy</t>
+        </is>
+      </c>
+      <c r="C69" s="43" t="inlineStr">
+        <is>
+          <t>sustain</t>
+        </is>
+      </c>
+      <c r="D69" s="43" t="n">
+        <v>6</v>
+      </c>
+      <c r="E69" s="43" t="inlineStr">
+        <is>
+          <t>Endless Belt</t>
+        </is>
+      </c>
+      <c r="F69" s="56">
+        <f>ROUND(Tuning!$B$21*POWER(Tuning!$B$22,D69-1),0)</f>
+        <v/>
+      </c>
+      <c r="G69" s="57" t="n"/>
+      <c r="H69" s="57" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="I69" s="57" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J69" s="57" t="n"/>
+      <c r="K69" s="57" t="n"/>
+      <c r="L69" s="57" t="n"/>
+      <c r="M69" s="57" t="n"/>
+      <c r="N69" s="57" t="n"/>
+      <c r="O69" s="57" t="n"/>
+      <c r="P69" s="57" t="n"/>
+      <c r="Q69" s="57" t="n"/>
+      <c r="R69" s="57" t="n"/>
+      <c r="S69" s="57" t="n"/>
+      <c r="T69" s="57" t="n"/>
+      <c r="U69" s="57" t="n"/>
+      <c r="V69" s="57" t="n"/>
+      <c r="W69" s="57" t="n"/>
+      <c r="X69" s="57" t="n"/>
+      <c r="Y69" s="57" t="n"/>
+      <c r="Z69" s="57" t="n"/>
+      <c r="AA69" s="57" t="n"/>
+      <c r="AB69" s="57" t="n"/>
+      <c r="AC69" s="57" t="n"/>
+      <c r="AD69" s="57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AE69" s="57" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AF69" s="57" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="AG69" s="57" t="n"/>
+      <c r="AH69" s="57" t="n"/>
+      <c r="AI69" s="57" t="n"/>
+      <c r="AX69" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="43" t="inlineStr">
+        <is>
+          <t>Big Game Hunter</t>
+        </is>
+      </c>
+      <c r="B70" s="43" t="inlineStr">
+        <is>
+          <t>Special Ammo</t>
+        </is>
+      </c>
+      <c r="C70" s="43" t="inlineStr">
+        <is>
+          <t>rounds</t>
+        </is>
+      </c>
+      <c r="D70" s="43" t="n">
+        <v>6</v>
+      </c>
+      <c r="E70" s="43" t="inlineStr">
+        <is>
+          <t>Powder Tips</t>
+        </is>
+      </c>
+      <c r="F70" s="56">
+        <f>ROUND(Tuning!$B$21*POWER(Tuning!$B$22,D70-1),0)</f>
+        <v/>
+      </c>
+      <c r="G70" s="57" t="n"/>
+      <c r="H70" s="57" t="n"/>
+      <c r="I70" s="57" t="n"/>
+      <c r="J70" s="57" t="n"/>
+      <c r="K70" s="57" t="n"/>
+      <c r="L70" s="57" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="M70" s="57" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="N70" s="57" t="n"/>
+      <c r="O70" s="57" t="n"/>
+      <c r="P70" s="57" t="n"/>
+      <c r="Q70" s="57" t="n"/>
+      <c r="R70" s="57" t="n"/>
+      <c r="S70" s="57" t="n"/>
+      <c r="T70" s="57" t="n"/>
+      <c r="U70" s="57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V70" s="57" t="n"/>
+      <c r="W70" s="57" t="n">
+        <v>1</v>
+      </c>
+      <c r="X70" s="57" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y70" s="57" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z70" s="57" t="n"/>
+      <c r="AA70" s="57" t="n">
+        <v>10</v>
+      </c>
+      <c r="AB70" s="57" t="n"/>
+      <c r="AC70" s="57" t="n"/>
+      <c r="AD70" s="57" t="n"/>
+      <c r="AE70" s="57" t="n"/>
+      <c r="AF70" s="57" t="n"/>
+      <c r="AG70" s="57" t="n"/>
+      <c r="AH70" s="57" t="n"/>
+      <c r="AI70" s="57" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="43" t="inlineStr">
+        <is>
+          <t>Brush Beater</t>
+        </is>
+      </c>
+      <c r="B71" s="43" t="inlineStr">
+        <is>
+          <t>Slug</t>
+        </is>
+      </c>
+      <c r="C71" s="43" t="inlineStr">
+        <is>
+          <t>reach</t>
+        </is>
+      </c>
+      <c r="D71" s="43" t="n">
+        <v>6</v>
+      </c>
+      <c r="E71" s="43" t="inlineStr">
+        <is>
+          <t>Thunder Slug</t>
+        </is>
+      </c>
+      <c r="F71" s="56">
+        <f>ROUND(Tuning!$B$21*POWER(Tuning!$B$22,D71-1),0)</f>
+        <v/>
+      </c>
+      <c r="G71" s="57" t="n"/>
+      <c r="H71" s="57" t="n"/>
+      <c r="I71" s="57" t="n"/>
+      <c r="J71" s="57" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="K71" s="57" t="n"/>
+      <c r="L71" s="57" t="n">
+        <v>3</v>
+      </c>
+      <c r="M71" s="57" t="n">
+        <v>1</v>
+      </c>
+      <c r="N71" s="57" t="n"/>
+      <c r="O71" s="57" t="n"/>
+      <c r="P71" s="57" t="n"/>
+      <c r="Q71" s="57" t="n">
+        <v>1</v>
+      </c>
+      <c r="R71" s="57" t="n"/>
+      <c r="S71" s="57" t="n">
+        <v>6</v>
+      </c>
+      <c r="T71" s="57" t="n"/>
+      <c r="U71" s="57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V71" s="57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W71" s="57" t="n"/>
+      <c r="X71" s="57" t="n"/>
+      <c r="Y71" s="57" t="n"/>
+      <c r="Z71" s="57" t="n"/>
+      <c r="AA71" s="57" t="n"/>
+      <c r="AB71" s="57" t="n"/>
+      <c r="AC71" s="57" t="n"/>
+      <c r="AD71" s="57" t="n"/>
+      <c r="AE71" s="57" t="n"/>
+      <c r="AF71" s="57" t="n"/>
+      <c r="AG71" s="57" t="n"/>
+      <c r="AH71" s="57" t="n"/>
+      <c r="AI71" s="57" t="n"/>
+      <c r="AS71" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="43" t="inlineStr">
+        <is>
+          <t>Brush Beater</t>
+        </is>
+      </c>
+      <c r="B72" s="43" t="inlineStr">
+        <is>
+          <t>Buckshot</t>
+        </is>
+      </c>
+      <c r="C72" s="43" t="inlineStr">
+        <is>
+          <t>crowds</t>
+        </is>
+      </c>
+      <c r="D72" s="43" t="n">
+        <v>6</v>
+      </c>
+      <c r="E72" s="43" t="inlineStr">
+        <is>
+          <t>Wildfire Drum</t>
+        </is>
+      </c>
+      <c r="F72" s="56">
+        <f>ROUND(Tuning!$B$21*POWER(Tuning!$B$22,D72-1),0)</f>
+        <v/>
+      </c>
+      <c r="G72" s="57" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="H72" s="57" t="n">
+        <v>3</v>
+      </c>
+      <c r="I72" s="57" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J72" s="57" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="K72" s="57" t="n"/>
+      <c r="L72" s="57" t="n"/>
+      <c r="M72" s="57" t="n"/>
+      <c r="N72" s="57" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="O72" s="57" t="n"/>
+      <c r="P72" s="57" t="n"/>
+      <c r="Q72" s="57" t="n">
+        <v>9</v>
+      </c>
+      <c r="R72" s="57" t="n"/>
+      <c r="S72" s="57" t="n"/>
+      <c r="T72" s="57" t="n"/>
+      <c r="U72" s="57" t="n"/>
+      <c r="V72" s="57" t="n"/>
+      <c r="W72" s="57" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="X72" s="57" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y72" s="57" t="n"/>
+      <c r="Z72" s="57" t="n"/>
+      <c r="AA72" s="57" t="n"/>
+      <c r="AB72" s="57" t="n"/>
+      <c r="AC72" s="57" t="n"/>
+      <c r="AD72" s="57" t="n"/>
+      <c r="AE72" s="57" t="n"/>
+      <c r="AF72" s="57" t="n"/>
+      <c r="AG72" s="57" t="n"/>
+      <c r="AH72" s="57" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AI72" s="57" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="AT72" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="43" t="inlineStr">
+        <is>
+          <t>Brush Beater</t>
+        </is>
+      </c>
+      <c r="B73" s="43" t="inlineStr">
+        <is>
+          <t>Point Blank</t>
+        </is>
+      </c>
+      <c r="C73" s="43" t="inlineStr">
+        <is>
+          <t>burst</t>
+        </is>
+      </c>
+      <c r="D73" s="43" t="n">
+        <v>6</v>
+      </c>
+      <c r="E73" s="43" t="inlineStr">
+        <is>
+          <t>Quad Barrel</t>
+        </is>
+      </c>
+      <c r="F73" s="56">
+        <f>ROUND(Tuning!$B$21*POWER(Tuning!$B$22,D73-1),0)</f>
+        <v/>
+      </c>
+      <c r="G73" s="57" t="n"/>
+      <c r="H73" s="57" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I73" s="57" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J73" s="57" t="n"/>
+      <c r="K73" s="57" t="n"/>
+      <c r="L73" s="57" t="n"/>
+      <c r="M73" s="57" t="n"/>
+      <c r="N73" s="57" t="n"/>
+      <c r="O73" s="57" t="n"/>
+      <c r="P73" s="57" t="n"/>
+      <c r="Q73" s="57" t="n"/>
+      <c r="R73" s="57" t="n">
+        <v>4</v>
+      </c>
+      <c r="S73" s="57" t="n"/>
+      <c r="T73" s="57" t="n"/>
+      <c r="U73" s="57" t="n"/>
+      <c r="V73" s="57" t="n"/>
+      <c r="W73" s="57" t="n"/>
+      <c r="X73" s="57" t="n"/>
+      <c r="Y73" s="57" t="n">
+        <v>5</v>
+      </c>
+      <c r="Z73" s="57" t="n">
+        <v>4</v>
+      </c>
+      <c r="AA73" s="57" t="n"/>
+      <c r="AB73" s="57" t="n"/>
+      <c r="AC73" s="57" t="n"/>
+      <c r="AD73" s="57" t="n"/>
+      <c r="AE73" s="57" t="n"/>
+      <c r="AF73" s="57" t="n"/>
+      <c r="AG73" s="57" t="n"/>
+      <c r="AH73" s="57" t="n"/>
+      <c r="AI73" s="57" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="43" t="inlineStr">
+        <is>
+          <t>Field Medic</t>
+        </is>
+      </c>
+      <c r="B74" s="43" t="inlineStr">
+        <is>
+          <t>Triage</t>
+        </is>
+      </c>
+      <c r="C74" s="43" t="inlineStr">
+        <is>
+          <t>ability</t>
+        </is>
+      </c>
+      <c r="D74" s="43" t="n">
+        <v>6</v>
+      </c>
+      <c r="E74" s="43" t="inlineStr">
+        <is>
+          <t>Rapid Response</t>
+        </is>
+      </c>
+      <c r="F74" s="56">
+        <f>ROUND(Tuning!$B$21*POWER(Tuning!$B$22,D74-1),0)</f>
+        <v/>
+      </c>
+      <c r="G74" s="57" t="n"/>
+      <c r="H74" s="57" t="n"/>
+      <c r="I74" s="57" t="n"/>
+      <c r="J74" s="57" t="n"/>
+      <c r="K74" s="57" t="n"/>
+      <c r="L74" s="57" t="n"/>
+      <c r="M74" s="57" t="n"/>
+      <c r="N74" s="57" t="n"/>
+      <c r="O74" s="57" t="n"/>
+      <c r="P74" s="57" t="n"/>
+      <c r="Q74" s="57" t="n"/>
+      <c r="R74" s="57" t="n"/>
+      <c r="S74" s="57" t="n"/>
+      <c r="T74" s="57" t="n"/>
+      <c r="U74" s="57" t="n"/>
+      <c r="V74" s="57" t="n"/>
+      <c r="W74" s="57" t="n"/>
+      <c r="X74" s="57" t="n"/>
+      <c r="Y74" s="57" t="n"/>
+      <c r="Z74" s="57" t="n"/>
+      <c r="AA74" s="57" t="n"/>
+      <c r="AB74" s="57" t="n"/>
+      <c r="AC74" s="57" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AD74" s="57" t="n"/>
+      <c r="AE74" s="57" t="n"/>
+      <c r="AF74" s="57" t="n"/>
+      <c r="AG74" s="57" t="n"/>
+      <c r="AH74" s="57" t="n"/>
+      <c r="AI74" s="57" t="n"/>
+      <c r="AJ74" s="81" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="AK74" s="81" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AL74" s="81" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AM74" s="81" t="n">
+        <v>30</v>
+      </c>
+      <c r="AN74" s="81" t="n">
+        <v>8</v>
+      </c>
+      <c r="BA74" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="43" t="inlineStr">
+        <is>
+          <t>Field Medic</t>
+        </is>
+      </c>
+      <c r="B75" s="43" t="inlineStr">
+        <is>
+          <t>Lever Action</t>
+        </is>
+      </c>
+      <c r="C75" s="43" t="inlineStr">
+        <is>
+          <t>handling</t>
+        </is>
+      </c>
+      <c r="D75" s="43" t="n">
+        <v>6</v>
+      </c>
+      <c r="E75" s="43" t="inlineStr">
+        <is>
+          <t>Tube Feed</t>
+        </is>
+      </c>
+      <c r="F75" s="56">
+        <f>ROUND(Tuning!$B$21*POWER(Tuning!$B$22,D75-1),0)</f>
+        <v/>
+      </c>
+      <c r="G75" s="57" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="H75" s="57" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="I75" s="57" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="J75" s="57" t="n"/>
+      <c r="K75" s="57" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L75" s="57" t="n"/>
+      <c r="M75" s="57" t="n"/>
+      <c r="N75" s="57" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="O75" s="57" t="n"/>
+      <c r="P75" s="57" t="n"/>
+      <c r="Q75" s="57" t="n"/>
+      <c r="R75" s="57" t="n"/>
+      <c r="S75" s="57" t="n"/>
+      <c r="T75" s="57" t="n"/>
+      <c r="U75" s="57" t="n"/>
+      <c r="V75" s="57" t="n"/>
+      <c r="W75" s="57" t="n"/>
+      <c r="X75" s="57" t="n"/>
+      <c r="Y75" s="57" t="n"/>
+      <c r="Z75" s="57" t="n"/>
+      <c r="AA75" s="57" t="n"/>
+      <c r="AB75" s="57" t="n"/>
+      <c r="AC75" s="57" t="n"/>
+      <c r="AD75" s="57" t="n"/>
+      <c r="AE75" s="57" t="n"/>
+      <c r="AF75" s="57" t="n"/>
+      <c r="AG75" s="57" t="n"/>
+      <c r="AH75" s="57" t="n"/>
+      <c r="AI75" s="57" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="43" t="inlineStr">
+        <is>
+          <t>Field Medic</t>
+        </is>
+      </c>
+      <c r="B76" s="43" t="inlineStr">
+        <is>
+          <t>Muzzle</t>
+        </is>
+      </c>
+      <c r="C76" s="43" t="inlineStr">
+        <is>
+          <t>protective rounds</t>
+        </is>
+      </c>
+      <c r="D76" s="43" t="n">
+        <v>6</v>
+      </c>
+      <c r="E76" s="43" t="inlineStr">
+        <is>
+          <t>Nightcap</t>
+        </is>
+      </c>
+      <c r="F76" s="56">
+        <f>ROUND(Tuning!$B$21*POWER(Tuning!$B$22,D76-1),0)</f>
+        <v/>
+      </c>
+      <c r="G76" s="57" t="n"/>
+      <c r="H76" s="57" t="n"/>
+      <c r="I76" s="57" t="n"/>
+      <c r="J76" s="57" t="n"/>
+      <c r="K76" s="57" t="n"/>
+      <c r="L76" s="57" t="n"/>
+      <c r="M76" s="57" t="n"/>
+      <c r="N76" s="57" t="n"/>
+      <c r="O76" s="57" t="n"/>
+      <c r="P76" s="57" t="n"/>
+      <c r="Q76" s="57" t="n"/>
+      <c r="R76" s="57" t="n"/>
+      <c r="S76" s="57" t="n"/>
+      <c r="T76" s="57" t="n"/>
+      <c r="U76" s="57" t="n"/>
+      <c r="V76" s="57" t="n"/>
+      <c r="W76" s="57" t="n"/>
+      <c r="X76" s="57" t="n"/>
+      <c r="Y76" s="57" t="n"/>
+      <c r="Z76" s="57" t="n"/>
+      <c r="AA76" s="57" t="n"/>
+      <c r="AB76" s="57" t="n"/>
+      <c r="AC76" s="57" t="n"/>
+      <c r="AD76" s="57" t="n"/>
+      <c r="AE76" s="57" t="n"/>
+      <c r="AF76" s="57" t="n"/>
+      <c r="AG76" s="57" t="n"/>
+      <c r="AH76" s="57" t="n"/>
+      <c r="AI76" s="57" t="n"/>
+      <c r="AO76" s="81" t="n">
+        <v>30</v>
+      </c>
+      <c r="AP76" s="81" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AQ76" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AR76" s="81" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
T53b: Heart Shot breaks 2 only scoped; Dino round 13 names (#170, #174-#176)
Heart Shot: new pure GunRules.sizeBreaks(stats, scoped) - on a scoped gun
only a scoped shot gets the gun's Size breaks, unscoped shots break 1;
Server/Hero passes the trigger's scoped flag into the direct-hit path.
Thunder Slug (no scope) still breaks 2 on every slug.

Names (sheet, re-exported; Config diff = these 11 strings only): Trick
Reload -> Bounce Back, Five-Round Burst -> Big Five, Powder Tips ->
Dynamite Rounds, Tube Feed -> Bottomless Tube, Nightcap -> Lights Out;
Mastery Field Dressing I-III -> First Aid, Quick Recovery I-III -> Back in
Action. Same renames in comments, spec titles and HEROES.md; HEROES "per
pop" -> "per take-down" and player-facing "break 2 sizes" -> "shrink a
dino 2 sizes". PLAN's tier-6 table left for the Director.

Spec: Heart Shot scoped vs a 3-size Pachy drops 2, unscoped 1; Thunder
Slug 2 either way. Not playtested.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Storm-Split-Balance.xlsx
+++ b/Storm-Split-Balance.xlsx
@@ -2267,7 +2267,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="21" t="inlineStr">
         <is>
@@ -2528,8 +2527,6 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="9"/>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
@@ -7409,7 +7406,6 @@
         </is>
       </c>
     </row>
-    <row r="103"/>
     <row r="104">
       <c r="A104" s="99" t="inlineStr">
         <is>
@@ -23601,7 +23597,7 @@
       </c>
       <c r="E67" s="43" t="inlineStr">
         <is>
-          <t>Trick Reload</t>
+          <t>Bounce Back</t>
         </is>
       </c>
       <c r="F67" s="56">
@@ -23670,7 +23666,7 @@
       </c>
       <c r="E68" s="43" t="inlineStr">
         <is>
-          <t>Five-Round Burst</t>
+          <t>Big Five</t>
         </is>
       </c>
       <c r="F68" s="56">
@@ -23824,7 +23820,7 @@
       </c>
       <c r="E70" s="43" t="inlineStr">
         <is>
-          <t>Powder Tips</t>
+          <t>Dynamite Rounds</t>
         </is>
       </c>
       <c r="F70" s="56">
@@ -24211,7 +24207,7 @@
       </c>
       <c r="E75" s="43" t="inlineStr">
         <is>
-          <t>Tube Feed</t>
+          <t>Bottomless Tube</t>
         </is>
       </c>
       <c r="F75" s="56">
@@ -24281,7 +24277,7 @@
       </c>
       <c r="E76" s="43" t="inlineStr">
         <is>
-          <t>Nightcap</t>
+          <t>Lights Out</t>
         </is>
       </c>
       <c r="F76" s="56">
@@ -24728,7 +24724,7 @@
       </c>
       <c r="E11" s="69" t="inlineStr">
         <is>
-          <t>Field Dressing I: heal 5 more HP when a round is cleared</t>
+          <t>First Aid I: heal 5 more HP when a round is cleared</t>
         </is>
       </c>
       <c r="F11" s="56" t="n">
@@ -24776,7 +24772,7 @@
       </c>
       <c r="E12" s="69" t="inlineStr">
         <is>
-          <t>Quick Recovery I: respawn 10% sooner</t>
+          <t>Back in Action I: respawn 10% sooner</t>
         </is>
       </c>
       <c r="F12" s="56" t="n">
@@ -24968,7 +24964,7 @@
       </c>
       <c r="E16" s="69" t="inlineStr">
         <is>
-          <t>Field Dressing II: heal 10 more HP when a round is cleared</t>
+          <t>First Aid II: heal 10 more HP when a round is cleared</t>
         </is>
       </c>
       <c r="F16" s="56" t="n">
@@ -25016,7 +25012,7 @@
       </c>
       <c r="E17" s="69" t="inlineStr">
         <is>
-          <t>Quick Recovery II: respawn 20% sooner</t>
+          <t>Back in Action II: respawn 20% sooner</t>
         </is>
       </c>
       <c r="F17" s="56" t="n">
@@ -25208,7 +25204,7 @@
       </c>
       <c r="E21" s="69" t="inlineStr">
         <is>
-          <t>Field Dressing III: heal 15 more HP when a round is cleared</t>
+          <t>First Aid III: heal 15 more HP when a round is cleared</t>
         </is>
       </c>
       <c r="F21" s="56" t="n">
@@ -25256,7 +25252,7 @@
       </c>
       <c r="E22" s="69" t="inlineStr">
         <is>
-          <t>Quick Recovery III: respawn 30% sooner</t>
+          <t>Back in Action III: respawn 30% sooner</t>
         </is>
       </c>
       <c r="F22" s="56" t="n">

</xml_diff>

<commit_message>
T58b: Lobby-only equip, budgeted leaderboard writes, round-14 names (#181-#187)
- Equip is Lobby-only on the server (Cosmetics.request); players see only
  "You can't equip that." / "Equip in the lobby."; internal reasons are logged.
- LevelBoard: unchanged XP is never written; a request-budget check
  (SetIncrementSortedAsync) before each write, 0 = skip and retry next tick.
- Cosmetics D25/D36/D58/D69/D79/D90/D113/D114 renamed; Config diff = the 8 names.
- Specs: lobby/playing equip, toast text, write-on-change, zero budget, trails
  add no parts (runner gains ColorSequence/NumberSequence). Hats were already
  inert and spec'd. Statically checked, not playtested.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Storm-Split-Balance.xlsx
+++ b/Storm-Split-Balance.xlsx
@@ -6501,7 +6501,7 @@
       </c>
       <c r="D25" s="81" t="inlineStr">
         <is>
-          <t>Trailblazer</t>
+          <t>Trapper</t>
         </is>
       </c>
       <c r="E25" s="81" t="inlineStr">
@@ -6831,7 +6831,7 @@
       </c>
       <c r="D36" s="81" t="inlineStr">
         <is>
-          <t>Trapper</t>
+          <t>Trailblazer</t>
         </is>
       </c>
       <c r="E36" s="81" t="inlineStr">
@@ -7491,7 +7491,7 @@
       </c>
       <c r="D58" s="81" t="inlineStr">
         <is>
-          <t>Trophy Hunter</t>
+          <t>Veteran Hunter</t>
         </is>
       </c>
       <c r="E58" s="81" t="inlineStr">
@@ -7821,7 +7821,7 @@
       </c>
       <c r="D69" s="81" t="inlineStr">
         <is>
-          <t>Warden</t>
+          <t>Game Warden</t>
         </is>
       </c>
       <c r="E69" s="81" t="inlineStr">
@@ -8116,7 +8116,7 @@
       </c>
       <c r="D79" s="81" t="inlineStr">
         <is>
-          <t>Star Marker</t>
+          <t>Claw Marker</t>
         </is>
       </c>
       <c r="E79" s="81" t="inlineStr">
@@ -8446,7 +8446,7 @@
       </c>
       <c r="D90" s="81" t="inlineStr">
         <is>
-          <t>Fern Trail</t>
+          <t>Footprint Trail</t>
         </is>
       </c>
       <c r="E90" s="81" t="inlineStr">
@@ -9141,7 +9141,7 @@
       </c>
       <c r="D113" s="81" t="inlineStr">
         <is>
-          <t>Apex Hunter</t>
+          <t>Master Hunter</t>
         </is>
       </c>
       <c r="E113" s="81" t="inlineStr">
@@ -9166,7 +9166,7 @@
       </c>
       <c r="D114" s="81" t="inlineStr">
         <is>
-          <t>Tar Pit Set</t>
+          <t>Volcano Set</t>
         </is>
       </c>
       <c r="E114" s="81" t="inlineStr">
@@ -22671,7 +22671,7 @@
           <t>Copper Wire</t>
         </is>
       </c>
-      <c r="BK110" t="n">
+      <c r="BK110" s="81" t="n">
         <v>6</v>
       </c>
     </row>
@@ -22727,10 +22727,10 @@
           <t>Long Arc</t>
         </is>
       </c>
-      <c r="BK111" t="n">
+      <c r="BK111" s="81" t="n">
         <v>6</v>
       </c>
-      <c r="BL111" t="n">
+      <c r="BL111" s="81" t="n">
         <v>15</v>
       </c>
     </row>
@@ -22786,13 +22786,13 @@
           <t>Fork Lightning</t>
         </is>
       </c>
-      <c r="BK112" t="n">
+      <c r="BK112" s="81" t="n">
         <v>6</v>
       </c>
-      <c r="BL112" t="n">
+      <c r="BL112" s="81" t="n">
         <v>15</v>
       </c>
-      <c r="BM112" t="n">
+      <c r="BM112" s="81" t="n">
         <v>2</v>
       </c>
     </row>
@@ -22848,13 +22848,13 @@
           <t>Jump Spark</t>
         </is>
       </c>
-      <c r="BK113" t="n">
+      <c r="BK113" s="81" t="n">
         <v>6</v>
       </c>
-      <c r="BL113" t="n">
+      <c r="BL113" s="81" t="n">
         <v>15</v>
       </c>
-      <c r="BM113" t="n">
+      <c r="BM113" s="81" t="n">
         <v>2</v>
       </c>
       <c r="BN113" s="46" t="inlineStr">
@@ -22915,13 +22915,13 @@
           <t>Power Grid</t>
         </is>
       </c>
-      <c r="BK114" t="n">
+      <c r="BK114" s="81" t="n">
         <v>6</v>
       </c>
-      <c r="BL114" t="n">
+      <c r="BL114" s="81" t="n">
         <v>15</v>
       </c>
-      <c r="BM114" t="n">
+      <c r="BM114" s="81" t="n">
         <v>2</v>
       </c>
       <c r="BN114" s="46" t="inlineStr">
@@ -23040,7 +23040,7 @@
           <t>Static Shock</t>
         </is>
       </c>
-      <c r="BP116" t="n">
+      <c r="BP116" s="81" t="n">
         <v>10</v>
       </c>
     </row>
@@ -23099,7 +23099,7 @@
       <c r="U117" s="57" t="n">
         <v>0.4</v>
       </c>
-      <c r="BP117" t="n">
+      <c r="BP117" s="81" t="n">
         <v>10</v>
       </c>
     </row>
@@ -23163,7 +23163,7 @@
       <c r="U118" s="57" t="n">
         <v>0.4</v>
       </c>
-      <c r="BP118" t="n">
+      <c r="BP118" s="81" t="n">
         <v>10</v>
       </c>
     </row>
@@ -23227,7 +23227,7 @@
       <c r="U119" s="57" t="n">
         <v>0.4</v>
       </c>
-      <c r="BP119" t="n">
+      <c r="BP119" s="81" t="n">
         <v>10</v>
       </c>
       <c r="BQ119" s="46" t="inlineStr">
@@ -23400,7 +23400,7 @@
       <c r="AB122" s="57" t="n">
         <v>10</v>
       </c>
-      <c r="BR122" t="n">
+      <c r="BR122" s="81" t="n">
         <v>4</v>
       </c>
     </row>
@@ -23462,7 +23462,7 @@
       <c r="AC123" s="57" t="n">
         <v>15</v>
       </c>
-      <c r="BR123" t="n">
+      <c r="BR123" s="81" t="n">
         <v>4</v>
       </c>
     </row>
@@ -23524,10 +23524,10 @@
       <c r="AC124" s="57" t="n">
         <v>15</v>
       </c>
-      <c r="BR124" t="n">
+      <c r="BR124" s="81" t="n">
         <v>4</v>
       </c>
-      <c r="BS124" t="n">
+      <c r="BS124" s="81" t="n">
         <v>50</v>
       </c>
     </row>

</xml_diff>

<commit_message>
T84b: parity buffs on Mastery Perks (Director's cells, #235)
Old values asserted before writing: F7 5->6, E8 3->3.5, F9 1.5->2.5,
F11 4->5, G12 10->14, plus their D texts as PLAN gives them. Exporter:
worth % M10 25/24/25/25 -> parity 1.04; summed 65/59/61/60 -> 1.10;
each L15 > L10, all <= 40. Config diff = these 5 values + 5 texts.
HEROES.md Mastery table and heroes.spec expectations follow the sheet.

Statically checked and headless-tested, not playtested.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Storm-Split-Balance.xlsx
+++ b/Storm-Split-Balance.xlsx
@@ -5665,11 +5665,11 @@
       </c>
       <c r="D7" s="43" t="inlineStr">
         <is>
-          <t>Rally Cry reaches 5 studs further</t>
+          <t>Rally Cry reaches 6 studs further</t>
         </is>
       </c>
       <c r="F7" s="27" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
@@ -5688,11 +5688,11 @@
       </c>
       <c r="D8" s="43" t="inlineStr">
         <is>
-          <t>Rally Cry lasts 3s longer</t>
+          <t>Rally Cry lasts 3.5s longer</t>
         </is>
       </c>
       <c r="E8" s="27" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="9">
@@ -5711,11 +5711,11 @@
       </c>
       <c r="D9" s="43" t="inlineStr">
         <is>
-          <t>Flare Strike reaches 1.5 studs further</t>
+          <t>Flare Strike reaches 2.5 studs further</t>
         </is>
       </c>
       <c r="F9" s="27" t="n">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="10">
@@ -5760,11 +5760,11 @@
       </c>
       <c r="D11" s="43" t="inlineStr">
         <is>
-          <t>Triage Kit reaches 4 studs further</t>
+          <t>Triage Kit reaches 5 studs further</t>
         </is>
       </c>
       <c r="F11" s="27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12">
@@ -5783,11 +5783,11 @@
       </c>
       <c r="D12" s="43" t="inlineStr">
         <is>
-          <t>Triage Kit heals 10 more HP</t>
+          <t>Triage Kit heals 14 more HP</t>
         </is>
       </c>
       <c r="G12" s="27" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Option-A Blurbs: one card line for every tier-4/5 option A
All 90 option-A Blurb cells (66 tower, 24 hero; hero tier 6 takes no
Blurb) were blank; each now holds a short kid-readable line of what that
step does, taken from the UPGRADES.md / HEROES.md effect text, or for the
plain stat steps from the row's own step columns, worded without numbers
the docs don't give ("shrinks a dino N sizes" for size breaks). Each cell
was asserted blank first; all <= 60 chars; no banned or old-theme words.
For the Dino agent's review.

Config diff: exactly 90 lines, blurb "" -> the new line; nothing else.
check clean, 706 specs, audit --strict 0, threat 0, value --breaks1 0.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Storm-Split-Balance.xlsx
+++ b/Storm-Split-Balance.xlsx
@@ -13262,7 +13262,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CJ170"/>
+  <dimension ref="A1:CJ169"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66667" defaultRowHeight="15" customHeight="1" outlineLevelRow="0"/>
   <cols>
     <col width="15" customWidth="1" style="81" min="1" max="1"/>
@@ -13832,12 +13832,12 @@
           <t>Aura vs slowed %</t>
         </is>
       </c>
-      <c r="CI4" t="inlineStr">
+      <c r="CI4" s="81" t="inlineStr">
         <is>
           <t>Option</t>
         </is>
       </c>
-      <c r="CJ4" t="inlineStr">
+      <c r="CJ4" s="81" t="inlineStr">
         <is>
           <t>Blurb</t>
         </is>
@@ -14188,9 +14188,14 @@
       <c r="AR8" s="57" t="n"/>
       <c r="AS8" s="57" t="n"/>
       <c r="AT8" s="57" t="n"/>
-      <c r="CI8" t="inlineStr">
+      <c r="CI8" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ8" t="inlineStr">
+        <is>
+          <t>Sees further, and shoots faster and harder</t>
         </is>
       </c>
     </row>
@@ -14285,9 +14290,14 @@
       <c r="AR9" s="57" t="n"/>
       <c r="AS9" s="57" t="n"/>
       <c r="AT9" s="57" t="n"/>
-      <c r="CI9" t="inlineStr">
+      <c r="CI9" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ9" t="inlineStr">
+        <is>
+          <t>Towers in range hit harder and can hurt armour</t>
         </is>
       </c>
     </row>
@@ -14636,9 +14646,14 @@
       <c r="AR13" s="57" t="n"/>
       <c r="AS13" s="57" t="n"/>
       <c r="AT13" s="57" t="n"/>
-      <c r="CI13" t="inlineStr">
+      <c r="CI13" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ13" t="inlineStr">
+        <is>
+          <t>Fires much faster and hits harder</t>
         </is>
       </c>
     </row>
@@ -14729,9 +14744,14 @@
       <c r="AR14" s="57" t="n"/>
       <c r="AS14" s="57" t="n"/>
       <c r="AT14" s="57" t="n"/>
-      <c r="CI14" t="inlineStr">
+      <c r="CI14" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ14" t="inlineStr">
+        <is>
+          <t>The fastest fire in the game</t>
         </is>
       </c>
     </row>
@@ -15095,9 +15115,14 @@
       <c r="BJ18" s="105" t="n">
         <v>2</v>
       </c>
-      <c r="CI18" t="inlineStr">
+      <c r="CI18" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ18" t="inlineStr">
+        <is>
+          <t>Each bullet goes through 3 dinos</t>
         </is>
       </c>
     </row>
@@ -15191,9 +15216,14 @@
       <c r="AS19" s="57" t="n"/>
       <c r="AT19" s="57" t="n"/>
       <c r="BJ19" s="105" t="n"/>
-      <c r="CI19" t="inlineStr">
+      <c r="CI19" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ19" t="inlineStr">
+        <is>
+          <t>Hits armoured dinos and bosses 4 times as hard</t>
         </is>
       </c>
     </row>
@@ -15559,9 +15589,14 @@
       <c r="BJ23" s="105" t="n">
         <v>2</v>
       </c>
-      <c r="CI23" t="inlineStr">
+      <c r="CI23" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ23" t="inlineStr">
+        <is>
+          <t>Shots go through more dinos, shrinking each 2 sizes</t>
         </is>
       </c>
     </row>
@@ -15655,9 +15690,14 @@
       <c r="BJ24" s="105" t="n">
         <v>3</v>
       </c>
-      <c r="CI24" t="inlineStr">
+      <c r="CI24" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ24" t="inlineStr">
+        <is>
+          <t>Each shot hits 10 dinos in a line, double damage</t>
         </is>
       </c>
     </row>
@@ -16008,9 +16048,14 @@
       <c r="AR28" s="57" t="n"/>
       <c r="AS28" s="57" t="n"/>
       <c r="AT28" s="57" t="n"/>
-      <c r="CI28" t="inlineStr">
+      <c r="CI28" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ28" t="inlineStr">
+        <is>
+          <t>Fires faster, and its mark hits harder</t>
         </is>
       </c>
     </row>
@@ -16103,9 +16148,14 @@
       <c r="AR29" s="57" t="n"/>
       <c r="AS29" s="57" t="n"/>
       <c r="AT29" s="57" t="n"/>
-      <c r="CI29" t="inlineStr">
+      <c r="CI29" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ29" t="inlineStr">
+        <is>
+          <t>A bigger mark, and towers in range shoot faster</t>
         </is>
       </c>
     </row>
@@ -16471,9 +16521,14 @@
       <c r="BJ33" s="105" t="n">
         <v>3</v>
       </c>
-      <c r="CI33" t="inlineStr">
+      <c r="CI33" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ33" t="inlineStr">
+        <is>
+          <t>Huge shots that stun and shrink a dino 3 sizes</t>
         </is>
       </c>
     </row>
@@ -16573,9 +16628,14 @@
       <c r="BJ34" s="105" t="n">
         <v>4</v>
       </c>
-      <c r="CI34" t="inlineStr">
+      <c r="CI34" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ34" t="inlineStr">
+        <is>
+          <t>10 times damage to bosses, and stuns them</t>
         </is>
       </c>
     </row>
@@ -16938,9 +16998,14 @@
       <c r="AR38" s="57" t="n"/>
       <c r="AS38" s="57" t="n"/>
       <c r="AT38" s="57" t="n"/>
-      <c r="CI38" t="inlineStr">
+      <c r="CI38" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ38" t="inlineStr">
+        <is>
+          <t>Bigger blasts that leave dinos burning</t>
         </is>
       </c>
     </row>
@@ -17035,9 +17100,14 @@
       <c r="AR39" s="57" t="n"/>
       <c r="AS39" s="57" t="n"/>
       <c r="AT39" s="57" t="n"/>
-      <c r="CI39" t="inlineStr">
+      <c r="CI39" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ39" t="inlineStr">
+        <is>
+          <t>Leaves a long burning stretch of track</t>
         </is>
       </c>
     </row>
@@ -17398,9 +17468,14 @@
       <c r="AR43" s="57" t="n"/>
       <c r="AS43" s="57" t="n"/>
       <c r="AT43" s="57" t="n"/>
-      <c r="CI43" t="inlineStr">
+      <c r="CI43" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ43" t="inlineStr">
+        <is>
+          <t>More bomblets and harder blasts</t>
         </is>
       </c>
     </row>
@@ -17491,9 +17566,14 @@
       <c r="AR44" s="57" t="n"/>
       <c r="AS44" s="57" t="n"/>
       <c r="AT44" s="57" t="n"/>
-      <c r="CI44" t="inlineStr">
+      <c r="CI44" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ44" t="inlineStr">
+        <is>
+          <t>Even more bomblets rain down</t>
         </is>
       </c>
     </row>
@@ -17864,9 +17944,14 @@
       <c r="AR48" s="57" t="n"/>
       <c r="AS48" s="57" t="n"/>
       <c r="AT48" s="57" t="n"/>
-      <c r="CI48" t="inlineStr">
+      <c r="CI48" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ48" t="inlineStr">
+        <is>
+          <t>Hits much harder and knocks dinos further back</t>
         </is>
       </c>
     </row>
@@ -17959,9 +18044,14 @@
       <c r="AR49" s="57" t="n"/>
       <c r="AS49" s="57" t="n"/>
       <c r="AT49" s="57" t="n"/>
-      <c r="CI49" t="inlineStr">
+      <c r="CI49" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ49" t="inlineStr">
+        <is>
+          <t>Stuns every dino it hits for a second</t>
         </is>
       </c>
     </row>
@@ -18318,9 +18408,14 @@
       <c r="AR53" s="57" t="n"/>
       <c r="AS53" s="57" t="n"/>
       <c r="AT53" s="57" t="n"/>
-      <c r="CI53" t="inlineStr">
+      <c r="CI53" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ53" t="inlineStr">
+        <is>
+          <t>A much stronger slow over a wider area</t>
         </is>
       </c>
     </row>
@@ -18417,9 +18512,14 @@
       <c r="AR54" s="57" t="n"/>
       <c r="AS54" s="57" t="n"/>
       <c r="AT54" s="57" t="n"/>
-      <c r="CI54" t="inlineStr">
+      <c r="CI54" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ54" t="inlineStr">
+        <is>
+          <t>Its slow works on bosses too</t>
         </is>
       </c>
     </row>
@@ -18784,9 +18884,14 @@
       <c r="AR58" s="57" t="n"/>
       <c r="AS58" s="57" t="n"/>
       <c r="AT58" s="57" t="n"/>
-      <c r="CI58" t="inlineStr">
+      <c r="CI58" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ58" t="inlineStr">
+        <is>
+          <t>Knockouts come sooner and hurt more</t>
         </is>
       </c>
     </row>
@@ -18883,9 +18988,14 @@
       <c r="AR59" s="57" t="n"/>
       <c r="AS59" s="57" t="n"/>
       <c r="AT59" s="57" t="n"/>
-      <c r="CI59" t="inlineStr">
+      <c r="CI59" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ59" t="inlineStr">
+        <is>
+          <t>A long knockout that even holds bosses</t>
         </is>
       </c>
     </row>
@@ -19250,9 +19360,14 @@
       <c r="AR63" s="57" t="n"/>
       <c r="AS63" s="57" t="n"/>
       <c r="AT63" s="57" t="n"/>
-      <c r="CI63" t="inlineStr">
+      <c r="CI63" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ63" t="inlineStr">
+        <is>
+          <t>Sedated dinos take even more damage</t>
         </is>
       </c>
     </row>
@@ -19345,9 +19460,14 @@
       <c r="AR64" s="57" t="n"/>
       <c r="AS64" s="57" t="n"/>
       <c r="AT64" s="57" t="n"/>
-      <c r="CI64" t="inlineStr">
+      <c r="CI64" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ64" t="inlineStr">
+        <is>
+          <t>Dinos take much more damage; towers in range hit harder</t>
         </is>
       </c>
     </row>
@@ -19702,9 +19822,14 @@
       <c r="AR68" s="57" t="n"/>
       <c r="AS68" s="57" t="n"/>
       <c r="AT68" s="57" t="n"/>
-      <c r="CI68" t="inlineStr">
+      <c r="CI68" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ68" t="inlineStr">
+        <is>
+          <t>Pays a lot more cash every round</t>
         </is>
       </c>
     </row>
@@ -19799,9 +19924,14 @@
       <c r="AR69" s="57" t="n"/>
       <c r="AS69" s="57" t="n"/>
       <c r="AT69" s="57" t="n"/>
-      <c r="CI69" t="inlineStr">
+      <c r="CI69" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ69" t="inlineStr">
+        <is>
+          <t>Earns interest on your banked cash</t>
         </is>
       </c>
     </row>
@@ -20164,9 +20294,14 @@
       </c>
       <c r="AS73" s="57" t="n"/>
       <c r="AT73" s="57" t="n"/>
-      <c r="CI73" t="inlineStr">
+      <c r="CI73" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ73" t="inlineStr">
+        <is>
+          <t>More chests land each round, worth more</t>
         </is>
       </c>
     </row>
@@ -20259,9 +20394,14 @@
       </c>
       <c r="AS74" s="57" t="n"/>
       <c r="AT74" s="57" t="n"/>
-      <c r="CI74" t="inlineStr">
+      <c r="CI74" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ74" t="inlineStr">
+        <is>
+          <t>The richest chests, and more of them</t>
         </is>
       </c>
     </row>
@@ -20618,9 +20758,14 @@
       <c r="AR78" s="57" t="n"/>
       <c r="AS78" s="57" t="n"/>
       <c r="AT78" s="57" t="n"/>
-      <c r="CI78" t="inlineStr">
+      <c r="CI78" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ78" t="inlineStr">
+        <is>
+          <t>Towers in range shoot faster</t>
         </is>
       </c>
     </row>
@@ -20713,9 +20858,14 @@
       <c r="AT79" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="CI79" t="inlineStr">
+      <c r="CI79" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ79" t="inlineStr">
+        <is>
+          <t>Towers in range cost less and sell for full price</t>
         </is>
       </c>
     </row>
@@ -21102,9 +21252,14 @@
       <c r="AY83" s="57" t="n"/>
       <c r="AZ83" s="57" t="n"/>
       <c r="BA83" s="57" t="n"/>
-      <c r="CI83" t="inlineStr">
+      <c r="CI83" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ83" t="inlineStr">
+        <is>
+          <t>Tougher armour, and biters take more damage back</t>
         </is>
       </c>
     </row>
@@ -21204,9 +21359,14 @@
       <c r="AY84" s="57" t="n"/>
       <c r="AZ84" s="57" t="n"/>
       <c r="BA84" s="57" t="n"/>
-      <c r="CI84" t="inlineStr">
+      <c r="CI84" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ84" t="inlineStr">
+        <is>
+          <t>The best armour; biting dinos get stunned (not bosses)</t>
         </is>
       </c>
     </row>
@@ -21599,9 +21759,14 @@
       <c r="AY88" s="57" t="n"/>
       <c r="AZ88" s="57" t="n"/>
       <c r="BA88" s="57" t="n"/>
-      <c r="CI88" t="inlineStr">
+      <c r="CI88" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ88" t="inlineStr">
+        <is>
+          <t>Towers in range hit harder and shoot faster</t>
         </is>
       </c>
     </row>
@@ -21701,9 +21866,14 @@
       <c r="AY89" s="57" t="n"/>
       <c r="AZ89" s="57" t="n"/>
       <c r="BA89" s="57" t="n"/>
-      <c r="CI89" t="inlineStr">
+      <c r="CI89" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ89" t="inlineStr">
+        <is>
+          <t>Towers in range hit much harder and faster</t>
         </is>
       </c>
     </row>
@@ -22090,9 +22260,14 @@
         <v>0.7</v>
       </c>
       <c r="BA93" s="57" t="n"/>
-      <c r="CI93" t="inlineStr">
+      <c r="CI93" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ93" t="inlineStr">
+        <is>
+          <t>Hunters in range shoot straighter</t>
         </is>
       </c>
     </row>
@@ -22196,9 +22371,14 @@
       <c r="BA94" s="57" t="n">
         <v>20</v>
       </c>
-      <c r="CI94" t="inlineStr">
+      <c r="CI94" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ94" t="inlineStr">
+        <is>
+          <t>Wider reach, and hunters in range fire faster</t>
         </is>
       </c>
     </row>
@@ -22619,9 +22799,14 @@
       <c r="BG98" s="57" t="n"/>
       <c r="BH98" s="57" t="n"/>
       <c r="BI98" s="57" t="n"/>
-      <c r="CI98" t="inlineStr">
+      <c r="CI98" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ98" t="inlineStr">
+        <is>
+          <t>Heals towers and hunters even faster</t>
         </is>
       </c>
     </row>
@@ -22729,9 +22914,14 @@
       <c r="BG99" s="57" t="n"/>
       <c r="BH99" s="57" t="n"/>
       <c r="BI99" s="57" t="n"/>
-      <c r="CI99" t="inlineStr">
+      <c r="CI99" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ99" t="inlineStr">
+        <is>
+          <t>The fastest heals; trampled towers revive at full speed</t>
         </is>
       </c>
     </row>
@@ -23146,9 +23336,14 @@
       <c r="BG103" s="57" t="n"/>
       <c r="BH103" s="57" t="n"/>
       <c r="BI103" s="57" t="n"/>
-      <c r="CI103" t="inlineStr">
+      <c r="CI103" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ103" t="inlineStr">
+        <is>
+          <t>Three med kits a round, and each heals more</t>
         </is>
       </c>
     </row>
@@ -23256,9 +23451,14 @@
       </c>
       <c r="BH104" s="57" t="n"/>
       <c r="BI104" s="57" t="n"/>
-      <c r="CI104" t="inlineStr">
+      <c r="CI104" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ104" t="inlineStr">
+        <is>
+          <t>Bigger kits and reach; downed hunters return sooner</t>
         </is>
       </c>
     </row>
@@ -23675,9 +23875,14 @@
         <v>35</v>
       </c>
       <c r="BI108" s="57" t="n"/>
-      <c r="CI108" t="inlineStr">
+      <c r="CI108" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ108" t="inlineStr">
+        <is>
+          <t>Towers in range get much more health</t>
         </is>
       </c>
     </row>
@@ -23787,9 +23992,14 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="CI109" t="inlineStr">
+      <c r="CI109" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ109" t="inlineStr">
+        <is>
+          <t>More health; once a round, saves a tower from trampling</t>
         </is>
       </c>
     </row>
@@ -24030,9 +24240,14 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="CI113" t="inlineStr">
+      <c r="CI113" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ113" t="inlineStr">
+        <is>
+          <t>Arcs can jump from one coil's range to another's</t>
         </is>
       </c>
     </row>
@@ -24097,9 +24312,14 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="CI114" t="inlineStr">
+      <c r="CI114" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ114" t="inlineStr">
+        <is>
+          <t>Strikes every dino near every coil; more coils, more power</t>
         </is>
       </c>
     </row>
@@ -24330,9 +24550,14 @@
       </c>
       <c r="U118" s="57" t="n"/>
       <c r="BP118" s="81" t="n"/>
-      <c r="CI118" t="inlineStr">
+      <c r="CI118" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ118" t="inlineStr">
+        <is>
+          <t>Hurts armoured dinos, and hits harder</t>
         </is>
       </c>
     </row>
@@ -24396,9 +24621,14 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="CI119" t="inlineStr">
+      <c r="CI119" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ119" t="inlineStr">
+        <is>
+          <t>A huge bolt shrinks the biggest dino 3 sizes</t>
         </is>
       </c>
     </row>
@@ -24627,9 +24857,14 @@
         <v>15</v>
       </c>
       <c r="BR123" s="81" t="n"/>
-      <c r="CI123" t="inlineStr">
+      <c r="CI123" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ123" t="inlineStr">
+        <is>
+          <t>Towers in range hit harder</t>
         </is>
       </c>
     </row>
@@ -24691,9 +24926,14 @@
       <c r="BS124" s="81" t="n">
         <v>50</v>
       </c>
-      <c r="CI124" t="inlineStr">
+      <c r="CI124" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ124" t="inlineStr">
+        <is>
+          <t>Towers in range chain their shots to one more dino</t>
         </is>
       </c>
     </row>
@@ -24923,9 +25163,14 @@
         <v>3</v>
       </c>
       <c r="BU128" s="81" t="n"/>
-      <c r="CI128" t="inlineStr">
+      <c r="CI128" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ128" t="inlineStr">
+        <is>
+          <t>Hurts armoured dinos; dives shrink a dino 3 sizes</t>
         </is>
       </c>
     </row>
@@ -24992,9 +25237,14 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="CI129" t="inlineStr">
+      <c r="CI129" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ129" t="inlineStr">
+        <is>
+          <t>One giant eagle dives, stuns and shrinks a dino 3 sizes</t>
         </is>
       </c>
     </row>
@@ -25219,9 +25469,14 @@
         </is>
       </c>
       <c r="BT133" s="81" t="n"/>
-      <c r="CI133" t="inlineStr">
+      <c r="CI133" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ133" t="inlineStr">
+        <is>
+          <t>The birds hunt much further out</t>
         </is>
       </c>
     </row>
@@ -25285,9 +25540,14 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="CI134" t="inlineStr">
+      <c r="CI134" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ134" t="inlineStr">
+        <is>
+          <t>A swarm of small birds pecks every dino in range</t>
         </is>
       </c>
     </row>
@@ -25516,9 +25776,14 @@
         <v>2</v>
       </c>
       <c r="BX138" s="81" t="n"/>
-      <c r="CI138" t="inlineStr">
+      <c r="CI138" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ138" t="inlineStr">
+        <is>
+          <t>Struck dinos get pulled back (not bosses)</t>
         </is>
       </c>
     </row>
@@ -25580,9 +25845,14 @@
       <c r="BY139" s="81" t="n">
         <v>15</v>
       </c>
-      <c r="CI139" t="inlineStr">
+      <c r="CI139" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ139" t="inlineStr">
+        <is>
+          <t>Towers in range shoot faster while a bird dives</t>
         </is>
       </c>
     </row>
@@ -25814,9 +26084,14 @@
         <v>3</v>
       </c>
       <c r="CC143" s="81" t="n"/>
-      <c r="CI143" t="inlineStr">
+      <c r="CI143" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ143" t="inlineStr">
+        <is>
+          <t>Dinos stay slowed for a while after they leave</t>
         </is>
       </c>
     </row>
@@ -25875,9 +26150,14 @@
       <c r="AE144" s="81" t="n"/>
       <c r="AF144" s="81" t="n"/>
       <c r="CC144" s="81" t="n"/>
-      <c r="CI144" t="inlineStr">
+      <c r="CI144" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ144" t="inlineStr">
+        <is>
+          <t>The pool covers three times as much track</t>
         </is>
       </c>
     </row>
@@ -26105,9 +26385,14 @@
       <c r="Y148" s="81" t="n">
         <v>2</v>
       </c>
-      <c r="CI148" t="inlineStr">
+      <c r="CI148" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ148" t="inlineStr">
+        <is>
+          <t>Dinos walk out of the tar still burning</t>
         </is>
       </c>
     </row>
@@ -26170,9 +26455,14 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="CI149" t="inlineStr">
+      <c r="CI149" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ149" t="inlineStr">
+        <is>
+          <t>A geyser shrinks every dino in the pool 2 sizes</t>
         </is>
       </c>
     </row>
@@ -26408,9 +26698,14 @@
       <c r="CG153" s="81" t="n">
         <v>15</v>
       </c>
-      <c r="CI153" t="inlineStr">
+      <c r="CI153" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ153" t="inlineStr">
+        <is>
+          <t>Dinos leaving the tar leave a slowing trail</t>
         </is>
       </c>
     </row>
@@ -26472,9 +26767,14 @@
       <c r="CH154" s="81" t="n">
         <v>15</v>
       </c>
-      <c r="CI154" t="inlineStr">
+      <c r="CI154" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ154" t="inlineStr">
+        <is>
+          <t>Towers in range hit slowed dinos harder</t>
         </is>
       </c>
     </row>
@@ -26700,9 +27000,14 @@
       <c r="BJ158" s="81" t="n">
         <v>3</v>
       </c>
-      <c r="CI158" t="inlineStr">
+      <c r="CI158" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ158" t="inlineStr">
+        <is>
+          <t>Pierces armour and shrinks a dino 3 sizes</t>
         </is>
       </c>
     </row>
@@ -26765,9 +27070,14 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="CI159" t="inlineStr">
+      <c r="CI159" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ159" t="inlineStr">
+        <is>
+          <t>The bolt flies on through every dino in its line</t>
         </is>
       </c>
     </row>
@@ -26989,9 +27299,14 @@
       <c r="W163" s="81" t="n">
         <v>6</v>
       </c>
-      <c r="CI163" t="inlineStr">
+      <c r="CI163" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ163" t="inlineStr">
+        <is>
+          <t>Drags the hit dino back along the track (not bosses)</t>
         </is>
       </c>
     </row>
@@ -27054,9 +27369,14 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="CI164" t="inlineStr">
+      <c r="CI164" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ164" t="inlineStr">
+        <is>
+          <t>Every 15 seconds, pulls a boss back along the track</t>
         </is>
       </c>
     </row>
@@ -27281,9 +27601,14 @@
         </is>
       </c>
       <c r="Q168" s="81" t="n"/>
-      <c r="CI168" t="inlineStr">
+      <c r="CI168" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="CJ168" t="inlineStr">
+        <is>
+          <t>Fires twice as fast</t>
         </is>
       </c>
     </row>
@@ -27347,13 +27672,17 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="CI169" t="inlineStr">
+      <c r="CI169" s="81" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-    </row>
-    <row r="170"/>
+      <c r="CJ169" t="inlineStr">
+        <is>
+          <t>Chained bolt pairs hit every dino between them</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811" footer="0.511811"/>
   <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" firstPageNumber="1" useFirstPageNumber="0" pageOrder="downThenOver"/>
@@ -27959,7 +28288,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BC77"/>
+  <dimension ref="A1:BC76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" style="90" min="1" max="1"/>
@@ -28011,7 +28340,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="21" t="inlineStr">
         <is>
@@ -28278,12 +28606,12 @@
           <t>Ability charges</t>
         </is>
       </c>
-      <c r="BB4" t="inlineStr">
+      <c r="BB4" s="81" t="inlineStr">
         <is>
           <t>Option</t>
         </is>
       </c>
-      <c r="BC4" t="inlineStr">
+      <c r="BC4" s="81" t="inlineStr">
         <is>
           <t>Blurb</t>
         </is>
@@ -28538,9 +28866,14 @@
       <c r="AG8" s="57" t="n"/>
       <c r="AH8" s="57" t="n"/>
       <c r="AI8" s="57" t="n"/>
-      <c r="BB8" t="inlineStr">
+      <c r="BB8" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="BC8" t="inlineStr">
+        <is>
+          <t>Fires faster and reloads quicker</t>
         </is>
       </c>
     </row>
@@ -28611,9 +28944,14 @@
       <c r="AG9" s="57" t="n"/>
       <c r="AH9" s="57" t="n"/>
       <c r="AI9" s="57" t="n"/>
-      <c r="BB9" t="inlineStr">
+      <c r="BB9" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="BC9" t="inlineStr">
+        <is>
+          <t>Both guns go full-auto</t>
         </is>
       </c>
     </row>
@@ -28874,9 +29212,14 @@
       <c r="AG13" s="57" t="n"/>
       <c r="AH13" s="57" t="n"/>
       <c r="AI13" s="57" t="n"/>
-      <c r="BB13" t="inlineStr">
+      <c r="BB13" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="BC13" t="inlineStr">
+        <is>
+          <t>Shots pierce armour</t>
         </is>
       </c>
     </row>
@@ -28945,9 +29288,14 @@
       <c r="AG14" s="57" t="n"/>
       <c r="AH14" s="57" t="n"/>
       <c r="AI14" s="57" t="n"/>
-      <c r="BB14" t="inlineStr">
+      <c r="BB14" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="BC14" t="inlineStr">
+        <is>
+          <t>Triple damage to marked dinos</t>
         </is>
       </c>
     </row>
@@ -29200,9 +29548,14 @@
       <c r="AG18" s="57" t="n"/>
       <c r="AH18" s="57" t="n"/>
       <c r="AI18" s="57" t="n"/>
-      <c r="BB18" t="inlineStr">
+      <c r="BB18" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="BC18" t="inlineStr">
+        <is>
+          <t>Your Tracking Dart is ready again sooner</t>
         </is>
       </c>
     </row>
@@ -29271,9 +29624,14 @@
       <c r="AG19" s="57" t="n"/>
       <c r="AH19" s="57" t="n"/>
       <c r="AI19" s="57" t="n"/>
-      <c r="BB19" t="inlineStr">
+      <c r="BB19" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="BC19" t="inlineStr">
+        <is>
+          <t>Shots bounce 4 times</t>
         </is>
       </c>
     </row>
@@ -29534,9 +29892,14 @@
       <c r="AG23" s="57" t="n"/>
       <c r="AH23" s="57" t="n"/>
       <c r="AI23" s="57" t="n"/>
-      <c r="BB23" t="inlineStr">
+      <c r="BB23" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="BC23" t="inlineStr">
+        <is>
+          <t>Less kick and longer reach</t>
         </is>
       </c>
     </row>
@@ -29609,9 +29972,14 @@
       <c r="AG24" s="57" t="n"/>
       <c r="AH24" s="57" t="n"/>
       <c r="AI24" s="57" t="n"/>
-      <c r="BB24" t="inlineStr">
+      <c r="BB24" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="BC24" t="inlineStr">
+        <is>
+          <t>4-round bursts with a much tighter grouping</t>
         </is>
       </c>
     </row>
@@ -29866,9 +30234,14 @@
       <c r="AG28" s="57" t="n"/>
       <c r="AH28" s="57" t="n"/>
       <c r="AI28" s="57" t="n"/>
-      <c r="BB28" t="inlineStr">
+      <c r="BB28" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="BC28" t="inlineStr">
+        <is>
+          <t>Much less kick while you stand still</t>
         </is>
       </c>
     </row>
@@ -29937,9 +30310,14 @@
       <c r="AG29" s="57" t="n"/>
       <c r="AH29" s="57" t="n"/>
       <c r="AI29" s="57" t="n"/>
-      <c r="BB29" t="inlineStr">
+      <c r="BB29" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="BC29" t="inlineStr">
+        <is>
+          <t>Fire rate climbs while you hold the trigger</t>
         </is>
       </c>
     </row>
@@ -30196,9 +30574,14 @@
       <c r="AG33" s="57" t="n"/>
       <c r="AH33" s="57" t="n"/>
       <c r="AI33" s="57" t="n"/>
-      <c r="BB33" t="inlineStr">
+      <c r="BB33" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="BC33" t="inlineStr">
+        <is>
+          <t>Hits harder and reaches further</t>
         </is>
       </c>
     </row>
@@ -30265,9 +30648,14 @@
       <c r="AG34" s="57" t="n"/>
       <c r="AH34" s="57" t="n"/>
       <c r="AI34" s="57" t="n"/>
-      <c r="BB34" t="inlineStr">
+      <c r="BB34" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="BC34" t="inlineStr">
+        <is>
+          <t>Shots burst with a small splash</t>
         </is>
       </c>
     </row>
@@ -30552,9 +30940,14 @@
       <c r="AG38" s="57" t="n"/>
       <c r="AH38" s="57" t="n"/>
       <c r="AI38" s="57" t="n"/>
-      <c r="BB38" t="inlineStr">
+      <c r="BB38" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="BC38" t="inlineStr">
+        <is>
+          <t>Tighter, longer slugs that go through 3 dinos</t>
         </is>
       </c>
     </row>
@@ -30623,9 +31016,14 @@
       <c r="AG39" s="57" t="n"/>
       <c r="AH39" s="57" t="n"/>
       <c r="AI39" s="57" t="n"/>
-      <c r="BB39" t="inlineStr">
+      <c r="BB39" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="BC39" t="inlineStr">
+        <is>
+          <t>Slugs go through 6 dinos</t>
         </is>
       </c>
     </row>
@@ -30884,9 +31282,14 @@
       <c r="AG43" s="57" t="n"/>
       <c r="AH43" s="57" t="n"/>
       <c r="AI43" s="57" t="n"/>
-      <c r="BB43" t="inlineStr">
+      <c r="BB43" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="BC43" t="inlineStr">
+        <is>
+          <t>Fires faster and reloads quicker</t>
         </is>
       </c>
     </row>
@@ -30959,9 +31362,14 @@
       <c r="AG44" s="57" t="n"/>
       <c r="AH44" s="57" t="n"/>
       <c r="AI44" s="57" t="n"/>
-      <c r="BB44" t="inlineStr">
+      <c r="BB44" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="BC44" t="inlineStr">
+        <is>
+          <t>A full-auto drum</t>
         </is>
       </c>
     </row>
@@ -31214,9 +31622,14 @@
       <c r="AG48" s="57" t="n"/>
       <c r="AH48" s="57" t="n"/>
       <c r="AI48" s="57" t="n"/>
-      <c r="BB48" t="inlineStr">
+      <c r="BB48" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="BC48" t="inlineStr">
+        <is>
+          <t>Blasts knock dinos back</t>
         </is>
       </c>
     </row>
@@ -31283,9 +31696,14 @@
       <c r="AG49" s="57" t="n"/>
       <c r="AH49" s="57" t="n"/>
       <c r="AI49" s="57" t="n"/>
-      <c r="BB49" t="inlineStr">
+      <c r="BB49" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="BC49" t="inlineStr">
+        <is>
+          <t>Shells explode on impact</t>
         </is>
       </c>
     </row>
@@ -31547,9 +31965,14 @@
         <v>1.5</v>
       </c>
       <c r="AL53" s="81" t="n"/>
-      <c r="BB53" t="inlineStr">
+      <c r="BB53" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="BC53" t="inlineStr">
+        <is>
+          <t>Your Triage Kit heals a wider area</t>
         </is>
       </c>
     </row>
@@ -31625,9 +32048,14 @@
       <c r="AN54" s="81" t="n">
         <v>8</v>
       </c>
-      <c r="BB54" t="inlineStr">
+      <c r="BB54" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="BC54" t="inlineStr">
+        <is>
+          <t>Everyone you heal takes less damage for a while</t>
         </is>
       </c>
     </row>
@@ -31890,9 +32318,14 @@
       <c r="AG58" s="57" t="n"/>
       <c r="AH58" s="57" t="n"/>
       <c r="AI58" s="57" t="n"/>
-      <c r="BB58" t="inlineStr">
+      <c r="BB58" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="BC58" t="inlineStr">
+        <is>
+          <t>Half the kick</t>
         </is>
       </c>
     </row>
@@ -31967,9 +32400,14 @@
       <c r="AG59" s="57" t="n"/>
       <c r="AH59" s="57" t="n"/>
       <c r="AI59" s="57" t="n"/>
-      <c r="BB59" t="inlineStr">
+      <c r="BB59" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="BC59" t="inlineStr">
+        <is>
+          <t>Goes full auto</t>
         </is>
       </c>
     </row>
@@ -32230,9 +32668,14 @@
       <c r="AQ63" s="81" t="n">
         <v>3</v>
       </c>
-      <c r="BB63" t="inlineStr">
+      <c r="BB63" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="BC63" t="inlineStr">
+        <is>
+          <t>Jaw Lock keeps a dino's jaws shut for longer</t>
         </is>
       </c>
     </row>
@@ -32299,9 +32742,14 @@
       <c r="AR64" s="81" t="n">
         <v>6</v>
       </c>
-      <c r="BB64" t="inlineStr">
+      <c r="BB64" s="81" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="BC64" t="inlineStr">
+        <is>
+          <t>Jaw Lock spreads to nearby dinos</t>
         </is>
       </c>
     </row>
@@ -33130,7 +33578,6 @@
         <v>9</v>
       </c>
     </row>
-    <row r="77"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
9f T121a: Tracker B/C options and the #298 gun-path worth metric
12 Tracker options appended to Hero Upgrades exactly as PLAN 9f (Cost =F of the A row,
no Damage x). value.py: hero_worth / hero_gun_worth (#298: (DPS x Hit + Burn) x Targets x
Hurt x Reach x Amp x Hold x Breaks, Tracker x (1 + Dart uptime); burst count no longer
multiplies rounds) replace hero_dps for the hero option bars and the T6 parity (Triage
and Muzzle keep hero_dps until the Field Medic commit). Bars: every Tracker slot within
0.8-1.25x; T6 builds per path x1.11 / x1.07 / x1.13. New herooptions spec: each option's
composed row, every T6 after any T5, Twin Burst = 3-round bursts from two guns (Hot Swap
still staggers), Hunter's Mark, Dart Storm. HEROES.md option table.

Statically checked and headless-tested; not playtested.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Storm-Split-Balance.xlsx
+++ b/Storm-Split-Balance.xlsx
@@ -37632,7 +37632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BC76"/>
+  <dimension ref="A1:CA88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" style="90" min="1" max="1"/>
@@ -42920,6 +42920,878 @@
       </c>
       <c r="AR76" s="81" t="n">
         <v>9</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="43" t="inlineStr">
+        <is>
+          <t>Tracker</t>
+        </is>
+      </c>
+      <c r="B77" s="43" t="inlineStr">
+        <is>
+          <t>Gunslinger</t>
+        </is>
+      </c>
+      <c r="C77" s="43" t="inlineStr">
+        <is>
+          <t>handling</t>
+        </is>
+      </c>
+      <c r="D77" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="E77" s="43" t="inlineStr">
+        <is>
+          <t>Deep Cylinders</t>
+        </is>
+      </c>
+      <c r="F77" s="56">
+        <f>F8</f>
+        <v/>
+      </c>
+      <c r="G77" s="57" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="H77" s="57" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I77" s="57" t="n"/>
+      <c r="J77" s="57" t="n"/>
+      <c r="K77" s="57" t="n"/>
+      <c r="L77" s="57" t="n"/>
+      <c r="M77" s="57" t="n"/>
+      <c r="N77" s="57" t="n"/>
+      <c r="O77" s="57" t="n"/>
+      <c r="P77" s="57" t="n"/>
+      <c r="Q77" s="57" t="n"/>
+      <c r="R77" s="57" t="n"/>
+      <c r="S77" s="57" t="n"/>
+      <c r="T77" s="57" t="n"/>
+      <c r="U77" s="57" t="n"/>
+      <c r="V77" s="57" t="n"/>
+      <c r="W77" s="57" t="n"/>
+      <c r="X77" s="57" t="n"/>
+      <c r="Y77" s="57" t="n"/>
+      <c r="Z77" s="57" t="n"/>
+      <c r="AA77" s="57" t="n"/>
+      <c r="AB77" s="57" t="n"/>
+      <c r="AC77" s="57" t="n"/>
+      <c r="AD77" s="57" t="n"/>
+      <c r="AE77" s="57" t="n"/>
+      <c r="AF77" s="57" t="n"/>
+      <c r="AG77" s="57" t="n"/>
+      <c r="AH77" s="57" t="n"/>
+      <c r="AI77" s="57" t="n"/>
+      <c r="BB77" s="81" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="BC77" s="81" t="inlineStr">
+        <is>
+          <t>Both guns hold 50% more and fire 15% faster</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="43" t="inlineStr">
+        <is>
+          <t>Tracker</t>
+        </is>
+      </c>
+      <c r="B78" s="43" t="inlineStr">
+        <is>
+          <t>Gunslinger</t>
+        </is>
+      </c>
+      <c r="C78" s="43" t="inlineStr">
+        <is>
+          <t>handling</t>
+        </is>
+      </c>
+      <c r="D78" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="E78" s="43" t="inlineStr">
+        <is>
+          <t>Crossdraw</t>
+        </is>
+      </c>
+      <c r="F78" s="56">
+        <f>F8</f>
+        <v/>
+      </c>
+      <c r="G78" s="57" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="H78" s="57" t="n"/>
+      <c r="I78" s="57" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J78" s="57" t="n"/>
+      <c r="K78" s="57" t="n"/>
+      <c r="L78" s="57" t="n"/>
+      <c r="M78" s="57" t="n"/>
+      <c r="N78" s="57" t="n"/>
+      <c r="O78" s="57" t="n"/>
+      <c r="P78" s="57" t="n"/>
+      <c r="Q78" s="57" t="n"/>
+      <c r="R78" s="57" t="n"/>
+      <c r="S78" s="57" t="n"/>
+      <c r="T78" s="57" t="n"/>
+      <c r="U78" s="57" t="n"/>
+      <c r="V78" s="57" t="n"/>
+      <c r="W78" s="57" t="n"/>
+      <c r="X78" s="57" t="n"/>
+      <c r="Y78" s="57" t="n"/>
+      <c r="Z78" s="57" t="n"/>
+      <c r="AA78" s="57" t="n"/>
+      <c r="AB78" s="57" t="n"/>
+      <c r="AC78" s="57" t="n"/>
+      <c r="AD78" s="57" t="n"/>
+      <c r="AE78" s="57" t="n"/>
+      <c r="AF78" s="57" t="n"/>
+      <c r="AG78" s="57" t="n"/>
+      <c r="AH78" s="57" t="n"/>
+      <c r="AI78" s="57" t="n"/>
+      <c r="BB78" s="81" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="BC78" s="81" t="inlineStr">
+        <is>
+          <t>Reload 35% faster, fire 15% faster</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="43" t="inlineStr">
+        <is>
+          <t>Tracker</t>
+        </is>
+      </c>
+      <c r="B79" s="43" t="inlineStr">
+        <is>
+          <t>Gunslinger</t>
+        </is>
+      </c>
+      <c r="C79" s="43" t="inlineStr">
+        <is>
+          <t>handling</t>
+        </is>
+      </c>
+      <c r="D79" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="E79" s="43" t="inlineStr">
+        <is>
+          <t>Twin Burst</t>
+        </is>
+      </c>
+      <c r="F79" s="56">
+        <f>F9</f>
+        <v/>
+      </c>
+      <c r="G79" s="57" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="H79" s="57" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="I79" s="57" t="n"/>
+      <c r="J79" s="57" t="n"/>
+      <c r="K79" s="57" t="n"/>
+      <c r="L79" s="57" t="n"/>
+      <c r="M79" s="57" t="n"/>
+      <c r="N79" s="57" t="inlineStr">
+        <is>
+          <t>burst</t>
+        </is>
+      </c>
+      <c r="O79" s="57" t="n">
+        <v>3</v>
+      </c>
+      <c r="P79" s="57" t="n"/>
+      <c r="Q79" s="57" t="n"/>
+      <c r="R79" s="57" t="n"/>
+      <c r="S79" s="57" t="n"/>
+      <c r="T79" s="57" t="n"/>
+      <c r="U79" s="57" t="n"/>
+      <c r="V79" s="57" t="n"/>
+      <c r="W79" s="57" t="n"/>
+      <c r="X79" s="57" t="n"/>
+      <c r="Y79" s="57" t="n"/>
+      <c r="Z79" s="57" t="n"/>
+      <c r="AA79" s="57" t="n"/>
+      <c r="AB79" s="57" t="n"/>
+      <c r="AC79" s="57" t="n"/>
+      <c r="AD79" s="57" t="n"/>
+      <c r="AE79" s="57" t="n"/>
+      <c r="AF79" s="57" t="n"/>
+      <c r="AG79" s="57" t="n"/>
+      <c r="AH79" s="57" t="n"/>
+      <c r="AI79" s="57" t="n"/>
+      <c r="BB79" s="81" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="BC79" s="81" t="inlineStr">
+        <is>
+          <t>Each click fires a 3-round burst, 30% faster</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="43" t="inlineStr">
+        <is>
+          <t>Tracker</t>
+        </is>
+      </c>
+      <c r="B80" s="43" t="inlineStr">
+        <is>
+          <t>Gunslinger</t>
+        </is>
+      </c>
+      <c r="C80" s="43" t="inlineStr">
+        <is>
+          <t>handling</t>
+        </is>
+      </c>
+      <c r="D80" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="E80" s="43" t="inlineStr">
+        <is>
+          <t>Steady Pair</t>
+        </is>
+      </c>
+      <c r="F80" s="56">
+        <f>F9</f>
+        <v/>
+      </c>
+      <c r="G80" s="57" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="H80" s="57" t="n"/>
+      <c r="I80" s="57" t="n"/>
+      <c r="J80" s="57" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K80" s="57" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L80" s="57" t="n"/>
+      <c r="M80" s="57" t="n"/>
+      <c r="N80" s="57" t="n"/>
+      <c r="O80" s="57" t="n"/>
+      <c r="P80" s="57" t="n"/>
+      <c r="Q80" s="57" t="n"/>
+      <c r="R80" s="57" t="n"/>
+      <c r="S80" s="57" t="n"/>
+      <c r="T80" s="57" t="n"/>
+      <c r="U80" s="57" t="n"/>
+      <c r="V80" s="57" t="n"/>
+      <c r="W80" s="57" t="n"/>
+      <c r="X80" s="57" t="n"/>
+      <c r="Y80" s="57" t="n"/>
+      <c r="Z80" s="57" t="n"/>
+      <c r="AA80" s="57" t="n"/>
+      <c r="AB80" s="57" t="n"/>
+      <c r="AC80" s="57" t="n"/>
+      <c r="AD80" s="57" t="n"/>
+      <c r="AE80" s="57" t="n"/>
+      <c r="AF80" s="57" t="n"/>
+      <c r="AG80" s="57" t="n"/>
+      <c r="AH80" s="57" t="n"/>
+      <c r="AI80" s="57" t="n"/>
+      <c r="BB80" s="81" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="BC80" s="81" t="inlineStr">
+        <is>
+          <t>Half the kick, tighter aim, 10% faster</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="43" t="inlineStr">
+        <is>
+          <t>Tracker</t>
+        </is>
+      </c>
+      <c r="B81" s="43" t="inlineStr">
+        <is>
+          <t>Marksman</t>
+        </is>
+      </c>
+      <c r="C81" s="43" t="inlineStr">
+        <is>
+          <t>accuracy</t>
+        </is>
+      </c>
+      <c r="D81" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="E81" s="43" t="inlineStr">
+        <is>
+          <t>Quick Cock</t>
+        </is>
+      </c>
+      <c r="F81" s="56">
+        <f>F13</f>
+        <v/>
+      </c>
+      <c r="G81" s="57" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H81" s="57" t="n"/>
+      <c r="I81" s="57" t="n"/>
+      <c r="J81" s="57" t="n"/>
+      <c r="K81" s="57" t="n"/>
+      <c r="L81" s="57" t="n"/>
+      <c r="M81" s="57" t="n"/>
+      <c r="N81" s="57" t="n"/>
+      <c r="O81" s="57" t="n"/>
+      <c r="P81" s="57" t="n"/>
+      <c r="Q81" s="57" t="n"/>
+      <c r="R81" s="57" t="n"/>
+      <c r="S81" s="57" t="n"/>
+      <c r="T81" s="57" t="n"/>
+      <c r="U81" s="57" t="n"/>
+      <c r="V81" s="57" t="n"/>
+      <c r="W81" s="57" t="n"/>
+      <c r="X81" s="57" t="n"/>
+      <c r="Y81" s="57" t="n"/>
+      <c r="Z81" s="57" t="n"/>
+      <c r="AA81" s="57" t="n"/>
+      <c r="AB81" s="57" t="n"/>
+      <c r="AC81" s="57" t="n"/>
+      <c r="AD81" s="57" t="n"/>
+      <c r="AE81" s="57" t="n"/>
+      <c r="AF81" s="57" t="n"/>
+      <c r="AG81" s="57" t="n"/>
+      <c r="AH81" s="57" t="n"/>
+      <c r="AI81" s="57" t="n"/>
+      <c r="BB81" s="81" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="BC81" s="81" t="inlineStr">
+        <is>
+          <t>Fire 20% faster, scope and all</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="43" t="inlineStr">
+        <is>
+          <t>Tracker</t>
+        </is>
+      </c>
+      <c r="B82" s="43" t="inlineStr">
+        <is>
+          <t>Marksman</t>
+        </is>
+      </c>
+      <c r="C82" s="43" t="inlineStr">
+        <is>
+          <t>accuracy</t>
+        </is>
+      </c>
+      <c r="D82" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="E82" s="43" t="inlineStr">
+        <is>
+          <t>Breath Control</t>
+        </is>
+      </c>
+      <c r="F82" s="56">
+        <f>F13</f>
+        <v/>
+      </c>
+      <c r="G82" s="57" t="n"/>
+      <c r="H82" s="57" t="n"/>
+      <c r="I82" s="57" t="n"/>
+      <c r="J82" s="57" t="n"/>
+      <c r="K82" s="57" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L82" s="57" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="M82" s="57" t="n"/>
+      <c r="N82" s="57" t="n"/>
+      <c r="O82" s="57" t="n"/>
+      <c r="P82" s="57" t="n"/>
+      <c r="Q82" s="57" t="n"/>
+      <c r="R82" s="57" t="n"/>
+      <c r="S82" s="57" t="n"/>
+      <c r="T82" s="57" t="n"/>
+      <c r="U82" s="57" t="n"/>
+      <c r="V82" s="57" t="n"/>
+      <c r="W82" s="57" t="n"/>
+      <c r="X82" s="57" t="n"/>
+      <c r="Y82" s="57" t="n"/>
+      <c r="Z82" s="57" t="n"/>
+      <c r="AA82" s="57" t="n"/>
+      <c r="AB82" s="57" t="n"/>
+      <c r="AC82" s="57" t="n"/>
+      <c r="AD82" s="57" t="n"/>
+      <c r="AE82" s="57" t="n"/>
+      <c r="AF82" s="57" t="n"/>
+      <c r="AG82" s="57" t="n"/>
+      <c r="AH82" s="57" t="n"/>
+      <c r="AI82" s="57" t="n"/>
+      <c r="BB82" s="81" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="BC82" s="81" t="inlineStr">
+        <is>
+          <t>Half the kick; the scope reaches 35% further</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="43" t="inlineStr">
+        <is>
+          <t>Tracker</t>
+        </is>
+      </c>
+      <c r="B83" s="43" t="inlineStr">
+        <is>
+          <t>Marksman</t>
+        </is>
+      </c>
+      <c r="C83" s="43" t="inlineStr">
+        <is>
+          <t>accuracy</t>
+        </is>
+      </c>
+      <c r="D83" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="E83" s="43" t="inlineStr">
+        <is>
+          <t>Quick Scope</t>
+        </is>
+      </c>
+      <c r="F83" s="56">
+        <f>F14</f>
+        <v/>
+      </c>
+      <c r="G83" s="57" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H83" s="57" t="n"/>
+      <c r="I83" s="57" t="n"/>
+      <c r="J83" s="57" t="n"/>
+      <c r="K83" s="57" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="L83" s="57" t="n"/>
+      <c r="M83" s="57" t="n"/>
+      <c r="N83" s="57" t="n"/>
+      <c r="O83" s="57" t="n"/>
+      <c r="P83" s="57" t="n"/>
+      <c r="Q83" s="57" t="n"/>
+      <c r="R83" s="57" t="n"/>
+      <c r="S83" s="57" t="n"/>
+      <c r="T83" s="57" t="n"/>
+      <c r="U83" s="57" t="n"/>
+      <c r="V83" s="57" t="n"/>
+      <c r="W83" s="57" t="n"/>
+      <c r="X83" s="57" t="n"/>
+      <c r="Y83" s="57" t="n"/>
+      <c r="Z83" s="57" t="n"/>
+      <c r="AA83" s="57" t="n"/>
+      <c r="AB83" s="57" t="n"/>
+      <c r="AC83" s="57" t="n"/>
+      <c r="AD83" s="57" t="n"/>
+      <c r="AE83" s="57" t="n"/>
+      <c r="AF83" s="57" t="n"/>
+      <c r="AG83" s="57" t="n"/>
+      <c r="AH83" s="57" t="n"/>
+      <c r="AI83" s="57" t="n"/>
+      <c r="BB83" s="81" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="BC83" s="81" t="inlineStr">
+        <is>
+          <t>Fire 70% faster with 30% less kick</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="43" t="inlineStr">
+        <is>
+          <t>Tracker</t>
+        </is>
+      </c>
+      <c r="B84" s="43" t="inlineStr">
+        <is>
+          <t>Marksman</t>
+        </is>
+      </c>
+      <c r="C84" s="43" t="inlineStr">
+        <is>
+          <t>accuracy</t>
+        </is>
+      </c>
+      <c r="D84" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="E84" s="43" t="inlineStr">
+        <is>
+          <t>Hunter's Mark</t>
+        </is>
+      </c>
+      <c r="F84" s="56">
+        <f>F14</f>
+        <v/>
+      </c>
+      <c r="G84" s="57" t="n"/>
+      <c r="H84" s="57" t="n"/>
+      <c r="I84" s="57" t="n"/>
+      <c r="J84" s="57" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K84" s="57" t="n"/>
+      <c r="L84" s="57" t="n"/>
+      <c r="M84" s="57" t="n"/>
+      <c r="N84" s="57" t="n"/>
+      <c r="O84" s="57" t="n"/>
+      <c r="P84" s="57" t="n"/>
+      <c r="Q84" s="57" t="n"/>
+      <c r="R84" s="57" t="n"/>
+      <c r="S84" s="57" t="n"/>
+      <c r="T84" s="57" t="n"/>
+      <c r="U84" s="57" t="n"/>
+      <c r="V84" s="57" t="n"/>
+      <c r="W84" s="57" t="n"/>
+      <c r="X84" s="57" t="n"/>
+      <c r="Y84" s="57" t="n"/>
+      <c r="Z84" s="57" t="n"/>
+      <c r="AA84" s="57" t="n">
+        <v>35</v>
+      </c>
+      <c r="AB84" s="57" t="n"/>
+      <c r="AC84" s="57" t="n"/>
+      <c r="AD84" s="57" t="n"/>
+      <c r="AE84" s="57" t="n"/>
+      <c r="AF84" s="57" t="n"/>
+      <c r="AG84" s="57" t="n"/>
+      <c r="AH84" s="57" t="n"/>
+      <c r="AI84" s="57" t="n"/>
+      <c r="BB84" s="81" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="BC84" s="81" t="inlineStr">
+        <is>
+          <t>Hits mark dinos: +35% from everything</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="43" t="inlineStr">
+        <is>
+          <t>Tracker</t>
+        </is>
+      </c>
+      <c r="B85" s="43" t="inlineStr">
+        <is>
+          <t>Trick Shot</t>
+        </is>
+      </c>
+      <c r="C85" s="43" t="inlineStr">
+        <is>
+          <t>utility</t>
+        </is>
+      </c>
+      <c r="D85" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="E85" s="43" t="inlineStr">
+        <is>
+          <t>Bank Shot</t>
+        </is>
+      </c>
+      <c r="F85" s="56">
+        <f>F18</f>
+        <v/>
+      </c>
+      <c r="G85" s="57" t="n"/>
+      <c r="H85" s="57" t="n"/>
+      <c r="I85" s="57" t="n"/>
+      <c r="J85" s="57" t="n"/>
+      <c r="K85" s="57" t="n"/>
+      <c r="L85" s="57" t="n"/>
+      <c r="M85" s="57" t="n"/>
+      <c r="N85" s="57" t="n"/>
+      <c r="O85" s="57" t="n"/>
+      <c r="P85" s="57" t="n"/>
+      <c r="Q85" s="57" t="n"/>
+      <c r="R85" s="57" t="n"/>
+      <c r="S85" s="57" t="n"/>
+      <c r="T85" s="57" t="n">
+        <v>2</v>
+      </c>
+      <c r="U85" s="57" t="n"/>
+      <c r="V85" s="57" t="n"/>
+      <c r="W85" s="57" t="n"/>
+      <c r="X85" s="57" t="n"/>
+      <c r="Y85" s="57" t="n"/>
+      <c r="Z85" s="57" t="n"/>
+      <c r="AA85" s="57" t="n"/>
+      <c r="AB85" s="57" t="n"/>
+      <c r="AC85" s="57" t="n"/>
+      <c r="AD85" s="57" t="n"/>
+      <c r="AE85" s="57" t="n"/>
+      <c r="AF85" s="57" t="n"/>
+      <c r="AG85" s="57" t="n"/>
+      <c r="AH85" s="57" t="n"/>
+      <c r="AI85" s="57" t="n"/>
+      <c r="BB85" s="81" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="BC85" s="81" t="inlineStr">
+        <is>
+          <t>Ricochets bounce twice</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="43" t="inlineStr">
+        <is>
+          <t>Tracker</t>
+        </is>
+      </c>
+      <c r="B86" s="43" t="inlineStr">
+        <is>
+          <t>Trick Shot</t>
+        </is>
+      </c>
+      <c r="C86" s="43" t="inlineStr">
+        <is>
+          <t>utility</t>
+        </is>
+      </c>
+      <c r="D86" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="E86" s="43" t="inlineStr">
+        <is>
+          <t>Quick Fingers</t>
+        </is>
+      </c>
+      <c r="F86" s="56">
+        <f>F18</f>
+        <v/>
+      </c>
+      <c r="G86" s="57" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="H86" s="57" t="n"/>
+      <c r="I86" s="57" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J86" s="57" t="n"/>
+      <c r="K86" s="57" t="n"/>
+      <c r="L86" s="57" t="n"/>
+      <c r="M86" s="57" t="n"/>
+      <c r="N86" s="57" t="n"/>
+      <c r="O86" s="57" t="n"/>
+      <c r="P86" s="57" t="n"/>
+      <c r="Q86" s="57" t="n"/>
+      <c r="R86" s="57" t="n"/>
+      <c r="S86" s="57" t="n"/>
+      <c r="T86" s="57" t="n"/>
+      <c r="U86" s="57" t="n"/>
+      <c r="V86" s="57" t="n"/>
+      <c r="W86" s="57" t="n"/>
+      <c r="X86" s="57" t="n"/>
+      <c r="Y86" s="57" t="n"/>
+      <c r="Z86" s="57" t="n"/>
+      <c r="AA86" s="57" t="n"/>
+      <c r="AB86" s="57" t="n"/>
+      <c r="AC86" s="57" t="n"/>
+      <c r="AD86" s="57" t="n"/>
+      <c r="AE86" s="57" t="n"/>
+      <c r="AF86" s="57" t="n"/>
+      <c r="AG86" s="57" t="n"/>
+      <c r="AH86" s="57" t="n"/>
+      <c r="AI86" s="57" t="n"/>
+      <c r="BB86" s="81" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="BC86" s="81" t="inlineStr">
+        <is>
+          <t>Reload 30% faster, fire a bit faster</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="43" t="inlineStr">
+        <is>
+          <t>Tracker</t>
+        </is>
+      </c>
+      <c r="B87" s="43" t="inlineStr">
+        <is>
+          <t>Trick Shot</t>
+        </is>
+      </c>
+      <c r="C87" s="43" t="inlineStr">
+        <is>
+          <t>utility</t>
+        </is>
+      </c>
+      <c r="D87" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="E87" s="43" t="inlineStr">
+        <is>
+          <t>Pinball</t>
+        </is>
+      </c>
+      <c r="F87" s="56">
+        <f>F19</f>
+        <v/>
+      </c>
+      <c r="G87" s="57" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="H87" s="57" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I87" s="57" t="n"/>
+      <c r="J87" s="57" t="n"/>
+      <c r="K87" s="57" t="n"/>
+      <c r="L87" s="57" t="n"/>
+      <c r="M87" s="57" t="n"/>
+      <c r="N87" s="57" t="n"/>
+      <c r="O87" s="57" t="n"/>
+      <c r="P87" s="57" t="n"/>
+      <c r="Q87" s="57" t="n"/>
+      <c r="R87" s="57" t="n"/>
+      <c r="S87" s="57" t="n"/>
+      <c r="T87" s="57" t="n">
+        <v>3</v>
+      </c>
+      <c r="U87" s="57" t="n"/>
+      <c r="V87" s="57" t="n"/>
+      <c r="W87" s="57" t="n"/>
+      <c r="X87" s="57" t="n"/>
+      <c r="Y87" s="57" t="n"/>
+      <c r="Z87" s="57" t="n"/>
+      <c r="AA87" s="57" t="n"/>
+      <c r="AB87" s="57" t="n"/>
+      <c r="AC87" s="57" t="n"/>
+      <c r="AD87" s="57" t="n"/>
+      <c r="AE87" s="57" t="n"/>
+      <c r="AF87" s="57" t="n"/>
+      <c r="AG87" s="57" t="n"/>
+      <c r="AH87" s="57" t="n"/>
+      <c r="AI87" s="57" t="n"/>
+      <c r="BB87" s="81" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="BC87" s="81" t="inlineStr">
+        <is>
+          <t>3 bounces, a bigger cylinder, faster shots</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="43" t="inlineStr">
+        <is>
+          <t>Tracker</t>
+        </is>
+      </c>
+      <c r="B88" s="43" t="inlineStr">
+        <is>
+          <t>Trick Shot</t>
+        </is>
+      </c>
+      <c r="C88" s="43" t="inlineStr">
+        <is>
+          <t>utility</t>
+        </is>
+      </c>
+      <c r="D88" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="E88" s="43" t="inlineStr">
+        <is>
+          <t>Dart Storm</t>
+        </is>
+      </c>
+      <c r="F88" s="56">
+        <f>F19</f>
+        <v/>
+      </c>
+      <c r="G88" s="57" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="H88" s="57" t="n"/>
+      <c r="I88" s="57" t="n"/>
+      <c r="J88" s="57" t="n"/>
+      <c r="K88" s="57" t="n"/>
+      <c r="L88" s="57" t="n"/>
+      <c r="M88" s="57" t="n"/>
+      <c r="N88" s="57" t="n"/>
+      <c r="O88" s="57" t="n"/>
+      <c r="P88" s="57" t="n"/>
+      <c r="Q88" s="57" t="n"/>
+      <c r="R88" s="57" t="n"/>
+      <c r="S88" s="57" t="n"/>
+      <c r="T88" s="57" t="n">
+        <v>3</v>
+      </c>
+      <c r="U88" s="57" t="n"/>
+      <c r="V88" s="57" t="n"/>
+      <c r="W88" s="57" t="n"/>
+      <c r="X88" s="57" t="n"/>
+      <c r="Y88" s="57" t="n"/>
+      <c r="Z88" s="57" t="n"/>
+      <c r="AA88" s="57" t="n"/>
+      <c r="AB88" s="57" t="n"/>
+      <c r="AC88" s="57" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AD88" s="57" t="n"/>
+      <c r="AE88" s="57" t="n"/>
+      <c r="AF88" s="57" t="n"/>
+      <c r="AG88" s="57" t="n"/>
+      <c r="AH88" s="57" t="n"/>
+      <c r="AI88" s="57" t="n"/>
+      <c r="BB88" s="81" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="BC88" s="81" t="inlineStr">
+        <is>
+          <t>3 bounces, faster shots, Tracking Dart sooner</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
9f T121b: Big Game Hunter B/C options
12 Big Game Hunter options appended to Hero Upgrades exactly as PLAN 9f (no Damage x).
Bars on the #298 gun metric: every slot within 0.8-1.25x; T6 builds per path x1.04
(Stalker) / x1.06 (Heavy) / x1.14 (Special Ammo). Specs: Big Five bursts 5 and Endless
Belt (spins up, no rounds once fully spun up) and Dynamite Rounds (6 m, pierces) after
every T5; Marking Burst, Bright Tracers marks; War Drum's Rally cooldown; Phosphor burn;
Fire Tips / Flat Tips blasts and reach. HEROES.md: option table and the Big Five /
Endless Belt / Dynamite Rounds rewording (#300).

Statically checked and headless-tested; not playtested.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Storm-Split-Balance.xlsx
+++ b/Storm-Split-Balance.xlsx
@@ -37632,7 +37632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CA88"/>
+  <dimension ref="A1:CA100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" style="90" min="1" max="1"/>
@@ -43791,6 +43791,870 @@
       <c r="BC88" s="81" t="inlineStr">
         <is>
           <t>3 bounces, faster shots, Tracking Dart sooner</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="43" t="inlineStr">
+        <is>
+          <t>Big Game Hunter</t>
+        </is>
+      </c>
+      <c r="B89" s="43" t="inlineStr">
+        <is>
+          <t>Stalker</t>
+        </is>
+      </c>
+      <c r="C89" s="43" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D89" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="E89" s="43" t="inlineStr">
+        <is>
+          <t>Snap Bursts</t>
+        </is>
+      </c>
+      <c r="F89" s="56">
+        <f>F23</f>
+        <v/>
+      </c>
+      <c r="G89" s="57" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H89" s="57" t="n"/>
+      <c r="I89" s="57" t="n"/>
+      <c r="J89" s="57" t="n"/>
+      <c r="K89" s="57" t="n"/>
+      <c r="L89" s="57" t="n"/>
+      <c r="M89" s="57" t="n"/>
+      <c r="N89" s="57" t="n"/>
+      <c r="O89" s="57" t="n"/>
+      <c r="P89" s="57" t="n"/>
+      <c r="Q89" s="57" t="n"/>
+      <c r="R89" s="57" t="n"/>
+      <c r="S89" s="57" t="n"/>
+      <c r="T89" s="57" t="n"/>
+      <c r="U89" s="57" t="n"/>
+      <c r="V89" s="57" t="n"/>
+      <c r="W89" s="57" t="n"/>
+      <c r="X89" s="57" t="n"/>
+      <c r="Y89" s="57" t="n"/>
+      <c r="Z89" s="57" t="n"/>
+      <c r="AA89" s="57" t="n"/>
+      <c r="AB89" s="57" t="n"/>
+      <c r="AC89" s="57" t="n"/>
+      <c r="AD89" s="57" t="n"/>
+      <c r="AE89" s="57" t="n"/>
+      <c r="AF89" s="57" t="n"/>
+      <c r="AG89" s="57" t="n"/>
+      <c r="AH89" s="57" t="n"/>
+      <c r="AI89" s="57" t="n"/>
+      <c r="BB89" s="81" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="BC89" s="81" t="inlineStr">
+        <is>
+          <t>Bursts come 20% faster</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="43" t="inlineStr">
+        <is>
+          <t>Big Game Hunter</t>
+        </is>
+      </c>
+      <c r="B90" s="43" t="inlineStr">
+        <is>
+          <t>Stalker</t>
+        </is>
+      </c>
+      <c r="C90" s="43" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D90" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="E90" s="43" t="inlineStr">
+        <is>
+          <t>Quick Mag</t>
+        </is>
+      </c>
+      <c r="F90" s="56">
+        <f>F23</f>
+        <v/>
+      </c>
+      <c r="G90" s="57" t="n"/>
+      <c r="H90" s="57" t="n"/>
+      <c r="I90" s="57" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J90" s="57" t="n"/>
+      <c r="K90" s="57" t="n"/>
+      <c r="L90" s="57" t="n"/>
+      <c r="M90" s="57" t="n"/>
+      <c r="N90" s="57" t="n"/>
+      <c r="O90" s="57" t="n"/>
+      <c r="P90" s="57" t="n"/>
+      <c r="Q90" s="57" t="n"/>
+      <c r="R90" s="57" t="n"/>
+      <c r="S90" s="57" t="n"/>
+      <c r="T90" s="57" t="n"/>
+      <c r="U90" s="57" t="n"/>
+      <c r="V90" s="57" t="n"/>
+      <c r="W90" s="57" t="n"/>
+      <c r="X90" s="57" t="n"/>
+      <c r="Y90" s="57" t="n"/>
+      <c r="Z90" s="57" t="n"/>
+      <c r="AA90" s="57" t="n"/>
+      <c r="AB90" s="57" t="n"/>
+      <c r="AC90" s="57" t="n"/>
+      <c r="AD90" s="57" t="n"/>
+      <c r="AE90" s="57" t="n"/>
+      <c r="AF90" s="57" t="n"/>
+      <c r="AG90" s="57" t="n"/>
+      <c r="AH90" s="57" t="n"/>
+      <c r="AI90" s="57" t="n"/>
+      <c r="BB90" s="81" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="BC90" s="81" t="inlineStr">
+        <is>
+          <t>Reload 25% faster</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="43" t="inlineStr">
+        <is>
+          <t>Big Game Hunter</t>
+        </is>
+      </c>
+      <c r="B91" s="43" t="inlineStr">
+        <is>
+          <t>Stalker</t>
+        </is>
+      </c>
+      <c r="C91" s="43" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D91" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="E91" s="43" t="inlineStr">
+        <is>
+          <t>Marking Burst</t>
+        </is>
+      </c>
+      <c r="F91" s="56">
+        <f>F24</f>
+        <v/>
+      </c>
+      <c r="G91" s="57" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="H91" s="57" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="I91" s="57" t="n"/>
+      <c r="J91" s="57" t="n"/>
+      <c r="K91" s="57" t="n"/>
+      <c r="L91" s="57" t="n"/>
+      <c r="M91" s="57" t="n"/>
+      <c r="N91" s="57" t="n"/>
+      <c r="O91" s="57" t="n">
+        <v>4</v>
+      </c>
+      <c r="P91" s="57" t="n"/>
+      <c r="Q91" s="57" t="n"/>
+      <c r="R91" s="57" t="n"/>
+      <c r="S91" s="57" t="n"/>
+      <c r="T91" s="57" t="n"/>
+      <c r="U91" s="57" t="n"/>
+      <c r="V91" s="57" t="n"/>
+      <c r="W91" s="57" t="n"/>
+      <c r="X91" s="57" t="n"/>
+      <c r="Y91" s="57" t="n"/>
+      <c r="Z91" s="57" t="n"/>
+      <c r="AA91" s="57" t="n">
+        <v>25</v>
+      </c>
+      <c r="AB91" s="57" t="n"/>
+      <c r="AC91" s="57" t="n"/>
+      <c r="AD91" s="57" t="n"/>
+      <c r="AE91" s="57" t="n"/>
+      <c r="AF91" s="57" t="n"/>
+      <c r="AG91" s="57" t="n"/>
+      <c r="AH91" s="57" t="n"/>
+      <c r="AI91" s="57" t="n"/>
+      <c r="BB91" s="81" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="BC91" s="81" t="inlineStr">
+        <is>
+          <t>4-round bursts that mark: +25% from everything</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="43" t="inlineStr">
+        <is>
+          <t>Big Game Hunter</t>
+        </is>
+      </c>
+      <c r="B92" s="43" t="inlineStr">
+        <is>
+          <t>Stalker</t>
+        </is>
+      </c>
+      <c r="C92" s="43" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D92" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="E92" s="43" t="inlineStr">
+        <is>
+          <t>Rapid Volley</t>
+        </is>
+      </c>
+      <c r="F92" s="56">
+        <f>F24</f>
+        <v/>
+      </c>
+      <c r="G92" s="57" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="H92" s="57" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I92" s="57" t="n"/>
+      <c r="J92" s="57" t="n"/>
+      <c r="K92" s="57" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L92" s="57" t="n"/>
+      <c r="M92" s="57" t="n"/>
+      <c r="N92" s="57" t="n"/>
+      <c r="O92" s="57" t="n"/>
+      <c r="P92" s="57" t="n"/>
+      <c r="Q92" s="57" t="n"/>
+      <c r="R92" s="57" t="n"/>
+      <c r="S92" s="57" t="n"/>
+      <c r="T92" s="57" t="n"/>
+      <c r="U92" s="57" t="n"/>
+      <c r="V92" s="57" t="n"/>
+      <c r="W92" s="57" t="n"/>
+      <c r="X92" s="57" t="n"/>
+      <c r="Y92" s="57" t="n"/>
+      <c r="Z92" s="57" t="n"/>
+      <c r="AA92" s="57" t="n"/>
+      <c r="AB92" s="57" t="n"/>
+      <c r="AC92" s="57" t="n"/>
+      <c r="AD92" s="57" t="n"/>
+      <c r="AE92" s="57" t="n"/>
+      <c r="AF92" s="57" t="n"/>
+      <c r="AG92" s="57" t="n"/>
+      <c r="AH92" s="57" t="n"/>
+      <c r="AI92" s="57" t="n"/>
+      <c r="BB92" s="81" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="BC92" s="81" t="inlineStr">
+        <is>
+          <t>Bursts 35% faster, half the kick, bigger mag</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="43" t="inlineStr">
+        <is>
+          <t>Big Game Hunter</t>
+        </is>
+      </c>
+      <c r="B93" s="43" t="inlineStr">
+        <is>
+          <t>Heavy</t>
+        </is>
+      </c>
+      <c r="C93" s="43" t="inlineStr">
+        <is>
+          <t>sustain</t>
+        </is>
+      </c>
+      <c r="D93" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="E93" s="43" t="inlineStr">
+        <is>
+          <t>Steady Sling</t>
+        </is>
+      </c>
+      <c r="F93" s="56">
+        <f>F28</f>
+        <v/>
+      </c>
+      <c r="G93" s="57" t="n"/>
+      <c r="H93" s="57" t="n"/>
+      <c r="I93" s="57" t="n"/>
+      <c r="J93" s="57" t="n"/>
+      <c r="K93" s="57" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L93" s="57" t="n"/>
+      <c r="M93" s="57" t="n"/>
+      <c r="N93" s="57" t="n"/>
+      <c r="O93" s="57" t="n"/>
+      <c r="P93" s="57" t="n"/>
+      <c r="Q93" s="57" t="n"/>
+      <c r="R93" s="57" t="n"/>
+      <c r="S93" s="57" t="n"/>
+      <c r="T93" s="57" t="n"/>
+      <c r="U93" s="57" t="n"/>
+      <c r="V93" s="57" t="n"/>
+      <c r="W93" s="57" t="n"/>
+      <c r="X93" s="57" t="n"/>
+      <c r="Y93" s="57" t="n"/>
+      <c r="Z93" s="57" t="n"/>
+      <c r="AA93" s="57" t="n"/>
+      <c r="AB93" s="57" t="n"/>
+      <c r="AC93" s="57" t="n"/>
+      <c r="AD93" s="57" t="n"/>
+      <c r="AE93" s="57" t="n"/>
+      <c r="AF93" s="57" t="n"/>
+      <c r="AG93" s="57" t="n"/>
+      <c r="AH93" s="57" t="n"/>
+      <c r="AI93" s="57" t="n"/>
+      <c r="BB93" s="81" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="BC93" s="81" t="inlineStr">
+        <is>
+          <t>35% less kick, moving or not</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="43" t="inlineStr">
+        <is>
+          <t>Big Game Hunter</t>
+        </is>
+      </c>
+      <c r="B94" s="43" t="inlineStr">
+        <is>
+          <t>Heavy</t>
+        </is>
+      </c>
+      <c r="C94" s="43" t="inlineStr">
+        <is>
+          <t>sustain</t>
+        </is>
+      </c>
+      <c r="D94" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="E94" s="43" t="inlineStr">
+        <is>
+          <t>Quick Belt</t>
+        </is>
+      </c>
+      <c r="F94" s="56">
+        <f>F28</f>
+        <v/>
+      </c>
+      <c r="G94" s="57" t="n"/>
+      <c r="H94" s="57" t="n"/>
+      <c r="I94" s="57" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J94" s="57" t="n"/>
+      <c r="K94" s="57" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L94" s="57" t="n"/>
+      <c r="M94" s="57" t="n"/>
+      <c r="N94" s="57" t="n"/>
+      <c r="O94" s="57" t="n"/>
+      <c r="P94" s="57" t="n"/>
+      <c r="Q94" s="57" t="n"/>
+      <c r="R94" s="57" t="n"/>
+      <c r="S94" s="57" t="n"/>
+      <c r="T94" s="57" t="n"/>
+      <c r="U94" s="57" t="n"/>
+      <c r="V94" s="57" t="n"/>
+      <c r="W94" s="57" t="n"/>
+      <c r="X94" s="57" t="n"/>
+      <c r="Y94" s="57" t="n"/>
+      <c r="Z94" s="57" t="n"/>
+      <c r="AA94" s="57" t="n"/>
+      <c r="AB94" s="57" t="n"/>
+      <c r="AC94" s="57" t="n"/>
+      <c r="AD94" s="57" t="n"/>
+      <c r="AE94" s="57" t="n"/>
+      <c r="AF94" s="57" t="n"/>
+      <c r="AG94" s="57" t="n"/>
+      <c r="AH94" s="57" t="n"/>
+      <c r="AI94" s="57" t="n"/>
+      <c r="BB94" s="81" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="BC94" s="81" t="inlineStr">
+        <is>
+          <t>Belt changes 30% faster; 20% less kick</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="43" t="inlineStr">
+        <is>
+          <t>Big Game Hunter</t>
+        </is>
+      </c>
+      <c r="B95" s="43" t="inlineStr">
+        <is>
+          <t>Heavy</t>
+        </is>
+      </c>
+      <c r="C95" s="43" t="inlineStr">
+        <is>
+          <t>sustain</t>
+        </is>
+      </c>
+      <c r="D95" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="E95" s="43" t="inlineStr">
+        <is>
+          <t>Hot Barrel</t>
+        </is>
+      </c>
+      <c r="F95" s="56">
+        <f>F29</f>
+        <v/>
+      </c>
+      <c r="G95" s="57" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H95" s="57" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="I95" s="57" t="n"/>
+      <c r="J95" s="57" t="n"/>
+      <c r="K95" s="57" t="n"/>
+      <c r="L95" s="57" t="n"/>
+      <c r="M95" s="57" t="n"/>
+      <c r="N95" s="57" t="n"/>
+      <c r="O95" s="57" t="n"/>
+      <c r="P95" s="57" t="n"/>
+      <c r="Q95" s="57" t="n"/>
+      <c r="R95" s="57" t="n"/>
+      <c r="S95" s="57" t="n"/>
+      <c r="T95" s="57" t="n"/>
+      <c r="U95" s="57" t="n"/>
+      <c r="V95" s="57" t="n"/>
+      <c r="W95" s="57" t="n"/>
+      <c r="X95" s="57" t="n"/>
+      <c r="Y95" s="57" t="n"/>
+      <c r="Z95" s="57" t="n"/>
+      <c r="AA95" s="57" t="n"/>
+      <c r="AB95" s="57" t="n"/>
+      <c r="AC95" s="57" t="n"/>
+      <c r="AD95" s="57" t="n"/>
+      <c r="AE95" s="57" t="n"/>
+      <c r="AF95" s="57" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="AG95" s="57" t="n"/>
+      <c r="AH95" s="57" t="n"/>
+      <c r="AI95" s="57" t="n"/>
+      <c r="BB95" s="81" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="BC95" s="81" t="inlineStr">
+        <is>
+          <t>50% faster at once, spins up to +60% more</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="43" t="inlineStr">
+        <is>
+          <t>Big Game Hunter</t>
+        </is>
+      </c>
+      <c r="B96" s="43" t="inlineStr">
+        <is>
+          <t>Heavy</t>
+        </is>
+      </c>
+      <c r="C96" s="43" t="inlineStr">
+        <is>
+          <t>sustain</t>
+        </is>
+      </c>
+      <c r="D96" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="E96" s="43" t="inlineStr">
+        <is>
+          <t>War Drum</t>
+        </is>
+      </c>
+      <c r="F96" s="56">
+        <f>F29</f>
+        <v/>
+      </c>
+      <c r="G96" s="57" t="n"/>
+      <c r="H96" s="57" t="n"/>
+      <c r="I96" s="57" t="n"/>
+      <c r="J96" s="57" t="n"/>
+      <c r="K96" s="57" t="n"/>
+      <c r="L96" s="57" t="n"/>
+      <c r="M96" s="57" t="n"/>
+      <c r="N96" s="57" t="n"/>
+      <c r="O96" s="57" t="n"/>
+      <c r="P96" s="57" t="n"/>
+      <c r="Q96" s="57" t="n"/>
+      <c r="R96" s="57" t="n"/>
+      <c r="S96" s="57" t="n"/>
+      <c r="T96" s="57" t="n"/>
+      <c r="U96" s="57" t="n"/>
+      <c r="V96" s="57" t="n"/>
+      <c r="W96" s="57" t="n"/>
+      <c r="X96" s="57" t="n"/>
+      <c r="Y96" s="57" t="n"/>
+      <c r="Z96" s="57" t="n"/>
+      <c r="AA96" s="57" t="n"/>
+      <c r="AB96" s="57" t="n"/>
+      <c r="AC96" s="57" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AD96" s="57" t="n"/>
+      <c r="AE96" s="57" t="n"/>
+      <c r="AF96" s="57" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="AG96" s="57" t="n"/>
+      <c r="AH96" s="57" t="n"/>
+      <c r="AI96" s="57" t="n"/>
+      <c r="BB96" s="81" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="BC96" s="81" t="inlineStr">
+        <is>
+          <t>Rally Cry twice as often; spins up to +130%</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="43" t="inlineStr">
+        <is>
+          <t>Big Game Hunter</t>
+        </is>
+      </c>
+      <c r="B97" s="43" t="inlineStr">
+        <is>
+          <t>Special Ammo</t>
+        </is>
+      </c>
+      <c r="C97" s="43" t="inlineStr">
+        <is>
+          <t>rounds</t>
+        </is>
+      </c>
+      <c r="D97" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="E97" s="43" t="inlineStr">
+        <is>
+          <t>Phosphor Rounds</t>
+        </is>
+      </c>
+      <c r="F97" s="56">
+        <f>F33</f>
+        <v/>
+      </c>
+      <c r="G97" s="57" t="n"/>
+      <c r="H97" s="57" t="n"/>
+      <c r="I97" s="57" t="n"/>
+      <c r="J97" s="57" t="n"/>
+      <c r="K97" s="57" t="n"/>
+      <c r="L97" s="57" t="n"/>
+      <c r="M97" s="57" t="n"/>
+      <c r="N97" s="57" t="n"/>
+      <c r="O97" s="57" t="n"/>
+      <c r="P97" s="57" t="n"/>
+      <c r="Q97" s="57" t="n"/>
+      <c r="R97" s="57" t="n"/>
+      <c r="S97" s="57" t="n"/>
+      <c r="T97" s="57" t="n"/>
+      <c r="U97" s="57" t="n"/>
+      <c r="V97" s="57" t="n"/>
+      <c r="W97" s="57" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="X97" s="57" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y97" s="57" t="n"/>
+      <c r="Z97" s="57" t="n"/>
+      <c r="AA97" s="57" t="n"/>
+      <c r="AB97" s="57" t="n"/>
+      <c r="AC97" s="57" t="n"/>
+      <c r="AD97" s="57" t="n"/>
+      <c r="AE97" s="57" t="n"/>
+      <c r="AF97" s="57" t="n"/>
+      <c r="AG97" s="57" t="n"/>
+      <c r="AH97" s="57" t="n"/>
+      <c r="AI97" s="57" t="n"/>
+      <c r="BB97" s="81" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="BC97" s="81" t="inlineStr">
+        <is>
+          <t>Fires burn 10% hotter and 50% longer</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="43" t="inlineStr">
+        <is>
+          <t>Big Game Hunter</t>
+        </is>
+      </c>
+      <c r="B98" s="43" t="inlineStr">
+        <is>
+          <t>Special Ammo</t>
+        </is>
+      </c>
+      <c r="C98" s="43" t="inlineStr">
+        <is>
+          <t>rounds</t>
+        </is>
+      </c>
+      <c r="D98" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="E98" s="43" t="inlineStr">
+        <is>
+          <t>Bright Tracers</t>
+        </is>
+      </c>
+      <c r="F98" s="56">
+        <f>F33</f>
+        <v/>
+      </c>
+      <c r="G98" s="57" t="n"/>
+      <c r="H98" s="57" t="n"/>
+      <c r="I98" s="57" t="n"/>
+      <c r="J98" s="57" t="n"/>
+      <c r="K98" s="57" t="n"/>
+      <c r="L98" s="57" t="n"/>
+      <c r="M98" s="57" t="n"/>
+      <c r="N98" s="57" t="n"/>
+      <c r="O98" s="57" t="n"/>
+      <c r="P98" s="57" t="n"/>
+      <c r="Q98" s="57" t="n"/>
+      <c r="R98" s="57" t="n"/>
+      <c r="S98" s="57" t="n"/>
+      <c r="T98" s="57" t="n"/>
+      <c r="U98" s="57" t="n"/>
+      <c r="V98" s="57" t="n"/>
+      <c r="W98" s="57" t="n"/>
+      <c r="X98" s="57" t="n"/>
+      <c r="Y98" s="57" t="n"/>
+      <c r="Z98" s="57" t="n"/>
+      <c r="AA98" s="57" t="n">
+        <v>30</v>
+      </c>
+      <c r="AB98" s="57" t="n"/>
+      <c r="AC98" s="57" t="n"/>
+      <c r="AD98" s="57" t="n"/>
+      <c r="AE98" s="57" t="n"/>
+      <c r="AF98" s="57" t="n"/>
+      <c r="AG98" s="57" t="n"/>
+      <c r="AH98" s="57" t="n"/>
+      <c r="AI98" s="57" t="n"/>
+      <c r="BB98" s="81" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="BC98" s="81" t="inlineStr">
+        <is>
+          <t>Hits mark dinos: +30% from everything</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="43" t="inlineStr">
+        <is>
+          <t>Big Game Hunter</t>
+        </is>
+      </c>
+      <c r="B99" s="43" t="inlineStr">
+        <is>
+          <t>Special Ammo</t>
+        </is>
+      </c>
+      <c r="C99" s="43" t="inlineStr">
+        <is>
+          <t>rounds</t>
+        </is>
+      </c>
+      <c r="D99" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="E99" s="43" t="inlineStr">
+        <is>
+          <t>Fire Tips</t>
+        </is>
+      </c>
+      <c r="F99" s="56">
+        <f>F34</f>
+        <v/>
+      </c>
+      <c r="G99" s="57" t="n"/>
+      <c r="H99" s="57" t="n"/>
+      <c r="I99" s="57" t="n"/>
+      <c r="J99" s="57" t="n"/>
+      <c r="K99" s="57" t="n"/>
+      <c r="L99" s="57" t="n"/>
+      <c r="M99" s="57" t="n"/>
+      <c r="N99" s="57" t="n"/>
+      <c r="O99" s="57" t="n"/>
+      <c r="P99" s="57" t="n"/>
+      <c r="Q99" s="57" t="n"/>
+      <c r="R99" s="57" t="n"/>
+      <c r="S99" s="57" t="n"/>
+      <c r="T99" s="57" t="n"/>
+      <c r="U99" s="57" t="n"/>
+      <c r="V99" s="57" t="n"/>
+      <c r="W99" s="57" t="n"/>
+      <c r="X99" s="57" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="Y99" s="57" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z99" s="57" t="n"/>
+      <c r="AA99" s="57" t="n"/>
+      <c r="AB99" s="57" t="n"/>
+      <c r="AC99" s="57" t="n"/>
+      <c r="AD99" s="57" t="n"/>
+      <c r="AE99" s="57" t="n"/>
+      <c r="AF99" s="57" t="n"/>
+      <c r="AG99" s="57" t="n"/>
+      <c r="AH99" s="57" t="n"/>
+      <c r="AI99" s="57" t="n"/>
+      <c r="BB99" s="81" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="BC99" s="81" t="inlineStr">
+        <is>
+          <t>Small blasts; dinos burn 25% longer</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="43" t="inlineStr">
+        <is>
+          <t>Big Game Hunter</t>
+        </is>
+      </c>
+      <c r="B100" s="43" t="inlineStr">
+        <is>
+          <t>Special Ammo</t>
+        </is>
+      </c>
+      <c r="C100" s="43" t="inlineStr">
+        <is>
+          <t>rounds</t>
+        </is>
+      </c>
+      <c r="D100" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="E100" s="43" t="inlineStr">
+        <is>
+          <t>Flat Tips</t>
+        </is>
+      </c>
+      <c r="F100" s="56">
+        <f>F34</f>
+        <v/>
+      </c>
+      <c r="G100" s="57" t="n"/>
+      <c r="H100" s="57" t="n"/>
+      <c r="I100" s="57" t="n"/>
+      <c r="J100" s="57" t="n"/>
+      <c r="K100" s="57" t="n"/>
+      <c r="L100" s="57" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="M100" s="57" t="n"/>
+      <c r="N100" s="57" t="n"/>
+      <c r="O100" s="57" t="n"/>
+      <c r="P100" s="57" t="n"/>
+      <c r="Q100" s="57" t="n"/>
+      <c r="R100" s="57" t="n"/>
+      <c r="S100" s="57" t="n"/>
+      <c r="T100" s="57" t="n"/>
+      <c r="U100" s="57" t="n"/>
+      <c r="V100" s="57" t="n"/>
+      <c r="W100" s="57" t="n"/>
+      <c r="X100" s="57" t="n"/>
+      <c r="Y100" s="57" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z100" s="57" t="n"/>
+      <c r="AA100" s="57" t="n"/>
+      <c r="AB100" s="57" t="n"/>
+      <c r="AC100" s="57" t="n"/>
+      <c r="AD100" s="57" t="n"/>
+      <c r="AE100" s="57" t="n"/>
+      <c r="AF100" s="57" t="n"/>
+      <c r="AG100" s="57" t="n"/>
+      <c r="AH100" s="57" t="n"/>
+      <c r="AI100" s="57" t="n"/>
+      <c r="BB100" s="81" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="BC100" s="81" t="inlineStr">
+        <is>
+          <t>Small blasts; rounds fly 25% further</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9f T122a: Brush Beater B/C options
12 Brush Beater options appended to Hero Upgrades exactly as PLAN 9f (no Damage x).
Bars on the #298 gun metric: every slot within 0.8-1.25x; T6 builds per path x1.13
(Slug) / x1.10 (Buckshot) / x1.14 (Point Blank). Specs: Twin Slug 2 slugs x pierce 4 per
pump (rounds per pump as Double Barrel), Slam Fire auto with 2 blasts and Quad Barrel 4
after it, Bird Shot hits air, Hot Shells burn, Flame Choke ignite. HEROES.md: option table,
Wildfire Drum rewording (#300).

Statically checked and headless-tested; not playtested.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Storm-Split-Balance.xlsx
+++ b/Storm-Split-Balance.xlsx
@@ -37632,7 +37632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CA100"/>
+  <dimension ref="A1:CA112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" style="90" min="1" max="1"/>
@@ -44655,6 +44655,878 @@
       <c r="BC100" s="81" t="inlineStr">
         <is>
           <t>Small blasts; rounds fly 25% further</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="43" t="inlineStr">
+        <is>
+          <t>Brush Beater</t>
+        </is>
+      </c>
+      <c r="B101" s="43" t="inlineStr">
+        <is>
+          <t>Slug</t>
+        </is>
+      </c>
+      <c r="C101" s="43" t="inlineStr">
+        <is>
+          <t>reach</t>
+        </is>
+      </c>
+      <c r="D101" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="E101" s="43" t="inlineStr">
+        <is>
+          <t>Quick Pump</t>
+        </is>
+      </c>
+      <c r="F101" s="56">
+        <f>F38</f>
+        <v/>
+      </c>
+      <c r="G101" s="57" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="H101" s="57" t="n"/>
+      <c r="I101" s="57" t="n"/>
+      <c r="J101" s="57" t="n"/>
+      <c r="K101" s="57" t="n"/>
+      <c r="L101" s="57" t="n"/>
+      <c r="M101" s="57" t="n"/>
+      <c r="N101" s="57" t="n"/>
+      <c r="O101" s="57" t="n"/>
+      <c r="P101" s="57" t="n"/>
+      <c r="Q101" s="57" t="n"/>
+      <c r="R101" s="57" t="n"/>
+      <c r="S101" s="57" t="n"/>
+      <c r="T101" s="57" t="n"/>
+      <c r="U101" s="57" t="n"/>
+      <c r="V101" s="57" t="n"/>
+      <c r="W101" s="57" t="n"/>
+      <c r="X101" s="57" t="n"/>
+      <c r="Y101" s="57" t="n"/>
+      <c r="Z101" s="57" t="n"/>
+      <c r="AA101" s="57" t="n"/>
+      <c r="AB101" s="57" t="n"/>
+      <c r="AC101" s="57" t="n"/>
+      <c r="AD101" s="57" t="n"/>
+      <c r="AE101" s="57" t="n"/>
+      <c r="AF101" s="57" t="n"/>
+      <c r="AG101" s="57" t="n"/>
+      <c r="AH101" s="57" t="n"/>
+      <c r="AI101" s="57" t="n"/>
+      <c r="BB101" s="81" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="BC101" s="81" t="inlineStr">
+        <is>
+          <t>Pump 25% faster</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="43" t="inlineStr">
+        <is>
+          <t>Brush Beater</t>
+        </is>
+      </c>
+      <c r="B102" s="43" t="inlineStr">
+        <is>
+          <t>Slug</t>
+        </is>
+      </c>
+      <c r="C102" s="43" t="inlineStr">
+        <is>
+          <t>reach</t>
+        </is>
+      </c>
+      <c r="D102" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="E102" s="43" t="inlineStr">
+        <is>
+          <t>Side Saddle</t>
+        </is>
+      </c>
+      <c r="F102" s="56">
+        <f>F38</f>
+        <v/>
+      </c>
+      <c r="G102" s="57" t="n"/>
+      <c r="H102" s="57" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I102" s="57" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J102" s="57" t="n"/>
+      <c r="K102" s="57" t="n"/>
+      <c r="L102" s="57" t="n"/>
+      <c r="M102" s="57" t="n"/>
+      <c r="N102" s="57" t="n"/>
+      <c r="O102" s="57" t="n"/>
+      <c r="P102" s="57" t="n"/>
+      <c r="Q102" s="57" t="n"/>
+      <c r="R102" s="57" t="n"/>
+      <c r="S102" s="57" t="n"/>
+      <c r="T102" s="57" t="n"/>
+      <c r="U102" s="57" t="n"/>
+      <c r="V102" s="57" t="n"/>
+      <c r="W102" s="57" t="n"/>
+      <c r="X102" s="57" t="n"/>
+      <c r="Y102" s="57" t="n"/>
+      <c r="Z102" s="57" t="n"/>
+      <c r="AA102" s="57" t="n"/>
+      <c r="AB102" s="57" t="n"/>
+      <c r="AC102" s="57" t="n"/>
+      <c r="AD102" s="57" t="n"/>
+      <c r="AE102" s="57" t="n"/>
+      <c r="AF102" s="57" t="n"/>
+      <c r="AG102" s="57" t="n"/>
+      <c r="AH102" s="57" t="n"/>
+      <c r="AI102" s="57" t="n"/>
+      <c r="BB102" s="81" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="BC102" s="81" t="inlineStr">
+        <is>
+          <t>Holds 50% more slugs, loads 20% faster</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="43" t="inlineStr">
+        <is>
+          <t>Brush Beater</t>
+        </is>
+      </c>
+      <c r="B103" s="43" t="inlineStr">
+        <is>
+          <t>Slug</t>
+        </is>
+      </c>
+      <c r="C103" s="43" t="inlineStr">
+        <is>
+          <t>reach</t>
+        </is>
+      </c>
+      <c r="D103" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="E103" s="43" t="inlineStr">
+        <is>
+          <t>Express Slug</t>
+        </is>
+      </c>
+      <c r="F103" s="56">
+        <f>F39</f>
+        <v/>
+      </c>
+      <c r="G103" s="57" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="H103" s="57" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I103" s="57" t="n"/>
+      <c r="J103" s="57" t="n"/>
+      <c r="K103" s="57" t="n"/>
+      <c r="L103" s="57" t="n"/>
+      <c r="M103" s="57" t="n"/>
+      <c r="N103" s="57" t="n"/>
+      <c r="O103" s="57" t="n"/>
+      <c r="P103" s="57" t="n"/>
+      <c r="Q103" s="57" t="n"/>
+      <c r="R103" s="57" t="n"/>
+      <c r="S103" s="57" t="n">
+        <v>6</v>
+      </c>
+      <c r="T103" s="57" t="n"/>
+      <c r="U103" s="57" t="n"/>
+      <c r="V103" s="57" t="n"/>
+      <c r="W103" s="57" t="n"/>
+      <c r="X103" s="57" t="n"/>
+      <c r="Y103" s="57" t="n"/>
+      <c r="Z103" s="57" t="n"/>
+      <c r="AA103" s="57" t="n"/>
+      <c r="AB103" s="57" t="n"/>
+      <c r="AC103" s="57" t="n"/>
+      <c r="AD103" s="57" t="n"/>
+      <c r="AE103" s="57" t="n"/>
+      <c r="AF103" s="57" t="n"/>
+      <c r="AG103" s="57" t="n"/>
+      <c r="AH103" s="57" t="n"/>
+      <c r="AI103" s="57" t="n"/>
+      <c r="BB103" s="81" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="BC103" s="81" t="inlineStr">
+        <is>
+          <t>Slugs through 6, 60% faster, bigger tube</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="43" t="inlineStr">
+        <is>
+          <t>Brush Beater</t>
+        </is>
+      </c>
+      <c r="B104" s="43" t="inlineStr">
+        <is>
+          <t>Slug</t>
+        </is>
+      </c>
+      <c r="C104" s="43" t="inlineStr">
+        <is>
+          <t>reach</t>
+        </is>
+      </c>
+      <c r="D104" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="E104" s="43" t="inlineStr">
+        <is>
+          <t>Twin Slug</t>
+        </is>
+      </c>
+      <c r="F104" s="56">
+        <f>F39</f>
+        <v/>
+      </c>
+      <c r="G104" s="57" t="n"/>
+      <c r="H104" s="57" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I104" s="57" t="n"/>
+      <c r="J104" s="57" t="n"/>
+      <c r="K104" s="57" t="n"/>
+      <c r="L104" s="57" t="n"/>
+      <c r="M104" s="57" t="n"/>
+      <c r="N104" s="57" t="n"/>
+      <c r="O104" s="57" t="n"/>
+      <c r="P104" s="57" t="n"/>
+      <c r="Q104" s="57" t="n"/>
+      <c r="R104" s="57" t="n">
+        <v>2</v>
+      </c>
+      <c r="S104" s="57" t="n">
+        <v>4</v>
+      </c>
+      <c r="T104" s="57" t="n"/>
+      <c r="U104" s="57" t="n"/>
+      <c r="V104" s="57" t="n"/>
+      <c r="W104" s="57" t="n"/>
+      <c r="X104" s="57" t="n"/>
+      <c r="Y104" s="57" t="n"/>
+      <c r="Z104" s="57" t="n"/>
+      <c r="AA104" s="57" t="n"/>
+      <c r="AB104" s="57" t="n"/>
+      <c r="AC104" s="57" t="n"/>
+      <c r="AD104" s="57" t="n"/>
+      <c r="AE104" s="57" t="n"/>
+      <c r="AF104" s="57" t="n"/>
+      <c r="AG104" s="57" t="n"/>
+      <c r="AH104" s="57" t="n"/>
+      <c r="AI104" s="57" t="n"/>
+      <c r="BB104" s="81" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="BC104" s="81" t="inlineStr">
+        <is>
+          <t>Two slugs per pump, each through 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="43" t="inlineStr">
+        <is>
+          <t>Brush Beater</t>
+        </is>
+      </c>
+      <c r="B105" s="43" t="inlineStr">
+        <is>
+          <t>Buckshot</t>
+        </is>
+      </c>
+      <c r="C105" s="43" t="inlineStr">
+        <is>
+          <t>crowds</t>
+        </is>
+      </c>
+      <c r="D105" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="E105" s="43" t="inlineStr">
+        <is>
+          <t>Hot Shells</t>
+        </is>
+      </c>
+      <c r="F105" s="56">
+        <f>F43</f>
+        <v/>
+      </c>
+      <c r="G105" s="57" t="n"/>
+      <c r="H105" s="57" t="n"/>
+      <c r="I105" s="57" t="n"/>
+      <c r="J105" s="57" t="n"/>
+      <c r="K105" s="57" t="n"/>
+      <c r="L105" s="57" t="n"/>
+      <c r="M105" s="57" t="n"/>
+      <c r="N105" s="57" t="n"/>
+      <c r="O105" s="57" t="n"/>
+      <c r="P105" s="57" t="n"/>
+      <c r="Q105" s="57" t="n"/>
+      <c r="R105" s="57" t="n"/>
+      <c r="S105" s="57" t="n"/>
+      <c r="T105" s="57" t="n"/>
+      <c r="U105" s="57" t="n"/>
+      <c r="V105" s="57" t="n"/>
+      <c r="W105" s="57" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="X105" s="57" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y105" s="57" t="n"/>
+      <c r="Z105" s="57" t="n"/>
+      <c r="AA105" s="57" t="n"/>
+      <c r="AB105" s="57" t="n"/>
+      <c r="AC105" s="57" t="n"/>
+      <c r="AD105" s="57" t="n"/>
+      <c r="AE105" s="57" t="n"/>
+      <c r="AF105" s="57" t="n"/>
+      <c r="AG105" s="57" t="n"/>
+      <c r="AH105" s="57" t="n"/>
+      <c r="AI105" s="57" t="n"/>
+      <c r="BB105" s="81" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="BC105" s="81" t="inlineStr">
+        <is>
+          <t>Fires burn more than twice as hot</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="43" t="inlineStr">
+        <is>
+          <t>Brush Beater</t>
+        </is>
+      </c>
+      <c r="B106" s="43" t="inlineStr">
+        <is>
+          <t>Buckshot</t>
+        </is>
+      </c>
+      <c r="C106" s="43" t="inlineStr">
+        <is>
+          <t>crowds</t>
+        </is>
+      </c>
+      <c r="D106" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="E106" s="43" t="inlineStr">
+        <is>
+          <t>Shell Belt</t>
+        </is>
+      </c>
+      <c r="F106" s="56">
+        <f>F43</f>
+        <v/>
+      </c>
+      <c r="G106" s="57" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H106" s="57" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I106" s="57" t="n"/>
+      <c r="J106" s="57" t="n"/>
+      <c r="K106" s="57" t="n"/>
+      <c r="L106" s="57" t="n"/>
+      <c r="M106" s="57" t="n"/>
+      <c r="N106" s="57" t="n"/>
+      <c r="O106" s="57" t="n"/>
+      <c r="P106" s="57" t="n"/>
+      <c r="Q106" s="57" t="n"/>
+      <c r="R106" s="57" t="n"/>
+      <c r="S106" s="57" t="n"/>
+      <c r="T106" s="57" t="n"/>
+      <c r="U106" s="57" t="n"/>
+      <c r="V106" s="57" t="n"/>
+      <c r="W106" s="57" t="n"/>
+      <c r="X106" s="57" t="n"/>
+      <c r="Y106" s="57" t="n"/>
+      <c r="Z106" s="57" t="n"/>
+      <c r="AA106" s="57" t="n"/>
+      <c r="AB106" s="57" t="n"/>
+      <c r="AC106" s="57" t="n"/>
+      <c r="AD106" s="57" t="n"/>
+      <c r="AE106" s="57" t="n"/>
+      <c r="AF106" s="57" t="n"/>
+      <c r="AG106" s="57" t="n"/>
+      <c r="AH106" s="57" t="n"/>
+      <c r="AI106" s="57" t="n"/>
+      <c r="BB106" s="81" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="BC106" s="81" t="inlineStr">
+        <is>
+          <t>Pump 50% faster; holds 50% more</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="43" t="inlineStr">
+        <is>
+          <t>Brush Beater</t>
+        </is>
+      </c>
+      <c r="B107" s="43" t="inlineStr">
+        <is>
+          <t>Buckshot</t>
+        </is>
+      </c>
+      <c r="C107" s="43" t="inlineStr">
+        <is>
+          <t>crowds</t>
+        </is>
+      </c>
+      <c r="D107" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="E107" s="43" t="inlineStr">
+        <is>
+          <t>Flame Choke</t>
+        </is>
+      </c>
+      <c r="F107" s="56">
+        <f>F44</f>
+        <v/>
+      </c>
+      <c r="G107" s="57" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H107" s="57" t="n"/>
+      <c r="I107" s="57" t="n"/>
+      <c r="J107" s="57" t="n"/>
+      <c r="K107" s="57" t="n"/>
+      <c r="L107" s="57" t="n"/>
+      <c r="M107" s="57" t="n"/>
+      <c r="N107" s="57" t="n"/>
+      <c r="O107" s="57" t="n"/>
+      <c r="P107" s="57" t="n"/>
+      <c r="Q107" s="57" t="n"/>
+      <c r="R107" s="57" t="n"/>
+      <c r="S107" s="57" t="n"/>
+      <c r="T107" s="57" t="n"/>
+      <c r="U107" s="57" t="n"/>
+      <c r="V107" s="57" t="n"/>
+      <c r="W107" s="57" t="n"/>
+      <c r="X107" s="57" t="n"/>
+      <c r="Y107" s="57" t="n"/>
+      <c r="Z107" s="57" t="n"/>
+      <c r="AA107" s="57" t="n"/>
+      <c r="AB107" s="57" t="n"/>
+      <c r="AC107" s="57" t="n"/>
+      <c r="AD107" s="57" t="n"/>
+      <c r="AE107" s="57" t="n"/>
+      <c r="AF107" s="57" t="n"/>
+      <c r="AG107" s="57" t="n"/>
+      <c r="AH107" s="57" t="n"/>
+      <c r="AI107" s="57" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="BB107" s="81" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="BC107" s="81" t="inlineStr">
+        <is>
+          <t>Dragon's Breath bursts for 70% of a shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="43" t="inlineStr">
+        <is>
+          <t>Brush Beater</t>
+        </is>
+      </c>
+      <c r="B108" s="43" t="inlineStr">
+        <is>
+          <t>Buckshot</t>
+        </is>
+      </c>
+      <c r="C108" s="43" t="inlineStr">
+        <is>
+          <t>crowds</t>
+        </is>
+      </c>
+      <c r="D108" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="E108" s="43" t="inlineStr">
+        <is>
+          <t>Pump Storm</t>
+        </is>
+      </c>
+      <c r="F108" s="56">
+        <f>F44</f>
+        <v/>
+      </c>
+      <c r="G108" s="57" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H108" s="57" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I108" s="57" t="n"/>
+      <c r="J108" s="57" t="n"/>
+      <c r="K108" s="57" t="n"/>
+      <c r="L108" s="57" t="n"/>
+      <c r="M108" s="57" t="n"/>
+      <c r="N108" s="57" t="n"/>
+      <c r="O108" s="57" t="n"/>
+      <c r="P108" s="57" t="n"/>
+      <c r="Q108" s="57" t="n"/>
+      <c r="R108" s="57" t="n"/>
+      <c r="S108" s="57" t="n"/>
+      <c r="T108" s="57" t="n"/>
+      <c r="U108" s="57" t="n"/>
+      <c r="V108" s="57" t="n"/>
+      <c r="W108" s="57" t="n"/>
+      <c r="X108" s="57" t="n"/>
+      <c r="Y108" s="57" t="n"/>
+      <c r="Z108" s="57" t="n"/>
+      <c r="AA108" s="57" t="n"/>
+      <c r="AB108" s="57" t="n"/>
+      <c r="AC108" s="57" t="n"/>
+      <c r="AD108" s="57" t="n"/>
+      <c r="AE108" s="57" t="n"/>
+      <c r="AF108" s="57" t="n"/>
+      <c r="AG108" s="57" t="n"/>
+      <c r="AH108" s="57" t="n"/>
+      <c r="AI108" s="57" t="n"/>
+      <c r="BB108" s="81" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="BC108" s="81" t="inlineStr">
+        <is>
+          <t>Pump 50% faster, bigger tube</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="43" t="inlineStr">
+        <is>
+          <t>Brush Beater</t>
+        </is>
+      </c>
+      <c r="B109" s="43" t="inlineStr">
+        <is>
+          <t>Point Blank</t>
+        </is>
+      </c>
+      <c r="C109" s="43" t="inlineStr">
+        <is>
+          <t>burst</t>
+        </is>
+      </c>
+      <c r="D109" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="E109" s="43" t="inlineStr">
+        <is>
+          <t>Quick Breech</t>
+        </is>
+      </c>
+      <c r="F109" s="56">
+        <f>F48</f>
+        <v/>
+      </c>
+      <c r="G109" s="57" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H109" s="57" t="n"/>
+      <c r="I109" s="57" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J109" s="57" t="n"/>
+      <c r="K109" s="57" t="n"/>
+      <c r="L109" s="57" t="n"/>
+      <c r="M109" s="57" t="n"/>
+      <c r="N109" s="57" t="n"/>
+      <c r="O109" s="57" t="n"/>
+      <c r="P109" s="57" t="n"/>
+      <c r="Q109" s="57" t="n"/>
+      <c r="R109" s="57" t="n"/>
+      <c r="S109" s="57" t="n"/>
+      <c r="T109" s="57" t="n"/>
+      <c r="U109" s="57" t="n"/>
+      <c r="V109" s="57" t="n"/>
+      <c r="W109" s="57" t="n"/>
+      <c r="X109" s="57" t="n"/>
+      <c r="Y109" s="57" t="n"/>
+      <c r="Z109" s="57" t="n"/>
+      <c r="AA109" s="57" t="n"/>
+      <c r="AB109" s="57" t="n"/>
+      <c r="AC109" s="57" t="n"/>
+      <c r="AD109" s="57" t="n"/>
+      <c r="AE109" s="57" t="n"/>
+      <c r="AF109" s="57" t="n"/>
+      <c r="AG109" s="57" t="n"/>
+      <c r="AH109" s="57" t="n"/>
+      <c r="AI109" s="57" t="n"/>
+      <c r="BB109" s="81" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="BC109" s="81" t="inlineStr">
+        <is>
+          <t>Reload 35% faster, fire 20% faster</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="43" t="inlineStr">
+        <is>
+          <t>Brush Beater</t>
+        </is>
+      </c>
+      <c r="B110" s="43" t="inlineStr">
+        <is>
+          <t>Point Blank</t>
+        </is>
+      </c>
+      <c r="C110" s="43" t="inlineStr">
+        <is>
+          <t>burst</t>
+        </is>
+      </c>
+      <c r="D110" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="E110" s="43" t="inlineStr">
+        <is>
+          <t>Bird Shot</t>
+        </is>
+      </c>
+      <c r="F110" s="56">
+        <f>F48</f>
+        <v/>
+      </c>
+      <c r="G110" s="57" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="H110" s="57" t="n"/>
+      <c r="I110" s="57" t="n"/>
+      <c r="J110" s="57" t="n"/>
+      <c r="K110" s="57" t="n"/>
+      <c r="L110" s="57" t="n"/>
+      <c r="M110" s="57" t="n"/>
+      <c r="N110" s="57" t="n"/>
+      <c r="O110" s="57" t="n"/>
+      <c r="P110" s="57" t="n"/>
+      <c r="Q110" s="57" t="n"/>
+      <c r="R110" s="57" t="n"/>
+      <c r="S110" s="57" t="n"/>
+      <c r="T110" s="57" t="n"/>
+      <c r="U110" s="57" t="n"/>
+      <c r="V110" s="57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W110" s="57" t="n"/>
+      <c r="X110" s="57" t="n"/>
+      <c r="Y110" s="57" t="n"/>
+      <c r="Z110" s="57" t="n"/>
+      <c r="AA110" s="57" t="n"/>
+      <c r="AB110" s="57" t="n"/>
+      <c r="AC110" s="57" t="n"/>
+      <c r="AD110" s="57" t="n"/>
+      <c r="AE110" s="57" t="n"/>
+      <c r="AF110" s="57" t="n"/>
+      <c r="AG110" s="57" t="n"/>
+      <c r="AH110" s="57" t="n"/>
+      <c r="AI110" s="57" t="n"/>
+      <c r="BB110" s="81" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="BC110" s="81" t="inlineStr">
+        <is>
+          <t>Blasts hit flying dinos; fire 15% faster</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="43" t="inlineStr">
+        <is>
+          <t>Brush Beater</t>
+        </is>
+      </c>
+      <c r="B111" s="43" t="inlineStr">
+        <is>
+          <t>Point Blank</t>
+        </is>
+      </c>
+      <c r="C111" s="43" t="inlineStr">
+        <is>
+          <t>burst</t>
+        </is>
+      </c>
+      <c r="D111" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="E111" s="43" t="inlineStr">
+        <is>
+          <t>Breech Loader</t>
+        </is>
+      </c>
+      <c r="F111" s="56">
+        <f>F49</f>
+        <v/>
+      </c>
+      <c r="G111" s="57" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="H111" s="57" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I111" s="57" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J111" s="57" t="n"/>
+      <c r="K111" s="57" t="n"/>
+      <c r="L111" s="57" t="n"/>
+      <c r="M111" s="57" t="n"/>
+      <c r="N111" s="57" t="n"/>
+      <c r="O111" s="57" t="n"/>
+      <c r="P111" s="57" t="n"/>
+      <c r="Q111" s="57" t="n"/>
+      <c r="R111" s="57" t="n"/>
+      <c r="S111" s="57" t="n"/>
+      <c r="T111" s="57" t="n"/>
+      <c r="U111" s="57" t="n"/>
+      <c r="V111" s="57" t="n"/>
+      <c r="W111" s="57" t="n"/>
+      <c r="X111" s="57" t="n"/>
+      <c r="Y111" s="57" t="n"/>
+      <c r="Z111" s="57" t="n"/>
+      <c r="AA111" s="57" t="n"/>
+      <c r="AB111" s="57" t="n"/>
+      <c r="AC111" s="57" t="n"/>
+      <c r="AD111" s="57" t="n"/>
+      <c r="AE111" s="57" t="n"/>
+      <c r="AF111" s="57" t="n"/>
+      <c r="AG111" s="57" t="n"/>
+      <c r="AH111" s="57" t="n"/>
+      <c r="AI111" s="57" t="n"/>
+      <c r="BB111" s="81" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="BC111" s="81" t="inlineStr">
+        <is>
+          <t>45% faster, bigger tube, quick reload</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="43" t="inlineStr">
+        <is>
+          <t>Brush Beater</t>
+        </is>
+      </c>
+      <c r="B112" s="43" t="inlineStr">
+        <is>
+          <t>Point Blank</t>
+        </is>
+      </c>
+      <c r="C112" s="43" t="inlineStr">
+        <is>
+          <t>burst</t>
+        </is>
+      </c>
+      <c r="D112" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="E112" s="43" t="inlineStr">
+        <is>
+          <t>Slam Fire</t>
+        </is>
+      </c>
+      <c r="F112" s="56">
+        <f>F49</f>
+        <v/>
+      </c>
+      <c r="G112" s="57" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H112" s="57" t="n"/>
+      <c r="I112" s="57" t="n"/>
+      <c r="J112" s="57" t="n"/>
+      <c r="K112" s="57" t="n"/>
+      <c r="L112" s="57" t="n"/>
+      <c r="M112" s="57" t="n"/>
+      <c r="N112" s="57" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="O112" s="57" t="n"/>
+      <c r="P112" s="57" t="n"/>
+      <c r="Q112" s="57" t="n"/>
+      <c r="R112" s="57" t="n"/>
+      <c r="S112" s="57" t="n"/>
+      <c r="T112" s="57" t="n"/>
+      <c r="U112" s="57" t="n"/>
+      <c r="V112" s="57" t="n"/>
+      <c r="W112" s="57" t="n"/>
+      <c r="X112" s="57" t="n"/>
+      <c r="Y112" s="57" t="n"/>
+      <c r="Z112" s="57" t="n"/>
+      <c r="AA112" s="57" t="n"/>
+      <c r="AB112" s="57" t="n"/>
+      <c r="AC112" s="57" t="n"/>
+      <c r="AD112" s="57" t="n"/>
+      <c r="AE112" s="57" t="n"/>
+      <c r="AF112" s="57" t="n"/>
+      <c r="AG112" s="57" t="n"/>
+      <c r="AH112" s="57" t="n"/>
+      <c r="AI112" s="57" t="n"/>
+      <c r="BB112" s="81" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="BC112" s="81" t="inlineStr">
+        <is>
+          <t>Hold to keep both barrels firing, 70% faster</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
9h T126c: Bone Totem fix + release (#331-#333)
Cells: Totem 800 -> 600 cash, Totem charge 8 -> 3, Spirit hunter damage 9 -> 8,
Bone cash 8/26/26, Bone Market 120, Bone Bonus 168. value.py prints the Roar T2
r11-20 c/e as a report (#332: Bone Pile T1-T2 payback is the round-20 bar).
ballista.spec exempts TOTEM/METEOR/VENT by key (#333). TOTEM released (450 Amber).
Measured: Roar c/e 377/693/290/153/174; Bone Pile payback 11/12/12; --breaks1
Ancient Roar S 203/391; --options, exporter clean. Not playtested.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Storm-Split-Balance.xlsx
+++ b/Storm-Split-Balance.xlsx
@@ -10178,7 +10178,6 @@
       </c>
       <c r="E38" s="17" t="n"/>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="31" t="inlineStr">
         <is>
@@ -10249,7 +10248,6 @@
         </is>
       </c>
     </row>
-    <row r="44"/>
     <row r="45">
       <c r="A45" s="31" t="inlineStr">
         <is>
@@ -10400,7 +10398,6 @@
         </is>
       </c>
     </row>
-    <row r="53"/>
     <row r="54">
       <c r="A54" s="31" t="inlineStr">
         <is>
@@ -10451,7 +10448,6 @@
         </is>
       </c>
     </row>
-    <row r="57"/>
     <row r="58">
       <c r="A58" s="31" t="inlineStr">
         <is>
@@ -10522,7 +10518,6 @@
         </is>
       </c>
     </row>
-    <row r="62"/>
     <row r="63">
       <c r="A63" s="31" t="inlineStr">
         <is>
@@ -10573,7 +10568,6 @@
         </is>
       </c>
     </row>
-    <row r="66"/>
     <row r="67">
       <c r="A67" s="31" t="inlineStr">
         <is>
@@ -10764,7 +10758,6 @@
         </is>
       </c>
     </row>
-    <row r="77"/>
     <row r="78">
       <c r="A78" s="31" t="inlineStr">
         <is>
@@ -10912,7 +10905,6 @@
         </is>
       </c>
     </row>
-    <row r="86"/>
     <row r="87">
       <c r="A87" s="31" t="inlineStr">
         <is>
@@ -11020,7 +11012,6 @@
         </is>
       </c>
     </row>
-    <row r="93"/>
     <row r="94" s="90">
       <c r="A94" s="31" t="inlineStr">
         <is>
@@ -11048,7 +11039,6 @@
         </is>
       </c>
     </row>
-    <row r="96"/>
     <row r="97">
       <c r="A97" s="31" t="inlineStr">
         <is>
@@ -11076,7 +11066,6 @@
         </is>
       </c>
     </row>
-    <row r="99"/>
     <row r="100">
       <c r="A100" s="99" t="inlineStr">
         <is>
@@ -11124,7 +11113,6 @@
         </is>
       </c>
     </row>
-    <row r="103"/>
     <row r="104">
       <c r="A104" s="99" t="inlineStr">
         <is>
@@ -11215,7 +11203,6 @@
         </is>
       </c>
     </row>
-    <row r="109"/>
     <row r="110">
       <c r="A110" s="99" t="inlineStr">
         <is>
@@ -11398,7 +11385,6 @@
         </is>
       </c>
     </row>
-    <row r="123"/>
     <row r="124">
       <c r="A124" s="99" t="inlineStr">
         <is>
@@ -11452,7 +11438,6 @@
         </is>
       </c>
     </row>
-    <row r="128"/>
     <row r="129">
       <c r="A129" s="99" t="inlineStr">
         <is>
@@ -11592,7 +11577,6 @@
         </is>
       </c>
     </row>
-    <row r="140"/>
     <row r="141">
       <c r="A141" s="99" t="inlineStr">
         <is>
@@ -12335,7 +12319,6 @@
         </is>
       </c>
     </row>
-    <row r="191"/>
     <row r="192">
       <c r="A192" s="81" t="inlineStr">
         <is>
@@ -12448,7 +12431,6 @@
         </is>
       </c>
     </row>
-    <row r="200"/>
     <row r="201">
       <c r="A201" s="81" t="inlineStr">
         <is>
@@ -12853,7 +12835,6 @@
         </is>
       </c>
     </row>
-    <row r="229"/>
     <row r="230">
       <c r="A230" s="81" t="inlineStr">
         <is>
@@ -12868,7 +12849,7 @@
         </is>
       </c>
       <c r="B231" s="81" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C231" s="81" t="inlineStr">
         <is>
@@ -12958,7 +12939,7 @@
         </is>
       </c>
       <c r="B237" s="81" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C237" s="81" t="inlineStr">
         <is>
@@ -14204,7 +14185,7 @@
         </is>
       </c>
       <c r="C21" s="81" t="n">
-        <v>800</v>
+        <v>600</v>
       </c>
       <c r="D21" s="81" t="n">
         <v>60</v>
@@ -42322,7 +42303,7 @@
       </c>
       <c r="DV366" s="81" t="n"/>
       <c r="EX366" s="81" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="367">
@@ -42381,7 +42362,7 @@
       <c r="AF367" s="81" t="n"/>
       <c r="DV367" s="81" t="n"/>
       <c r="EX367" s="81" t="n">
-        <v>14</v>
+        <v>26</v>
       </c>
     </row>
     <row r="368">
@@ -42442,10 +42423,10 @@
       <c r="DN368" s="81" t="n"/>
       <c r="DV368" s="81" t="n"/>
       <c r="ER368" s="81" t="n">
-        <v>400</v>
+        <v>120</v>
       </c>
       <c r="EX368" s="81" t="n">
-        <v>14</v>
+        <v>26</v>
       </c>
     </row>
     <row r="369">
@@ -43183,7 +43164,7 @@
       </c>
       <c r="DP380" s="81" t="n"/>
       <c r="ER380" s="81" t="n">
-        <v>560</v>
+        <v>168</v>
       </c>
     </row>
     <row r="381">

</xml_diff>

<commit_message>
9h T125c: Treetop Pass, Belt Gun known, Blimp round-20 bar (#341-#343)
Door Gun T3 "Strafing Run" -> "Treetop Pass" (sheet M385, UPGRADES.md,
blimp.spec; Config diff = that one name); Falcon Roost Flock T5C keeps
"Strafing Run". value.py: KNOWN_DEAD tags accepted DEAD tiers with their
decision (Belt Gun #342, plus #165/#194/#332); the Blimp's Door Gun T2
r11-20 c/e is printed, not gated (586 vs 386, #343: Cargo payback
8.6/10/8.9 is the round-20 bar). No number changes. audit --strict 0;
test.sh 807 green; value/--breaks1/--options/threat exit 0. Not playtested.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Storm-Split-Balance.xlsx
+++ b/Storm-Split-Balance.xlsx
@@ -13023,112 +13023,112 @@
       </c>
     </row>
     <row r="244">
-      <c r="A244" t="inlineStr">
+      <c r="A244" s="81" t="inlineStr">
         <is>
           <t>SPOTTER BLIMP</t>
         </is>
       </c>
     </row>
     <row r="245">
-      <c r="A245" t="inlineStr">
+      <c r="A245" s="81" t="inlineStr">
         <is>
           <t>Blimp speed (studs/s)</t>
         </is>
       </c>
-      <c r="B245" t="n">
+      <c r="B245" s="81" t="n">
         <v>40</v>
       </c>
-      <c r="C245" t="inlineStr">
+      <c r="C245" s="81" t="inlineStr">
         <is>
           <t>the blimp's flying speed along its side's track (x Blimp speed x); a lap = spawn end to exit end and back (Shared/Blimp)</t>
         </is>
       </c>
     </row>
     <row r="246">
-      <c r="A246" t="inlineStr">
+      <c r="A246" s="81" t="inlineStr">
         <is>
           <t>Paratrooper HP</t>
         </is>
       </c>
-      <c r="B246" t="n">
+      <c r="B246" s="81" t="n">
         <v>80</v>
       </c>
-      <c r="C246" t="inlineStr">
+      <c r="C246" s="81" t="inlineStr">
         <is>
           <t>a Paratroopers ranger's HP (the 9g walker, fight mode)</t>
         </is>
       </c>
     </row>
     <row r="247">
-      <c r="A247" t="inlineStr">
+      <c r="A247" s="81" t="inlineStr">
         <is>
           <t>Paratrooper damage</t>
         </is>
       </c>
-      <c r="B247" t="n">
+      <c r="B247" s="81" t="n">
         <v>40</v>
       </c>
-      <c r="C247" t="inlineStr">
+      <c r="C247" s="81" t="inlineStr">
         <is>
           <t>a paratrooper's shot (x the team's level)</t>
         </is>
       </c>
     </row>
     <row r="248">
-      <c r="A248" t="inlineStr">
+      <c r="A248" s="81" t="inlineStr">
         <is>
           <t>Paratrooper rate</t>
         </is>
       </c>
-      <c r="B248" t="n">
+      <c r="B248" s="81" t="n">
         <v>1.5</v>
       </c>
-      <c r="C248" t="inlineStr">
+      <c r="C248" s="81" t="inlineStr">
         <is>
           <t>shots a second per paratrooper</t>
         </is>
       </c>
     </row>
     <row r="249">
-      <c r="A249" t="inlineStr">
+      <c r="A249" s="81" t="inlineStr">
         <is>
           <t>Paratrooper reach</t>
         </is>
       </c>
-      <c r="B249" t="n">
+      <c r="B249" s="81" t="n">
         <v>14</v>
       </c>
-      <c r="C249" t="inlineStr">
+      <c r="C249" s="81" t="inlineStr">
         <is>
           <t>studs: paratroopers hunt dinos within this of where they land</t>
         </is>
       </c>
     </row>
     <row r="250">
-      <c r="A250" t="inlineStr">
+      <c r="A250" s="81" t="inlineStr">
         <is>
           <t>Paratrooper speed</t>
         </is>
       </c>
-      <c r="B250" t="n">
+      <c r="B250" s="81" t="n">
         <v>14</v>
       </c>
-      <c r="C250" t="inlineStr">
+      <c r="C250" s="81" t="inlineStr">
         <is>
           <t>studs/s a paratrooper walks</t>
         </is>
       </c>
     </row>
     <row r="251">
-      <c r="A251" t="inlineStr">
+      <c r="A251" s="81" t="inlineStr">
         <is>
           <t>Hook max sizes</t>
         </is>
       </c>
-      <c r="B251" t="n">
+      <c r="B251" s="81" t="n">
         <v>2</v>
       </c>
-      <c r="C251" t="inlineStr">
+      <c r="C251" s="81" t="inlineStr">
         <is>
           <t>Sky Hook takes only a non-boss dino with at most this many sizes left</t>
         </is>
@@ -14354,72 +14354,72 @@
       <c r="Z21" s="81" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="81" t="inlineStr">
         <is>
           <t>Spotter Blimp</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="81" t="inlineStr">
         <is>
           <t>Flies your track: a door gun, a searchlight or cargo</t>
         </is>
       </c>
-      <c r="C22" t="n">
+      <c r="C22" s="81" t="n">
         <v>600</v>
       </c>
-      <c r="D22" t="n">
+      <c r="D22" s="81" t="n">
         <v>5</v>
       </c>
-      <c r="E22" t="n">
+      <c r="E22" s="81" t="n">
         <v>2</v>
       </c>
-      <c r="F22" t="n">
-        <v>1</v>
-      </c>
-      <c r="G22">
+      <c r="F22" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="81">
         <f>D22*E22*F22</f>
         <v/>
       </c>
-      <c r="H22" t="n">
+      <c r="H22" s="81" t="n">
         <v>14</v>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="I22" s="81" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="J22" t="n">
+      <c r="J22" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="K22" t="inlineStr">
+      <c r="K22" s="81" t="inlineStr">
         <is>
           <t>Its mooring mast is placed like any tower; the blimp flies your track there and back. Can't be damaged (#148).</t>
         </is>
       </c>
-      <c r="L22" t="n">
+      <c r="L22" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="M22" t="n">
+      <c r="M22" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="N22" t="n">
+      <c r="N22" s="81" t="n">
         <v>400</v>
       </c>
-      <c r="O22" t="inlineStr">
+      <c r="O22" s="81" t="inlineStr">
         <is>
           <t>BLIMP</t>
         </is>
       </c>
-      <c r="P22" t="n">
+      <c r="P22" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="Q22" t="n">
+      <c r="Q22" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="R22" t="n">
+      <c r="R22" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="T22" t="inlineStr">
+      <c r="T22" s="81" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -14445,7 +14445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:FM409"/>
+  <dimension ref="A1:FL409"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66667" defaultRowHeight="15" customHeight="1" outlineLevelRow="0"/>
   <cols>
     <col width="15" customWidth="1" style="81" min="1" max="1"/>
@@ -15370,57 +15370,57 @@
           <t>Aura range %</t>
         </is>
       </c>
-      <c r="FB4" t="inlineStr">
+      <c r="FB4" s="81" t="inlineStr">
         <is>
           <t>Blimp speed x</t>
         </is>
       </c>
-      <c r="FC4" t="inlineStr">
+      <c r="FC4" s="81" t="inlineStr">
         <is>
           <t>Lap chests</t>
         </is>
       </c>
-      <c r="FD4" t="inlineStr">
+      <c r="FD4" s="81" t="inlineStr">
         <is>
           <t>Lap repairs</t>
         </is>
       </c>
-      <c r="FE4" t="inlineStr">
+      <c r="FE4" s="81" t="inlineStr">
         <is>
           <t>Crate heal %</t>
         </is>
       </c>
-      <c r="FF4" t="inlineStr">
+      <c r="FF4" s="81" t="inlineStr">
         <is>
           <t>Paratroopers</t>
         </is>
       </c>
-      <c r="FG4" t="inlineStr">
+      <c r="FG4" s="81" t="inlineStr">
         <is>
           <t>Airlift</t>
         </is>
       </c>
-      <c r="FH4" t="inlineStr">
+      <c r="FH4" s="81" t="inlineStr">
         <is>
           <t>Throw miss %</t>
         </is>
       </c>
-      <c r="FI4" t="inlineStr">
+      <c r="FI4" s="81" t="inlineStr">
         <is>
           <t>Aura reach x</t>
         </is>
       </c>
-      <c r="FJ4" t="inlineStr">
+      <c r="FJ4" s="81" t="inlineStr">
         <is>
           <t>Dino outlines</t>
         </is>
       </c>
-      <c r="FK4" t="inlineStr">
+      <c r="FK4" s="81" t="inlineStr">
         <is>
           <t>Bombing run</t>
         </is>
       </c>
-      <c r="FL4" t="inlineStr">
+      <c r="FL4" s="81" t="inlineStr">
         <is>
           <t>Hook every (s)</t>
         </is>
@@ -43536,1665 +43536,1665 @@
       </c>
     </row>
     <row r="383">
-      <c r="A383" t="inlineStr">
+      <c r="A383" s="81" t="inlineStr">
         <is>
           <t>Spotter Blimp</t>
         </is>
       </c>
-      <c r="B383" t="inlineStr">
+      <c r="B383" s="81" t="inlineStr">
         <is>
           <t>Door Gun</t>
         </is>
       </c>
-      <c r="C383" t="inlineStr">
+      <c r="C383" s="81" t="inlineStr">
         <is>
           <t>damage</t>
         </is>
       </c>
-      <c r="D383" t="n">
-        <v>1</v>
-      </c>
-      <c r="E383">
+      <c r="D383" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="E383" s="81">
         <f>ROUND('Towers'!$C$22*POWER('Tuning'!$B$12,D383),0)</f>
         <v/>
       </c>
-      <c r="F383">
+      <c r="F383" s="81">
         <f>'Towers'!$C$22+E383</f>
         <v/>
       </c>
-      <c r="G383" t="n">
+      <c r="G383" s="81" t="n">
         <v>1.5</v>
       </c>
-      <c r="H383" t="n">
+      <c r="H383" s="81" t="n">
         <v>1.2</v>
       </c>
-      <c r="I383" t="n">
-        <v>1</v>
-      </c>
-      <c r="J383">
+      <c r="I383" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J383" s="81">
         <f>'Towers'!$G$22*G383*H383*I383</f>
         <v/>
       </c>
-      <c r="K383">
+      <c r="K383" s="81">
         <f>IF(J383=0,0,F383/J383)</f>
         <v/>
       </c>
-      <c r="L383" t="n">
-        <v>1</v>
-      </c>
-      <c r="M383" t="inlineStr">
+      <c r="L383" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M383" s="81" t="inlineStr">
         <is>
           <t>Belt Gun</t>
         </is>
       </c>
     </row>
     <row r="384">
-      <c r="A384" t="inlineStr">
+      <c r="A384" s="81" t="inlineStr">
         <is>
           <t>Spotter Blimp</t>
         </is>
       </c>
-      <c r="B384" t="inlineStr">
+      <c r="B384" s="81" t="inlineStr">
         <is>
           <t>Door Gun</t>
         </is>
       </c>
-      <c r="C384" t="inlineStr">
+      <c r="C384" s="81" t="inlineStr">
         <is>
           <t>damage</t>
         </is>
       </c>
-      <c r="D384" t="n">
+      <c r="D384" s="81" t="n">
         <v>2</v>
       </c>
-      <c r="E384">
+      <c r="E384" s="81">
         <f>ROUND('Towers'!$C$22*POWER('Tuning'!$B$12,D384),0)</f>
         <v/>
       </c>
-      <c r="F384">
+      <c r="F384" s="81">
         <f>F383+E384</f>
         <v/>
       </c>
-      <c r="G384" t="n">
+      <c r="G384" s="81" t="n">
         <v>1.5</v>
       </c>
-      <c r="H384" t="n">
+      <c r="H384" s="81" t="n">
         <v>1.2</v>
       </c>
-      <c r="I384" t="n">
-        <v>1</v>
-      </c>
-      <c r="J384">
+      <c r="I384" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J384" s="81">
         <f>'Towers'!$G$22*G384*H384*I384</f>
         <v/>
       </c>
-      <c r="K384">
+      <c r="K384" s="81">
         <f>IF(J384=0,0,F384/J384)</f>
         <v/>
       </c>
-      <c r="L384" t="n">
-        <v>1</v>
-      </c>
-      <c r="M384" t="inlineStr">
+      <c r="L384" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M384" s="81" t="inlineStr">
         <is>
           <t>Twin Mount</t>
         </is>
       </c>
-      <c r="Q384" t="n">
+      <c r="Q384" s="81" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="385">
-      <c r="A385" t="inlineStr">
+      <c r="A385" s="81" t="inlineStr">
         <is>
           <t>Spotter Blimp</t>
         </is>
       </c>
-      <c r="B385" t="inlineStr">
+      <c r="B385" s="81" t="inlineStr">
         <is>
           <t>Door Gun</t>
         </is>
       </c>
-      <c r="C385" t="inlineStr">
+      <c r="C385" s="81" t="inlineStr">
         <is>
           <t>damage</t>
         </is>
       </c>
-      <c r="D385" t="n">
+      <c r="D385" s="81" t="n">
         <v>3</v>
       </c>
-      <c r="E385">
+      <c r="E385" s="81">
         <f>ROUND('Towers'!$C$22*POWER('Tuning'!$B$12,D385),0)</f>
         <v/>
       </c>
-      <c r="F385">
+      <c r="F385" s="81">
         <f>F384+E385</f>
         <v/>
       </c>
-      <c r="G385" t="n">
+      <c r="G385" s="81" t="n">
         <v>2.6</v>
       </c>
-      <c r="H385" t="n">
+      <c r="H385" s="81" t="n">
         <v>1.2</v>
       </c>
-      <c r="I385" t="n">
-        <v>1</v>
-      </c>
-      <c r="J385">
+      <c r="I385" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J385" s="81">
         <f>'Towers'!$G$22*G385*H385*I385</f>
         <v/>
       </c>
-      <c r="K385">
+      <c r="K385" s="81">
         <f>IF(J385=0,0,F385/J385)</f>
         <v/>
       </c>
-      <c r="L385" t="n">
-        <v>1</v>
-      </c>
-      <c r="M385" t="inlineStr">
-        <is>
-          <t>Strafing Run</t>
-        </is>
-      </c>
-      <c r="Q385" t="n">
+      <c r="L385" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M385" s="81" t="inlineStr">
+        <is>
+          <t>Treetop Pass</t>
+        </is>
+      </c>
+      <c r="Q385" s="81" t="n">
         <v>2</v>
       </c>
-      <c r="R385" t="n">
+      <c r="R385" s="81" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="386">
-      <c r="A386" t="inlineStr">
+      <c r="A386" s="81" t="inlineStr">
         <is>
           <t>Spotter Blimp</t>
         </is>
       </c>
-      <c r="B386" t="inlineStr">
+      <c r="B386" s="81" t="inlineStr">
         <is>
           <t>Door Gun</t>
         </is>
       </c>
-      <c r="C386" t="inlineStr">
+      <c r="C386" s="81" t="inlineStr">
         <is>
           <t>damage</t>
         </is>
       </c>
-      <c r="D386" t="n">
+      <c r="D386" s="81" t="n">
         <v>4</v>
       </c>
-      <c r="E386">
+      <c r="E386" s="81">
         <f>ROUND('Towers'!$C$22*POWER('Tuning'!$B$12,D386),0)</f>
         <v/>
       </c>
-      <c r="F386">
+      <c r="F386" s="81">
         <f>F385+E386</f>
         <v/>
       </c>
-      <c r="G386" t="n">
+      <c r="G386" s="81" t="n">
         <v>1.7</v>
       </c>
-      <c r="H386" t="n">
-        <v>1</v>
-      </c>
-      <c r="I386" t="n">
-        <v>1</v>
-      </c>
-      <c r="J386">
+      <c r="H386" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I386" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J386" s="81">
         <f>J385*G386*H386*I386</f>
         <v/>
       </c>
-      <c r="K386">
+      <c r="K386" s="81">
         <f>IF(J386=0,0,F386/J386)</f>
         <v/>
       </c>
-      <c r="L386" t="n">
-        <v>1</v>
-      </c>
-      <c r="M386" t="inlineStr">
+      <c r="L386" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M386" s="81" t="inlineStr">
         <is>
           <t>Heavy Mount</t>
         </is>
       </c>
-      <c r="N386" t="inlineStr">
+      <c r="N386" s="81" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="BJ386" t="n">
+      <c r="BJ386" s="81" t="n">
         <v>2</v>
       </c>
-      <c r="CI386" t="inlineStr">
+      <c r="CI386" s="81" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="CJ386" t="inlineStr">
+      <c r="CJ386" s="81" t="inlineStr">
         <is>
           <t>Shoots through armour, breaks 2</t>
         </is>
       </c>
     </row>
     <row r="387">
-      <c r="A387" t="inlineStr">
+      <c r="A387" s="81" t="inlineStr">
         <is>
           <t>Spotter Blimp</t>
         </is>
       </c>
-      <c r="B387" t="inlineStr">
+      <c r="B387" s="81" t="inlineStr">
         <is>
           <t>Door Gun</t>
         </is>
       </c>
-      <c r="C387" t="inlineStr">
+      <c r="C387" s="81" t="inlineStr">
         <is>
           <t>damage</t>
         </is>
       </c>
-      <c r="D387" t="n">
+      <c r="D387" s="81" t="n">
         <v>5</v>
       </c>
-      <c r="E387">
+      <c r="E387" s="81">
         <f>ROUND('Towers'!$C$22*POWER('Tuning'!$B$12,D387),0)</f>
         <v/>
       </c>
-      <c r="F387">
+      <c r="F387" s="81">
         <f>F386+E387</f>
         <v/>
       </c>
-      <c r="G387" t="n">
+      <c r="G387" s="81" t="n">
         <v>0.78</v>
       </c>
-      <c r="H387" t="n">
-        <v>1</v>
-      </c>
-      <c r="I387" t="n">
-        <v>1</v>
-      </c>
-      <c r="J387">
+      <c r="H387" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I387" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J387" s="81">
         <f>J386*G387*H387*I387</f>
         <v/>
       </c>
-      <c r="K387">
+      <c r="K387" s="81">
         <f>IF(J387=0,0,F387/J387)</f>
         <v/>
       </c>
-      <c r="L387" t="n">
-        <v>1</v>
-      </c>
-      <c r="M387" t="inlineStr">
+      <c r="L387" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M387" s="81" t="inlineStr">
         <is>
           <t>Gunship</t>
         </is>
       </c>
-      <c r="Q387" t="n">
+      <c r="Q387" s="81" t="n">
         <v>4</v>
       </c>
-      <c r="Z387" t="n">
+      <c r="Z387" s="81" t="n">
         <v>2</v>
       </c>
-      <c r="AA387" t="n">
-        <v>1</v>
-      </c>
-      <c r="CI387" t="inlineStr">
+      <c r="AA387" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="CI387" s="81" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="CJ387" t="inlineStr">
+      <c r="CJ387" s="81" t="inlineStr">
         <is>
           <t>Faster, four guns and rockets</t>
         </is>
       </c>
-      <c r="FB387" t="n">
+      <c r="FB387" s="81" t="n">
         <v>1.5</v>
       </c>
     </row>
     <row r="388">
-      <c r="A388" t="inlineStr">
+      <c r="A388" s="81" t="inlineStr">
         <is>
           <t>Spotter Blimp</t>
         </is>
       </c>
-      <c r="B388" t="inlineStr">
+      <c r="B388" s="81" t="inlineStr">
         <is>
           <t>Searchlight</t>
         </is>
       </c>
-      <c r="C388" t="inlineStr">
+      <c r="C388" s="81" t="inlineStr">
         <is>
           <t>support</t>
         </is>
       </c>
-      <c r="D388" t="n">
-        <v>1</v>
-      </c>
-      <c r="E388">
+      <c r="D388" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="E388" s="81">
         <f>ROUND('Towers'!$C$22*POWER('Tuning'!$B$12,D388),0)</f>
         <v/>
       </c>
-      <c r="F388">
+      <c r="F388" s="81">
         <f>'Towers'!$C$22+E388</f>
         <v/>
       </c>
-      <c r="G388" t="n">
-        <v>1</v>
-      </c>
-      <c r="H388" t="n">
-        <v>1</v>
-      </c>
-      <c r="I388" t="n">
-        <v>1</v>
-      </c>
-      <c r="J388">
+      <c r="G388" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="H388" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I388" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J388" s="81">
         <f>'Towers'!$G$22*G388*H388*I388</f>
         <v/>
       </c>
-      <c r="K388">
+      <c r="K388" s="81">
         <f>IF(J388=0,0,F388/J388)</f>
         <v/>
       </c>
-      <c r="L388" t="n">
-        <v>1</v>
-      </c>
-      <c r="M388" t="inlineStr">
+      <c r="L388" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M388" s="81" t="inlineStr">
         <is>
           <t>Spotlight</t>
         </is>
       </c>
-      <c r="AL388" t="n">
+      <c r="AL388" s="81" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="389">
-      <c r="A389" t="inlineStr">
+      <c r="A389" s="81" t="inlineStr">
         <is>
           <t>Spotter Blimp</t>
         </is>
       </c>
-      <c r="B389" t="inlineStr">
+      <c r="B389" s="81" t="inlineStr">
         <is>
           <t>Searchlight</t>
         </is>
       </c>
-      <c r="C389" t="inlineStr">
+      <c r="C389" s="81" t="inlineStr">
         <is>
           <t>support</t>
         </is>
       </c>
-      <c r="D389" t="n">
+      <c r="D389" s="81" t="n">
         <v>2</v>
       </c>
-      <c r="E389">
+      <c r="E389" s="81">
         <f>ROUND('Towers'!$C$22*POWER('Tuning'!$B$12,D389),0)</f>
         <v/>
       </c>
-      <c r="F389">
+      <c r="F389" s="81">
         <f>F388+E389</f>
         <v/>
       </c>
-      <c r="G389" t="n">
-        <v>1</v>
-      </c>
-      <c r="H389" t="n">
-        <v>1</v>
-      </c>
-      <c r="I389" t="n">
-        <v>1</v>
-      </c>
-      <c r="J389">
+      <c r="G389" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="H389" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I389" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J389" s="81">
         <f>'Towers'!$G$22*G389*H389*I389</f>
         <v/>
       </c>
-      <c r="K389">
+      <c r="K389" s="81">
         <f>IF(J389=0,0,F389/J389)</f>
         <v/>
       </c>
-      <c r="L389" t="n">
+      <c r="L389" s="81" t="n">
         <v>1.3</v>
       </c>
-      <c r="M389" t="inlineStr">
+      <c r="M389" s="81" t="inlineStr">
         <is>
           <t>Wide Beam</t>
         </is>
       </c>
-      <c r="AL389" t="n">
+      <c r="AL389" s="81" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="390">
-      <c r="A390" t="inlineStr">
+      <c r="A390" s="81" t="inlineStr">
         <is>
           <t>Spotter Blimp</t>
         </is>
       </c>
-      <c r="B390" t="inlineStr">
+      <c r="B390" s="81" t="inlineStr">
         <is>
           <t>Searchlight</t>
         </is>
       </c>
-      <c r="C390" t="inlineStr">
+      <c r="C390" s="81" t="inlineStr">
         <is>
           <t>support</t>
         </is>
       </c>
-      <c r="D390" t="n">
+      <c r="D390" s="81" t="n">
         <v>3</v>
       </c>
-      <c r="E390">
+      <c r="E390" s="81">
         <f>ROUND('Towers'!$C$22*POWER('Tuning'!$B$12,D390),0)</f>
         <v/>
       </c>
-      <c r="F390">
+      <c r="F390" s="81">
         <f>F389+E390</f>
         <v/>
       </c>
-      <c r="G390" t="n">
-        <v>1</v>
-      </c>
-      <c r="H390" t="n">
-        <v>1</v>
-      </c>
-      <c r="I390" t="n">
-        <v>1</v>
-      </c>
-      <c r="J390">
+      <c r="G390" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="H390" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I390" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J390" s="81">
         <f>'Towers'!$G$22*G390*H390*I390</f>
         <v/>
       </c>
-      <c r="K390">
+      <c r="K390" s="81">
         <f>IF(J390=0,0,F390/J390)</f>
         <v/>
       </c>
-      <c r="L390" t="n">
+      <c r="L390" s="81" t="n">
         <v>1.3</v>
       </c>
-      <c r="M390" t="inlineStr">
+      <c r="M390" s="81" t="inlineStr">
         <is>
           <t>Night Hunt</t>
         </is>
       </c>
-      <c r="AL390" t="n">
+      <c r="AL390" s="81" t="n">
         <v>10</v>
       </c>
-      <c r="FA390" t="n">
+      <c r="FA390" s="81" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="391">
-      <c r="A391" t="inlineStr">
+      <c r="A391" s="81" t="inlineStr">
         <is>
           <t>Spotter Blimp</t>
         </is>
       </c>
-      <c r="B391" t="inlineStr">
+      <c r="B391" s="81" t="inlineStr">
         <is>
           <t>Searchlight</t>
         </is>
       </c>
-      <c r="C391" t="inlineStr">
+      <c r="C391" s="81" t="inlineStr">
         <is>
           <t>support</t>
         </is>
       </c>
-      <c r="D391" t="n">
+      <c r="D391" s="81" t="n">
         <v>4</v>
       </c>
-      <c r="E391">
+      <c r="E391" s="81">
         <f>ROUND('Towers'!$C$22*POWER('Tuning'!$B$12,D391),0)</f>
         <v/>
       </c>
-      <c r="F391">
+      <c r="F391" s="81">
         <f>F390+E391</f>
         <v/>
       </c>
-      <c r="G391" t="n">
-        <v>1</v>
-      </c>
-      <c r="H391" t="n">
-        <v>1</v>
-      </c>
-      <c r="I391" t="n">
-        <v>1</v>
-      </c>
-      <c r="J391">
+      <c r="G391" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="H391" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I391" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J391" s="81">
         <f>J390*G391*H391*I391</f>
         <v/>
       </c>
-      <c r="K391">
+      <c r="K391" s="81">
         <f>IF(J391=0,0,F391/J391)</f>
         <v/>
       </c>
-      <c r="L391" t="n">
+      <c r="L391" s="81" t="n">
         <v>1.6</v>
       </c>
-      <c r="M391" t="inlineStr">
+      <c r="M391" s="81" t="inlineStr">
         <is>
           <t>Floodlights</t>
         </is>
       </c>
-      <c r="CI391" t="inlineStr">
+      <c r="CI391" s="81" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="CJ391" t="inlineStr">
+      <c r="CJ391" s="81" t="inlineStr">
         <is>
           <t>Lights a much wider circle</t>
         </is>
       </c>
     </row>
     <row r="392">
-      <c r="A392" t="inlineStr">
+      <c r="A392" s="81" t="inlineStr">
         <is>
           <t>Spotter Blimp</t>
         </is>
       </c>
-      <c r="B392" t="inlineStr">
+      <c r="B392" s="81" t="inlineStr">
         <is>
           <t>Searchlight</t>
         </is>
       </c>
-      <c r="C392" t="inlineStr">
+      <c r="C392" s="81" t="inlineStr">
         <is>
           <t>support</t>
         </is>
       </c>
-      <c r="D392" t="n">
+      <c r="D392" s="81" t="n">
         <v>5</v>
       </c>
-      <c r="E392">
+      <c r="E392" s="81">
         <f>ROUND('Towers'!$C$22*POWER('Tuning'!$B$12,D392),0)</f>
         <v/>
       </c>
-      <c r="F392">
+      <c r="F392" s="81">
         <f>F391+E392</f>
         <v/>
       </c>
-      <c r="G392" t="n">
-        <v>1</v>
-      </c>
-      <c r="H392" t="n">
-        <v>1</v>
-      </c>
-      <c r="I392" t="n">
-        <v>1</v>
-      </c>
-      <c r="J392">
+      <c r="G392" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="H392" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I392" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J392" s="81">
         <f>J391*G392*H392*I392</f>
         <v/>
       </c>
-      <c r="K392">
+      <c r="K392" s="81">
         <f>IF(J392=0,0,F392/J392)</f>
         <v/>
       </c>
-      <c r="L392" t="n">
-        <v>1</v>
-      </c>
-      <c r="M392" t="inlineStr">
+      <c r="L392" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M392" s="81" t="inlineStr">
         <is>
           <t>All-Seeing Eye</t>
         </is>
       </c>
-      <c r="AL392" t="n">
+      <c r="AL392" s="81" t="n">
         <v>25</v>
       </c>
-      <c r="CI392" t="inlineStr">
+      <c r="CI392" s="81" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="CJ392" t="inlineStr">
+      <c r="CJ392" s="81" t="inlineStr">
         <is>
           <t>Every dino under the blimp marked +25%</t>
         </is>
       </c>
     </row>
     <row r="393">
-      <c r="A393" t="inlineStr">
+      <c r="A393" s="81" t="inlineStr">
         <is>
           <t>Spotter Blimp</t>
         </is>
       </c>
-      <c r="B393" t="inlineStr">
+      <c r="B393" s="81" t="inlineStr">
         <is>
           <t>Cargo</t>
         </is>
       </c>
-      <c r="C393" t="inlineStr">
+      <c r="C393" s="81" t="inlineStr">
         <is>
           <t>cash</t>
         </is>
       </c>
-      <c r="D393" t="n">
-        <v>1</v>
-      </c>
-      <c r="E393">
+      <c r="D393" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="E393" s="81">
         <f>ROUND('Towers'!$C$22*POWER('Tuning'!$B$12,D393),0)</f>
         <v/>
       </c>
-      <c r="F393">
+      <c r="F393" s="81">
         <f>'Towers'!$C$22+E393</f>
         <v/>
       </c>
-      <c r="G393" t="n">
-        <v>1</v>
-      </c>
-      <c r="H393" t="n">
-        <v>1</v>
-      </c>
-      <c r="I393" t="n">
-        <v>1</v>
-      </c>
-      <c r="J393">
+      <c r="G393" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="H393" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I393" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J393" s="81">
         <f>'Towers'!$G$22*G393*H393*I393</f>
         <v/>
       </c>
-      <c r="K393">
+      <c r="K393" s="81">
         <f>IF(J393=0,0,F393/J393)</f>
         <v/>
       </c>
-      <c r="L393" t="n">
-        <v>1</v>
-      </c>
-      <c r="M393" t="inlineStr">
+      <c r="L393" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M393" s="81" t="inlineStr">
         <is>
           <t>Supply Crates</t>
         </is>
       </c>
-      <c r="AQ393" t="n">
-        <v>1</v>
-      </c>
-      <c r="AR393" t="n">
+      <c r="AQ393" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR393" s="81" t="n">
         <v>200</v>
       </c>
     </row>
     <row r="394">
-      <c r="A394" t="inlineStr">
+      <c r="A394" s="81" t="inlineStr">
         <is>
           <t>Spotter Blimp</t>
         </is>
       </c>
-      <c r="B394" t="inlineStr">
+      <c r="B394" s="81" t="inlineStr">
         <is>
           <t>Cargo</t>
         </is>
       </c>
-      <c r="C394" t="inlineStr">
+      <c r="C394" s="81" t="inlineStr">
         <is>
           <t>cash</t>
         </is>
       </c>
-      <c r="D394" t="n">
+      <c r="D394" s="81" t="n">
         <v>2</v>
       </c>
-      <c r="E394">
+      <c r="E394" s="81">
         <f>ROUND('Towers'!$C$22*POWER('Tuning'!$B$12,D394),0)</f>
         <v/>
       </c>
-      <c r="F394">
+      <c r="F394" s="81">
         <f>F393+E394</f>
         <v/>
       </c>
-      <c r="G394" t="n">
-        <v>1</v>
-      </c>
-      <c r="H394" t="n">
-        <v>1</v>
-      </c>
-      <c r="I394" t="n">
-        <v>1</v>
-      </c>
-      <c r="J394">
+      <c r="G394" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="H394" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I394" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J394" s="81">
         <f>'Towers'!$G$22*G394*H394*I394</f>
         <v/>
       </c>
-      <c r="K394">
+      <c r="K394" s="81">
         <f>IF(J394=0,0,F394/J394)</f>
         <v/>
       </c>
-      <c r="L394" t="n">
-        <v>1</v>
-      </c>
-      <c r="M394" t="inlineStr">
+      <c r="L394" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M394" s="81" t="inlineStr">
         <is>
           <t>Ammo Drop</t>
         </is>
       </c>
-      <c r="AQ394" t="n">
-        <v>1</v>
-      </c>
-      <c r="AR394" t="n">
+      <c r="AQ394" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR394" s="81" t="n">
         <v>550</v>
       </c>
-      <c r="AY394" t="n">
+      <c r="AY394" s="81" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="395">
-      <c r="A395" t="inlineStr">
+      <c r="A395" s="81" t="inlineStr">
         <is>
           <t>Spotter Blimp</t>
         </is>
       </c>
-      <c r="B395" t="inlineStr">
+      <c r="B395" s="81" t="inlineStr">
         <is>
           <t>Cargo</t>
         </is>
       </c>
-      <c r="C395" t="inlineStr">
+      <c r="C395" s="81" t="inlineStr">
         <is>
           <t>cash</t>
         </is>
       </c>
-      <c r="D395" t="n">
+      <c r="D395" s="81" t="n">
         <v>3</v>
       </c>
-      <c r="E395">
+      <c r="E395" s="81">
         <f>ROUND('Towers'!$C$22*POWER('Tuning'!$B$12,D395),0)</f>
         <v/>
       </c>
-      <c r="F395">
+      <c r="F395" s="81">
         <f>F394+E395</f>
         <v/>
       </c>
-      <c r="G395" t="n">
-        <v>1</v>
-      </c>
-      <c r="H395" t="n">
-        <v>1</v>
-      </c>
-      <c r="I395" t="n">
-        <v>1</v>
-      </c>
-      <c r="J395">
+      <c r="G395" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="H395" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I395" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J395" s="81">
         <f>'Towers'!$G$22*G395*H395*I395</f>
         <v/>
       </c>
-      <c r="K395">
+      <c r="K395" s="81">
         <f>IF(J395=0,0,F395/J395)</f>
         <v/>
       </c>
-      <c r="L395" t="n">
-        <v>1</v>
-      </c>
-      <c r="M395" t="inlineStr">
+      <c r="L395" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M395" s="81" t="inlineStr">
         <is>
           <t>Med Drop</t>
         </is>
       </c>
-      <c r="AQ395" t="n">
-        <v>1</v>
-      </c>
-      <c r="AR395" t="n">
+      <c r="AQ395" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR395" s="81" t="n">
         <v>1550</v>
       </c>
-      <c r="AY395" t="n">
+      <c r="AY395" s="81" t="n">
         <v>0.8</v>
       </c>
-      <c r="BE395" t="n">
-        <v>1</v>
-      </c>
-      <c r="BF395" t="n">
+      <c r="BE395" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF395" s="81" t="n">
         <v>40</v>
       </c>
     </row>
     <row r="396">
-      <c r="A396" t="inlineStr">
+      <c r="A396" s="81" t="inlineStr">
         <is>
           <t>Spotter Blimp</t>
         </is>
       </c>
-      <c r="B396" t="inlineStr">
+      <c r="B396" s="81" t="inlineStr">
         <is>
           <t>Cargo</t>
         </is>
       </c>
-      <c r="C396" t="inlineStr">
+      <c r="C396" s="81" t="inlineStr">
         <is>
           <t>cash</t>
         </is>
       </c>
-      <c r="D396" t="n">
+      <c r="D396" s="81" t="n">
         <v>4</v>
       </c>
-      <c r="E396">
+      <c r="E396" s="81">
         <f>ROUND('Towers'!$C$22*POWER('Tuning'!$B$12,D396),0)</f>
         <v/>
       </c>
-      <c r="F396">
+      <c r="F396" s="81">
         <f>F395+E396</f>
         <v/>
       </c>
-      <c r="G396" t="n">
-        <v>1</v>
-      </c>
-      <c r="H396" t="n">
-        <v>1</v>
-      </c>
-      <c r="I396" t="n">
-        <v>1</v>
-      </c>
-      <c r="J396">
+      <c r="G396" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="H396" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I396" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J396" s="81">
         <f>J395*G396*H396*I396</f>
         <v/>
       </c>
-      <c r="K396">
+      <c r="K396" s="81">
         <f>IF(J396=0,0,F396/J396)</f>
         <v/>
       </c>
-      <c r="L396" t="n">
-        <v>1</v>
-      </c>
-      <c r="M396" t="inlineStr">
+      <c r="L396" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M396" s="81" t="inlineStr">
         <is>
           <t>Heavy Cargo</t>
         </is>
       </c>
-      <c r="AR396" t="n">
+      <c r="AR396" s="81" t="n">
         <v>2000</v>
       </c>
-      <c r="CI396" t="inlineStr">
+      <c r="CI396" s="81" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="CJ396" t="inlineStr">
+      <c r="CJ396" s="81" t="inlineStr">
         <is>
           <t>Bigger crates</t>
         </is>
       </c>
     </row>
     <row r="397">
-      <c r="A397" t="inlineStr">
+      <c r="A397" s="81" t="inlineStr">
         <is>
           <t>Spotter Blimp</t>
         </is>
       </c>
-      <c r="B397" t="inlineStr">
+      <c r="B397" s="81" t="inlineStr">
         <is>
           <t>Cargo</t>
         </is>
       </c>
-      <c r="C397" t="inlineStr">
+      <c r="C397" s="81" t="inlineStr">
         <is>
           <t>cash</t>
         </is>
       </c>
-      <c r="D397" t="n">
+      <c r="D397" s="81" t="n">
         <v>5</v>
       </c>
-      <c r="E397">
+      <c r="E397" s="81">
         <f>ROUND('Towers'!$C$22*POWER('Tuning'!$B$12,D397),0)</f>
         <v/>
       </c>
-      <c r="F397">
+      <c r="F397" s="81">
         <f>F396+E397</f>
         <v/>
       </c>
-      <c r="G397" t="n">
-        <v>1</v>
-      </c>
-      <c r="H397" t="n">
-        <v>1</v>
-      </c>
-      <c r="I397" t="n">
-        <v>1</v>
-      </c>
-      <c r="J397">
+      <c r="G397" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="H397" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I397" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J397" s="81">
         <f>J396*G397*H397*I397</f>
         <v/>
       </c>
-      <c r="K397">
+      <c r="K397" s="81">
         <f>IF(J397=0,0,F397/J397)</f>
         <v/>
       </c>
-      <c r="L397" t="n">
-        <v>1</v>
-      </c>
-      <c r="M397" t="inlineStr">
+      <c r="L397" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M397" s="81" t="inlineStr">
         <is>
           <t>Cargo Run</t>
         </is>
       </c>
-      <c r="CI397" t="inlineStr">
+      <c r="CI397" s="81" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="CJ397" t="inlineStr">
+      <c r="CJ397" s="81" t="inlineStr">
         <is>
           <t>A big crate every lap</t>
         </is>
       </c>
-      <c r="FC397" t="inlineStr">
+      <c r="FC397" s="81" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="398">
-      <c r="A398" t="inlineStr">
+      <c r="A398" s="81" t="inlineStr">
         <is>
           <t>Spotter Blimp</t>
         </is>
       </c>
-      <c r="B398" t="inlineStr">
+      <c r="B398" s="81" t="inlineStr">
         <is>
           <t>Door Gun</t>
         </is>
       </c>
-      <c r="C398" t="inlineStr">
+      <c r="C398" s="81" t="inlineStr">
         <is>
           <t>damage</t>
         </is>
       </c>
-      <c r="D398" t="n">
+      <c r="D398" s="81" t="n">
         <v>4</v>
       </c>
-      <c r="E398">
+      <c r="E398" s="81">
         <f>E386</f>
         <v/>
       </c>
-      <c r="F398">
+      <c r="F398" s="81">
         <f>F386</f>
         <v/>
       </c>
-      <c r="G398" t="n">
+      <c r="G398" s="81" t="n">
         <v>1.4</v>
       </c>
-      <c r="H398" t="n">
-        <v>1</v>
-      </c>
-      <c r="I398" t="n">
-        <v>1</v>
-      </c>
-      <c r="L398" t="n">
-        <v>1</v>
-      </c>
-      <c r="M398" t="inlineStr">
+      <c r="H398" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I398" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="L398" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M398" s="81" t="inlineStr">
         <is>
           <t>Rocket Pods</t>
         </is>
       </c>
-      <c r="Z398" t="n">
+      <c r="Z398" s="81" t="n">
         <v>3</v>
       </c>
-      <c r="AA398" t="n">
-        <v>1</v>
-      </c>
-      <c r="CI398" t="inlineStr">
+      <c r="AA398" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="CI398" s="81" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="CJ398" t="inlineStr">
+      <c r="CJ398" s="81" t="inlineStr">
         <is>
           <t>Rockets that splash</t>
         </is>
       </c>
     </row>
     <row r="399">
-      <c r="A399" t="inlineStr">
+      <c r="A399" s="81" t="inlineStr">
         <is>
           <t>Spotter Blimp</t>
         </is>
       </c>
-      <c r="B399" t="inlineStr">
+      <c r="B399" s="81" t="inlineStr">
         <is>
           <t>Door Gun</t>
         </is>
       </c>
-      <c r="C399" t="inlineStr">
+      <c r="C399" s="81" t="inlineStr">
         <is>
           <t>damage</t>
         </is>
       </c>
-      <c r="D399" t="n">
+      <c r="D399" s="81" t="n">
         <v>4</v>
       </c>
-      <c r="E399">
+      <c r="E399" s="81">
         <f>E386</f>
         <v/>
       </c>
-      <c r="F399">
+      <c r="F399" s="81">
         <f>F386</f>
         <v/>
       </c>
-      <c r="G399" t="n">
+      <c r="G399" s="81" t="n">
         <v>1.75</v>
       </c>
-      <c r="H399" t="n">
-        <v>1</v>
-      </c>
-      <c r="I399" t="n">
-        <v>1</v>
-      </c>
-      <c r="L399" t="n">
-        <v>1</v>
-      </c>
-      <c r="M399" t="inlineStr">
+      <c r="H399" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I399" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="L399" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M399" s="81" t="inlineStr">
         <is>
           <t>Tracer Belt</t>
         </is>
       </c>
-      <c r="T399" t="n">
+      <c r="T399" s="81" t="n">
         <v>15</v>
       </c>
-      <c r="CI399" t="inlineStr">
+      <c r="CI399" s="81" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="CJ399" t="inlineStr">
+      <c r="CJ399" s="81" t="inlineStr">
         <is>
           <t>Hit dinos are marked +15%</t>
         </is>
       </c>
     </row>
     <row r="400">
-      <c r="A400" t="inlineStr">
+      <c r="A400" s="81" t="inlineStr">
         <is>
           <t>Spotter Blimp</t>
         </is>
       </c>
-      <c r="B400" t="inlineStr">
+      <c r="B400" s="81" t="inlineStr">
         <is>
           <t>Door Gun</t>
         </is>
       </c>
-      <c r="C400" t="inlineStr">
+      <c r="C400" s="81" t="inlineStr">
         <is>
           <t>damage</t>
         </is>
       </c>
-      <c r="D400" t="n">
+      <c r="D400" s="81" t="n">
         <v>5</v>
       </c>
-      <c r="E400">
+      <c r="E400" s="81">
         <f>E387</f>
         <v/>
       </c>
-      <c r="F400">
+      <c r="F400" s="81">
         <f>F387</f>
         <v/>
       </c>
-      <c r="G400" t="n">
+      <c r="G400" s="81" t="n">
         <v>1.6</v>
       </c>
-      <c r="H400" t="n">
-        <v>1</v>
-      </c>
-      <c r="I400" t="n">
-        <v>1</v>
-      </c>
-      <c r="L400" t="n">
-        <v>1</v>
-      </c>
-      <c r="M400" t="inlineStr">
+      <c r="H400" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I400" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="L400" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M400" s="81" t="inlineStr">
         <is>
           <t>Bombing Run</t>
         </is>
       </c>
-      <c r="CI400" t="inlineStr">
+      <c r="CI400" s="81" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="CJ400" t="inlineStr">
+      <c r="CJ400" s="81" t="inlineStr">
         <is>
           <t>Bombs the whole track once a round</t>
         </is>
       </c>
-      <c r="CS400" t="n">
+      <c r="CS400" s="81" t="n">
         <v>12</v>
       </c>
-      <c r="FK400" t="inlineStr">
+      <c r="FK400" s="81" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="401">
-      <c r="A401" t="inlineStr">
+      <c r="A401" s="81" t="inlineStr">
         <is>
           <t>Spotter Blimp</t>
         </is>
       </c>
-      <c r="B401" t="inlineStr">
+      <c r="B401" s="81" t="inlineStr">
         <is>
           <t>Door Gun</t>
         </is>
       </c>
-      <c r="C401" t="inlineStr">
+      <c r="C401" s="81" t="inlineStr">
         <is>
           <t>damage</t>
         </is>
       </c>
-      <c r="D401" t="n">
+      <c r="D401" s="81" t="n">
         <v>5</v>
       </c>
-      <c r="E401">
+      <c r="E401" s="81">
         <f>E387</f>
         <v/>
       </c>
-      <c r="F401">
+      <c r="F401" s="81">
         <f>F387</f>
         <v/>
       </c>
-      <c r="G401" t="n">
+      <c r="G401" s="81" t="n">
         <v>1.75</v>
       </c>
-      <c r="H401" t="n">
-        <v>1</v>
-      </c>
-      <c r="I401" t="n">
-        <v>1</v>
-      </c>
-      <c r="L401" t="n">
-        <v>1</v>
-      </c>
-      <c r="M401" t="inlineStr">
+      <c r="H401" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I401" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="L401" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M401" s="81" t="inlineStr">
         <is>
           <t>Sky Hook</t>
         </is>
       </c>
-      <c r="CI401" t="inlineStr">
+      <c r="CI401" s="81" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="CJ401" t="inlineStr">
+      <c r="CJ401" s="81" t="inlineStr">
         <is>
           <t>Snatches the smallest dino every 5 s</t>
         </is>
       </c>
-      <c r="FL401" t="n">
+      <c r="FL401" s="81" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="402">
-      <c r="A402" t="inlineStr">
+      <c r="A402" s="81" t="inlineStr">
         <is>
           <t>Spotter Blimp</t>
         </is>
       </c>
-      <c r="B402" t="inlineStr">
+      <c r="B402" s="81" t="inlineStr">
         <is>
           <t>Searchlight</t>
         </is>
       </c>
-      <c r="C402" t="inlineStr">
+      <c r="C402" s="81" t="inlineStr">
         <is>
           <t>support</t>
         </is>
       </c>
-      <c r="D402" t="n">
+      <c r="D402" s="81" t="n">
         <v>4</v>
       </c>
-      <c r="E402">
+      <c r="E402" s="81">
         <f>E391</f>
         <v/>
       </c>
-      <c r="F402">
+      <c r="F402" s="81">
         <f>F391</f>
         <v/>
       </c>
-      <c r="G402" t="n">
-        <v>1</v>
-      </c>
-      <c r="H402" t="n">
-        <v>1</v>
-      </c>
-      <c r="I402" t="n">
-        <v>1</v>
-      </c>
-      <c r="L402" t="n">
-        <v>1</v>
-      </c>
-      <c r="M402" t="inlineStr">
+      <c r="G402" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="H402" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I402" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="L402" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M402" s="81" t="inlineStr">
         <is>
           <t>Tracking Beam</t>
         </is>
       </c>
-      <c r="AL402" t="n">
+      <c r="AL402" s="81" t="n">
         <v>14</v>
       </c>
-      <c r="CI402" t="inlineStr">
+      <c r="CI402" s="81" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="CJ402" t="inlineStr">
+      <c r="CJ402" s="81" t="inlineStr">
         <is>
           <t>The light follows the biggest dino</t>
         </is>
       </c>
-      <c r="CU402" t="inlineStr">
+      <c r="CU402" s="81" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="403">
-      <c r="A403" t="inlineStr">
+      <c r="A403" s="81" t="inlineStr">
         <is>
           <t>Spotter Blimp</t>
         </is>
       </c>
-      <c r="B403" t="inlineStr">
+      <c r="B403" s="81" t="inlineStr">
         <is>
           <t>Searchlight</t>
         </is>
       </c>
-      <c r="C403" t="inlineStr">
+      <c r="C403" s="81" t="inlineStr">
         <is>
           <t>support</t>
         </is>
       </c>
-      <c r="D403" t="n">
+      <c r="D403" s="81" t="n">
         <v>4</v>
       </c>
-      <c r="E403">
+      <c r="E403" s="81">
         <f>E391</f>
         <v/>
       </c>
-      <c r="F403">
+      <c r="F403" s="81">
         <f>F391</f>
         <v/>
       </c>
-      <c r="G403" t="n">
-        <v>1</v>
-      </c>
-      <c r="H403" t="n">
-        <v>1</v>
-      </c>
-      <c r="I403" t="n">
-        <v>1</v>
-      </c>
-      <c r="L403" t="n">
-        <v>1</v>
-      </c>
-      <c r="M403" t="inlineStr">
+      <c r="G403" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="H403" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I403" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="L403" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M403" s="81" t="inlineStr">
         <is>
           <t>Blinding Glare</t>
         </is>
       </c>
-      <c r="AL403" t="n">
+      <c r="AL403" s="81" t="n">
         <v>15</v>
       </c>
-      <c r="CI403" t="inlineStr">
+      <c r="CI403" s="81" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="CJ403" t="inlineStr">
+      <c r="CJ403" s="81" t="inlineStr">
         <is>
           <t>Dinos in the light miss throws</t>
         </is>
       </c>
-      <c r="FH403" t="n">
+      <c r="FH403" s="81" t="n">
         <v>25</v>
       </c>
     </row>
     <row r="404">
-      <c r="A404" t="inlineStr">
+      <c r="A404" s="81" t="inlineStr">
         <is>
           <t>Spotter Blimp</t>
         </is>
       </c>
-      <c r="B404" t="inlineStr">
+      <c r="B404" s="81" t="inlineStr">
         <is>
           <t>Searchlight</t>
         </is>
       </c>
-      <c r="C404" t="inlineStr">
+      <c r="C404" s="81" t="inlineStr">
         <is>
           <t>support</t>
         </is>
       </c>
-      <c r="D404" t="n">
+      <c r="D404" s="81" t="n">
         <v>5</v>
       </c>
-      <c r="E404">
+      <c r="E404" s="81">
         <f>E392</f>
         <v/>
       </c>
-      <c r="F404">
+      <c r="F404" s="81">
         <f>F392</f>
         <v/>
       </c>
-      <c r="G404" t="n">
-        <v>1</v>
-      </c>
-      <c r="H404" t="n">
-        <v>1</v>
-      </c>
-      <c r="I404" t="n">
-        <v>1</v>
-      </c>
-      <c r="L404" t="n">
-        <v>1</v>
-      </c>
-      <c r="M404" t="inlineStr">
+      <c r="G404" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="H404" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I404" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="L404" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M404" s="81" t="inlineStr">
         <is>
           <t>Lighthouse</t>
         </is>
       </c>
-      <c r="AC404" t="n">
+      <c r="AC404" s="81" t="n">
         <v>10</v>
       </c>
-      <c r="CI404" t="inlineStr">
+      <c r="CI404" s="81" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="CJ404" t="inlineStr">
+      <c r="CJ404" s="81" t="inlineStr">
         <is>
           <t>Towers near its path +10% damage</t>
         </is>
       </c>
-      <c r="FI404" t="n">
+      <c r="FI404" s="81" t="n">
         <v>1.5</v>
       </c>
     </row>
     <row r="405">
-      <c r="A405" t="inlineStr">
+      <c r="A405" s="81" t="inlineStr">
         <is>
           <t>Spotter Blimp</t>
         </is>
       </c>
-      <c r="B405" t="inlineStr">
+      <c r="B405" s="81" t="inlineStr">
         <is>
           <t>Searchlight</t>
         </is>
       </c>
-      <c r="C405" t="inlineStr">
+      <c r="C405" s="81" t="inlineStr">
         <is>
           <t>support</t>
         </is>
       </c>
-      <c r="D405" t="n">
+      <c r="D405" s="81" t="n">
         <v>5</v>
       </c>
-      <c r="E405">
+      <c r="E405" s="81">
         <f>E392</f>
         <v/>
       </c>
-      <c r="F405">
+      <c r="F405" s="81">
         <f>F392</f>
         <v/>
       </c>
-      <c r="G405" t="n">
-        <v>1</v>
-      </c>
-      <c r="H405" t="n">
-        <v>1</v>
-      </c>
-      <c r="I405" t="n">
-        <v>1</v>
-      </c>
-      <c r="L405" t="n">
-        <v>1</v>
-      </c>
-      <c r="M405" t="inlineStr">
+      <c r="G405" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="H405" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I405" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="L405" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M405" s="81" t="inlineStr">
         <is>
           <t>Spotter's Map</t>
         </is>
       </c>
-      <c r="AL405" t="n">
+      <c r="AL405" s="81" t="n">
         <v>22</v>
       </c>
-      <c r="CI405" t="inlineStr">
+      <c r="CI405" s="81" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="CJ405" t="inlineStr">
+      <c r="CJ405" s="81" t="inlineStr">
         <is>
           <t>See every dino through walls</t>
         </is>
       </c>
-      <c r="FJ405" t="inlineStr">
+      <c r="FJ405" s="81" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="406">
-      <c r="A406" t="inlineStr">
+      <c r="A406" s="81" t="inlineStr">
         <is>
           <t>Spotter Blimp</t>
         </is>
       </c>
-      <c r="B406" t="inlineStr">
+      <c r="B406" s="81" t="inlineStr">
         <is>
           <t>Cargo</t>
         </is>
       </c>
-      <c r="C406" t="inlineStr">
+      <c r="C406" s="81" t="inlineStr">
         <is>
           <t>cash</t>
         </is>
       </c>
-      <c r="D406" t="n">
+      <c r="D406" s="81" t="n">
         <v>4</v>
       </c>
-      <c r="E406">
+      <c r="E406" s="81">
         <f>E396</f>
         <v/>
       </c>
-      <c r="F406">
+      <c r="F406" s="81">
         <f>F396</f>
         <v/>
       </c>
-      <c r="G406" t="n">
-        <v>1</v>
-      </c>
-      <c r="H406" t="n">
-        <v>1</v>
-      </c>
-      <c r="I406" t="n">
-        <v>1</v>
-      </c>
-      <c r="L406" t="n">
-        <v>1</v>
-      </c>
-      <c r="M406" t="inlineStr">
+      <c r="G406" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="H406" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I406" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="L406" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M406" s="81" t="inlineStr">
         <is>
           <t>Rebuild Kits</t>
         </is>
       </c>
-      <c r="CI406" t="inlineStr">
+      <c r="CI406" s="81" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="CJ406" t="inlineStr">
+      <c r="CJ406" s="81" t="inlineStr">
         <is>
           <t>Fixes a Trampled tower each lap</t>
         </is>
       </c>
-      <c r="FD406" t="n">
+      <c r="FD406" s="81" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="407">
-      <c r="A407" t="inlineStr">
+      <c r="A407" s="81" t="inlineStr">
         <is>
           <t>Spotter Blimp</t>
         </is>
       </c>
-      <c r="B407" t="inlineStr">
+      <c r="B407" s="81" t="inlineStr">
         <is>
           <t>Cargo</t>
         </is>
       </c>
-      <c r="C407" t="inlineStr">
+      <c r="C407" s="81" t="inlineStr">
         <is>
           <t>cash</t>
         </is>
       </c>
-      <c r="D407" t="n">
+      <c r="D407" s="81" t="n">
         <v>4</v>
       </c>
-      <c r="E407">
+      <c r="E407" s="81">
         <f>E396</f>
         <v/>
       </c>
-      <c r="F407">
+      <c r="F407" s="81">
         <f>F396</f>
         <v/>
       </c>
-      <c r="G407" t="n">
-        <v>1</v>
-      </c>
-      <c r="H407" t="n">
-        <v>1</v>
-      </c>
-      <c r="I407" t="n">
-        <v>1</v>
-      </c>
-      <c r="L407" t="n">
-        <v>1</v>
-      </c>
-      <c r="M407" t="inlineStr">
+      <c r="G407" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="H407" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I407" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="L407" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M407" s="81" t="inlineStr">
         <is>
           <t>Spare Parts</t>
         </is>
       </c>
-      <c r="AR407" t="n">
+      <c r="AR407" s="81" t="n">
         <v>1900</v>
       </c>
-      <c r="CI407" t="inlineStr">
+      <c r="CI407" s="81" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="CJ407" t="inlineStr">
+      <c r="CJ407" s="81" t="inlineStr">
         <is>
           <t>A crate heals the closest tower</t>
         </is>
       </c>
-      <c r="FE407" t="n">
+      <c r="FE407" s="81" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="408">
-      <c r="A408" t="inlineStr">
+      <c r="A408" s="81" t="inlineStr">
         <is>
           <t>Spotter Blimp</t>
         </is>
       </c>
-      <c r="B408" t="inlineStr">
+      <c r="B408" s="81" t="inlineStr">
         <is>
           <t>Cargo</t>
         </is>
       </c>
-      <c r="C408" t="inlineStr">
+      <c r="C408" s="81" t="inlineStr">
         <is>
           <t>cash</t>
         </is>
       </c>
-      <c r="D408" t="n">
+      <c r="D408" s="81" t="n">
         <v>5</v>
       </c>
-      <c r="E408">
+      <c r="E408" s="81">
         <f>E397</f>
         <v/>
       </c>
-      <c r="F408">
+      <c r="F408" s="81">
         <f>F397</f>
         <v/>
       </c>
-      <c r="G408" t="n">
-        <v>1</v>
-      </c>
-      <c r="H408" t="n">
-        <v>1</v>
-      </c>
-      <c r="I408" t="n">
-        <v>1</v>
-      </c>
-      <c r="L408" t="n">
-        <v>1</v>
-      </c>
-      <c r="M408" t="inlineStr">
+      <c r="G408" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="H408" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I408" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="L408" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M408" s="81" t="inlineStr">
         <is>
           <t>Paratroopers</t>
         </is>
       </c>
-      <c r="CI408" t="inlineStr">
+      <c r="CI408" s="81" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="CJ408" t="inlineStr">
+      <c r="CJ408" s="81" t="inlineStr">
         <is>
           <t>Drops 2 rangers a round</t>
         </is>
       </c>
-      <c r="FF408" t="n">
+      <c r="FF408" s="81" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="409">
-      <c r="A409" t="inlineStr">
+      <c r="A409" s="81" t="inlineStr">
         <is>
           <t>Spotter Blimp</t>
         </is>
       </c>
-      <c r="B409" t="inlineStr">
+      <c r="B409" s="81" t="inlineStr">
         <is>
           <t>Cargo</t>
         </is>
       </c>
-      <c r="C409" t="inlineStr">
+      <c r="C409" s="81" t="inlineStr">
         <is>
           <t>cash</t>
         </is>
       </c>
-      <c r="D409" t="n">
+      <c r="D409" s="81" t="n">
         <v>5</v>
       </c>
-      <c r="E409">
+      <c r="E409" s="81">
         <f>E397</f>
         <v/>
       </c>
-      <c r="F409">
+      <c r="F409" s="81">
         <f>F397</f>
         <v/>
       </c>
-      <c r="G409" t="n">
-        <v>1</v>
-      </c>
-      <c r="H409" t="n">
-        <v>1</v>
-      </c>
-      <c r="I409" t="n">
-        <v>1</v>
-      </c>
-      <c r="L409" t="n">
-        <v>1</v>
-      </c>
-      <c r="M409" t="inlineStr">
+      <c r="G409" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="H409" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I409" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="L409" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M409" s="81" t="inlineStr">
         <is>
           <t>Airlift</t>
         </is>
       </c>
-      <c r="AR409" t="n">
+      <c r="AR409" s="81" t="n">
         <v>2700</v>
       </c>
-      <c r="CI409" t="inlineStr">
+      <c r="CI409" s="81" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="CJ409" t="inlineStr">
+      <c r="CJ409" s="81" t="inlineStr">
         <is>
           <t>Fixes the first Trampled tower each round</t>
         </is>
       </c>
-      <c r="FG409" t="inlineStr">
+      <c r="FG409" s="81" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>

</xml_diff>

<commit_message>
9i T127 step 1: Meteor Beacon rows, metrics, Shared/Meteor (unreleased)
Towers row 23 METEOR (600 cash, 40 x 0.125/s on 6, splash 8, 150 HP,
600 Amber), Tuning METEOR BEACON block, 14 new Tower Upgrades columns
(FM-FZ, KEY_ONLY METEOR; Throw miss % and Bombing run shared with it),
27 rows (PLAN 9i, #337). BREAK_PATHS += Meteor Impact; --breaks1 bar 3
reported for area strikes (#338); Impact T1/T2, Sky Rocks T1 DEAD known.

value.py meteor_edps / meteor_aftermath reproduce the Director's check
except Comet Tail: the PLAN metric's sweep term (Field strike x 6 on 10
dinos / 50 s) adds ~35 eDPS the harness left out, so Starfall after B4
fell to 0.78x its slot. Rule 7: Starfall Damage x 2.8 -> 3.388 (two 10%
steps; 0.80x). Measured: Impact T5 433/388/388, 353/315/315, 395/400/400;
damage T5 c/e 157-268 (<= 177 / 284); best T2 r11-20 179 (<= 386);
Aftermath slots match. Unreleased. Not playtested.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Storm-Split-Balance.xlsx
+++ b/Storm-Split-Balance.xlsx
@@ -9500,7 +9500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E251"/>
+  <dimension ref="A1:E266"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66667" defaultRowHeight="15" customHeight="1" outlineLevelRow="0"/>
   <cols>
     <col width="34" customWidth="1" style="81" min="1" max="1"/>
@@ -13131,6 +13131,208 @@
       <c r="C251" s="81" t="inlineStr">
         <is>
           <t>Sky Hook takes only a non-boss dino with at most this many sizes left</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="81" t="inlineStr">
+        <is>
+          <t>METEOR BEACON</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="81" t="inlineStr">
+        <is>
+          <t>Bunch radius (studs)</t>
+        </is>
+      </c>
+      <c r="B254" s="81" t="n">
+        <v>8</v>
+      </c>
+      <c r="C254" s="81" t="inlineStr">
+        <is>
+          <t>studs: a meteor aims at the track point with the most dinos within this (a boss counts 3; Shared/Meteor)</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="81" t="inlineStr">
+        <is>
+          <t>Strike warning (s)</t>
+        </is>
+      </c>
+      <c r="B255" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="C255" s="81" t="inlineStr">
+        <is>
+          <t>s the red warning ring shows before a meteor lands</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="81" t="inlineStr">
+        <is>
+          <t>Crater radius</t>
+        </is>
+      </c>
+      <c r="B256" s="81" t="n">
+        <v>6</v>
+      </c>
+      <c r="C256" s="81" t="inlineStr">
+        <is>
+          <t>studs: the burning crater a strike's densest-point meteor leaves</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="81" t="inlineStr">
+        <is>
+          <t>Crater (s)</t>
+        </is>
+      </c>
+      <c r="B257" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="C257" s="81" t="inlineStr">
+        <is>
+          <t>s a crater lasts when the build sets no Crater (s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="81" t="inlineStr">
+        <is>
+          <t>Crater burn DPS</t>
+        </is>
+      </c>
+      <c r="B258" s="81" t="n">
+        <v>10</v>
+      </c>
+      <c r="C258" s="81" t="inlineStr">
+        <is>
+          <t>a crater's burn a second when the build sets no Burn DPS (x the team's level)</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="81" t="inlineStr">
+        <is>
+          <t>Small meteor x</t>
+        </is>
+      </c>
+      <c r="B259" s="81" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C259" s="81" t="inlineStr">
+        <is>
+          <t>x the meteor's damage for each small meteor (Sky Rocks, Endless Rain, Starfall)</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="81" t="inlineStr">
+        <is>
+          <t>Small splash x</t>
+        </is>
+      </c>
+      <c r="B260" s="81" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="C260" s="81" t="inlineStr">
+        <is>
+          <t>x the splash radius for each small meteor</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="81" t="inlineStr">
+        <is>
+          <t>Extinction min bunch</t>
+        </is>
+      </c>
+      <c r="B261" s="81" t="n">
+        <v>6</v>
+      </c>
+      <c r="C261" s="81" t="inlineStr">
+        <is>
+          <t>Extinction Event fires itself on a boss or this many dinos in the bunch (else at the last spawn)</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="81" t="inlineStr">
+        <is>
+          <t>Extinction x</t>
+        </is>
+      </c>
+      <c r="B262" s="81" t="n">
+        <v>3</v>
+      </c>
+      <c r="C262" s="81" t="inlineStr">
+        <is>
+          <t>x the meteor's damage on every dino on your side (Extinction Event, once per round played)</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="81" t="inlineStr">
+        <is>
+          <t>Extinction breaks</t>
+        </is>
+      </c>
+      <c r="B263" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="C263" s="81" t="inlineStr">
+        <is>
+          <t>sizes the Extinction Event breaks on the densest bunch's dinos (the rest break 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="81" t="inlineStr">
+        <is>
+          <t>Starfall meteors</t>
+        </is>
+      </c>
+      <c r="B264" s="81" t="n">
+        <v>20</v>
+      </c>
+      <c r="C264" s="81" t="inlineStr">
+        <is>
+          <t>Starfall: small meteors on the densest points across your side, in place of the strike</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="81" t="inlineStr">
+        <is>
+          <t>Fire line gap (studs)</t>
+        </is>
+      </c>
+      <c r="B265" s="81" t="n">
+        <v>30</v>
+      </c>
+      <c r="C265" s="81" t="inlineStr">
+        <is>
+          <t>Fire Line: craters this close along the track join into one burning strip while both last</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="81" t="inlineStr">
+        <is>
+          <t>Streak length (studs)</t>
+        </is>
+      </c>
+      <c r="B266" s="81" t="n">
+        <v>10</v>
+      </c>
+      <c r="C266" s="81" t="inlineStr">
+        <is>
+          <t>Cinder Trail: each small meteor leaves a burning strip this long for 3 s</t>
         </is>
       </c>
     </row>
@@ -13154,7 +13356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z22"/>
+  <dimension ref="A1:Z23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66667" defaultRowHeight="15" customHeight="1" outlineLevelRow="0"/>
   <cols>
     <col width="15" customWidth="1" style="81" min="1" max="1"/>
@@ -14425,6 +14627,73 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="81" t="inlineStr">
+        <is>
+          <t>Meteor Beacon</t>
+        </is>
+      </c>
+      <c r="B23" s="81" t="inlineStr">
+        <is>
+          <t>Meteors on the biggest bunch: area hits and burning craters</t>
+        </is>
+      </c>
+      <c r="C23" s="81" t="n">
+        <v>600</v>
+      </c>
+      <c r="D23" s="81" t="n">
+        <v>40</v>
+      </c>
+      <c r="E23" s="81" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="F23" s="81" t="n">
+        <v>6</v>
+      </c>
+      <c r="G23" s="81">
+        <f>D23*E23*F23</f>
+        <v/>
+      </c>
+      <c r="H23" s="81" t="n">
+        <v>999</v>
+      </c>
+      <c r="I23" s="81" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J23" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="81" t="inlineStr">
+        <is>
+          <t>Every 8 s calls a meteor on the biggest bunch of dinos on your side: area hit + burning crater. Ground only.</t>
+        </is>
+      </c>
+      <c r="L23" s="81" t="n">
+        <v>8</v>
+      </c>
+      <c r="M23" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" s="81" t="n">
+        <v>600</v>
+      </c>
+      <c r="O23" s="81" t="inlineStr">
+        <is>
+          <t>METEOR</t>
+        </is>
+      </c>
+      <c r="P23" s="81" t="n">
+        <v>150</v>
+      </c>
+      <c r="Q23" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="R23" s="81" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811" footer="0.511811"/>
   <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" firstPageNumber="1" useFirstPageNumber="0" pageOrder="downThenOver"/>
@@ -14445,7 +14714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:FL409"/>
+  <dimension ref="A1:FZ436"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66667" defaultRowHeight="15" customHeight="1" outlineLevelRow="0"/>
   <cols>
     <col width="15" customWidth="1" style="81" min="1" max="1"/>
@@ -15423,6 +15692,76 @@
       <c r="FL4" s="81" t="inlineStr">
         <is>
           <t>Hook every (s)</t>
+        </is>
+      </c>
+      <c r="FM4" s="81" t="inlineStr">
+        <is>
+          <t>Meteors</t>
+        </is>
+      </c>
+      <c r="FN4" s="81" t="inlineStr">
+        <is>
+          <t>Scatter</t>
+        </is>
+      </c>
+      <c r="FO4" s="81" t="inlineStr">
+        <is>
+          <t>Meteor every (s)</t>
+        </is>
+      </c>
+      <c r="FP4" s="81" t="inlineStr">
+        <is>
+          <t>Starfall every (s)</t>
+        </is>
+      </c>
+      <c r="FQ4" s="81" t="inlineStr">
+        <is>
+          <t>Crater (s)</t>
+        </is>
+      </c>
+      <c r="FR4" s="81" t="inlineStr">
+        <is>
+          <t>Crater amp %</t>
+        </is>
+      </c>
+      <c r="FS4" s="81" t="inlineStr">
+        <is>
+          <t>Bite miss %</t>
+        </is>
+      </c>
+      <c r="FT4" s="81" t="inlineStr">
+        <is>
+          <t>Crater freeze (s)</t>
+        </is>
+      </c>
+      <c r="FU4" s="81" t="inlineStr">
+        <is>
+          <t>Fire line</t>
+        </is>
+      </c>
+      <c r="FV4" s="81" t="inlineStr">
+        <is>
+          <t>Burn streak</t>
+        </is>
+      </c>
+      <c r="FW4" s="81" t="inlineStr">
+        <is>
+          <t>Extinction</t>
+        </is>
+      </c>
+      <c r="FX4" s="81" t="inlineStr">
+        <is>
+          <t>Side slow %</t>
+        </is>
+      </c>
+      <c r="FY4" s="81" t="inlineStr">
+        <is>
+          <t>Side slow (s)</t>
+        </is>
+      </c>
+      <c r="FZ4" s="81" t="inlineStr">
+        <is>
+          <t>Biggest breaks +</t>
         </is>
       </c>
     </row>
@@ -45198,6 +45537,1654 @@
         <is>
           <t>Yes</t>
         </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" s="81" t="inlineStr">
+        <is>
+          <t>Meteor Beacon</t>
+        </is>
+      </c>
+      <c r="B410" s="81" t="inlineStr">
+        <is>
+          <t>Impact</t>
+        </is>
+      </c>
+      <c r="C410" s="81" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D410" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="E410" s="81">
+        <f>ROUND('Towers'!$C$23*POWER('Tuning'!$B$12,D410),0)</f>
+        <v/>
+      </c>
+      <c r="F410" s="81">
+        <f>'Towers'!$C$23+E410</f>
+        <v/>
+      </c>
+      <c r="G410" s="81" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H410" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I410" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J410" s="81">
+        <f>'Towers'!$G$23*G410*H410*I410</f>
+        <v/>
+      </c>
+      <c r="K410" s="81">
+        <f>IF(J410=0,0,F410/J410)</f>
+        <v/>
+      </c>
+      <c r="L410" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M410" s="81" t="inlineStr">
+        <is>
+          <t>Heavier Rock</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" s="81" t="inlineStr">
+        <is>
+          <t>Meteor Beacon</t>
+        </is>
+      </c>
+      <c r="B411" s="81" t="inlineStr">
+        <is>
+          <t>Impact</t>
+        </is>
+      </c>
+      <c r="C411" s="81" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D411" s="81" t="n">
+        <v>2</v>
+      </c>
+      <c r="E411" s="81">
+        <f>ROUND('Towers'!$C$23*POWER('Tuning'!$B$12,D411),0)</f>
+        <v/>
+      </c>
+      <c r="F411" s="81">
+        <f>F410+E411</f>
+        <v/>
+      </c>
+      <c r="G411" s="81" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="H411" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I411" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J411" s="81">
+        <f>'Towers'!$G$23*G411*H411*I411</f>
+        <v/>
+      </c>
+      <c r="K411" s="81">
+        <f>IF(J411=0,0,F411/J411)</f>
+        <v/>
+      </c>
+      <c r="L411" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M411" s="81" t="inlineStr">
+        <is>
+          <t>Iron Core</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" s="81" t="inlineStr">
+        <is>
+          <t>Meteor Beacon</t>
+        </is>
+      </c>
+      <c r="B412" s="81" t="inlineStr">
+        <is>
+          <t>Impact</t>
+        </is>
+      </c>
+      <c r="C412" s="81" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D412" s="81" t="n">
+        <v>3</v>
+      </c>
+      <c r="E412" s="81">
+        <f>ROUND('Towers'!$C$23*POWER('Tuning'!$B$12,D412),0)</f>
+        <v/>
+      </c>
+      <c r="F412" s="81">
+        <f>F411+E412</f>
+        <v/>
+      </c>
+      <c r="G412" s="81" t="n">
+        <v>6</v>
+      </c>
+      <c r="H412" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I412" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J412" s="81">
+        <f>'Towers'!$G$23*G412*H412*I412</f>
+        <v/>
+      </c>
+      <c r="K412" s="81">
+        <f>IF(J412=0,0,F412/J412)</f>
+        <v/>
+      </c>
+      <c r="L412" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M412" s="81" t="inlineStr">
+        <is>
+          <t>Ground Zero</t>
+        </is>
+      </c>
+      <c r="BJ412" s="81" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" s="81" t="inlineStr">
+        <is>
+          <t>Meteor Beacon</t>
+        </is>
+      </c>
+      <c r="B413" s="81" t="inlineStr">
+        <is>
+          <t>Impact</t>
+        </is>
+      </c>
+      <c r="C413" s="81" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D413" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="E413" s="81">
+        <f>ROUND('Towers'!$C$23*POWER('Tuning'!$B$12,D413),0)</f>
+        <v/>
+      </c>
+      <c r="F413" s="81">
+        <f>F412+E413</f>
+        <v/>
+      </c>
+      <c r="G413" s="81" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="H413" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I413" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J413" s="81">
+        <f>J412*G413*H413*I413</f>
+        <v/>
+      </c>
+      <c r="K413" s="81">
+        <f>IF(J413=0,0,F413/J413)</f>
+        <v/>
+      </c>
+      <c r="L413" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M413" s="81" t="inlineStr">
+        <is>
+          <t>Planet Killer</t>
+        </is>
+      </c>
+      <c r="P413" s="81" t="n">
+        <v>2</v>
+      </c>
+      <c r="BJ413" s="81" t="n">
+        <v>3</v>
+      </c>
+      <c r="CI413" s="81" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="CJ413" s="81" t="inlineStr">
+        <is>
+          <t>Breaks 3, ×2 on bosses</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" s="81" t="inlineStr">
+        <is>
+          <t>Meteor Beacon</t>
+        </is>
+      </c>
+      <c r="B414" s="81" t="inlineStr">
+        <is>
+          <t>Impact</t>
+        </is>
+      </c>
+      <c r="C414" s="81" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D414" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="E414" s="81">
+        <f>ROUND('Towers'!$C$23*POWER('Tuning'!$B$12,D414),0)</f>
+        <v/>
+      </c>
+      <c r="F414" s="81">
+        <f>F413+E414</f>
+        <v/>
+      </c>
+      <c r="G414" s="81" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="H414" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I414" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J414" s="81">
+        <f>J413*G414*H414*I414</f>
+        <v/>
+      </c>
+      <c r="K414" s="81">
+        <f>IF(J414=0,0,F414/J414)</f>
+        <v/>
+      </c>
+      <c r="L414" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M414" s="81" t="inlineStr">
+        <is>
+          <t>Extinction Event</t>
+        </is>
+      </c>
+      <c r="CI414" s="81" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="CJ414" s="81" t="inlineStr">
+        <is>
+          <t>One giant meteor a round, fires itself</t>
+        </is>
+      </c>
+      <c r="FW414" s="81" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" s="81" t="inlineStr">
+        <is>
+          <t>Meteor Beacon</t>
+        </is>
+      </c>
+      <c r="B415" s="81" t="inlineStr">
+        <is>
+          <t>Sky Rocks</t>
+        </is>
+      </c>
+      <c r="C415" s="81" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D415" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="E415" s="81">
+        <f>ROUND('Towers'!$C$23*POWER('Tuning'!$B$12,D415),0)</f>
+        <v/>
+      </c>
+      <c r="F415" s="81">
+        <f>'Towers'!$C$23+E415</f>
+        <v/>
+      </c>
+      <c r="G415" s="81" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="H415" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I415" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J415" s="81">
+        <f>'Towers'!$G$23*G415*H415*I415</f>
+        <v/>
+      </c>
+      <c r="K415" s="81">
+        <f>IF(J415=0,0,F415/J415)</f>
+        <v/>
+      </c>
+      <c r="L415" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M415" s="81" t="inlineStr">
+        <is>
+          <t>Rock Chunks</t>
+        </is>
+      </c>
+      <c r="FM415" s="81" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" s="81" t="inlineStr">
+        <is>
+          <t>Meteor Beacon</t>
+        </is>
+      </c>
+      <c r="B416" s="81" t="inlineStr">
+        <is>
+          <t>Sky Rocks</t>
+        </is>
+      </c>
+      <c r="C416" s="81" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D416" s="81" t="n">
+        <v>2</v>
+      </c>
+      <c r="E416" s="81">
+        <f>ROUND('Towers'!$C$23*POWER('Tuning'!$B$12,D416),0)</f>
+        <v/>
+      </c>
+      <c r="F416" s="81">
+        <f>F415+E416</f>
+        <v/>
+      </c>
+      <c r="G416" s="81" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="H416" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I416" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J416" s="81">
+        <f>'Towers'!$G$23*G416*H416*I416</f>
+        <v/>
+      </c>
+      <c r="K416" s="81">
+        <f>IF(J416=0,0,F416/J416)</f>
+        <v/>
+      </c>
+      <c r="L416" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M416" s="81" t="inlineStr">
+        <is>
+          <t>Twin Fall</t>
+        </is>
+      </c>
+      <c r="FM416" s="81" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" s="81" t="inlineStr">
+        <is>
+          <t>Meteor Beacon</t>
+        </is>
+      </c>
+      <c r="B417" s="81" t="inlineStr">
+        <is>
+          <t>Sky Rocks</t>
+        </is>
+      </c>
+      <c r="C417" s="81" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D417" s="81" t="n">
+        <v>3</v>
+      </c>
+      <c r="E417" s="81">
+        <f>ROUND('Towers'!$C$23*POWER('Tuning'!$B$12,D417),0)</f>
+        <v/>
+      </c>
+      <c r="F417" s="81">
+        <f>F416+E417</f>
+        <v/>
+      </c>
+      <c r="G417" s="81" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="H417" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I417" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J417" s="81">
+        <f>'Towers'!$G$23*G417*H417*I417</f>
+        <v/>
+      </c>
+      <c r="K417" s="81">
+        <f>IF(J417=0,0,F417/J417)</f>
+        <v/>
+      </c>
+      <c r="L417" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M417" s="81" t="inlineStr">
+        <is>
+          <t>Fireball Flurry</t>
+        </is>
+      </c>
+      <c r="FM417" s="81" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" s="81" t="inlineStr">
+        <is>
+          <t>Meteor Beacon</t>
+        </is>
+      </c>
+      <c r="B418" s="81" t="inlineStr">
+        <is>
+          <t>Sky Rocks</t>
+        </is>
+      </c>
+      <c r="C418" s="81" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D418" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="E418" s="81">
+        <f>ROUND('Towers'!$C$23*POWER('Tuning'!$B$12,D418),0)</f>
+        <v/>
+      </c>
+      <c r="F418" s="81">
+        <f>F417+E418</f>
+        <v/>
+      </c>
+      <c r="G418" s="81" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="H418" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I418" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J418" s="81">
+        <f>J417*G418*H418*I418</f>
+        <v/>
+      </c>
+      <c r="K418" s="81">
+        <f>IF(J418=0,0,F418/J418)</f>
+        <v/>
+      </c>
+      <c r="L418" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M418" s="81" t="inlineStr">
+        <is>
+          <t>Endless Rain</t>
+        </is>
+      </c>
+      <c r="CI418" s="81" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="CJ418" s="81" t="inlineStr">
+        <is>
+          <t>A small meteor every 4 s</t>
+        </is>
+      </c>
+      <c r="FO418" s="81" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" s="81" t="inlineStr">
+        <is>
+          <t>Meteor Beacon</t>
+        </is>
+      </c>
+      <c r="B419" s="81" t="inlineStr">
+        <is>
+          <t>Sky Rocks</t>
+        </is>
+      </c>
+      <c r="C419" s="81" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D419" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="E419" s="81">
+        <f>ROUND('Towers'!$C$23*POWER('Tuning'!$B$12,D419),0)</f>
+        <v/>
+      </c>
+      <c r="F419" s="81">
+        <f>F418+E419</f>
+        <v/>
+      </c>
+      <c r="G419" s="81" t="n">
+        <v>3.388</v>
+      </c>
+      <c r="H419" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I419" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J419" s="81">
+        <f>J418*G419*H419*I419</f>
+        <v/>
+      </c>
+      <c r="K419" s="81">
+        <f>IF(J419=0,0,F419/J419)</f>
+        <v/>
+      </c>
+      <c r="L419" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M419" s="81" t="inlineStr">
+        <is>
+          <t>Starfall</t>
+        </is>
+      </c>
+      <c r="CI419" s="81" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="CJ419" s="81" t="inlineStr">
+        <is>
+          <t>20 meteors across your side every 15 s</t>
+        </is>
+      </c>
+      <c r="FP419" s="81" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" s="81" t="inlineStr">
+        <is>
+          <t>Meteor Beacon</t>
+        </is>
+      </c>
+      <c r="B420" s="81" t="inlineStr">
+        <is>
+          <t>Aftermath</t>
+        </is>
+      </c>
+      <c r="C420" s="81" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D420" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="E420" s="81">
+        <f>ROUND('Towers'!$C$23*POWER('Tuning'!$B$12,D420),0)</f>
+        <v/>
+      </c>
+      <c r="F420" s="81">
+        <f>'Towers'!$C$23+E420</f>
+        <v/>
+      </c>
+      <c r="G420" s="81" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="H420" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I420" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J420" s="81">
+        <f>'Towers'!$G$23*G420*H420*I420</f>
+        <v/>
+      </c>
+      <c r="K420" s="81">
+        <f>IF(J420=0,0,F420/J420)</f>
+        <v/>
+      </c>
+      <c r="L420" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M420" s="81" t="inlineStr">
+        <is>
+          <t>Hot Crater</t>
+        </is>
+      </c>
+      <c r="X420" s="81" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" s="81" t="inlineStr">
+        <is>
+          <t>Meteor Beacon</t>
+        </is>
+      </c>
+      <c r="B421" s="81" t="inlineStr">
+        <is>
+          <t>Aftermath</t>
+        </is>
+      </c>
+      <c r="C421" s="81" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D421" s="81" t="n">
+        <v>2</v>
+      </c>
+      <c r="E421" s="81">
+        <f>ROUND('Towers'!$C$23*POWER('Tuning'!$B$12,D421),0)</f>
+        <v/>
+      </c>
+      <c r="F421" s="81">
+        <f>F420+E421</f>
+        <v/>
+      </c>
+      <c r="G421" s="81" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="H421" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I421" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J421" s="81">
+        <f>'Towers'!$G$23*G421*H421*I421</f>
+        <v/>
+      </c>
+      <c r="K421" s="81">
+        <f>IF(J421=0,0,F421/J421)</f>
+        <v/>
+      </c>
+      <c r="L421" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M421" s="81" t="inlineStr">
+        <is>
+          <t>Ash Cloud</t>
+        </is>
+      </c>
+      <c r="X421" s="81" t="n">
+        <v>20</v>
+      </c>
+      <c r="FH421" s="81" t="n">
+        <v>30</v>
+      </c>
+      <c r="FS421" s="81" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" s="81" t="inlineStr">
+        <is>
+          <t>Meteor Beacon</t>
+        </is>
+      </c>
+      <c r="B422" s="81" t="inlineStr">
+        <is>
+          <t>Aftermath</t>
+        </is>
+      </c>
+      <c r="C422" s="81" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D422" s="81" t="n">
+        <v>3</v>
+      </c>
+      <c r="E422" s="81">
+        <f>ROUND('Towers'!$C$23*POWER('Tuning'!$B$12,D422),0)</f>
+        <v/>
+      </c>
+      <c r="F422" s="81">
+        <f>F421+E422</f>
+        <v/>
+      </c>
+      <c r="G422" s="81" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="H422" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I422" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J422" s="81">
+        <f>'Towers'!$G$23*G422*H422*I422</f>
+        <v/>
+      </c>
+      <c r="K422" s="81">
+        <f>IF(J422=0,0,F422/J422)</f>
+        <v/>
+      </c>
+      <c r="L422" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M422" s="81" t="inlineStr">
+        <is>
+          <t>Shockwave Ring</t>
+        </is>
+      </c>
+      <c r="W422" s="81" t="n">
+        <v>6</v>
+      </c>
+      <c r="X422" s="81" t="n">
+        <v>30</v>
+      </c>
+      <c r="FH422" s="81" t="n">
+        <v>30</v>
+      </c>
+      <c r="FS422" s="81" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" s="81" t="inlineStr">
+        <is>
+          <t>Meteor Beacon</t>
+        </is>
+      </c>
+      <c r="B423" s="81" t="inlineStr">
+        <is>
+          <t>Aftermath</t>
+        </is>
+      </c>
+      <c r="C423" s="81" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D423" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="E423" s="81">
+        <f>ROUND('Towers'!$C$23*POWER('Tuning'!$B$12,D423),0)</f>
+        <v/>
+      </c>
+      <c r="F423" s="81">
+        <f>F422+E423</f>
+        <v/>
+      </c>
+      <c r="G423" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="H423" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I423" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J423" s="81">
+        <f>J422*G423*H423*I423</f>
+        <v/>
+      </c>
+      <c r="K423" s="81">
+        <f>IF(J423=0,0,F423/J423)</f>
+        <v/>
+      </c>
+      <c r="L423" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M423" s="81" t="inlineStr">
+        <is>
+          <t>Long Burn</t>
+        </is>
+      </c>
+      <c r="X423" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="CI423" s="81" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="CJ423" s="81" t="inlineStr">
+        <is>
+          <t>Craters last 8 s, hotter</t>
+        </is>
+      </c>
+      <c r="FQ423" s="81" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" s="81" t="inlineStr">
+        <is>
+          <t>Meteor Beacon</t>
+        </is>
+      </c>
+      <c r="B424" s="81" t="inlineStr">
+        <is>
+          <t>Aftermath</t>
+        </is>
+      </c>
+      <c r="C424" s="81" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D424" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="E424" s="81">
+        <f>ROUND('Towers'!$C$23*POWER('Tuning'!$B$12,D424),0)</f>
+        <v/>
+      </c>
+      <c r="F424" s="81">
+        <f>F423+E424</f>
+        <v/>
+      </c>
+      <c r="G424" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="H424" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I424" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J424" s="81">
+        <f>J423*G424*H424*I424</f>
+        <v/>
+      </c>
+      <c r="K424" s="81">
+        <f>IF(J424=0,0,F424/J424)</f>
+        <v/>
+      </c>
+      <c r="L424" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M424" s="81" t="inlineStr">
+        <is>
+          <t>Fire Line</t>
+        </is>
+      </c>
+      <c r="X424" s="81" t="n">
+        <v>54</v>
+      </c>
+      <c r="CI424" s="81" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="CJ424" s="81" t="inlineStr">
+        <is>
+          <t>Craters join into one burning strip</t>
+        </is>
+      </c>
+      <c r="FU424" s="81" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" s="81" t="inlineStr">
+        <is>
+          <t>Meteor Beacon</t>
+        </is>
+      </c>
+      <c r="B425" s="81" t="inlineStr">
+        <is>
+          <t>Impact</t>
+        </is>
+      </c>
+      <c r="C425" s="81" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D425" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="E425" s="81">
+        <f>E413</f>
+        <v/>
+      </c>
+      <c r="F425" s="81">
+        <f>F413</f>
+        <v/>
+      </c>
+      <c r="G425" s="81" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="H425" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I425" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="L425" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M425" s="81" t="inlineStr">
+        <is>
+          <t>Plate Cracker</t>
+        </is>
+      </c>
+      <c r="N425" s="81" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="CI425" s="81" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="CJ425" s="81" t="inlineStr">
+        <is>
+          <t>Meteors cut through armour</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" s="81" t="inlineStr">
+        <is>
+          <t>Meteor Beacon</t>
+        </is>
+      </c>
+      <c r="B426" s="81" t="inlineStr">
+        <is>
+          <t>Impact</t>
+        </is>
+      </c>
+      <c r="C426" s="81" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D426" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="E426" s="81">
+        <f>E413</f>
+        <v/>
+      </c>
+      <c r="F426" s="81">
+        <f>F413</f>
+        <v/>
+      </c>
+      <c r="G426" s="81" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="H426" s="81" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I426" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="L426" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M426" s="81" t="inlineStr">
+        <is>
+          <t>Quick Call</t>
+        </is>
+      </c>
+      <c r="CI426" s="81" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="CJ426" s="81" t="inlineStr">
+        <is>
+          <t>Meteors fall 50% more often</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" s="81" t="inlineStr">
+        <is>
+          <t>Meteor Beacon</t>
+        </is>
+      </c>
+      <c r="B427" s="81" t="inlineStr">
+        <is>
+          <t>Impact</t>
+        </is>
+      </c>
+      <c r="C427" s="81" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D427" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="E427" s="81">
+        <f>E414</f>
+        <v/>
+      </c>
+      <c r="F427" s="81">
+        <f>F414</f>
+        <v/>
+      </c>
+      <c r="G427" s="81" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="H427" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I427" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="L427" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M427" s="81" t="inlineStr">
+        <is>
+          <t>Dino Killer</t>
+        </is>
+      </c>
+      <c r="CI427" s="81" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="CJ427" s="81" t="inlineStr">
+        <is>
+          <t>Breaks the biggest dino it hits 2 extra sizes</t>
+        </is>
+      </c>
+      <c r="FZ427" s="81" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" s="81" t="inlineStr">
+        <is>
+          <t>Meteor Beacon</t>
+        </is>
+      </c>
+      <c r="B428" s="81" t="inlineStr">
+        <is>
+          <t>Impact</t>
+        </is>
+      </c>
+      <c r="C428" s="81" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D428" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="E428" s="81">
+        <f>E414</f>
+        <v/>
+      </c>
+      <c r="F428" s="81">
+        <f>F414</f>
+        <v/>
+      </c>
+      <c r="G428" s="81" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="H428" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I428" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="L428" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M428" s="81" t="inlineStr">
+        <is>
+          <t>Impact Winter</t>
+        </is>
+      </c>
+      <c r="CI428" s="81" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="CJ428" s="81" t="inlineStr">
+        <is>
+          <t>Every dino on your side slowed after each hit</t>
+        </is>
+      </c>
+      <c r="FX428" s="81" t="n">
+        <v>30</v>
+      </c>
+      <c r="FY428" s="81" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" s="81" t="inlineStr">
+        <is>
+          <t>Meteor Beacon</t>
+        </is>
+      </c>
+      <c r="B429" s="81" t="inlineStr">
+        <is>
+          <t>Sky Rocks</t>
+        </is>
+      </c>
+      <c r="C429" s="81" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D429" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="E429" s="81">
+        <f>E418</f>
+        <v/>
+      </c>
+      <c r="F429" s="81">
+        <f>F418</f>
+        <v/>
+      </c>
+      <c r="G429" s="81" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="H429" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I429" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="L429" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M429" s="81" t="inlineStr">
+        <is>
+          <t>Scatter Field</t>
+        </is>
+      </c>
+      <c r="CI429" s="81" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="CJ429" s="81" t="inlineStr">
+        <is>
+          <t>Meteors land all along the track</t>
+        </is>
+      </c>
+      <c r="FN429" s="81" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" s="81" t="inlineStr">
+        <is>
+          <t>Meteor Beacon</t>
+        </is>
+      </c>
+      <c r="B430" s="81" t="inlineStr">
+        <is>
+          <t>Sky Rocks</t>
+        </is>
+      </c>
+      <c r="C430" s="81" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D430" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="E430" s="81">
+        <f>E418</f>
+        <v/>
+      </c>
+      <c r="F430" s="81">
+        <f>F418</f>
+        <v/>
+      </c>
+      <c r="G430" s="81" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="H430" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I430" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="L430" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M430" s="81" t="inlineStr">
+        <is>
+          <t>Cinder Trail</t>
+        </is>
+      </c>
+      <c r="X430" s="81" t="n">
+        <v>20</v>
+      </c>
+      <c r="CI430" s="81" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="CJ430" s="81" t="inlineStr">
+        <is>
+          <t>Small meteors leave a burning streak</t>
+        </is>
+      </c>
+      <c r="FV430" s="81" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" s="81" t="inlineStr">
+        <is>
+          <t>Meteor Beacon</t>
+        </is>
+      </c>
+      <c r="B431" s="81" t="inlineStr">
+        <is>
+          <t>Sky Rocks</t>
+        </is>
+      </c>
+      <c r="C431" s="81" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D431" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="E431" s="81">
+        <f>E419</f>
+        <v/>
+      </c>
+      <c r="F431" s="81">
+        <f>F419</f>
+        <v/>
+      </c>
+      <c r="G431" s="81" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H431" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I431" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="L431" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M431" s="81" t="inlineStr">
+        <is>
+          <t>Comet Tail</t>
+        </is>
+      </c>
+      <c r="CI431" s="81" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="CJ431" s="81" t="inlineStr">
+        <is>
+          <t>A comet sweeps the whole track once a round</t>
+        </is>
+      </c>
+      <c r="CS431" s="81" t="n">
+        <v>6</v>
+      </c>
+      <c r="FK431" s="81" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" s="81" t="inlineStr">
+        <is>
+          <t>Meteor Beacon</t>
+        </is>
+      </c>
+      <c r="B432" s="81" t="inlineStr">
+        <is>
+          <t>Sky Rocks</t>
+        </is>
+      </c>
+      <c r="C432" s="81" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D432" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="E432" s="81">
+        <f>E419</f>
+        <v/>
+      </c>
+      <c r="F432" s="81">
+        <f>F419</f>
+        <v/>
+      </c>
+      <c r="G432" s="81" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="H432" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I432" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="L432" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M432" s="81" t="inlineStr">
+        <is>
+          <t>Shooting Stars</t>
+        </is>
+      </c>
+      <c r="CI432" s="81" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="CJ432" s="81" t="inlineStr">
+        <is>
+          <t>Meteors can hit flyers</t>
+        </is>
+      </c>
+      <c r="DW432" s="81" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" s="81" t="inlineStr">
+        <is>
+          <t>Meteor Beacon</t>
+        </is>
+      </c>
+      <c r="B433" s="81" t="inlineStr">
+        <is>
+          <t>Aftermath</t>
+        </is>
+      </c>
+      <c r="C433" s="81" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D433" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="E433" s="81">
+        <f>E423</f>
+        <v/>
+      </c>
+      <c r="F433" s="81">
+        <f>F423</f>
+        <v/>
+      </c>
+      <c r="G433" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="H433" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I433" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="L433" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M433" s="81" t="inlineStr">
+        <is>
+          <t>Glass Crater</t>
+        </is>
+      </c>
+      <c r="X433" s="81" t="n">
+        <v>40</v>
+      </c>
+      <c r="AM433" s="81" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="CI433" s="81" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="CJ433" s="81" t="inlineStr">
+        <is>
+          <t>Craters strip armour</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" s="81" t="inlineStr">
+        <is>
+          <t>Meteor Beacon</t>
+        </is>
+      </c>
+      <c r="B434" s="81" t="inlineStr">
+        <is>
+          <t>Aftermath</t>
+        </is>
+      </c>
+      <c r="C434" s="81" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D434" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="E434" s="81">
+        <f>E423</f>
+        <v/>
+      </c>
+      <c r="F434" s="81">
+        <f>F423</f>
+        <v/>
+      </c>
+      <c r="G434" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="H434" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I434" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="L434" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M434" s="81" t="inlineStr">
+        <is>
+          <t>Scorch Marks</t>
+        </is>
+      </c>
+      <c r="X434" s="81" t="n">
+        <v>40</v>
+      </c>
+      <c r="CI434" s="81" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="CJ434" s="81" t="inlineStr">
+        <is>
+          <t>Dinos crossing a crater take +15%</t>
+        </is>
+      </c>
+      <c r="FR434" s="81" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" s="81" t="inlineStr">
+        <is>
+          <t>Meteor Beacon</t>
+        </is>
+      </c>
+      <c r="B435" s="81" t="inlineStr">
+        <is>
+          <t>Aftermath</t>
+        </is>
+      </c>
+      <c r="C435" s="81" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D435" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="E435" s="81">
+        <f>E424</f>
+        <v/>
+      </c>
+      <c r="F435" s="81">
+        <f>F424</f>
+        <v/>
+      </c>
+      <c r="G435" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="H435" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I435" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="L435" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M435" s="81" t="inlineStr">
+        <is>
+          <t>Blinding Dust</t>
+        </is>
+      </c>
+      <c r="X435" s="81" t="n">
+        <v>55</v>
+      </c>
+      <c r="CI435" s="81" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="CJ435" s="81" t="inlineStr">
+        <is>
+          <t>Dinos in the ash can't bite or throw</t>
+        </is>
+      </c>
+      <c r="FH435" s="81" t="n">
+        <v>100</v>
+      </c>
+      <c r="FS435" s="81" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" s="81" t="inlineStr">
+        <is>
+          <t>Meteor Beacon</t>
+        </is>
+      </c>
+      <c r="B436" s="81" t="inlineStr">
+        <is>
+          <t>Aftermath</t>
+        </is>
+      </c>
+      <c r="C436" s="81" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D436" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="E436" s="81">
+        <f>E424</f>
+        <v/>
+      </c>
+      <c r="F436" s="81">
+        <f>F424</f>
+        <v/>
+      </c>
+      <c r="G436" s="81" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="H436" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="I436" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="L436" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M436" s="81" t="inlineStr">
+        <is>
+          <t>New Ice Age</t>
+        </is>
+      </c>
+      <c r="CI436" s="81" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="CJ436" s="81" t="inlineStr">
+        <is>
+          <t>Craters freeze dinos solid for 2 s</t>
+        </is>
+      </c>
+      <c r="FT436" s="81" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
9i T128 step 1: Volcano Vent rows, metrics, Shared/Vent, Near track (unreleased)
Towers row 24 VENT (600 cash, 30 x 0.0833/s on 4, range 20, 200 HP,
600 Amber) and the new Towers column AA Near track (studs) = 8 (the
Vent only; Shared/Placement.checkNear, measured to the lane), Tuning
VOLCANO VENT block, 14 new Tower Upgrades columns (GA-GN, KEY_ONLY
VENT; Throw miss % and the Resin Wall (s) shared with it), 27 rows
(PLAN 9i, #339). Vent stays off BREAK_PATHS.

value.py vent_edps / vent_obsidian reproduce the Director's check
exactly: Magma T4 159/194/165, T5 304/277/330, 339/321/406,
319/288/344; Pressure T4 142/142/164, T5 291/261/247 (x2), 319/286/282;
Obsidian slots as #339. Damage T5 c/e 167-274 (<= 177 / 284); best T2
r11-20 202 (<= 386); no DEAD/DOMINANT; options clean. Unreleased. Not
playtested.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Storm-Split-Balance.xlsx
+++ b/Storm-Split-Balance.xlsx
@@ -9500,7 +9500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E266"/>
+  <dimension ref="A1:E281"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66667" defaultRowHeight="15" customHeight="1" outlineLevelRow="0"/>
   <cols>
     <col width="34" customWidth="1" style="81" min="1" max="1"/>
@@ -10178,6 +10178,7 @@
       </c>
       <c r="E38" s="17" t="n"/>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="31" t="inlineStr">
         <is>
@@ -10248,6 +10249,7 @@
         </is>
       </c>
     </row>
+    <row r="44"/>
     <row r="45">
       <c r="A45" s="31" t="inlineStr">
         <is>
@@ -10398,6 +10400,7 @@
         </is>
       </c>
     </row>
+    <row r="53"/>
     <row r="54">
       <c r="A54" s="31" t="inlineStr">
         <is>
@@ -10448,6 +10451,7 @@
         </is>
       </c>
     </row>
+    <row r="57"/>
     <row r="58">
       <c r="A58" s="31" t="inlineStr">
         <is>
@@ -10518,6 +10522,7 @@
         </is>
       </c>
     </row>
+    <row r="62"/>
     <row r="63">
       <c r="A63" s="31" t="inlineStr">
         <is>
@@ -10568,6 +10573,7 @@
         </is>
       </c>
     </row>
+    <row r="66"/>
     <row r="67">
       <c r="A67" s="31" t="inlineStr">
         <is>
@@ -10758,6 +10764,7 @@
         </is>
       </c>
     </row>
+    <row r="77"/>
     <row r="78">
       <c r="A78" s="31" t="inlineStr">
         <is>
@@ -10905,6 +10912,7 @@
         </is>
       </c>
     </row>
+    <row r="86"/>
     <row r="87">
       <c r="A87" s="31" t="inlineStr">
         <is>
@@ -11012,6 +11020,7 @@
         </is>
       </c>
     </row>
+    <row r="93"/>
     <row r="94" s="90">
       <c r="A94" s="31" t="inlineStr">
         <is>
@@ -11039,6 +11048,7 @@
         </is>
       </c>
     </row>
+    <row r="96"/>
     <row r="97">
       <c r="A97" s="31" t="inlineStr">
         <is>
@@ -11066,6 +11076,7 @@
         </is>
       </c>
     </row>
+    <row r="99"/>
     <row r="100">
       <c r="A100" s="99" t="inlineStr">
         <is>
@@ -11113,6 +11124,7 @@
         </is>
       </c>
     </row>
+    <row r="103"/>
     <row r="104">
       <c r="A104" s="99" t="inlineStr">
         <is>
@@ -11203,6 +11215,7 @@
         </is>
       </c>
     </row>
+    <row r="109"/>
     <row r="110">
       <c r="A110" s="99" t="inlineStr">
         <is>
@@ -11385,6 +11398,7 @@
         </is>
       </c>
     </row>
+    <row r="123"/>
     <row r="124">
       <c r="A124" s="99" t="inlineStr">
         <is>
@@ -11438,6 +11452,7 @@
         </is>
       </c>
     </row>
+    <row r="128"/>
     <row r="129">
       <c r="A129" s="99" t="inlineStr">
         <is>
@@ -11577,6 +11592,7 @@
         </is>
       </c>
     </row>
+    <row r="140"/>
     <row r="141">
       <c r="A141" s="99" t="inlineStr">
         <is>
@@ -12319,6 +12335,7 @@
         </is>
       </c>
     </row>
+    <row r="191"/>
     <row r="192">
       <c r="A192" s="81" t="inlineStr">
         <is>
@@ -12431,6 +12448,7 @@
         </is>
       </c>
     </row>
+    <row r="200"/>
     <row r="201">
       <c r="A201" s="81" t="inlineStr">
         <is>
@@ -12835,6 +12853,7 @@
         </is>
       </c>
     </row>
+    <row r="229"/>
     <row r="230">
       <c r="A230" s="81" t="inlineStr">
         <is>
@@ -13022,6 +13041,7 @@
         </is>
       </c>
     </row>
+    <row r="243"/>
     <row r="244">
       <c r="A244" s="81" t="inlineStr">
         <is>
@@ -13134,6 +13154,7 @@
         </is>
       </c>
     </row>
+    <row r="252"/>
     <row r="253">
       <c r="A253" s="81" t="inlineStr">
         <is>
@@ -13333,6 +13354,208 @@
       <c r="C266" s="81" t="inlineStr">
         <is>
           <t>Cinder Trail: each small meteor leaves a burning strip this long for 3 s</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>VOLCANO VENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>Flow length (studs)</t>
+        </is>
+      </c>
+      <c r="B269" t="n">
+        <v>24</v>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>studs of track a Volcano Vent's lava covers, centred on the track point nearest it (x Flow length x; Shared/Vent)</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>Flow (s)</t>
+        </is>
+      </c>
+      <c r="B270" t="n">
+        <v>6</v>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>s the lava stays down when the build sets no Flow (s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>Flow burn DPS</t>
+        </is>
+      </c>
+      <c r="B271" t="n">
+        <v>8</v>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>lava burn a second on each dino in it (x Damage x x the team's level)</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>Flow shove (studs/s)</t>
+        </is>
+      </c>
+      <c r="B272" t="n">
+        <v>3</v>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>studs a second the lava shoves a dino off its path (not a slow; bosses aren't shoved)</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>Shove max (studs)</t>
+        </is>
+      </c>
+      <c r="B273" t="n">
+        <v>4</v>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>the furthest the lava shoves a dino off its path (it walks back after the flow)</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>Geyser x</t>
+        </is>
+      </c>
+      <c r="B274" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>x the eruption's damage for a Geyser burst between eruptions</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>Crust (s)</t>
+        </is>
+      </c>
+      <c r="B275" t="n">
+        <v>6</v>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>s a flow's stretch stays crust after the lava (Obsidian)</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>Crust slow %</t>
+        </is>
+      </c>
+      <c r="B276" t="n">
+        <v>30</v>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>dinos on the crust are slowed this much</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>Lava bomb x</t>
+        </is>
+      </c>
+      <c r="B277" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>x the eruption's damage for each Lava Bombs bomb</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>Lava bombs</t>
+        </is>
+      </c>
+      <c r="B278" t="n">
+        <v>6</v>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>bombs Lava Bombs throws at the biggest dinos in range each eruption</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>Extra vent x</t>
+        </is>
+      </c>
+      <c r="B279" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>Ring of Fire: each small vent's eruption, x the main one's size</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>Supervolcano (s)</t>
+        </is>
+      </c>
+      <c r="B280" t="n">
+        <v>4</v>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>Supervolcano: once per round played every dino on your side is in lava this long</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>Ash (s)</t>
+        </is>
+      </c>
+      <c r="B281" t="n">
+        <v>5</v>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>Ash Blanket: s the ash after each eruption makes dinos on your side miss throws</t>
         </is>
       </c>
     </row>
@@ -13356,7 +13579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z23"/>
+  <dimension ref="A1:AA24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66667" defaultRowHeight="15" customHeight="1" outlineLevelRow="0"/>
   <cols>
     <col width="15" customWidth="1" style="81" min="1" max="1"/>
@@ -13559,6 +13782,11 @@
           <t>Walkers</t>
         </is>
       </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>Near track (studs)</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="13.65" customHeight="1" s="90">
       <c r="A5" s="43" t="inlineStr">
@@ -14692,6 +14920,76 @@
       </c>
       <c r="R23" s="81" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Volcano Vent</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Lava on one stretch of track: burns, shoves, crust</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>600</v>
+      </c>
+      <c r="D24" t="n">
+        <v>30</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="F24" t="n">
+        <v>4</v>
+      </c>
+      <c r="G24">
+        <f>D24*E24*F24</f>
+        <v/>
+      </c>
+      <c r="H24" t="n">
+        <v>20</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Erupts every 12 s: lava floods its stretch of track for 6 s; dinos burn and are shoved aside.</t>
+        </is>
+      </c>
+      <c r="L24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" t="n">
+        <v>600</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>VENT</t>
+        </is>
+      </c>
+      <c r="P24" t="n">
+        <v>200</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>0</v>
+      </c>
+      <c r="R24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA24" t="n">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -14714,7 +15012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:FZ436"/>
+  <dimension ref="A1:GN463"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66667" defaultRowHeight="15" customHeight="1" outlineLevelRow="0"/>
   <cols>
     <col width="15" customWidth="1" style="81" min="1" max="1"/>
@@ -15762,6 +16060,76 @@
       <c r="FZ4" s="81" t="inlineStr">
         <is>
           <t>Biggest breaks +</t>
+        </is>
+      </c>
+      <c r="GA4" t="inlineStr">
+        <is>
+          <t>Flow (s)</t>
+        </is>
+      </c>
+      <c r="GB4" t="inlineStr">
+        <is>
+          <t>Flow length x</t>
+        </is>
+      </c>
+      <c r="GC4" t="inlineStr">
+        <is>
+          <t>Burn breaks</t>
+        </is>
+      </c>
+      <c r="GD4" t="inlineStr">
+        <is>
+          <t>Geyser every (s)</t>
+        </is>
+      </c>
+      <c r="GE4" t="inlineStr">
+        <is>
+          <t>Extra vents</t>
+        </is>
+      </c>
+      <c r="GF4" t="inlineStr">
+        <is>
+          <t>Lava bombs</t>
+        </is>
+      </c>
+      <c r="GG4" t="inlineStr">
+        <is>
+          <t>Boss erupt</t>
+        </is>
+      </c>
+      <c r="GH4" t="inlineStr">
+        <is>
+          <t>Side throw miss %</t>
+        </is>
+      </c>
+      <c r="GI4" t="inlineStr">
+        <is>
+          <t>Supervolcano</t>
+        </is>
+      </c>
+      <c r="GJ4" t="inlineStr">
+        <is>
+          <t>Crust</t>
+        </is>
+      </c>
+      <c r="GK4" t="inlineStr">
+        <is>
+          <t>Crust DPS</t>
+        </is>
+      </c>
+      <c r="GL4" t="inlineStr">
+        <is>
+          <t>Maze (studs)</t>
+        </is>
+      </c>
+      <c r="GM4" t="inlineStr">
+        <is>
+          <t>Freeze flow (s)</t>
+        </is>
+      </c>
+      <c r="GN4" t="inlineStr">
+        <is>
+          <t>Throw resist %</t>
         </is>
       </c>
     </row>
@@ -47184,6 +47552,1630 @@
         </is>
       </c>
       <c r="FT436" s="81" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>Volcano Vent</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>Magma</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D437" t="n">
+        <v>1</v>
+      </c>
+      <c r="E437">
+        <f>ROUND('Towers'!$C$24*POWER('Tuning'!$B$12,D437),0)</f>
+        <v/>
+      </c>
+      <c r="F437">
+        <f>'Towers'!$C$24+E437</f>
+        <v/>
+      </c>
+      <c r="G437" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="H437" t="n">
+        <v>1</v>
+      </c>
+      <c r="I437" t="n">
+        <v>1</v>
+      </c>
+      <c r="J437">
+        <f>'Towers'!$G$24*G437*H437*I437</f>
+        <v/>
+      </c>
+      <c r="K437">
+        <f>IF(J437=0,0,F437/J437)</f>
+        <v/>
+      </c>
+      <c r="L437" t="n">
+        <v>1</v>
+      </c>
+      <c r="M437" t="inlineStr">
+        <is>
+          <t>Hot Rock</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>Volcano Vent</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>Magma</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D438" t="n">
+        <v>2</v>
+      </c>
+      <c r="E438">
+        <f>ROUND('Towers'!$C$24*POWER('Tuning'!$B$12,D438),0)</f>
+        <v/>
+      </c>
+      <c r="F438">
+        <f>F437+E438</f>
+        <v/>
+      </c>
+      <c r="G438" t="n">
+        <v>3</v>
+      </c>
+      <c r="H438" t="n">
+        <v>1</v>
+      </c>
+      <c r="I438" t="n">
+        <v>1</v>
+      </c>
+      <c r="J438">
+        <f>'Towers'!$G$24*G438*H438*I438</f>
+        <v/>
+      </c>
+      <c r="K438">
+        <f>IF(J438=0,0,F438/J438)</f>
+        <v/>
+      </c>
+      <c r="L438" t="n">
+        <v>1</v>
+      </c>
+      <c r="M438" t="inlineStr">
+        <is>
+          <t>Searing Flow</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>Volcano Vent</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>Magma</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D439" t="n">
+        <v>3</v>
+      </c>
+      <c r="E439">
+        <f>ROUND('Towers'!$C$24*POWER('Tuning'!$B$12,D439),0)</f>
+        <v/>
+      </c>
+      <c r="F439">
+        <f>F438+E439</f>
+        <v/>
+      </c>
+      <c r="G439" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="H439" t="n">
+        <v>1</v>
+      </c>
+      <c r="I439" t="n">
+        <v>1</v>
+      </c>
+      <c r="J439">
+        <f>'Towers'!$G$24*G439*H439*I439</f>
+        <v/>
+      </c>
+      <c r="K439">
+        <f>IF(J439=0,0,F439/J439)</f>
+        <v/>
+      </c>
+      <c r="L439" t="n">
+        <v>1</v>
+      </c>
+      <c r="M439" t="inlineStr">
+        <is>
+          <t>Lava Lake</t>
+        </is>
+      </c>
+      <c r="GA439" t="n">
+        <v>10</v>
+      </c>
+      <c r="GC439" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>Volcano Vent</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>Magma</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D440" t="n">
+        <v>4</v>
+      </c>
+      <c r="E440">
+        <f>ROUND('Towers'!$C$24*POWER('Tuning'!$B$12,D440),0)</f>
+        <v/>
+      </c>
+      <c r="F440">
+        <f>F439+E440</f>
+        <v/>
+      </c>
+      <c r="G440" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="H440" t="n">
+        <v>1</v>
+      </c>
+      <c r="I440" t="n">
+        <v>1</v>
+      </c>
+      <c r="J440">
+        <f>J439*G440*H440*I440</f>
+        <v/>
+      </c>
+      <c r="K440">
+        <f>IF(J440=0,0,F440/J440)</f>
+        <v/>
+      </c>
+      <c r="L440" t="n">
+        <v>1</v>
+      </c>
+      <c r="M440" t="inlineStr">
+        <is>
+          <t>White Hot</t>
+        </is>
+      </c>
+      <c r="N440" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="CI440" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="CJ440" t="inlineStr">
+        <is>
+          <t>Lava melts armour</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>Volcano Vent</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>Magma</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D441" t="n">
+        <v>5</v>
+      </c>
+      <c r="E441">
+        <f>ROUND('Towers'!$C$24*POWER('Tuning'!$B$12,D441),0)</f>
+        <v/>
+      </c>
+      <c r="F441">
+        <f>F440+E441</f>
+        <v/>
+      </c>
+      <c r="G441" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H441" t="n">
+        <v>1</v>
+      </c>
+      <c r="I441" t="n">
+        <v>1</v>
+      </c>
+      <c r="J441">
+        <f>J440*G441*H441*I441</f>
+        <v/>
+      </c>
+      <c r="K441">
+        <f>IF(J441=0,0,F441/J441)</f>
+        <v/>
+      </c>
+      <c r="L441" t="n">
+        <v>1</v>
+      </c>
+      <c r="M441" t="inlineStr">
+        <is>
+          <t>Supervolcano</t>
+        </is>
+      </c>
+      <c r="CI441" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="CJ441" t="inlineStr">
+        <is>
+          <t>Floods the whole track once a round</t>
+        </is>
+      </c>
+      <c r="GI441" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>Volcano Vent</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>Pressure</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D442" t="n">
+        <v>1</v>
+      </c>
+      <c r="E442">
+        <f>ROUND('Towers'!$C$24*POWER('Tuning'!$B$12,D442),0)</f>
+        <v/>
+      </c>
+      <c r="F442">
+        <f>'Towers'!$C$24+E442</f>
+        <v/>
+      </c>
+      <c r="G442" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H442" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="I442" t="n">
+        <v>1</v>
+      </c>
+      <c r="J442">
+        <f>'Towers'!$G$24*G442*H442*I442</f>
+        <v/>
+      </c>
+      <c r="K442">
+        <f>IF(J442=0,0,F442/J442)</f>
+        <v/>
+      </c>
+      <c r="L442" t="n">
+        <v>1</v>
+      </c>
+      <c r="M442" t="inlineStr">
+        <is>
+          <t>Shorter Fuse</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>Volcano Vent</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>Pressure</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D443" t="n">
+        <v>2</v>
+      </c>
+      <c r="E443">
+        <f>ROUND('Towers'!$C$24*POWER('Tuning'!$B$12,D443),0)</f>
+        <v/>
+      </c>
+      <c r="F443">
+        <f>F442+E443</f>
+        <v/>
+      </c>
+      <c r="G443" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H443" t="n">
+        <v>2</v>
+      </c>
+      <c r="I443" t="n">
+        <v>1</v>
+      </c>
+      <c r="J443">
+        <f>'Towers'!$G$24*G443*H443*I443</f>
+        <v/>
+      </c>
+      <c r="K443">
+        <f>IF(J443=0,0,F443/J443)</f>
+        <v/>
+      </c>
+      <c r="L443" t="n">
+        <v>1</v>
+      </c>
+      <c r="M443" t="inlineStr">
+        <is>
+          <t>Twin Vents</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>Volcano Vent</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>Pressure</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D444" t="n">
+        <v>3</v>
+      </c>
+      <c r="E444">
+        <f>ROUND('Towers'!$C$24*POWER('Tuning'!$B$12,D444),0)</f>
+        <v/>
+      </c>
+      <c r="F444">
+        <f>F443+E444</f>
+        <v/>
+      </c>
+      <c r="G444" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H444" t="n">
+        <v>2</v>
+      </c>
+      <c r="I444" t="n">
+        <v>1</v>
+      </c>
+      <c r="J444">
+        <f>'Towers'!$G$24*G444*H444*I444</f>
+        <v/>
+      </c>
+      <c r="K444">
+        <f>IF(J444=0,0,F444/J444)</f>
+        <v/>
+      </c>
+      <c r="L444" t="n">
+        <v>1</v>
+      </c>
+      <c r="M444" t="inlineStr">
+        <is>
+          <t>Geyser</t>
+        </is>
+      </c>
+      <c r="GD444" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>Volcano Vent</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>Pressure</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D445" t="n">
+        <v>4</v>
+      </c>
+      <c r="E445">
+        <f>ROUND('Towers'!$C$24*POWER('Tuning'!$B$12,D445),0)</f>
+        <v/>
+      </c>
+      <c r="F445">
+        <f>F444+E445</f>
+        <v/>
+      </c>
+      <c r="G445" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="H445" t="n">
+        <v>1</v>
+      </c>
+      <c r="I445" t="n">
+        <v>1</v>
+      </c>
+      <c r="J445">
+        <f>J444*G445*H445*I445</f>
+        <v/>
+      </c>
+      <c r="K445">
+        <f>IF(J445=0,0,F445/J445)</f>
+        <v/>
+      </c>
+      <c r="L445" t="n">
+        <v>1</v>
+      </c>
+      <c r="M445" t="inlineStr">
+        <is>
+          <t>Steam Burst</t>
+        </is>
+      </c>
+      <c r="W445" t="n">
+        <v>6</v>
+      </c>
+      <c r="CI445" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="CJ445" t="inlineStr">
+        <is>
+          <t>Eruptions knock small dinos back</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>Volcano Vent</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>Pressure</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D446" t="n">
+        <v>5</v>
+      </c>
+      <c r="E446">
+        <f>ROUND('Towers'!$C$24*POWER('Tuning'!$B$12,D446),0)</f>
+        <v/>
+      </c>
+      <c r="F446">
+        <f>F445+E446</f>
+        <v/>
+      </c>
+      <c r="G446" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H446" t="n">
+        <v>1</v>
+      </c>
+      <c r="I446" t="n">
+        <v>1</v>
+      </c>
+      <c r="J446">
+        <f>J445*G446*H446*I446</f>
+        <v/>
+      </c>
+      <c r="K446">
+        <f>IF(J446=0,0,F446/J446)</f>
+        <v/>
+      </c>
+      <c r="L446" t="n">
+        <v>1</v>
+      </c>
+      <c r="M446" t="inlineStr">
+        <is>
+          <t>Ring of Fire</t>
+        </is>
+      </c>
+      <c r="CI446" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="CJ446" t="inlineStr">
+        <is>
+          <t>3 small vents erupt in turn</t>
+        </is>
+      </c>
+      <c r="GE446" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>Volcano Vent</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>Obsidian</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D447" t="n">
+        <v>1</v>
+      </c>
+      <c r="E447">
+        <f>ROUND('Towers'!$C$24*POWER('Tuning'!$B$12,D447),0)</f>
+        <v/>
+      </c>
+      <c r="F447">
+        <f>'Towers'!$C$24+E447</f>
+        <v/>
+      </c>
+      <c r="G447" t="n">
+        <v>1</v>
+      </c>
+      <c r="H447" t="n">
+        <v>1</v>
+      </c>
+      <c r="I447" t="n">
+        <v>1</v>
+      </c>
+      <c r="J447">
+        <f>'Towers'!$G$24*G447*H447*I447</f>
+        <v/>
+      </c>
+      <c r="K447">
+        <f>IF(J447=0,0,F447/J447)</f>
+        <v/>
+      </c>
+      <c r="L447" t="n">
+        <v>1</v>
+      </c>
+      <c r="M447" t="inlineStr">
+        <is>
+          <t>Cooling Crust</t>
+        </is>
+      </c>
+      <c r="GJ447" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>Volcano Vent</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>Obsidian</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D448" t="n">
+        <v>2</v>
+      </c>
+      <c r="E448">
+        <f>ROUND('Towers'!$C$24*POWER('Tuning'!$B$12,D448),0)</f>
+        <v/>
+      </c>
+      <c r="F448">
+        <f>F447+E448</f>
+        <v/>
+      </c>
+      <c r="G448" t="n">
+        <v>1</v>
+      </c>
+      <c r="H448" t="n">
+        <v>1</v>
+      </c>
+      <c r="I448" t="n">
+        <v>1</v>
+      </c>
+      <c r="J448">
+        <f>'Towers'!$G$24*G448*H448*I448</f>
+        <v/>
+      </c>
+      <c r="K448">
+        <f>IF(J448=0,0,F448/J448)</f>
+        <v/>
+      </c>
+      <c r="L448" t="n">
+        <v>1</v>
+      </c>
+      <c r="M448" t="inlineStr">
+        <is>
+          <t>Sharp Glass</t>
+        </is>
+      </c>
+      <c r="AM448" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="GJ448" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>Volcano Vent</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>Obsidian</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D449" t="n">
+        <v>3</v>
+      </c>
+      <c r="E449">
+        <f>ROUND('Towers'!$C$24*POWER('Tuning'!$B$12,D449),0)</f>
+        <v/>
+      </c>
+      <c r="F449">
+        <f>F448+E449</f>
+        <v/>
+      </c>
+      <c r="G449" t="n">
+        <v>1</v>
+      </c>
+      <c r="H449" t="n">
+        <v>1</v>
+      </c>
+      <c r="I449" t="n">
+        <v>1</v>
+      </c>
+      <c r="J449">
+        <f>'Towers'!$G$24*G449*H449*I449</f>
+        <v/>
+      </c>
+      <c r="K449">
+        <f>IF(J449=0,0,F449/J449)</f>
+        <v/>
+      </c>
+      <c r="L449" t="n">
+        <v>1</v>
+      </c>
+      <c r="M449" t="inlineStr">
+        <is>
+          <t>Obsidian Wall</t>
+        </is>
+      </c>
+      <c r="AM449" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="DL449" t="n">
+        <v>2</v>
+      </c>
+      <c r="GJ449" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>Volcano Vent</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>Obsidian</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D450" t="n">
+        <v>4</v>
+      </c>
+      <c r="E450">
+        <f>ROUND('Towers'!$C$24*POWER('Tuning'!$B$12,D450),0)</f>
+        <v/>
+      </c>
+      <c r="F450">
+        <f>F449+E450</f>
+        <v/>
+      </c>
+      <c r="G450" t="n">
+        <v>1</v>
+      </c>
+      <c r="H450" t="n">
+        <v>1</v>
+      </c>
+      <c r="I450" t="n">
+        <v>1</v>
+      </c>
+      <c r="J450">
+        <f>J449*G450*H450*I450</f>
+        <v/>
+      </c>
+      <c r="K450">
+        <f>IF(J450=0,0,F450/J450)</f>
+        <v/>
+      </c>
+      <c r="L450" t="n">
+        <v>1</v>
+      </c>
+      <c r="M450" t="inlineStr">
+        <is>
+          <t>Jagged Crust</t>
+        </is>
+      </c>
+      <c r="CI450" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="CJ450" t="inlineStr">
+        <is>
+          <t>The crust cuts dinos</t>
+        </is>
+      </c>
+      <c r="GK450" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>Volcano Vent</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>Obsidian</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D451" t="n">
+        <v>5</v>
+      </c>
+      <c r="E451">
+        <f>ROUND('Towers'!$C$24*POWER('Tuning'!$B$12,D451),0)</f>
+        <v/>
+      </c>
+      <c r="F451">
+        <f>F450+E451</f>
+        <v/>
+      </c>
+      <c r="G451" t="n">
+        <v>1</v>
+      </c>
+      <c r="H451" t="n">
+        <v>1</v>
+      </c>
+      <c r="I451" t="n">
+        <v>1</v>
+      </c>
+      <c r="J451">
+        <f>J450*G451*H451*I451</f>
+        <v/>
+      </c>
+      <c r="K451">
+        <f>IF(J451=0,0,F451/J451)</f>
+        <v/>
+      </c>
+      <c r="L451" t="n">
+        <v>1</v>
+      </c>
+      <c r="M451" t="inlineStr">
+        <is>
+          <t>Glass Maze</t>
+        </is>
+      </c>
+      <c r="CI451" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="CJ451" t="inlineStr">
+        <is>
+          <t>The crust makes dinos walk 12 studs further</t>
+        </is>
+      </c>
+      <c r="GL451" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>Volcano Vent</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>Magma</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D452" t="n">
+        <v>4</v>
+      </c>
+      <c r="E452">
+        <f>E440</f>
+        <v/>
+      </c>
+      <c r="F452">
+        <f>F440</f>
+        <v/>
+      </c>
+      <c r="G452" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="H452" t="n">
+        <v>1</v>
+      </c>
+      <c r="I452" t="n">
+        <v>1</v>
+      </c>
+      <c r="L452" t="n">
+        <v>1</v>
+      </c>
+      <c r="M452" t="inlineStr">
+        <is>
+          <t>Rivers of Fire</t>
+        </is>
+      </c>
+      <c r="CI452" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="CJ452" t="inlineStr">
+        <is>
+          <t>The lava runs 20 studs further</t>
+        </is>
+      </c>
+      <c r="GB452" t="n">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>Volcano Vent</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>Magma</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D453" t="n">
+        <v>4</v>
+      </c>
+      <c r="E453">
+        <f>E440</f>
+        <v/>
+      </c>
+      <c r="F453">
+        <f>F440</f>
+        <v/>
+      </c>
+      <c r="G453" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="H453" t="n">
+        <v>1</v>
+      </c>
+      <c r="I453" t="n">
+        <v>1</v>
+      </c>
+      <c r="L453" t="n">
+        <v>1</v>
+      </c>
+      <c r="M453" t="inlineStr">
+        <is>
+          <t>Ember Rain</t>
+        </is>
+      </c>
+      <c r="CI453" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="CJ453" t="inlineStr">
+        <is>
+          <t>Embers hit low flyers</t>
+        </is>
+      </c>
+      <c r="DW453" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>Volcano Vent</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>Magma</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D454" t="n">
+        <v>5</v>
+      </c>
+      <c r="E454">
+        <f>E441</f>
+        <v/>
+      </c>
+      <c r="F454">
+        <f>F441</f>
+        <v/>
+      </c>
+      <c r="G454" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H454" t="n">
+        <v>1</v>
+      </c>
+      <c r="I454" t="n">
+        <v>1</v>
+      </c>
+      <c r="L454" t="n">
+        <v>1</v>
+      </c>
+      <c r="M454" t="inlineStr">
+        <is>
+          <t>Lava Bombs</t>
+        </is>
+      </c>
+      <c r="CI454" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="CJ454" t="inlineStr">
+        <is>
+          <t>Throws 6 lava bombs at big dinos</t>
+        </is>
+      </c>
+      <c r="GF454" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>Volcano Vent</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>Magma</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D455" t="n">
+        <v>5</v>
+      </c>
+      <c r="E455">
+        <f>E441</f>
+        <v/>
+      </c>
+      <c r="F455">
+        <f>F441</f>
+        <v/>
+      </c>
+      <c r="G455" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="H455" t="n">
+        <v>1</v>
+      </c>
+      <c r="I455" t="n">
+        <v>2</v>
+      </c>
+      <c r="L455" t="n">
+        <v>1</v>
+      </c>
+      <c r="M455" t="inlineStr">
+        <is>
+          <t>Fire Mountain</t>
+        </is>
+      </c>
+      <c r="CI455" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="CJ455" t="inlineStr">
+        <is>
+          <t>Eruptions twice as big</t>
+        </is>
+      </c>
+      <c r="GB455" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>Volcano Vent</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>Pressure</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D456" t="n">
+        <v>4</v>
+      </c>
+      <c r="E456">
+        <f>E445</f>
+        <v/>
+      </c>
+      <c r="F456">
+        <f>F445</f>
+        <v/>
+      </c>
+      <c r="G456" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="H456" t="n">
+        <v>1</v>
+      </c>
+      <c r="I456" t="n">
+        <v>1</v>
+      </c>
+      <c r="L456" t="n">
+        <v>1</v>
+      </c>
+      <c r="M456" t="inlineStr">
+        <is>
+          <t>Rumble</t>
+        </is>
+      </c>
+      <c r="AE456" t="n">
+        <v>20</v>
+      </c>
+      <c r="CI456" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="CJ456" t="inlineStr">
+        <is>
+          <t>Dinos nearby stumble: −20% speed</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>Volcano Vent</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>Pressure</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D457" t="n">
+        <v>4</v>
+      </c>
+      <c r="E457">
+        <f>E445</f>
+        <v/>
+      </c>
+      <c r="F457">
+        <f>F445</f>
+        <v/>
+      </c>
+      <c r="G457" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="H457" t="n">
+        <v>1</v>
+      </c>
+      <c r="I457" t="n">
+        <v>1</v>
+      </c>
+      <c r="L457" t="n">
+        <v>1</v>
+      </c>
+      <c r="M457" t="inlineStr">
+        <is>
+          <t>Pressure Valve</t>
+        </is>
+      </c>
+      <c r="CI457" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="CJ457" t="inlineStr">
+        <is>
+          <t>Erupts early when a boss comes</t>
+        </is>
+      </c>
+      <c r="GG457" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>Volcano Vent</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>Pressure</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D458" t="n">
+        <v>5</v>
+      </c>
+      <c r="E458">
+        <f>E446</f>
+        <v/>
+      </c>
+      <c r="F458">
+        <f>F446</f>
+        <v/>
+      </c>
+      <c r="G458" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H458" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I458" t="n">
+        <v>1</v>
+      </c>
+      <c r="L458" t="n">
+        <v>1</v>
+      </c>
+      <c r="M458" t="inlineStr">
+        <is>
+          <t>Old Faithful</t>
+        </is>
+      </c>
+      <c r="CI458" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="CJ458" t="inlineStr">
+        <is>
+          <t>Erupts 2.5× as often, smaller</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>Volcano Vent</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>Pressure</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D459" t="n">
+        <v>5</v>
+      </c>
+      <c r="E459">
+        <f>E446</f>
+        <v/>
+      </c>
+      <c r="F459">
+        <f>F446</f>
+        <v/>
+      </c>
+      <c r="G459" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="H459" t="n">
+        <v>1</v>
+      </c>
+      <c r="I459" t="n">
+        <v>1</v>
+      </c>
+      <c r="L459" t="n">
+        <v>1</v>
+      </c>
+      <c r="M459" t="inlineStr">
+        <is>
+          <t>Ash Blanket</t>
+        </is>
+      </c>
+      <c r="CI459" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="CJ459" t="inlineStr">
+        <is>
+          <t>Ash makes dinos miss 30% of throws</t>
+        </is>
+      </c>
+      <c r="GH459" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>Volcano Vent</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>Obsidian</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D460" t="n">
+        <v>4</v>
+      </c>
+      <c r="E460">
+        <f>E450</f>
+        <v/>
+      </c>
+      <c r="F460">
+        <f>F450</f>
+        <v/>
+      </c>
+      <c r="G460" t="n">
+        <v>1</v>
+      </c>
+      <c r="H460" t="n">
+        <v>1</v>
+      </c>
+      <c r="I460" t="n">
+        <v>1</v>
+      </c>
+      <c r="L460" t="n">
+        <v>1</v>
+      </c>
+      <c r="M460" t="inlineStr">
+        <is>
+          <t>Black Glass</t>
+        </is>
+      </c>
+      <c r="CI460" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="CJ460" t="inlineStr">
+        <is>
+          <t>Nearby towers see 15% further</t>
+        </is>
+      </c>
+      <c r="FA460" t="n">
+        <v>15</v>
+      </c>
+      <c r="GK460" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>Volcano Vent</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>Obsidian</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D461" t="n">
+        <v>4</v>
+      </c>
+      <c r="E461">
+        <f>E450</f>
+        <v/>
+      </c>
+      <c r="F461">
+        <f>F450</f>
+        <v/>
+      </c>
+      <c r="G461" t="n">
+        <v>1</v>
+      </c>
+      <c r="H461" t="n">
+        <v>1</v>
+      </c>
+      <c r="I461" t="n">
+        <v>1</v>
+      </c>
+      <c r="L461" t="n">
+        <v>1</v>
+      </c>
+      <c r="M461" t="inlineStr">
+        <is>
+          <t>Heat Shimmer</t>
+        </is>
+      </c>
+      <c r="CI461" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="CJ461" t="inlineStr">
+        <is>
+          <t>Dinos on the crust can't throw</t>
+        </is>
+      </c>
+      <c r="FH461" t="n">
+        <v>100</v>
+      </c>
+      <c r="GK461" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>Volcano Vent</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>Obsidian</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D462" t="n">
+        <v>5</v>
+      </c>
+      <c r="E462">
+        <f>E451</f>
+        <v/>
+      </c>
+      <c r="F462">
+        <f>F451</f>
+        <v/>
+      </c>
+      <c r="G462" t="n">
+        <v>1</v>
+      </c>
+      <c r="H462" t="n">
+        <v>1</v>
+      </c>
+      <c r="I462" t="n">
+        <v>1</v>
+      </c>
+      <c r="L462" t="n">
+        <v>1</v>
+      </c>
+      <c r="M462" t="inlineStr">
+        <is>
+          <t>Obsidian Armour</t>
+        </is>
+      </c>
+      <c r="CI462" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="CJ462" t="inlineStr">
+        <is>
+          <t>Nearby towers take 30% less from throws</t>
+        </is>
+      </c>
+      <c r="GK462" t="n">
+        <v>15</v>
+      </c>
+      <c r="GN462" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>Volcano Vent</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>Obsidian</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D463" t="n">
+        <v>5</v>
+      </c>
+      <c r="E463">
+        <f>E451</f>
+        <v/>
+      </c>
+      <c r="F463">
+        <f>F451</f>
+        <v/>
+      </c>
+      <c r="G463" t="n">
+        <v>1</v>
+      </c>
+      <c r="H463" t="n">
+        <v>1</v>
+      </c>
+      <c r="I463" t="n">
+        <v>1</v>
+      </c>
+      <c r="L463" t="n">
+        <v>1</v>
+      </c>
+      <c r="M463" t="inlineStr">
+        <is>
+          <t>Frozen Fire</t>
+        </is>
+      </c>
+      <c r="CI463" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="CJ463" t="inlineStr">
+        <is>
+          <t>The whole flow hardens: 2 s stop</t>
+        </is>
+      </c>
+      <c r="GM463" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
T139b Training finish price: 2,000 Amber per remaining minute (#403)
Tuning "Training finish Amber per min" = 2000 (was blank); Config diff is
that one row. Shared/Training.finishPrice = ceil(remaining min) x 2,000 and
nil when nothing is left (no button) or the stat is maxed. The Training panel
already shows the price via Theme.formatAmber and the server charges it
between matches.

Spec: 510 s -> 9 min, 1 s -> 1 min, 60 s -> 1 min, 61 s -> 2 min, 0 left =
no button, level 10 = 200K, a whole stat = 1.1M, K/M label, blank = not for
sale.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Storm-Split-Balance.xlsx
+++ b/Storm-Split-Balance.xlsx
@@ -14737,96 +14737,99 @@
       </c>
     </row>
     <row r="321">
-      <c r="A321" t="inlineStr">
+      <c r="A321" s="81" t="inlineStr">
         <is>
           <t>TRAINING</t>
         </is>
       </c>
     </row>
     <row r="322">
-      <c r="A322" t="inlineStr">
+      <c r="A322" s="81" t="inlineStr">
         <is>
           <t>Training levels</t>
         </is>
       </c>
-      <c r="B322" t="n">
+      <c r="B322" s="81" t="n">
         <v>10</v>
       </c>
-      <c r="C322" t="inlineStr">
+      <c r="C322" s="81" t="inlineStr">
         <is>
           <t>levels per trained stat; each level adds Trained &lt;stat&gt; max / this (#370, #397: +2 % Reach, +1.5 % Speed, +1 % Health, +3 % Throw)</t>
         </is>
       </c>
     </row>
     <row r="323">
-      <c r="A323" t="inlineStr">
+      <c r="A323" s="81" t="inlineStr">
         <is>
           <t>Train minutes</t>
         </is>
       </c>
-      <c r="B323" t="n">
+      <c r="B323" s="81" t="n">
         <v>10</v>
       </c>
-      <c r="C323" t="inlineStr">
+      <c r="C323" s="81" t="inlineStr">
         <is>
           <t>min x L: level L takes this x L minutes of full-rate training (#371: 550 min a stat)</t>
         </is>
       </c>
     </row>
     <row r="324">
-      <c r="A324" t="inlineStr">
+      <c r="A324" s="81" t="inlineStr">
         <is>
           <t>Training elsewhere rate</t>
         </is>
       </c>
-      <c r="B324" t="n">
+      <c r="B324" s="81" t="n">
         <v>0.5</v>
       </c>
-      <c r="C324" t="inlineStr">
+      <c r="C324" s="81" t="inlineStr">
         <is>
           <t>x the full rate while online but away from the stat's station (in a match, around camp); nothing offline (#391; Shared/Training)</t>
         </is>
       </c>
     </row>
     <row r="325">
-      <c r="A325" t="inlineStr">
+      <c r="A325" s="81" t="inlineStr">
         <is>
           <t>Training slots</t>
         </is>
       </c>
-      <c r="B325" t="n">
-        <v>1</v>
-      </c>
-      <c r="C325" t="inlineStr">
+      <c r="B325" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="C325" s="81" t="inlineStr">
         <is>
           <t>stats that train at once (#371; the 2nd-slot Game Pass comes with the Store, T143)</t>
         </is>
       </c>
     </row>
     <row r="326">
-      <c r="A326" t="inlineStr">
+      <c r="A326" s="81" t="inlineStr">
         <is>
           <t>Training bank (s)</t>
         </is>
       </c>
-      <c r="B326" t="n">
+      <c r="B326" s="81" t="n">
         <v>60</v>
       </c>
-      <c r="C326" t="inlineStr">
+      <c r="C326" s="81" t="inlineStr">
         <is>
           <t>s between saves of training progress (also on leave and shutdown; the idle kick loses at most this, #391)</t>
         </is>
       </c>
     </row>
     <row r="327">
-      <c r="A327" t="inlineStr">
+      <c r="A327" s="81" t="inlineStr">
         <is>
           <t>Training finish Amber per min</t>
         </is>
       </c>
-      <c r="C327" t="inlineStr">
-        <is>
-          <t>Amber per remaining minute to finish a level (#373); BLANK = not for sale until the Director sets it (Shared/Training)</t>
+      <c r="B327" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C327" s="81" t="inlineStr">
+        <is>
+          <t>Amber per remaining minute to finish a level, whole minutes rounded up (#373, #403: ~2/3 of a played minute; a whole level 10 = 200K, a stat 1.1M) (Shared/Training)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
T144: Phase-10 wording from Dino Round 23
Must-fixes: Amber skin/decoration buttons "Buy 25K Amber"; training
"Finish now — 24K Amber"; Hatchery heading "Warming eggs (1/2)"; full
hut "Your Hatchery Hut is full — hatch an egg first"; Home "100K Amber".
Nice-to-haves: training row "+6% (max +20%)"; the melee button counts
down its cooldown like the grenade; counter header and prompt "Outpost
Shop"; price label "R$49"; Hatch now rows named "Hatch now — Speckled
Egg" / "— Golden Egg" on the sheet (the card no longer appends the egg).
Honker's line left as is: #407 honks at the nearest boss, else the dino
with the most HP, so "a boss dino" would not be true.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Storm-Split-Balance.xlsx
+++ b/Storm-Split-Balance.xlsx
@@ -17536,7 +17536,7 @@
       </c>
       <c r="D11" s="81" t="inlineStr">
         <is>
-          <t>Hatch now</t>
+          <t>Hatch now — Speckled Egg</t>
         </is>
       </c>
       <c r="E11" s="81" t="n">
@@ -17581,7 +17581,7 @@
       </c>
       <c r="D12" s="81" t="inlineStr">
         <is>
-          <t>Hatch now</t>
+          <t>Hatch now — Golden Egg</t>
         </is>
       </c>
       <c r="E12" s="81" t="n">

</xml_diff>